<commit_message>
RAC entra na atualização automática (seg-sex 12h, junto com Emergências)
Adiciona atualizar_do_drive() em extrair_rac.py, inclui rac em
executar_atualizacao.py e no workflow do GitHub Actions (mesmo horário de
Emergências). Também atualiza a documentação de atualizações e o CLAUDE.md
raiz para refletir a migração de launchd (Mac) para GitHub Actions (nuvem).
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -492,12 +492,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -511,21 +511,21 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -535,20 +535,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Dentro do contrato</t>
+          <t>Fora do contrato</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -567,16 +567,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="F5" t="n">
-        <v>25</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -595,21 +595,21 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="F6" t="n">
-        <v>87</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -623,49 +623,49 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="F7" t="n">
-        <v>136</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2702</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>EPCAR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Desmontada</t>
+          <t>Montada</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fora do contrato</t>
+          <t>Dentro do contrato</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2702</t>
+          <t>2703</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EPCAR</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -688,12 +688,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2703</t>
+          <t>2704</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>PAMALS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -716,12 +716,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2704</t>
+          <t>2708</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PAMALS</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -744,12 +744,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2708</t>
+          <t>2709</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>6º ETA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -772,12 +772,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2709</t>
+          <t>2719</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>2ª ETA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -800,12 +800,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2719</t>
+          <t>2720</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2ª ETA</t>
+          <t>6º ETA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -828,12 +828,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2720</t>
+          <t>2722</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>2ª ETA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -856,12 +856,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2722</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2ª ETA</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1495,22 +1495,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3122678-04</t>
+          <t>P7036368-01</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FUEL CONTROL UNIT</t>
+          <t>PROPELLER ASSEMBLY</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1520,12 +1520,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1545,7 +1545,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1595,12 +1595,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1620,22 +1620,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>P7036368-01</t>
+          <t>2643007-1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PROPELLER ASSEMBLY</t>
+          <t>SHIMMY DAMP AS</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1645,12 +1645,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1670,7 +1670,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1720,22 +1720,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2643007-1</t>
+          <t>C611505-0201</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SHIMMY DAMP AS</t>
+          <t>ALTERNATOR</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1745,12 +1745,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1770,7 +1770,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1795,7 +1795,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1820,22 +1820,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C611505-0201</t>
+          <t>2651022-20-1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ALTERNATOR</t>
+          <t>RING ASSY ENGI</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1845,12 +1845,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1870,12 +1870,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1895,22 +1895,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2651022-20-1</t>
+          <t>2643100-206</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RING ASSY ENGI</t>
+          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2643100-206</t>
+          <t>162-10700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+          <t>OUTER WHEEL HALF ASSY</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>162-10700</t>
+          <t>D20B-14489-KA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>OUTER WHEEL HALF ASSY</t>
+          <t>SLEEVE</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1980,12 +1980,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>D20B-14489-KA</t>
+          <t>400454</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SLEEVE</t>
+          <t>SEAL,PLAIN ENCASED</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2005,27 +2005,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>400454</t>
+          <t>AE3663163K0600</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SEAL,PLAIN ENCASED</t>
+          <t>HOSE ASSY</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2039,13 +2039,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2064,18 +2064,18 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2095,22 +2095,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AE3663163K0600</t>
+          <t>2641013-6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>HOSE ASSY</t>
+          <t>SPRING-MAIN GEAR LH &amp; RH</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2120,12 +2120,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2145,12 +2145,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2164,32 +2164,32 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2641013-6</t>
+          <t>154-03000</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR LH &amp; RH</t>
+          <t>SEAL MOLDED</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -2205,27 +2205,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>154-03000</t>
+          <t>M81934/2-32C032</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SEAL MOLDED</t>
+          <t>BEARING,SLEEVE</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2245,22 +2245,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>M81934/2-32C032</t>
+          <t>2611137-7</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BEARING,SLEEVE</t>
+          <t>CAP MAIN LAND</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2280,16 +2280,16 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2611137-7</t>
+          <t>2621013-2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CAP MAIN LAND</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Atualização automática: rac (07/07/2026 21:07)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1316,27 +1304,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (08/07/2026 14:33)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,32 +430,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -508,12 +520,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -527,21 +539,21 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -551,25 +563,25 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fora do contrato</t>
+          <t>Dentro do contrato</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -579,20 +591,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fora do contrato</t>
+          <t>Dentro do contrato</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>87</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -611,21 +623,21 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>136</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -639,77 +651,77 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="F8" t="n">
-        <v>230</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2702</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EPCAR</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Montada</t>
+          <t>Desmontada</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dentro do contrato</t>
+          <t>Fora do contrato</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2703</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Montada</t>
+          <t>Desmontada</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Dentro do contrato</t>
+          <t>Fora do contrato</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2704</t>
+          <t>2702</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PAMALS</t>
+          <t>EPCAR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -732,7 +744,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2708</t>
+          <t>2703</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -760,12 +772,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2719</t>
+          <t>2704</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2ª ETA</t>
+          <t>PAMALS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -788,12 +800,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2720</t>
+          <t>2708</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -816,7 +828,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2722</t>
+          <t>2719</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -844,12 +856,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2720</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>6º ETA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -872,12 +884,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2727</t>
+          <t>2722</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1/15 GAV</t>
+          <t>2ª ETA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -900,12 +912,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2729</t>
+          <t>2727</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1/15 GAV</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -928,12 +940,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2731</t>
+          <t>2729</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1ª ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -956,12 +968,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2733</t>
+          <t>2731</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1ª ETA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1300,31 +1312,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E210"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>
@@ -1393,12 +1405,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3044000</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ENGINE PT6A-114A</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1408,22 +1420,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3044000</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ENGINE PT6A-114A</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1433,12 +1445,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2721</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>6º ETA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1458,12 +1470,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1483,12 +1495,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1508,22 +1520,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2721</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>066-3046-07</t>
+          <t>3044000</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CONTROL,INDICATOR</t>
+          <t>ENGINE PT6A-114A</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1533,22 +1545,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>P7036368-01</t>
+          <t>3044000</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PROPELLER ASSEMBLY</t>
+          <t>ENGINE PT6A-114A</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1558,12 +1570,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1583,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1608,7 +1620,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1633,12 +1645,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1658,22 +1670,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2643007-1</t>
+          <t>P7036368-01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SHIMMY DAMP AS</t>
+          <t>PROPELLER ASSEMBLY</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1683,12 +1695,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1708,7 +1720,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1733,7 +1745,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1758,22 +1770,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>C611505-0201</t>
+          <t>2643007-1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ALTERNATOR</t>
+          <t>SHIMMY DAMP AS</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1783,12 +1795,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1808,7 +1820,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1833,7 +1845,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1858,22 +1870,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2651022-20-1</t>
+          <t>C611505-0201</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RING ASSY ENGI</t>
+          <t>ALTERNATOR</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1883,12 +1895,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1908,12 +1920,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1933,22 +1945,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2641011-5</t>
+          <t>2651022-20-1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AXLE-MAIN GEAR</t>
+          <t>RING ASSY ENGI</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1958,12 +1970,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1977,32 +1989,32 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2643100-206</t>
+          <t>2641011-5</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+          <t>AXLE-MAIN GEAR</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -2018,12 +2030,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>162-10700</t>
+          <t>2643100-206</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OUTER WHEEL HALF ASSY</t>
+          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2043,12 +2055,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>D20B-14489-KA</t>
+          <t>162-10700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SLEEVE</t>
+          <t>OUTER WHEEL HALF ASSY</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2068,12 +2080,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>400454</t>
+          <t>D20B-14489-KA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SEAL,PLAIN ENCASED</t>
+          <t>SLEEVE</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2093,27 +2105,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AE3663163K0600</t>
+          <t>400454</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>HOSE ASSY</t>
+          <t>SEAL,PLAIN ENCASED</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2127,13 +2139,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2152,18 +2164,18 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2183,22 +2195,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2641013-6</t>
+          <t>AE3663163K0600</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR LH &amp; RH</t>
+          <t>HOSE ASSY</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2208,12 +2220,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2233,12 +2245,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2252,43 +2264,43 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2611112-2</t>
+          <t>2641013-6</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>STRAP</t>
+          <t>SPRING-MAIN GEAR LH &amp; RH</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2302,18 +2314,18 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2327,28 +2339,28 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2601119-1</t>
+          <t>2611112-2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>JACK PAD LH</t>
+          <t>STRAP</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2358,12 +2370,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2377,32 +2389,32 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>154-03000</t>
+          <t>2601119-1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SEAL MOLDED</t>
+          <t>JACK PAD LH</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2418,12 +2430,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2621013-2</t>
+          <t>154-03000</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>SEAL MOLDED</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2443,27 +2455,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>M81934/2-32C032</t>
+          <t>2621013-2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>BEARING,SLEEVE</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2483,22 +2495,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2611137-7</t>
+          <t>M81934/2-32C032</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CAP MAIN LAND</t>
+          <t>BEARING,SLEEVE</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2508,47 +2520,47 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>2611137-7</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>CAP MAIN LAND</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>3122678-04</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2558,7 +2570,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2583,12 +2595,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2608,7 +2620,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2618,12 +2630,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2600100-7</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>LINE ASSY-PROP</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2633,22 +2645,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2600100-7</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>LINE ASSY-PROP</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -2658,7 +2670,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2683,7 +2695,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2693,12 +2705,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2698010-7</t>
+          <t>2600100-7</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PASSENGER DOOR - LOW</t>
+          <t>LINE ASSY-PROP</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2718,12 +2730,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2698010-7</t>
+          <t>2600100-7</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>PASSENGER DOOR - LOW</t>
+          <t>LINE ASSY-PROP</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2743,12 +2755,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>2698010-7</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>PASSENGER DOOR - LOW</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2768,12 +2780,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>2698010-7</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>PASSENGER DOOR - LOW</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2793,12 +2805,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2818,12 +2830,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2843,12 +2855,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2868,12 +2880,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2893,22 +2905,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2918,22 +2930,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2958,12 +2970,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2983,7 +2995,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2993,12 +3005,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2115040-8</t>
+          <t>030-18200</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CYLINDER GAS S</t>
+          <t>MAIN WHEEL BRAKE</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3008,22 +3020,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2115040-8</t>
+          <t>030-18200</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>CYLINDER GAS S</t>
+          <t>MAIN WHEEL BRAKE</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -3033,7 +3045,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3058,7 +3070,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3068,12 +3080,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>S1053K16T</t>
+          <t>2115040-8</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>CYLINDER GAS S</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -3083,7 +3095,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3093,12 +3105,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>S1053K16T</t>
+          <t>2115040-8</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>CYLINDER GAS S</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -3108,7 +3120,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3127,18 +3139,18 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3152,13 +3164,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3168,47 +3180,47 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>42854-11</t>
+          <t>S1053K16T</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>FITTING A S TR</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>799-1</t>
+          <t>S1053K16T</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>TRANSDUCER</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3218,27 +3230,27 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>799-1</t>
+          <t>42854-11</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>TRANSDUCER</t>
+          <t>FITTING A S TR</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3258,7 +3270,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3268,12 +3280,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>S1053K24T</t>
+          <t>799-1</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>TRANSDUCER</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -3283,22 +3295,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>S1053K24T</t>
+          <t>799-1</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>TRANSDUCER</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3308,12 +3320,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3327,13 +3339,13 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3343,12 +3355,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>C352TS</t>
+          <t>S1053K24T</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>EXTINGUISHER,FIRE</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -3358,26 +3370,26 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>C352TS</t>
+          <t>S1053K24T</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>EXTINGUISHER,FIRE</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -3393,12 +3405,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AN929-4W</t>
+          <t>C352TS</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>CAP,TUBE</t>
+          <t>EXTINGUISHER,FIRE</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -3418,12 +3430,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AN929-4W</t>
+          <t>C352TS</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>CAP,TUBE</t>
+          <t>EXTINGUISHER,FIRE</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3443,12 +3455,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2601266-2</t>
+          <t>AN929-4W</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>COUPLING-SPLINED</t>
+          <t>CAP,TUBE</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -3458,22 +3470,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2601266-2</t>
+          <t>AN929-4W</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>COUPLING-SPLINED</t>
+          <t>CAP,TUBE</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -3493,12 +3505,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>30994-001</t>
+          <t>2601266-2</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>BATTERY-MARATHON TSP410 NICAD</t>
+          <t>COUPLING-SPLINED</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -3518,12 +3530,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>30994-001</t>
+          <t>2601266-2</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>BATTERY-MARATHON TSP410 NICAD</t>
+          <t>COUPLING-SPLINED</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3543,12 +3555,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2641018-25</t>
+          <t>30994-001</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>FAIRING ASSY LH</t>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3558,22 +3570,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2641018-26</t>
+          <t>30994-001</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>FAIRING ASSY RH</t>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -3593,12 +3605,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>S2814-2</t>
+          <t>2641018-25</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CABLE ASSY-DOOR PULL</t>
+          <t>FAIRING ASSY LH</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -3618,12 +3630,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>S2574-1</t>
+          <t>2641018-26</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>NUT-DIODE ATTACH</t>
+          <t>FAIRING ASSY RH</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3643,12 +3655,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2601393-1</t>
+          <t>S2814-2</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SUPORT PLATE</t>
+          <t>CABLE ASSY-DOOR PULL</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -3668,12 +3680,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2601188-9</t>
+          <t>S2574-1</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>COMPRESSOR DRIVE ASS</t>
+          <t>NUT-DIODE ATTACH</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -3693,12 +3705,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2601392-1</t>
+          <t>2601393-1</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>ADJUSTER PLATE</t>
+          <t>SUPORT PLATE</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -3718,12 +3730,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2622236-6</t>
+          <t>2601188-9</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>COVER ACCESS RH</t>
+          <t>COMPRESSOR DRIVE ASS</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -3743,22 +3755,22 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>S2837-1</t>
+          <t>2601392-1</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>CABLE ASSY-PASSENGER</t>
+          <t>ADJUSTER PLATE</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3768,27 +3780,27 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>S2837-1</t>
+          <t>2622236-6</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>CABLE ASSY-PASSENGER</t>
+          <t>COVER ACCESS RH</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3808,7 +3820,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3818,12 +3830,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>S51-14</t>
+          <t>S2837-1</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+          <t>CABLE ASSY-PASSENGER</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -3833,22 +3845,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>S51-14</t>
+          <t>S2837-1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+          <t>CABLE ASSY-PASSENGER</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -3868,12 +3880,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>1134380-5</t>
+          <t>S51-14</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -3883,7 +3895,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3893,12 +3905,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>1H101-4</t>
+          <t>S51-14</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>FLOW CONTROL VALVE</t>
+          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -3918,12 +3930,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>5950017-11</t>
+          <t>1134380-5</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>REDUCER ASSEMBY</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -3943,12 +3955,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>040-0043</t>
+          <t>1H101-4</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>STROB TUB</t>
+          <t>FLOW CONTROL VALVE</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -3968,16 +3980,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>DLS4-02303</t>
+          <t>5950017-11</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>IMOBILIZADOR</t>
+          <t>REDUCER ASSEMBY</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -3993,16 +4005,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>DLS4-01786</t>
+          <t>040-0043</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>BLOQUEIO DA VENTILAÇ</t>
+          <t>STROB TUB</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -4018,22 +4030,22 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>A1635-133</t>
+          <t>DLS4-02303</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>SCREW</t>
+          <t>IMOBILIZADOR</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4043,22 +4055,22 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>A1635-133</t>
+          <t>DLS4-01786</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>SCREW</t>
+          <t>BLOQUEIO DA VENTILAÇ</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -4068,41 +4080,41 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2641014-5</t>
+          <t>A1635-133</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR CEN</t>
+          <t>SCREW</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2641014-5</t>
+          <t>A1635-133</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR CEN</t>
+          <t>SCREW</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113">
@@ -4118,12 +4130,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>205842-1</t>
+          <t>2641014-5</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>CONNECTOR</t>
+          <t>SPRING-MAIN GEAR CEN</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -4133,22 +4145,22 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>AN804D4</t>
+          <t>2641014-5</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>TEE,TUBE</t>
+          <t>SPRING-MAIN GEAR CEN</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4168,12 +4180,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>453-5060</t>
+          <t>205842-1</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>BEACON,DISTRESS</t>
+          <t>CONNECTOR</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4193,12 +4205,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>S3465-2-0132</t>
+          <t>AN804D4</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAKE CYL</t>
+          <t>TEE,TUBE</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4218,12 +4230,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>S3465-2-0146</t>
+          <t>453-5060</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAK</t>
+          <t>BEACON,DISTRESS</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4243,12 +4255,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>200276-2</t>
+          <t>S3465-2-0132</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>CONNECTOR BODY,RECEP</t>
+          <t>HOSE ASSY BRAKE CYL</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -4268,12 +4280,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>51539-012N</t>
+          <t>S3465-2-0146</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>CONTROL UNIT,GENERA</t>
+          <t>HOSE ASSY BRAK</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -4293,12 +4305,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>M83248/1-904</t>
+          <t>200276-2</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ANEL-O</t>
+          <t>CONNECTOR BODY,RECEP</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4318,12 +4330,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2643065-2</t>
+          <t>51539-012N</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>BUNGEE ASSY</t>
+          <t>CONTROL UNIT,GENERA</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -4343,12 +4355,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>723908</t>
+          <t>M83248/1-904</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>ANEL-O</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -4368,12 +4380,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2601271-18</t>
+          <t>2643065-2</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DRIVE PULLEY</t>
+          <t>BUNGEE ASSY</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4393,12 +4405,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>1134380-4</t>
+          <t>723908</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4418,12 +4430,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2652016-21</t>
+          <t>2601271-18</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>DOOR ASSY COWL LH</t>
+          <t>DRIVE PULLEY</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4443,12 +4455,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>S1053K22T144.00</t>
+          <t>1134380-4</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4468,12 +4480,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>S1915-3</t>
+          <t>2652016-21</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>CAPACITOR-6.0 MF 150</t>
+          <t>DOOR ASSY COWL LH</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4493,12 +4505,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2619020-37</t>
+          <t>S1053K22T144.00</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>SEAT ASSEMBLY - BENCH</t>
+          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4518,12 +4530,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>011-00870-00</t>
+          <t>S1915-3</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>MAGNETOMETER GMU 44</t>
+          <t>CAPACITOR-6.0 MF 150</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4543,12 +4555,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>011-00877-00</t>
+          <t>2619020-37</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>GSA-80 TORQUE SERVO</t>
+          <t>SEAT ASSEMBLY - BENCH</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4568,12 +4580,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>011-00878-10</t>
+          <t>011-00870-00</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>GSA-81 TORQUE SERVO</t>
+          <t>MAGNETOMETER GMU 44</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -4593,12 +4605,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>011-01020-10</t>
+          <t>011-00877-00</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>AFCS MODE CONTROLLER</t>
+          <t>GSA-80 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4618,12 +4630,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SL6015-4</t>
+          <t>011-00878-10</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>CLIP</t>
+          <t>GSA-81 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4643,12 +4655,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>EA5175-29PTL-CES</t>
+          <t>011-01020-10</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>AIRSPEED INDICATOR</t>
+          <t>AFCS MODE CONTROLLER</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -4668,12 +4680,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2650032-4</t>
+          <t>SL6015-4</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>CLIP</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4693,12 +4705,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>011-01105-01</t>
+          <t>EA5175-29PTL-CES</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>INTEGRATED AVIONICS</t>
+          <t>AIRSPEED INDICATOR</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -4718,12 +4730,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>2650032-4</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -4743,16 +4755,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2654013-4</t>
+          <t>011-01105-01</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>INTEGRATED AVIONICS</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -4768,16 +4780,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2115040-206</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>GAS SPRING</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -4793,12 +4805,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>5211369-8</t>
+          <t>2654013-4</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>EXTENDER-CREW, (WHEN</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -4818,12 +4830,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>MS16674-5021</t>
+          <t>2115040-206</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>RETAINING RING</t>
+          <t>GAS SPRING</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -4843,12 +4855,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>302-120-302</t>
+          <t>5211369-8</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>TUBE MAIN 850X10</t>
+          <t>EXTENDER-CREW, (WHEN</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -4868,12 +4880,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>1570301-1</t>
+          <t>MS16674-5021</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>DIMMING ASSY,SPEC</t>
+          <t>RETAINING RING</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -4893,16 +4905,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>71014</t>
+          <t>302-120-302</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>TUBE MAIN 850X10</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -4918,16 +4930,16 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>NAS1149F0363P</t>
+          <t>1570301-1</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>WASHER, FLAT</t>
+          <t>DIMMING ASSY,SPEC</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146">
@@ -4943,16 +4955,16 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>AN3-5A</t>
+          <t>71014</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>BOLT,MACHINE</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147">
@@ -4968,66 +4980,66 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>DD2W</t>
+          <t>NAS1149F0363P</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>STATIC WICK</t>
+          <t>WASHER, FLAT</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2641012-14</t>
+          <t>AN3-5A</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY-RH-MAI</t>
+          <t>BOLT,MACHINE</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>5950028-10</t>
+          <t>DD2W</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>VANT,BREATHER</t>
+          <t>STATIC WICK</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150">
@@ -5043,12 +5055,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>S2889-3-0112</t>
+          <t>2641012-14</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>HOSE ASSY TEE</t>
+          <t>TRUNNION ASSY-RH-MAI</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -5068,12 +5080,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1J18-10</t>
+          <t>5950028-10</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>FUEL FILTER ASSY</t>
+          <t>VANT,BREATHER</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -5093,12 +5105,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>C668050-1103</t>
+          <t>S2889-3-0112</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>TRANSMITER FUEL</t>
+          <t>HOSE ASSY TEE</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -5118,12 +5130,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2651023-23</t>
+          <t>1J18-10</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT ASSEMBL</t>
+          <t>FUEL FILTER ASSY</t>
         </is>
       </c>
       <c r="E153" t="n">
@@ -5143,12 +5155,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>S133-6P58</t>
+          <t>C668050-1103</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>TRANSMITER FUEL</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -5168,12 +5180,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>9910338-6</t>
+          <t>2651023-23</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>TRANSMITTER,RATE OF FLOW</t>
+          <t>ENGINE MOUNT ASSEMBL</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -5193,12 +5205,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>162-11800</t>
+          <t>S133-6P58</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-OUTER</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -5218,12 +5230,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>244-18922</t>
+          <t>9910338-6</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>CABLE FIRE DET</t>
+          <t>TRANSMITTER,RATE OF FLOW</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -5243,12 +5255,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2632020-14</t>
+          <t>162-11800</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>HINGE BKT INBD</t>
+          <t>WHEEL HALF ASSY-OUTER</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -5268,12 +5280,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>9919105-1</t>
+          <t>244-18922</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>RESTRAINT ASSY</t>
+          <t>CABLE FIRE DET</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -5293,12 +5305,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2643055-5</t>
+          <t>2632020-14</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>SUPPORT ASSY AFT NOSE GEAR</t>
+          <t>HINGE BKT INBD</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -5318,12 +5330,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2641030-2</t>
+          <t>9919105-1</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>COVER</t>
+          <t>RESTRAINT ASSY</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -5343,12 +5355,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2613439-1</t>
+          <t>2643055-5</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>SHIELD</t>
+          <t>SUPPORT ASSY AFT NOSE GEAR</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -5368,12 +5380,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2682004-1</t>
+          <t>2641030-2</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>RESERVOIR ASSY-BRAKE</t>
+          <t>COVER</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -5393,12 +5405,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2621000-24</t>
+          <t>2613439-1</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>STRUT ASSY-RH WING</t>
+          <t>SHIELD</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -5418,12 +5430,12 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2662018-5</t>
+          <t>2682004-1</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>TUBE ASSY-LONG</t>
+          <t>RESERVOIR ASSY-BRAKE</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -5443,12 +5455,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2661215-6</t>
+          <t>2621000-24</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>SCREW INTERNAL</t>
+          <t>STRUT ASSY-RH WING</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -5468,12 +5480,12 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2622185-22</t>
+          <t>2662018-5</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>RIB ASSY-RH-AILERON</t>
+          <t>TUBE ASSY-LONG</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -5493,12 +5505,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>AN6289D3</t>
+          <t>2661215-6</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>LOCKNUT,TUBE F</t>
+          <t>SCREW INTERNAL</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -5518,12 +5530,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2643057-1</t>
+          <t>2622185-22</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>BOOT N G STEER</t>
+          <t>RIB ASSY-RH-AILERON</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -5543,12 +5555,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>S2889-3-0160</t>
+          <t>AN6289D3</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>HOSE ASSY ELBOW</t>
+          <t>LOCKNUT,TUBE F</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -5568,12 +5580,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2617015-18</t>
+          <t>2643057-1</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>HINGE DOOR LH</t>
+          <t>BOOT N G STEER</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -5593,12 +5605,12 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2615018-1</t>
+          <t>S2889-3-0160</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>MOLDING-WINDOW</t>
+          <t>HOSE ASSY ELBOW</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -5618,12 +5630,12 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2615035-5</t>
+          <t>2617015-18</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-LH CREW</t>
+          <t>HINGE DOOR LH</t>
         </is>
       </c>
       <c r="E173" t="n">
@@ -5643,12 +5655,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2615035-6</t>
+          <t>2615018-1</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-RH CREW</t>
+          <t>MOLDING-WINDOW</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -5668,12 +5680,12 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>AT-RL1019</t>
+          <t>2615035-5</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>PLATE - COVER</t>
+          <t>SCUFF PLATE-LH CREW</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -5693,12 +5705,12 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2615011-2</t>
+          <t>2615035-6</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>WINDOW MOLDING</t>
+          <t>SCUFF PLATE-RH CREW</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -5718,12 +5730,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2641012-13</t>
+          <t>AT-RL1019</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY</t>
+          <t>PLATE - COVER</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -5743,12 +5755,12 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2650113-5</t>
+          <t>2615011-2</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>WINDOW MOLDING</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -5768,12 +5780,12 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2601072-14</t>
+          <t>2641012-13</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>BRACKET ASSY-95 AMP</t>
+          <t>TRUNNION ASSY</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -5793,12 +5805,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>C622010-0102</t>
+          <t>2650113-5</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>LIGHT STROBE RH</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -5818,16 +5830,16 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>C662041-0102</t>
+          <t>2601072-14</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>INDICATOR FUEL</t>
+          <t>BRACKET ASSY-95 AMP</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -5843,16 +5855,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2617015-22</t>
+          <t>C622010-0102</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>HINGE-DOOR LH</t>
+          <t>LIGHT STROBE RH</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -5868,12 +5880,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2621011-3</t>
+          <t>C662041-0102</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>WASHER</t>
+          <t>INDICATOR FUEL</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -5893,12 +5905,12 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2621008-202</t>
+          <t>2617015-22</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT U</t>
+          <t>HINGE-DOOR LH</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -5918,12 +5930,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2552-070</t>
+          <t>2621011-3</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>NUT,SELF-LOCKI</t>
+          <t>WASHER</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -5943,12 +5955,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>C262023-0107</t>
+          <t>2621008-202</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>TUBE 850X10</t>
+          <t>FITTING-WING STRUT U</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -5968,12 +5980,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2661215-1</t>
+          <t>2552-070</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>ACTUATOR ASSY-ELEVAT</t>
+          <t>NUT,SELF-LOCKI</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -5993,12 +6005,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2622184-3</t>
+          <t>C262023-0107</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>PUSH ROD ASSY</t>
+          <t>TUBE 850X10</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -6018,12 +6030,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>NAS464P12-37</t>
+          <t>2661215-1</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>BOLT,SHEAR</t>
+          <t>ACTUATOR ASSY-ELEVAT</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -6043,12 +6055,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>NAS464P14-76</t>
+          <t>2622184-3</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>BOLT,SHEAR</t>
+          <t>PUSH ROD ASSY</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -6068,12 +6080,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>MS24462-5</t>
+          <t>NAS464P12-37</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>BEARING ROLLER</t>
+          <t>BOLT,SHEAR</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -6093,12 +6105,12 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>161-12800</t>
+          <t>NAS464P14-76</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-INNE</t>
+          <t>BOLT,SHEAR</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -6118,16 +6130,16 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2614076-63</t>
+          <t>MS24462-5</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>PASSENGER SEAT UPHOL</t>
+          <t>BEARING ROLLER</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194">
@@ -6143,16 +6155,16 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>C299501-0402</t>
+          <t>161-12800</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>WHEEL HALF ASSY-INNE</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195">
@@ -6168,16 +6180,16 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>214-01400</t>
+          <t>2614076-63</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>CONE AND ROLLERS,TAP</t>
+          <t>PASSENGER SEAT UPHOL</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="196">
@@ -6193,16 +6205,16 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2621009-2</t>
+          <t>C299501-0402</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT L</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="197">
@@ -6218,12 +6230,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>NAS1336C5C19K</t>
+          <t>214-01400</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>PIN-LOCWELL SINGLE A</t>
+          <t>CONE AND ROLLERS,TAP</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -6243,12 +6255,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2614021-13</t>
+          <t>2621009-2</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>FITTING-WING STRUT L</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -6268,12 +6280,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2616031-1</t>
+          <t>NAS1336C5C19K</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>VALVE</t>
+          <t>PIN-LOCWELL SINGLE A</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -6293,16 +6305,16 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>6361620-11</t>
+          <t>2614021-13</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SPROCKET</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="201">
@@ -6318,16 +6330,16 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2601347-1</t>
+          <t>2616031-1</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>BRACKET CARGO PAD</t>
+          <t>VALVE</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="202">
@@ -6343,16 +6355,16 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>9910333-1</t>
+          <t>6361620-11</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT</t>
+          <t>SPROCKET</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="203">
@@ -6368,16 +6380,16 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>S2357-3</t>
+          <t>2601347-1</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>CLAMP, LOOP</t>
+          <t>BRACKET CARGO PAD</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="204">
@@ -6393,16 +6405,16 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>R221485</t>
+          <t>9910333-1</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>MANGUEIRA</t>
+          <t>ENGINE MOUNT</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205">
@@ -6418,16 +6430,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>R221487</t>
+          <t>S2357-3</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>MANGUEIRA</t>
+          <t>CLAMP, LOOP</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="206">
@@ -6443,16 +6455,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>S3354-1</t>
+          <t>R221485</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>MANGUEIRA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="207">
@@ -6468,16 +6480,16 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>657735</t>
+          <t>R221487</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>CLIP, LOCKING</t>
+          <t>MANGUEIRA</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="208">
@@ -6493,16 +6505,16 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>MS27641-6G</t>
+          <t>S3354-1</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>BEARING</t>
+          <t>BOLT</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="209">
@@ -6518,16 +6530,16 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23541</t>
+          <t>657735</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>BUSHING,CABLE CLAMP</t>
+          <t>CLIP, LOCKING</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="210">
@@ -6543,15 +6555,65 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
+          <t>MS27641-6G</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>BEARING</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>23541</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>BUSHING,CABLE CLAMP</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2726</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1º ETA</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
           <t>2670067-1</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr">
+      <c r="D212" t="inlineStr">
         <is>
           <t>POST LIGHT ASS</t>
         </is>
       </c>
-      <c r="E210" t="n">
+      <c r="E212" t="n">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (09/07/2026 15:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -539,10 +539,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -623,10 +623,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -707,10 +707,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F10" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
@@ -1312,7 +1312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2545,12 +2545,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2733</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2570,22 +2570,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>3122678-04</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2595,7 +2595,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2620,7 +2620,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2645,12 +2645,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2670,22 +2670,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2600100-7</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>LINE ASSY-PROP</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2695,7 +2695,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2720,7 +2720,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2745,7 +2745,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2698010-7</t>
+          <t>2600100-7</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PASSENGER DOOR - LOW</t>
+          <t>LINE ASSY-PROP</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2770,7 +2770,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2795,7 +2795,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2805,12 +2805,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>2698010-7</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>PASSENGER DOOR - LOW</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2845,7 +2845,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2880,12 +2880,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2905,22 +2905,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>030-18200</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>MAIN WHEEL BRAKE</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2930,22 +2930,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>030-18200</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>MAIN WHEEL BRAKE</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2970,12 +2970,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2995,7 +2995,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>2115040-8</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>CYLINDER GAS S</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3020,22 +3020,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>2115040-8</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>CYLINDER GAS S</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -3045,7 +3045,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3070,7 +3070,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3080,12 +3080,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2115040-8</t>
+          <t>S1053K16T</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>CYLINDER GAS S</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -3095,7 +3095,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3105,12 +3105,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2115040-8</t>
+          <t>S1053K16T</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>CYLINDER GAS S</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -3120,7 +3120,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3139,18 +3139,18 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3164,13 +3164,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3180,47 +3180,47 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>S1053K16T</t>
+          <t>42854-11</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>FITTING A S TR</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>S1053K16T</t>
+          <t>799-1</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>TRANSDUCER</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3230,27 +3230,27 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>42854-11</t>
+          <t>799-1</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>FITTING A S TR</t>
+          <t>TRANSDUCER</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3270,7 +3270,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3280,12 +3280,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>799-1</t>
+          <t>S1053K24T</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>TRANSDUCER</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -3295,22 +3295,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>799-1</t>
+          <t>S1053K24T</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TRANSDUCER</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3320,12 +3320,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3339,13 +3339,13 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>S1053K24T</t>
+          <t>C352TS</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>EXTINGUISHER,FIRE</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -3370,26 +3370,26 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>S1053K24T</t>
+          <t>C352TS</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>EXTINGUISHER,FIRE</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -3405,12 +3405,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>C352TS</t>
+          <t>AN929-4W</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>EXTINGUISHER,FIRE</t>
+          <t>CAP,TUBE</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -3430,12 +3430,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>C352TS</t>
+          <t>AN929-4W</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>EXTINGUISHER,FIRE</t>
+          <t>CAP,TUBE</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3455,12 +3455,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>AN929-4W</t>
+          <t>2601266-2</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>CAP,TUBE</t>
+          <t>COUPLING-SPLINED</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -3470,22 +3470,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AN929-4W</t>
+          <t>2601266-2</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>CAP,TUBE</t>
+          <t>COUPLING-SPLINED</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -3505,12 +3505,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2601266-2</t>
+          <t>30994-001</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>COUPLING-SPLINED</t>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -3530,12 +3530,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2601266-2</t>
+          <t>30994-001</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>COUPLING-SPLINED</t>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3555,12 +3555,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>30994-001</t>
+          <t>2641018-25</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>BATTERY-MARATHON TSP410 NICAD</t>
+          <t>FAIRING ASSY LH</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3570,22 +3570,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>30994-001</t>
+          <t>2641018-26</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>BATTERY-MARATHON TSP410 NICAD</t>
+          <t>FAIRING ASSY RH</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -3605,12 +3605,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2641018-25</t>
+          <t>S2814-2</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>FAIRING ASSY LH</t>
+          <t>CABLE ASSY-DOOR PULL</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -3630,12 +3630,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2641018-26</t>
+          <t>S2574-1</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>FAIRING ASSY RH</t>
+          <t>NUT-DIODE ATTACH</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3655,12 +3655,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>S2814-2</t>
+          <t>2601393-1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>CABLE ASSY-DOOR PULL</t>
+          <t>SUPORT PLATE</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -3680,12 +3680,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>S2574-1</t>
+          <t>2601188-9</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>NUT-DIODE ATTACH</t>
+          <t>COMPRESSOR DRIVE ASS</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -3705,12 +3705,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2601393-1</t>
+          <t>2601392-1</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>SUPORT PLATE</t>
+          <t>ADJUSTER PLATE</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -3730,12 +3730,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2601188-9</t>
+          <t>2622236-6</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>COMPRESSOR DRIVE ASS</t>
+          <t>COVER ACCESS RH</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -3755,22 +3755,22 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2601392-1</t>
+          <t>S2837-1</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>ADJUSTER PLATE</t>
+          <t>CABLE ASSY-PASSENGER</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3780,27 +3780,27 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2622236-6</t>
+          <t>S2837-1</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>COVER ACCESS RH</t>
+          <t>CABLE ASSY-PASSENGER</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3820,7 +3820,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3830,12 +3830,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>S2837-1</t>
+          <t>S51-14</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CABLE ASSY-PASSENGER</t>
+          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -3845,22 +3845,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>S2837-1</t>
+          <t>S51-14</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>CABLE ASSY-PASSENGER</t>
+          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -3880,12 +3880,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>S51-14</t>
+          <t>1134380-5</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -3895,7 +3895,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3905,12 +3905,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>S51-14</t>
+          <t>1H101-4</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+          <t>FLOW CONTROL VALVE</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -3930,12 +3930,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>1134380-5</t>
+          <t>5950017-11</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>REDUCER ASSEMBY</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -3955,12 +3955,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>1H101-4</t>
+          <t>040-0043</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>FLOW CONTROL VALVE</t>
+          <t>STROB TUB</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -3980,16 +3980,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>5950017-11</t>
+          <t>DLS4-02303</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>REDUCER ASSEMBY</t>
+          <t>IMOBILIZADOR</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="108">
@@ -4005,16 +4005,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>040-0043</t>
+          <t>DLS4-01786</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>STROB TUB</t>
+          <t>BLOQUEIO DA VENTILAÇ</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="109">
@@ -4030,22 +4030,22 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>DLS4-02303</t>
+          <t>A1635-133</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>IMOBILIZADOR</t>
+          <t>SCREW</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4055,22 +4055,22 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>DLS4-01786</t>
+          <t>A1635-133</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>BLOQUEIO DA VENTILAÇ</t>
+          <t>SCREW</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -4080,41 +4080,41 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>A1635-133</t>
+          <t>2641014-5</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>SCREW</t>
+          <t>SPRING-MAIN GEAR CEN</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A1635-133</t>
+          <t>2641014-5</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SCREW</t>
+          <t>SPRING-MAIN GEAR CEN</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2641014-5</t>
+          <t>205842-1</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR CEN</t>
+          <t>CONNECTOR</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -4145,22 +4145,22 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2641014-5</t>
+          <t>AN804D4</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR CEN</t>
+          <t>TEE,TUBE</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4180,12 +4180,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>205842-1</t>
+          <t>453-5060</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>CONNECTOR</t>
+          <t>BEACON,DISTRESS</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4205,12 +4205,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>AN804D4</t>
+          <t>S3465-2-0132</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>TEE,TUBE</t>
+          <t>HOSE ASSY BRAKE CYL</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>453-5060</t>
+          <t>S3465-2-0146</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>BEACON,DISTRESS</t>
+          <t>HOSE ASSY BRAK</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4255,12 +4255,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>S3465-2-0132</t>
+          <t>200276-2</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAKE CYL</t>
+          <t>CONNECTOR BODY,RECEP</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -4280,12 +4280,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>S3465-2-0146</t>
+          <t>51539-012N</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAK</t>
+          <t>CONTROL UNIT,GENERA</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -4305,12 +4305,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>200276-2</t>
+          <t>M83248/1-904</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>CONNECTOR BODY,RECEP</t>
+          <t>ANEL-O</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4330,12 +4330,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>51539-012N</t>
+          <t>2643065-2</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>CONTROL UNIT,GENERA</t>
+          <t>BUNGEE ASSY</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -4355,12 +4355,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>M83248/1-904</t>
+          <t>723908</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ANEL-O</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2643065-2</t>
+          <t>2601271-18</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>BUNGEE ASSY</t>
+          <t>DRIVE PULLEY</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4405,12 +4405,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>723908</t>
+          <t>1134380-4</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4430,12 +4430,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2601271-18</t>
+          <t>2652016-21</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>DRIVE PULLEY</t>
+          <t>DOOR ASSY COWL LH</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4455,12 +4455,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>1134380-4</t>
+          <t>S1053K22T144.00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4480,12 +4480,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2652016-21</t>
+          <t>S1915-3</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>DOOR ASSY COWL LH</t>
+          <t>CAPACITOR-6.0 MF 150</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4505,12 +4505,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>S1053K22T144.00</t>
+          <t>2619020-37</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
+          <t>SEAT ASSEMBLY - BENCH</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>S1915-3</t>
+          <t>011-00870-00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>CAPACITOR-6.0 MF 150</t>
+          <t>MAGNETOMETER GMU 44</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4555,12 +4555,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2619020-37</t>
+          <t>011-00877-00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>SEAT ASSEMBLY - BENCH</t>
+          <t>GSA-80 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4580,12 +4580,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>011-00870-00</t>
+          <t>011-00878-10</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>MAGNETOMETER GMU 44</t>
+          <t>GSA-81 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -4605,12 +4605,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>011-00877-00</t>
+          <t>011-01020-10</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>GSA-80 TORQUE SERVO</t>
+          <t>AFCS MODE CONTROLLER</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4630,12 +4630,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>011-00878-10</t>
+          <t>SL6015-4</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>GSA-81 TORQUE SERVO</t>
+          <t>CLIP</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4655,12 +4655,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>011-01020-10</t>
+          <t>EA5175-29PTL-CES</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>AFCS MODE CONTROLLER</t>
+          <t>AIRSPEED INDICATOR</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SL6015-4</t>
+          <t>2650032-4</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>CLIP</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4705,12 +4705,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>EA5175-29PTL-CES</t>
+          <t>011-01105-01</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>AIRSPEED INDICATOR</t>
+          <t>INTEGRATED AVIONICS</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -4730,12 +4730,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2650032-4</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -4755,16 +4755,16 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>011-01105-01</t>
+          <t>2654013-4</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>INTEGRATED AVIONICS</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139">
@@ -4780,16 +4780,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>2115040-206</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>GAS SPRING</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140">
@@ -4805,12 +4805,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2654013-4</t>
+          <t>5211369-8</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>EXTENDER-CREW, (WHEN</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -4830,12 +4830,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2115040-206</t>
+          <t>MS16674-5021</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>GAS SPRING</t>
+          <t>RETAINING RING</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -4855,12 +4855,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>5211369-8</t>
+          <t>302-120-302</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>EXTENDER-CREW, (WHEN</t>
+          <t>TUBE MAIN 850X10</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -4880,12 +4880,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>MS16674-5021</t>
+          <t>1570301-1</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>RETAINING RING</t>
+          <t>DIMMING ASSY,SPEC</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -4905,16 +4905,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>302-120-302</t>
+          <t>71014</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>TUBE MAIN 850X10</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="145">
@@ -4930,16 +4930,16 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>1570301-1</t>
+          <t>NAS1149F0363P</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIMMING ASSY,SPEC</t>
+          <t>WASHER, FLAT</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="146">
@@ -4955,16 +4955,16 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>71014</t>
+          <t>AN3-5A</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>BOLT,MACHINE</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="147">
@@ -4980,66 +4980,66 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>NAS1149F0363P</t>
+          <t>DD2W</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>WASHER, FLAT</t>
+          <t>STATIC WICK</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AN3-5A</t>
+          <t>2641012-14</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>BOLT,MACHINE</t>
+          <t>TRUNNION ASSY-RH-MAI</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>DD2W</t>
+          <t>5950028-10</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>STATIC WICK</t>
+          <t>VANT,BREATHER</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -5055,12 +5055,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2641012-14</t>
+          <t>S2889-3-0112</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY-RH-MAI</t>
+          <t>HOSE ASSY TEE</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -5080,12 +5080,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>5950028-10</t>
+          <t>1J18-10</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>VANT,BREATHER</t>
+          <t>FUEL FILTER ASSY</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -5105,12 +5105,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>S2889-3-0112</t>
+          <t>C668050-1103</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>HOSE ASSY TEE</t>
+          <t>TRANSMITER FUEL</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -5130,12 +5130,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>1J18-10</t>
+          <t>2651023-23</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>FUEL FILTER ASSY</t>
+          <t>ENGINE MOUNT ASSEMBL</t>
         </is>
       </c>
       <c r="E153" t="n">
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>C668050-1103</t>
+          <t>S133-6P58</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>TRANSMITER FUEL</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -5180,12 +5180,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2651023-23</t>
+          <t>9910338-6</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT ASSEMBL</t>
+          <t>TRANSMITTER,RATE OF FLOW</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -5205,12 +5205,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>S133-6P58</t>
+          <t>162-11800</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>WHEEL HALF ASSY-OUTER</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -5230,12 +5230,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>9910338-6</t>
+          <t>244-18922</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>TRANSMITTER,RATE OF FLOW</t>
+          <t>CABLE FIRE DET</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -5255,12 +5255,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>162-11800</t>
+          <t>2632020-14</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-OUTER</t>
+          <t>HINGE BKT INBD</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -5280,12 +5280,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>244-18922</t>
+          <t>9919105-1</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>CABLE FIRE DET</t>
+          <t>RESTRAINT ASSY</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -5305,12 +5305,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2632020-14</t>
+          <t>2643055-5</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HINGE BKT INBD</t>
+          <t>SUPPORT ASSY AFT NOSE GEAR</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -5330,12 +5330,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>9919105-1</t>
+          <t>2641030-2</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>RESTRAINT ASSY</t>
+          <t>COVER</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -5355,12 +5355,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2643055-5</t>
+          <t>2613439-1</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>SUPPORT ASSY AFT NOSE GEAR</t>
+          <t>SHIELD</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -5380,12 +5380,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2641030-2</t>
+          <t>2682004-1</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>COVER</t>
+          <t>RESERVOIR ASSY-BRAKE</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2613439-1</t>
+          <t>2621000-24</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>SHIELD</t>
+          <t>STRUT ASSY-RH WING</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -5430,12 +5430,12 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2682004-1</t>
+          <t>2662018-5</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>RESERVOIR ASSY-BRAKE</t>
+          <t>TUBE ASSY-LONG</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -5455,12 +5455,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2621000-24</t>
+          <t>2661215-6</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>STRUT ASSY-RH WING</t>
+          <t>SCREW INTERNAL</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -5480,12 +5480,12 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2662018-5</t>
+          <t>2622185-22</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>TUBE ASSY-LONG</t>
+          <t>RIB ASSY-RH-AILERON</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -5505,12 +5505,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2661215-6</t>
+          <t>AN6289D3</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>SCREW INTERNAL</t>
+          <t>LOCKNUT,TUBE F</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -5530,12 +5530,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2622185-22</t>
+          <t>2643057-1</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>RIB ASSY-RH-AILERON</t>
+          <t>BOOT N G STEER</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -5555,12 +5555,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AN6289D3</t>
+          <t>S2889-3-0160</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>LOCKNUT,TUBE F</t>
+          <t>HOSE ASSY ELBOW</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -5580,12 +5580,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2643057-1</t>
+          <t>2617015-18</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>BOOT N G STEER</t>
+          <t>HINGE DOOR LH</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>S2889-3-0160</t>
+          <t>2615018-1</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>HOSE ASSY ELBOW</t>
+          <t>MOLDING-WINDOW</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -5630,12 +5630,12 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2617015-18</t>
+          <t>2615035-5</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>HINGE DOOR LH</t>
+          <t>SCUFF PLATE-LH CREW</t>
         </is>
       </c>
       <c r="E173" t="n">
@@ -5655,12 +5655,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2615018-1</t>
+          <t>2615035-6</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>MOLDING-WINDOW</t>
+          <t>SCUFF PLATE-RH CREW</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -5680,12 +5680,12 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2615035-5</t>
+          <t>AT-RL1019</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-LH CREW</t>
+          <t>PLATE - COVER</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -5705,12 +5705,12 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2615035-6</t>
+          <t>2615011-2</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-RH CREW</t>
+          <t>WINDOW MOLDING</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -5730,12 +5730,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>AT-RL1019</t>
+          <t>2641012-13</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>PLATE - COVER</t>
+          <t>TRUNNION ASSY</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -5755,12 +5755,12 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2615011-2</t>
+          <t>2650113-5</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>WINDOW MOLDING</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -5780,12 +5780,12 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2641012-13</t>
+          <t>2601072-14</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY</t>
+          <t>BRACKET ASSY-95 AMP</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -5805,12 +5805,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2650113-5</t>
+          <t>C622010-0102</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>LIGHT STROBE RH</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -5830,16 +5830,16 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2601072-14</t>
+          <t>C662041-0102</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>BRACKET ASSY-95 AMP</t>
+          <t>INDICATOR FUEL</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="182">
@@ -5855,16 +5855,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>C622010-0102</t>
+          <t>2617015-22</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>LIGHT STROBE RH</t>
+          <t>HINGE-DOOR LH</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="183">
@@ -5880,12 +5880,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>C662041-0102</t>
+          <t>2621011-3</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>INDICATOR FUEL</t>
+          <t>WASHER</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -5905,12 +5905,12 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2617015-22</t>
+          <t>2621008-202</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>HINGE-DOOR LH</t>
+          <t>FITTING-WING STRUT U</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -5930,12 +5930,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2621011-3</t>
+          <t>2552-070</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>WASHER</t>
+          <t>NUT,SELF-LOCKI</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -5955,12 +5955,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2621008-202</t>
+          <t>C262023-0107</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT U</t>
+          <t>TUBE 850X10</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -5980,12 +5980,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2552-070</t>
+          <t>2661215-1</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>NUT,SELF-LOCKI</t>
+          <t>ACTUATOR ASSY-ELEVAT</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -6005,12 +6005,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>C262023-0107</t>
+          <t>2622184-3</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>TUBE 850X10</t>
+          <t>PUSH ROD ASSY</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -6030,12 +6030,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2661215-1</t>
+          <t>NAS464P12-37</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>ACTUATOR ASSY-ELEVAT</t>
+          <t>BOLT,SHEAR</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -6055,12 +6055,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2622184-3</t>
+          <t>NAS464P14-76</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>PUSH ROD ASSY</t>
+          <t>BOLT,SHEAR</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -6080,12 +6080,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>NAS464P12-37</t>
+          <t>MS24462-5</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>BOLT,SHEAR</t>
+          <t>BEARING ROLLER</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>NAS464P14-76</t>
+          <t>161-12800</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>BOLT,SHEAR</t>
+          <t>WHEEL HALF ASSY-INNE</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -6130,16 +6130,16 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>MS24462-5</t>
+          <t>2614076-63</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>BEARING ROLLER</t>
+          <t>PASSENGER SEAT UPHOL</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="194">
@@ -6155,16 +6155,16 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>161-12800</t>
+          <t>C299501-0402</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-INNE</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="195">
@@ -6180,16 +6180,16 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2614076-63</t>
+          <t>214-01400</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>PASSENGER SEAT UPHOL</t>
+          <t>CONE AND ROLLERS,TAP</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="196">
@@ -6205,16 +6205,16 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>C299501-0402</t>
+          <t>2621009-2</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>FITTING-WING STRUT L</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="197">
@@ -6230,12 +6230,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>214-01400</t>
+          <t>NAS1336C5C19K</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>CONE AND ROLLERS,TAP</t>
+          <t>PIN-LOCWELL SINGLE A</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -6255,12 +6255,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2621009-2</t>
+          <t>2614021-13</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT L</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -6280,12 +6280,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>NAS1336C5C19K</t>
+          <t>2616031-1</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>PIN-LOCWELL SINGLE A</t>
+          <t>VALVE</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -6305,16 +6305,16 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2614021-13</t>
+          <t>6361620-11</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>SPROCKET</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="201">
@@ -6330,16 +6330,16 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2616031-1</t>
+          <t>2601347-1</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>VALVE</t>
+          <t>BRACKET CARGO PAD</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="202">
@@ -6355,16 +6355,16 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>6361620-11</t>
+          <t>9910333-1</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SPROCKET</t>
+          <t>ENGINE MOUNT</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="203">
@@ -6380,16 +6380,16 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2601347-1</t>
+          <t>S2357-3</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>BRACKET CARGO PAD</t>
+          <t>CLAMP, LOOP</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="204">
@@ -6405,16 +6405,16 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>9910333-1</t>
+          <t>R221485</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT</t>
+          <t>MANGUEIRA</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="205">
@@ -6430,16 +6430,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>S2357-3</t>
+          <t>R221487</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>CLAMP, LOOP</t>
+          <t>MANGUEIRA</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="206">
@@ -6455,16 +6455,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>R221485</t>
+          <t>S3354-1</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>MANGUEIRA</t>
+          <t>BOLT</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="207">
@@ -6480,16 +6480,16 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>R221487</t>
+          <t>657735</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>MANGUEIRA</t>
+          <t>CLIP, LOCKING</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="208">
@@ -6505,16 +6505,16 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>S3354-1</t>
+          <t>MS27641-6G</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="209">
@@ -6530,16 +6530,16 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>657735</t>
+          <t>23541</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>CLIP, LOCKING</t>
+          <t>BUSHING,CABLE CLAMP</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="210">
@@ -6555,16 +6555,16 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>MS27641-6G</t>
+          <t>2670067-1</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>BEARING</t>
+          <t>POST LIGHT ASS</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="211">
@@ -6580,41 +6580,16 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23541</t>
+          <t>060-0015-00</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>BUSHING,CABLE CLAMP</t>
+          <t>CONTROL,DIRECTIONAL</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>2726</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>1º ETA</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>2670067-1</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>POST LIGHT ASS</t>
-        </is>
-      </c>
-      <c r="E212" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (09/07/2026 23:47)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1316,27 +1304,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (10/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,32 +430,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -536,12 +548,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,21 +567,21 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2733</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -583,10 +595,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -1304,27 +1316,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>
@@ -1558,22 +1570,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>P7036368-01</t>
+          <t>3122678-04</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PROPELLER ASSEMBLY</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1583,22 +1595,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>P7036368-01</t>
+          <t>3122678-04</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PROPELLER ASSEMBLY</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1608,12 +1620,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1633,7 +1645,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1658,12 +1670,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1683,22 +1695,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2643007-1</t>
+          <t>P7036368-01</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SHIMMY DAMP AS</t>
+          <t>PROPELLER ASSEMBLY</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1708,22 +1720,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2643007-1</t>
+          <t>P7036368-01</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SHIMMY DAMP AS</t>
+          <t>PROPELLER ASSEMBLY</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1733,12 +1745,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1758,7 +1770,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1783,22 +1795,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>C611505-0201</t>
+          <t>2643007-1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ALTERNATOR</t>
+          <t>SHIMMY DAMP AS</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1808,7 +1820,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1818,12 +1830,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C611505-0201</t>
+          <t>2643007-1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ALTERNATOR</t>
+          <t>SHIMMY DAMP AS</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1833,12 +1845,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1858,7 +1870,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1883,22 +1895,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2651022-20-1</t>
+          <t>C611505-0201</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RING ASSY ENGI</t>
+          <t>ALTERNATOR</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1908,7 +1920,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1918,12 +1930,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2651022-20-1</t>
+          <t>C611505-0201</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RING ASSY ENGI</t>
+          <t>ALTERNATOR</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1933,12 +1945,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1958,22 +1970,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2641011-5</t>
+          <t>2651022-20-1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AXLE-MAIN GEAR</t>
+          <t>RING ASSY ENGI</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1993,16 +2005,16 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2641011-5</t>
+          <t>2651022-20-1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AXLE-MAIN GEAR</t>
+          <t>RING ASSY ENGI</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2018,12 +2030,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2643100-206</t>
+          <t>2641011-5</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+          <t>AXLE-MAIN GEAR</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2033,26 +2045,26 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>162-10700</t>
+          <t>2641011-5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>OUTER WHEEL HALF ASSY</t>
+          <t>AXLE-MAIN GEAR</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -2068,12 +2080,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>D20B-14489-KA</t>
+          <t>2643100-206</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SLEEVE</t>
+          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2093,12 +2105,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>400454</t>
+          <t>162-10700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SEAL,PLAIN ENCASED</t>
+          <t>OUTER WHEEL HALF ASSY</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2118,52 +2130,52 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AE3663163K0600</t>
+          <t>D20B-14489-KA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>HOSE ASSY</t>
+          <t>SLEEVE</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AE3663163K0600</t>
+          <t>400454</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>HOSE ASSY</t>
+          <t>SEAL,PLAIN ENCASED</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2183,12 +2195,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2202,28 +2214,28 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2641013-6</t>
+          <t>AE3663163K0600</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR LH &amp; RH</t>
+          <t>HOSE ASSY</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2233,22 +2245,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2641013-6</t>
+          <t>AE3663163K0600</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR LH &amp; RH</t>
+          <t>HOSE ASSY</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2258,12 +2270,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2277,28 +2289,28 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2611112-2</t>
+          <t>2641013-6</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>STRAP</t>
+          <t>SPRING-MAIN GEAR LH &amp; RH</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2308,37 +2320,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2611112-2</t>
+          <t>2641013-6</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>STRAP</t>
+          <t>SPRING-MAIN GEAR LH &amp; RH</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2358,26 +2370,26 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2601119-1</t>
+          <t>2611112-2</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>JACK PAD LH</t>
+          <t>STRAP</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
@@ -2393,16 +2405,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2601119-1</t>
+          <t>2611112-2</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>JACK PAD LH</t>
+          <t>STRAP</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
@@ -2418,12 +2430,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>154-03000</t>
+          <t>2601119-1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SEAL MOLDED</t>
+          <t>JACK PAD LH</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2433,26 +2445,26 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2621013-2</t>
+          <t>2601119-1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>JACK PAD LH</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -2468,41 +2480,41 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>M81934/2-32C032</t>
+          <t>154-03000</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>BEARING,SLEEVE</t>
+          <t>SEAL MOLDED</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>M81934/2-32C032</t>
+          <t>2621013-2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BEARING,SLEEVE</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -2518,12 +2530,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2611137-7</t>
+          <t>M81934/2-32C032</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CAP MAIN LAND</t>
+          <t>BEARING,SLEEVE</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -2533,51 +2545,51 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3122678-04</t>
+          <t>M81934/2-32C032</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>FUEL CONTROL UNIT</t>
+          <t>BEARING,SLEEVE</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2733</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3122678-04</t>
+          <t>2611137-7</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>FUEL CONTROL UNIT</t>
+          <t>CAP MAIN LAND</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Atualização automática: rac (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1316,27 +1304,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (10/07/2026 16:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,32 +430,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1304,27 +1316,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (10/07/2026 22:38)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1316,27 +1304,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (10/07/2026 20:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,32 +430,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1304,27 +1316,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (11/07/2026 07:19)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,32 +418,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>contrato</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>total_pendencias</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>soma_unidades_faltantes</t>
         </is>
@@ -1316,27 +1304,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unidade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>quantidade_faltante</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: rac (14/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Desmontada</t>
+          <t>Montada</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -583,10 +583,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -602,7 +602,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Desmontada</t>
+          <t>Montada</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -611,10 +611,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -726,7 +726,7 @@
         <v>82</v>
       </c>
       <c r="F11" t="n">
-        <v>231</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Montada</t>
+          <t>Desmontada</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1199,10 +1199,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1300,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1333,7 +1333,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2709</t>
+          <t>2721</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1368,12 +1368,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C145-00-46</t>
+          <t>066-3046-07</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TRANSMISSION ASSY</t>
+          <t>CONTROL,INDICATOR</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1383,12 +1383,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2721</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1408,22 +1408,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2721</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>6º ETA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>066-3046-07</t>
+          <t>3044000</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CONTROL,INDICATOR</t>
+          <t>ENGINE PT6A-114A</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1433,12 +1433,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2721</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1458,12 +1458,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1483,12 +1483,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2741</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BABV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1533,12 +1533,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1558,22 +1558,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2723</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3044000</t>
+          <t>3122678-04</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ENGINE PT6A-114A</t>
+          <t>FUEL CONTROL UNIT</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1583,12 +1583,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2723</t>
+          <t>2733</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1608,22 +1608,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2733</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3122678-04</t>
+          <t>P7036368-01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FUEL CONTROL UNIT</t>
+          <t>PROPELLER ASSEMBLY</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1633,12 +1633,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1658,7 +1658,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1708,12 +1708,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1733,22 +1733,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>P7036368-01</t>
+          <t>2643007-1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PROPELLER ASSEMBLY</t>
+          <t>SHIMMY DAMP AS</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1758,12 +1758,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1783,7 +1783,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1808,7 +1808,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1833,22 +1833,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2643007-1</t>
+          <t>C611505-0201</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SHIMMY DAMP AS</t>
+          <t>ALTERNATOR</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1858,12 +1858,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1883,7 +1883,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1908,7 +1908,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1933,22 +1933,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>C611505-0201</t>
+          <t>2651022-20-1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ALTERNATOR</t>
+          <t>RING ASSY ENGI</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1958,12 +1958,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1983,12 +1983,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2008,22 +2008,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2651022-20-1</t>
+          <t>2641011-5</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RING ASSY ENGI</t>
+          <t>AXLE-MAIN GEAR</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2033,12 +2033,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2052,32 +2052,32 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2641011-5</t>
+          <t>2643100-206</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AXLE-MAIN GEAR</t>
+          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2093,12 +2093,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2643100-206</t>
+          <t>162-10700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+          <t>OUTER WHEEL HALF ASSY</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2118,12 +2118,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>162-10700</t>
+          <t>D20B-14489-KA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>OUTER WHEEL HALF ASSY</t>
+          <t>SLEEVE</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2143,12 +2143,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>D20B-14489-KA</t>
+          <t>400454</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SLEEVE</t>
+          <t>SEAL,PLAIN ENCASED</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2168,27 +2168,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>400454</t>
+          <t>AE3663163K0600</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SEAL,PLAIN ENCASED</t>
+          <t>HOSE ASSY</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2202,13 +2202,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2227,18 +2227,18 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2258,22 +2258,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AE3663163K0600</t>
+          <t>2641013-6</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>HOSE ASSY</t>
+          <t>SPRING-MAIN GEAR LH &amp; RH</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -2283,12 +2283,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2308,12 +2308,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2327,43 +2327,43 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2641013-6</t>
+          <t>2611112-2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR LH &amp; RH</t>
+          <t>STRAP</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2377,18 +2377,18 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2402,28 +2402,28 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2611112-2</t>
+          <t>2601119-1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>STRAP</t>
+          <t>JACK PAD LH</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2433,12 +2433,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2452,32 +2452,32 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2601119-1</t>
+          <t>154-03000</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>JACK PAD LH</t>
+          <t>SEAL MOLDED</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -2493,12 +2493,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>154-03000</t>
+          <t>2621013-2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>SEAL MOLDED</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2518,27 +2518,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2621013-2</t>
+          <t>M81934/2-32C032</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>BEARING,SLEEVE</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2558,22 +2558,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2728</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>1º/5º GAV</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>M81934/2-32C032</t>
+          <t>2611137-7</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BEARING,SLEEVE</t>
+          <t>CAP MAIN LAND</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2583,32 +2583,32 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2728</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1º/5º GAV</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2611137-7</t>
+          <t>1H75-21</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CAP MAIN LAND</t>
+          <t>PRESSURE REGULATOR</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2633,7 +2633,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2658,12 +2658,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2683,22 +2683,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1H75-21</t>
+          <t>2600100-7</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PRESSURE REGULATOR</t>
+          <t>LINE ASSY-PROP</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2708,7 +2708,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2733,7 +2733,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2600100-7</t>
+          <t>2698010-7</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>LINE ASSY-PROP</t>
+          <t>PASSENGER DOOR - LOW</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2783,7 +2783,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2808,7 +2808,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2818,22 +2818,22 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2698010-7</t>
+          <t>030-18200</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>PASSENGER DOOR - LOW</t>
+          <t>MAIN WHEEL BRAKE</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2858,7 +2858,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2883,12 +2883,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2908,22 +2908,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>030-18200</t>
+          <t>2115040-8</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MAIN WHEEL BRAKE</t>
+          <t>CYLINDER GAS S</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -2933,7 +2933,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2958,7 +2958,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2983,7 +2983,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2993,12 +2993,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2115040-8</t>
+          <t>S1053K16T</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CYLINDER GAS S</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3008,7 +3008,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3033,7 +3033,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3052,18 +3052,18 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3083,32 +3083,32 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2732</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>S1053K16T</t>
+          <t>42854-11</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>FITTING A S TR</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2732</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3118,22 +3118,22 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>42854-11</t>
+          <t>799-1</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>FITTING A S TR</t>
+          <t>TRANSDUCER</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3158,12 +3158,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3183,22 +3183,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>799-1</t>
+          <t>S1053K24T</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>TRANSDUCER</t>
+          <t>HOSE,AIR DUCT</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -3208,7 +3208,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3233,12 +3233,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3252,38 +3252,38 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>S1053K24T</t>
+          <t>C352TS</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT</t>
+          <t>EXTINGUISHER,FIRE</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3308,7 +3308,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3318,12 +3318,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>C352TS</t>
+          <t>AN929-4W</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>EXTINGUISHER,FIRE</t>
+          <t>CAP,TUBE</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -3333,7 +3333,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3358,7 +3358,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3368,12 +3368,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AN929-4W</t>
+          <t>2601266-2</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>CAP,TUBE</t>
+          <t>COUPLING-SPLINED</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -3383,12 +3383,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3408,22 +3408,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2601266-2</t>
+          <t>30994-001</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>COUPLING-SPLINED</t>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3433,12 +3433,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3458,22 +3458,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>30994-001</t>
+          <t>2641018-25</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>BATTERY-MARATHON TSP410 NICAD</t>
+          <t>FAIRING ASSY LH</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2641018-25</t>
+          <t>2641018-26</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>FAIRING ASSY LH</t>
+          <t>FAIRING ASSY RH</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -3518,12 +3518,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2641018-26</t>
+          <t>S2814-2</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>FAIRING ASSY RH</t>
+          <t>CABLE ASSY-DOOR PULL</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>S2814-2</t>
+          <t>S2574-1</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>CABLE ASSY-DOOR PULL</t>
+          <t>NUT-DIODE ATTACH</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3568,12 +3568,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>S2574-1</t>
+          <t>2601393-1</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>NUT-DIODE ATTACH</t>
+          <t>SUPORT PLATE</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -3593,12 +3593,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2601393-1</t>
+          <t>2601188-9</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>SUPORT PLATE</t>
+          <t>COMPRESSOR DRIVE ASS</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -3618,12 +3618,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2601188-9</t>
+          <t>2601392-1</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>COMPRESSOR DRIVE ASS</t>
+          <t>ADJUSTER PLATE</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2601392-1</t>
+          <t>2622236-6</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ADJUSTER PLATE</t>
+          <t>COVER ACCESS RH</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -3668,22 +3668,22 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2622236-6</t>
+          <t>S2837-1</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>COVER ACCESS RH</t>
+          <t>CABLE ASSY-PASSENGER</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3708,12 +3708,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3733,22 +3733,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>S2837-1</t>
+          <t>S51-14</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>CABLE ASSY-PASSENGER</t>
+          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -3758,7 +3758,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3783,7 +3783,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2730</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3793,12 +3793,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>S51-14</t>
+          <t>1134380-5</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1134380-5</t>
+          <t>1H101-4</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>FLOW CONTROL VALVE</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -3843,12 +3843,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>1H101-4</t>
+          <t>5950017-11</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>FLOW CONTROL VALVE</t>
+          <t>REDUCER ASSEMBY</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -3868,12 +3868,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>5950017-11</t>
+          <t>040-0043</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>REDUCER ASSEMBY</t>
+          <t>STROB TUB</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -3893,16 +3893,16 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>040-0043</t>
+          <t>DLS4-02303</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>STROB TUB</t>
+          <t>IMOBILIZADOR</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105">
@@ -3918,16 +3918,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>DLS4-02303</t>
+          <t>DLS4-01786</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>IMOBILIZADOR</t>
+          <t>BLOQUEIO DA VENTILAÇ</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="106">
@@ -3943,22 +3943,22 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>DLS4-01786</t>
+          <t>A1635-133</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>BLOQUEIO DA VENTILAÇ</t>
+          <t>SCREW</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2730</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3993,27 +3993,27 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>A1635-133</t>
+          <t>2641014-5</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>SCREW</t>
+          <t>SPRING-MAIN GEAR CEN</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4033,22 +4033,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2734</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>7º ETA</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2641014-5</t>
+          <t>MS24392-10</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>SPRING-MAIN GEAR CEN</t>
+          <t>NIPPLE,TUBE</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>MS24392-10</t>
+          <t>AS5174D1210</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>NIPPLE,TUBE</t>
+          <t>REDUCER, TUBE</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -4093,12 +4093,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>AS5174D1210</t>
+          <t>24540-100</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>REDUCER, TUBE</t>
+          <t>COUPLING,CLAMP,GROOV</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4118,12 +4118,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>24540-100</t>
+          <t>205842-1</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>COUPLING,CLAMP,GROOV</t>
+          <t>CONNECTOR</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -4143,12 +4143,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>205842-1</t>
+          <t>AN804D4</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>CONNECTOR</t>
+          <t>TEE,TUBE</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4168,12 +4168,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>AN804D4</t>
+          <t>453-5060</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>TEE,TUBE</t>
+          <t>BEACON,DISTRESS</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4193,12 +4193,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>453-5060</t>
+          <t>S3465-2-0132</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>BEACON,DISTRESS</t>
+          <t>HOSE ASSY BRAKE CYL</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4218,12 +4218,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>S3465-2-0132</t>
+          <t>S3465-2-0146</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAKE CYL</t>
+          <t>HOSE ASSY BRAK</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4243,12 +4243,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>S3465-2-0146</t>
+          <t>200276-2</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>HOSE ASSY BRAK</t>
+          <t>CONNECTOR BODY,RECEP</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -4268,12 +4268,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>200276-2</t>
+          <t>51539-012N</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>CONNECTOR BODY,RECEP</t>
+          <t>CONTROL UNIT,GENERA</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -4293,12 +4293,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>51539-012N</t>
+          <t>M83248/1-904</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>CONTROL UNIT,GENERA</t>
+          <t>ANEL-O</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4318,12 +4318,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>M83248/1-904</t>
+          <t>2643065-2</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ANEL-O</t>
+          <t>BUNGEE ASSY</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -4343,12 +4343,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2643065-2</t>
+          <t>723908</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>BUNGEE ASSY</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -4368,12 +4368,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>723908</t>
+          <t>2601271-18</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>DRIVE PULLEY</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4393,12 +4393,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2601271-18</t>
+          <t>1134380-4</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>DRIVE PULLEY</t>
+          <t>EVAPORATOR MODULE AS</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4418,12 +4418,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>1134380-4</t>
+          <t>2652016-21</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>EVAPORATOR MODULE AS</t>
+          <t>DOOR ASSY COWL LH</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4443,12 +4443,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2652016-21</t>
+          <t>S1053K22T144.00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>DOOR ASSY COWL LH</t>
+          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4468,12 +4468,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>S1053K22T144.00</t>
+          <t>S1915-3</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
+          <t>CAPACITOR-6.0 MF 150</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4493,12 +4493,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>S1915-3</t>
+          <t>2619020-37</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>CAPACITOR-6.0 MF 150</t>
+          <t>SEAT ASSEMBLY - BENCH</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4518,12 +4518,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2619020-37</t>
+          <t>011-00870-00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>SEAT ASSEMBLY - BENCH</t>
+          <t>MAGNETOMETER GMU 44</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4543,12 +4543,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>011-00870-00</t>
+          <t>011-00877-00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>MAGNETOMETER GMU 44</t>
+          <t>GSA-80 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4568,12 +4568,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>011-00877-00</t>
+          <t>011-00878-10</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>GSA-80 TORQUE SERVO</t>
+          <t>GSA-81 TORQUE SERVO</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -4593,12 +4593,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>011-00878-10</t>
+          <t>011-01020-10</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>GSA-81 TORQUE SERVO</t>
+          <t>AFCS MODE CONTROLLER</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4618,12 +4618,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>011-01020-10</t>
+          <t>SL6015-4</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>AFCS MODE CONTROLLER</t>
+          <t>CLIP</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4643,12 +4643,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SL6015-4</t>
+          <t>EA5175-29PTL-CES</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>CLIP</t>
+          <t>AIRSPEED INDICATOR</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -4668,12 +4668,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>EA5175-29PTL-CES</t>
+          <t>2650032-4</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>AIRSPEED INDICATOR</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2650032-4</t>
+          <t>011-01105-01</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>INTEGRATED AVIONICS</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -4718,12 +4718,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>011-01105-01</t>
+          <t>011-00883-20</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>INTEGRATED AVIONICS</t>
+          <t>RADAR GWX 68 WEATHER</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -4743,12 +4743,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>011-00883-20</t>
+          <t>S2655-1</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>RADAR GWX 68 WEATHER</t>
+          <t>DUCT-FLEX</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -4768,16 +4768,16 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>S2655-1</t>
+          <t>2654013-4</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>DUCT-FLEX</t>
+          <t>GASKET</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140">
@@ -4793,12 +4793,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2654013-4</t>
+          <t>2115040-206</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>GASKET</t>
+          <t>GAS SPRING</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -4818,12 +4818,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2115040-206</t>
+          <t>5211369-8</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>GAS SPRING</t>
+          <t>EXTENDER-CREW, (WHEN</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -4843,12 +4843,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>5211369-8</t>
+          <t>MS16674-5021</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>EXTENDER-CREW, (WHEN</t>
+          <t>RETAINING RING</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -4868,12 +4868,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>MS16674-5021</t>
+          <t>302-120-302</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>RETAINING RING</t>
+          <t>TUBE MAIN 850X10</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -4893,12 +4893,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>302-120-302</t>
+          <t>1570301-1</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>TUBE MAIN 850X10</t>
+          <t>DIMMING ASSY,SPEC</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -4918,16 +4918,16 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>1570301-1</t>
+          <t>71014</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIMMING ASSY,SPEC</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
@@ -4943,16 +4943,16 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>71014</t>
+          <t>NAS1149F0363P</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>WASHER, FLAT</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="147">
@@ -4968,12 +4968,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>NAS1149F0363P</t>
+          <t>AN3-5A</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>WASHER, FLAT</t>
+          <t>BOLT,MACHINE</t>
         </is>
       </c>
       <c r="E147" t="n">
@@ -4993,41 +4993,41 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AN3-5A</t>
+          <t>DD2W</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>BOLT,MACHINE</t>
+          <t>STATIC WICK</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2734</t>
+          <t>2726</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>7º ETA</t>
+          <t>1º ETA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>DD2W</t>
+          <t>2641012-14</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>STATIC WICK</t>
+          <t>TRUNNION ASSY-RH-MAI</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -5043,12 +5043,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2641012-14</t>
+          <t>5950028-10</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY-RH-MAI</t>
+          <t>VANT,BREATHER</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -5068,12 +5068,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>5950028-10</t>
+          <t>S2889-3-0112</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>VANT,BREATHER</t>
+          <t>HOSE ASSY TEE</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -5093,12 +5093,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>S2889-3-0112</t>
+          <t>1J18-10</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>HOSE ASSY TEE</t>
+          <t>FUEL FILTER ASSY</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -5118,12 +5118,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>1J18-10</t>
+          <t>C668050-1103</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>FUEL FILTER ASSY</t>
+          <t>TRANSMITER FUEL</t>
         </is>
       </c>
       <c r="E153" t="n">
@@ -5143,12 +5143,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>C668050-1103</t>
+          <t>2651023-23</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>TRANSMITER FUEL</t>
+          <t>ENGINE MOUNT ASSEMBL</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -5168,12 +5168,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2651023-23</t>
+          <t>S133-6P58</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT ASSEMBL</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -5193,12 +5193,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>S133-6P58</t>
+          <t>9910338-6</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>TRANSMITTER,RATE OF FLOW</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -5218,12 +5218,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>9910338-6</t>
+          <t>162-11800</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>TRANSMITTER,RATE OF FLOW</t>
+          <t>WHEEL HALF ASSY-OUTER</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -5243,12 +5243,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>162-11800</t>
+          <t>244-18922</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-OUTER</t>
+          <t>CABLE FIRE DET</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -5268,12 +5268,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>244-18922</t>
+          <t>2632020-14</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>CABLE FIRE DET</t>
+          <t>HINGE BKT INBD</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -5293,12 +5293,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2632020-14</t>
+          <t>9919105-1</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HINGE BKT INBD</t>
+          <t>RESTRAINT ASSY</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -5318,12 +5318,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>9919105-1</t>
+          <t>2643055-5</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>RESTRAINT ASSY</t>
+          <t>SUPPORT ASSY AFT NOSE GEAR</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -5343,12 +5343,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2643055-5</t>
+          <t>2641030-2</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>SUPPORT ASSY AFT NOSE GEAR</t>
+          <t>COVER</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -5368,12 +5368,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2641030-2</t>
+          <t>2613439-1</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>COVER</t>
+          <t>SHIELD</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -5393,12 +5393,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2613439-1</t>
+          <t>2682004-1</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>SHIELD</t>
+          <t>RESERVOIR ASSY-BRAKE</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -5418,12 +5418,12 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2682004-1</t>
+          <t>2621000-24</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>RESERVOIR ASSY-BRAKE</t>
+          <t>STRUT ASSY-RH WING</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2621000-24</t>
+          <t>2662018-5</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>STRUT ASSY-RH WING</t>
+          <t>TUBE ASSY-LONG</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -5468,12 +5468,12 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2662018-5</t>
+          <t>2661215-6</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>TUBE ASSY-LONG</t>
+          <t>SCREW INTERNAL</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -5493,12 +5493,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2661215-6</t>
+          <t>2622185-22</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>SCREW INTERNAL</t>
+          <t>RIB ASSY-RH-AILERON</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -5518,12 +5518,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2622185-22</t>
+          <t>AN6289D3</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>RIB ASSY-RH-AILERON</t>
+          <t>LOCKNUT,TUBE F</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -5543,12 +5543,12 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AN6289D3</t>
+          <t>2643057-1</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>LOCKNUT,TUBE F</t>
+          <t>BOOT N G STEER</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2643057-1</t>
+          <t>S2889-3-0160</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>BOOT N G STEER</t>
+          <t>HOSE ASSY ELBOW</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -5593,12 +5593,12 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>S2889-3-0160</t>
+          <t>2617015-18</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>HOSE ASSY ELBOW</t>
+          <t>HINGE DOOR LH</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -5618,16 +5618,16 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2617015-18</t>
+          <t>2615018-1</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>HINGE DOOR LH</t>
+          <t>MOLDING-WINDOW</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174">
@@ -5643,12 +5643,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2615018-1</t>
+          <t>2615035-5</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>MOLDING-WINDOW</t>
+          <t>SCUFF PLATE-LH CREW</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -5668,12 +5668,12 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2615035-5</t>
+          <t>2615035-6</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-LH CREW</t>
+          <t>SCUFF PLATE-RH CREW</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2615035-6</t>
+          <t>AT-RL1019</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>SCUFF PLATE-RH CREW</t>
+          <t>PLATE - COVER</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -5718,12 +5718,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>AT-RL1019</t>
+          <t>2615011-2</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>PLATE - COVER</t>
+          <t>WINDOW MOLDING</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -5743,12 +5743,12 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2615011-2</t>
+          <t>2641012-13</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>WINDOW MOLDING</t>
+          <t>TRUNNION ASSY</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -5768,12 +5768,12 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2641012-13</t>
+          <t>2650113-5</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>TRUNNION ASSY</t>
+          <t>BRACKET</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -5793,12 +5793,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2650113-5</t>
+          <t>2601072-14</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>BRACKET</t>
+          <t>BRACKET ASSY-95 AMP</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -5818,12 +5818,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2601072-14</t>
+          <t>C622010-0102</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>BRACKET ASSY-95 AMP</t>
+          <t>LIGHT STROBE RH</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -5843,12 +5843,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>C622010-0102</t>
+          <t>060-0015-00</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>LIGHT STROBE RH</t>
+          <t>CONTROL,DIRECTIONAL</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -5868,16 +5868,16 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>060-0015-00</t>
+          <t>C662041-0102</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>CONTROL,DIRECTIONAL</t>
+          <t>INDICATOR FUEL</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
@@ -5893,12 +5893,12 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>C662041-0102</t>
+          <t>2617015-22</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>INDICATOR FUEL</t>
+          <t>HINGE-DOOR LH</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -5918,12 +5918,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2617015-22</t>
+          <t>2621011-3</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>HINGE-DOOR LH</t>
+          <t>WASHER</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -5943,12 +5943,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2621011-3</t>
+          <t>2621008-202</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>WASHER</t>
+          <t>FITTING-WING STRUT U</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -5968,16 +5968,16 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2621008-202</t>
+          <t>2552-070</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT U</t>
+          <t>NUT,SELF-LOCKI</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="188">
@@ -5993,12 +5993,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2552-070</t>
+          <t>C262023-0107</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>NUT,SELF-LOCKI</t>
+          <t>TUBE 850X10</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -6018,12 +6018,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>C262023-0107</t>
+          <t>2661215-1</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>TUBE 850X10</t>
+          <t>ACTUATOR ASSY-ELEVAT</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -6043,12 +6043,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2661215-1</t>
+          <t>2622184-3</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>ACTUATOR ASSY-ELEVAT</t>
+          <t>PUSH ROD ASSY</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -6068,12 +6068,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2622184-3</t>
+          <t>NAS464P12-37</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>PUSH ROD ASSY</t>
+          <t>BOLT,SHEAR</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>NAS464P12-37</t>
+          <t>NAS464P14-76</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -6118,12 +6118,12 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>NAS464P14-76</t>
+          <t>MS24462-5</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>BOLT,SHEAR</t>
+          <t>BEARING ROLLER</t>
         </is>
       </c>
       <c r="E193" t="n">
@@ -6143,12 +6143,12 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>MS24462-5</t>
+          <t>161-12800</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>BEARING ROLLER</t>
+          <t>WHEEL HALF ASSY-INNE</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -6168,16 +6168,16 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>161-12800</t>
+          <t>2614076-63</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>WHEEL HALF ASSY-INNE</t>
+          <t>PASSENGER SEAT UPHOL</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="196">
@@ -6193,16 +6193,16 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2614076-63</t>
+          <t>C299501-0402</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>PASSENGER SEAT UPHOL</t>
+          <t>SPACER</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="197">
@@ -6218,16 +6218,16 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>C299501-0402</t>
+          <t>214-01400</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SPACER</t>
+          <t>CONE AND ROLLERS,TAP</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="198">
@@ -6243,12 +6243,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>214-01400</t>
+          <t>2621009-2</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>CONE AND ROLLERS,TAP</t>
+          <t>FITTING-WING STRUT L</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -6268,12 +6268,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2621009-2</t>
+          <t>NAS1336C5C19K</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>FITTING-WING STRUT L</t>
+          <t>PIN-LOCWELL SINGLE A</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -6293,12 +6293,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>NAS1336C5C19K</t>
+          <t>2614021-13</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>PIN-LOCWELL SINGLE A</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -6318,12 +6318,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2614021-13</t>
+          <t>2616031-1</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>VALVE</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -6343,16 +6343,16 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2616031-1</t>
+          <t>6361620-11</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>VALVE</t>
+          <t>SPROCKET</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="203">
@@ -6368,16 +6368,16 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>6361620-11</t>
+          <t>2601347-1</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SPROCKET</t>
+          <t>BRACKET CARGO PAD</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="204">
@@ -6393,16 +6393,16 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2601347-1</t>
+          <t>9910333-1</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>BRACKET CARGO PAD</t>
+          <t>ENGINE MOUNT</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205">
@@ -6418,16 +6418,16 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>9910333-1</t>
+          <t>S2357-3</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT</t>
+          <t>CLAMP, LOOP</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="206">
@@ -6443,16 +6443,16 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>S2357-3</t>
+          <t>R221485</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>CLAMP, LOOP</t>
+          <t>MANGUEIRA</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="207">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>R221485</t>
+          <t>R221487</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -6493,16 +6493,16 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>R221487</t>
+          <t>S3354-1</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>MANGUEIRA</t>
+          <t>BOLT</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="209">
@@ -6518,12 +6518,12 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>S3354-1</t>
+          <t>657735</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>CLIP, LOCKING</t>
         </is>
       </c>
       <c r="E209" t="n">
@@ -6543,16 +6543,16 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>657735</t>
+          <t>MS27641-6G</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>CLIP, LOCKING</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="211">
@@ -6568,16 +6568,16 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>MS27641-6G</t>
+          <t>23541</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>BEARING</t>
+          <t>BUSHING,CABLE CLAMP</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="212">
@@ -6593,41 +6593,66 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23541</t>
+          <t>2670067-1</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>BUSHING,CABLE CLAMP</t>
+          <t>POST LIGHT ASS</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2726</t>
+          <t>2743</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>1º ETA</t>
+          <t>5º ETA</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2670067-1</t>
+          <t>C611008-0101</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>POST LIGHT ASS</t>
+          <t>ALTERNATOR CONTROL UNIT ASSY</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1º/5º GAV</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>067-06300</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>SPACER MAIN GE</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza RAC/Disponibilidade manualmente + janela de 2 anos na Diagonal TBO/HSI
RAC e Disponibilidade Diária estavam com o ciclo automático atrasado essa
manhã — busquei manualmente (RAC: 30 aeronaves/214 pendências; Disponibilidade:
relatório de 15/07 que ainda não tinha sido buscado, agora 10 relatórios).

Linha do tempo TBO/HSI (Motores) passa a ser sempre "ano atual + próximo"
em vez de um intervalo fixo 2026-2030 — rola sozinha com o tempo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="362">
   <si>
     <t>matricula</t>
   </si>
@@ -38,6 +38,9 @@
     <t>2721</t>
   </si>
   <si>
+    <t>2722</t>
+  </si>
+  <si>
     <t>2743</t>
   </si>
   <si>
@@ -83,9 +86,6 @@
     <t>2720</t>
   </si>
   <si>
-    <t>2722</t>
-  </si>
-  <si>
     <t>2727</t>
   </si>
   <si>
@@ -128,6 +128,9 @@
     <t>6º ETA</t>
   </si>
   <si>
+    <t>2ª ETA</t>
+  </si>
+  <si>
     <t>5º ETA</t>
   </si>
   <si>
@@ -149,9 +152,6 @@
     <t>PAMALS</t>
   </si>
   <si>
-    <t>2ª ETA</t>
-  </si>
-  <si>
     <t>1/15 GAV</t>
   </si>
   <si>
@@ -428,9 +428,6 @@
     <t>2650032-4</t>
   </si>
   <si>
-    <t>011-01105-01</t>
-  </si>
-  <si>
     <t>011-00883-20</t>
   </si>
   <si>
@@ -891,9 +888,6 @@
   </si>
   <si>
     <t>BRACKET</t>
-  </si>
-  <si>
-    <t>INTEGRATED AVIONICS</t>
   </si>
   <si>
     <t>RADAR GWX 68 WEATHER</t>
@@ -1113,8 +1107,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1130,7 +1132,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1138,12 +1140,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1442,22 +1462,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1515,10 +1535,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1535,10 +1555,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1555,10 +1575,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1572,13 +1592,13 @@
         <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1586,7 +1606,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1595,10 +1615,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="F8">
-        <v>87</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1606,7 +1626,7 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
@@ -1615,10 +1635,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="F9">
-        <v>137</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1626,7 +1646,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
         <v>50</v>
@@ -1635,10 +1655,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="F10">
-        <v>242</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1646,19 +1666,19 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1666,7 +1686,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1686,7 +1706,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1706,7 +1726,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1726,7 +1746,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1746,7 +1766,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1766,7 +1786,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1786,7 +1806,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1826,7 +1846,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1866,7 +1886,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
@@ -1886,7 +1906,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s">
         <v>51</v>
@@ -1926,7 +1946,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -1946,7 +1966,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
         <v>51</v>
@@ -2006,7 +2026,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
@@ -2026,7 +2046,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
@@ -2068,23 +2088,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E214"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2099,7 +2119,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2116,7 +2136,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2124,16 +2144,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2150,7 +2170,7 @@
         <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2158,16 +2178,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2175,16 +2195,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
         <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2192,16 +2212,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
         <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2209,16 +2229,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2226,16 +2246,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2252,7 +2272,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2266,10 +2286,10 @@
         <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2286,7 +2306,7 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2300,10 +2320,10 @@
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2320,7 +2340,7 @@
         <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2331,13 +2351,13 @@
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
         <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2348,13 +2368,13 @@
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
         <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2365,13 +2385,13 @@
         <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
         <v>63</v>
       </c>
       <c r="D18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2379,16 +2399,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
         <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2405,7 +2425,7 @@
         <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2416,13 +2436,13 @@
         <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2433,13 +2453,13 @@
         <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
         <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2447,16 +2467,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2473,7 +2493,7 @@
         <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2484,13 +2504,13 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C25" t="s">
         <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2501,13 +2521,13 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2515,16 +2535,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2532,7 +2552,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
         <v>41</v>
@@ -2541,7 +2561,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2549,16 +2569,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2566,16 +2586,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2583,50 +2603,50 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
         <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
         <v>40</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2634,16 +2654,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2651,16 +2671,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2668,24 +2688,24 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
         <v>41</v>
@@ -2694,10 +2714,10 @@
         <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2705,16 +2725,16 @@
         <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2722,13 +2742,13 @@
         <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2736,16 +2756,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B40" t="s">
         <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2753,7 +2773,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B41" t="s">
         <v>41</v>
@@ -2762,7 +2782,7 @@
         <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E41">
         <v>2</v>
@@ -2773,38 +2793,38 @@
         <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C42" t="s">
         <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
         <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
         <v>41</v>
@@ -2813,10 +2833,10 @@
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2824,30 +2844,30 @@
         <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C45" t="s">
         <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
         <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2855,50 +2875,50 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C47" t="s">
         <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
         <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D49" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2906,33 +2926,33 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D50" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
         <v>78</v>
       </c>
       <c r="D51" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -2940,16 +2960,16 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
         <v>40</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D52" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E52">
         <v>4</v>
@@ -2963,13 +2983,13 @@
         <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D53" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2977,13 +2997,13 @@
         <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C54" t="s">
         <v>80</v>
       </c>
       <c r="D54" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -2994,13 +3014,13 @@
         <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C55" t="s">
         <v>80</v>
       </c>
       <c r="D55" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3011,13 +3031,13 @@
         <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C56" t="s">
         <v>80</v>
       </c>
       <c r="D56" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3025,16 +3045,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D57" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3045,13 +3065,13 @@
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C58" t="s">
         <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3062,13 +3082,13 @@
         <v>13</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C59" t="s">
         <v>81</v>
       </c>
       <c r="D59" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3076,16 +3096,16 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C60" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D60" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3093,16 +3113,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C61" t="s">
         <v>82</v>
       </c>
       <c r="D61" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3110,19 +3130,19 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C62" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D62" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3130,13 +3150,13 @@
         <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C63" t="s">
         <v>83</v>
       </c>
       <c r="D63" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3147,13 +3167,13 @@
         <v>13</v>
       </c>
       <c r="B64" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C64" t="s">
         <v>83</v>
       </c>
       <c r="D64" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3164,13 +3184,13 @@
         <v>14</v>
       </c>
       <c r="B65" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C65" t="s">
         <v>83</v>
       </c>
       <c r="D65" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3178,16 +3198,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B66" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D66" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3198,13 +3218,13 @@
         <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C67" t="s">
         <v>84</v>
       </c>
       <c r="D67" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3215,13 +3235,13 @@
         <v>13</v>
       </c>
       <c r="B68" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C68" t="s">
         <v>84</v>
       </c>
       <c r="D68" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3229,16 +3249,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C69" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D69" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3249,13 +3269,13 @@
         <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C70" t="s">
         <v>85</v>
       </c>
       <c r="D70" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3266,16 +3286,16 @@
         <v>13</v>
       </c>
       <c r="B71" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C71" t="s">
         <v>85</v>
       </c>
       <c r="D71" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3283,13 +3303,13 @@
         <v>14</v>
       </c>
       <c r="B72" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C72" t="s">
         <v>85</v>
       </c>
       <c r="D72" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E72">
         <v>4</v>
@@ -3297,19 +3317,19 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D73" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E73">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3317,16 +3337,16 @@
         <v>12</v>
       </c>
       <c r="B74" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C74" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D74" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3334,13 +3354,13 @@
         <v>13</v>
       </c>
       <c r="B75" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C75" t="s">
         <v>87</v>
       </c>
       <c r="D75" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3351,13 +3371,13 @@
         <v>14</v>
       </c>
       <c r="B76" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C76" t="s">
         <v>87</v>
       </c>
       <c r="D76" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E76">
         <v>1</v>
@@ -3365,16 +3385,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D77" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3385,13 +3405,13 @@
         <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C78" t="s">
         <v>88</v>
       </c>
       <c r="D78" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3402,33 +3422,33 @@
         <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C79" t="s">
         <v>88</v>
       </c>
       <c r="D79" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E79">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D80" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3436,13 +3456,13 @@
         <v>13</v>
       </c>
       <c r="B81" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C81" t="s">
         <v>89</v>
       </c>
       <c r="D81" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3450,16 +3470,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C82" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D82" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3470,13 +3490,13 @@
         <v>13</v>
       </c>
       <c r="B83" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C83" t="s">
         <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3484,16 +3504,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C84" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D84" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3501,16 +3521,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B85" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C85" t="s">
         <v>91</v>
       </c>
       <c r="D85" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3518,16 +3538,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D86" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3535,16 +3555,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C87" t="s">
         <v>92</v>
       </c>
       <c r="D87" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3552,16 +3572,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B88" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D88" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3569,16 +3589,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B89" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D89" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3586,16 +3606,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3603,16 +3623,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D91" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3620,16 +3640,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C92" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D92" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3637,16 +3657,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C93" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D93" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3654,16 +3674,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C94" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D94" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3671,16 +3691,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C95" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D95" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3688,19 +3708,19 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C96" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D96" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E96">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -3708,13 +3728,13 @@
         <v>13</v>
       </c>
       <c r="B97" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C97" t="s">
         <v>101</v>
       </c>
       <c r="D97" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E97">
         <v>2</v>
@@ -3725,13 +3745,13 @@
         <v>14</v>
       </c>
       <c r="B98" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C98" t="s">
         <v>101</v>
       </c>
       <c r="D98" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E98">
         <v>2</v>
@@ -3739,16 +3759,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B99" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C99" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D99" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E99">
         <v>2</v>
@@ -3759,13 +3779,13 @@
         <v>13</v>
       </c>
       <c r="B100" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C100" t="s">
         <v>102</v>
       </c>
       <c r="D100" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E100">
         <v>2</v>
@@ -3773,16 +3793,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C101" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D101" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E101">
         <v>2</v>
@@ -3790,16 +3810,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C102" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D102" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E102">
         <v>2</v>
@@ -3807,16 +3827,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C103" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E103">
         <v>2</v>
@@ -3824,16 +3844,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B104" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C104" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D104" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E104">
         <v>2</v>
@@ -3841,53 +3861,53 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B105" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D105" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E105">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B106" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D106" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E106">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B107" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C107" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D107" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E107">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -3895,13 +3915,13 @@
         <v>13</v>
       </c>
       <c r="B108" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C108" t="s">
         <v>109</v>
       </c>
       <c r="D108" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E108">
         <v>30</v>
@@ -3909,33 +3929,33 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B109" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C109" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D109" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C110" t="s">
         <v>110</v>
       </c>
       <c r="D110" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3943,16 +3963,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B111" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C111" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -3960,16 +3980,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B112" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D112" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -3977,16 +3997,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B113" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C113" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D113" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E113">
         <v>1</v>
@@ -3994,16 +4014,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B114" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C114" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D114" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E114">
         <v>1</v>
@@ -4011,16 +4031,16 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C115" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D115" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E115">
         <v>1</v>
@@ -4028,16 +4048,16 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B116" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C116" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D116" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E116">
         <v>1</v>
@@ -4045,16 +4065,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C117" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D117" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E117">
         <v>1</v>
@@ -4062,16 +4082,16 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B118" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C118" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D118" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E118">
         <v>1</v>
@@ -4079,16 +4099,16 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B119" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C119" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D119" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E119">
         <v>1</v>
@@ -4096,16 +4116,16 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C120" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E120">
         <v>1</v>
@@ -4113,16 +4133,16 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B121" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C121" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D121" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E121">
         <v>1</v>
@@ -4130,16 +4150,16 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B122" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C122" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D122" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E122">
         <v>1</v>
@@ -4147,16 +4167,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B123" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C123" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D123" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4164,16 +4184,16 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B124" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C124" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D124" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4181,16 +4201,16 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B125" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C125" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D125" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4198,16 +4218,16 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B126" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C126" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D126" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4215,16 +4235,16 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B127" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C127" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D127" t="s">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4232,16 +4252,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B128" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C128" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D128" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4249,16 +4269,16 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B129" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C129" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D129" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4266,16 +4286,16 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C130" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D130" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4283,16 +4303,16 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C131" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D131" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4300,16 +4320,16 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B132" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C132" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D132" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4317,16 +4337,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B133" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C133" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D133" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4334,16 +4354,16 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B134" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C134" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D134" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4351,16 +4371,16 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B135" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C135" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D135" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4368,16 +4388,16 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B136" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C136" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D136" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4385,16 +4405,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B137" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C137" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D137" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4402,16 +4422,16 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B138" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D138" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4419,16 +4439,16 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B139" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C139" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D139" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4436,33 +4456,33 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B140" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C140" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D140" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="E140">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B141" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C141" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D141" t="s">
-        <v>295</v>
+        <v>278</v>
       </c>
       <c r="E141">
         <v>2</v>
@@ -4470,16 +4490,16 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B142" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C142" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D142" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="E142">
         <v>2</v>
@@ -4487,16 +4507,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B143" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C143" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D143" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E143">
         <v>2</v>
@@ -4504,16 +4524,16 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B144" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C144" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D144" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E144">
         <v>2</v>
@@ -4521,16 +4541,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B145" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C145" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D145" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E145">
         <v>2</v>
@@ -4538,50 +4558,50 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B146" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C146" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D146" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E146">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B147" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C147" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D147" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="E147">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B148" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C148" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D148" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E148">
         <v>8</v>
@@ -4589,19 +4609,19 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B149" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C149" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D149" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E149">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -4609,30 +4629,30 @@
         <v>14</v>
       </c>
       <c r="B150" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C150" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D150" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E150">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B151" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D151" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4640,16 +4660,16 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B152" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D152" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4657,16 +4677,16 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B153" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D153" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4674,16 +4694,16 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B154" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D154" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4691,16 +4711,16 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B155" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D155" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4708,16 +4728,16 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B156" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D156" t="s">
-        <v>234</v>
+        <v>307</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4725,16 +4745,16 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B157" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D157" t="s">
-        <v>310</v>
+        <v>233</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4742,16 +4762,16 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B158" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D158" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4759,16 +4779,16 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B159" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D159" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4776,16 +4796,16 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B160" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D160" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4793,16 +4813,16 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B161" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C161" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D161" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4810,16 +4830,16 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B162" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D162" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4827,16 +4847,16 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B163" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D163" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4844,16 +4864,16 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B164" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C164" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D164" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4861,16 +4881,16 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B165" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C165" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D165" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4878,16 +4898,16 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B166" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C166" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D166" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4895,16 +4915,16 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B167" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C167" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D167" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4912,16 +4932,16 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B168" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C168" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D168" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4929,16 +4949,16 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B169" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D169" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4946,16 +4966,16 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D170" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4963,16 +4983,16 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B171" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D171" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4980,16 +5000,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B172" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D172" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -4997,16 +5017,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B173" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D173" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5014,33 +5034,33 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B174" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D174" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="E174">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B175" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D175" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5048,16 +5068,16 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B176" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D176" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5065,16 +5085,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B177" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D177" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5082,16 +5102,16 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B178" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D178" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5099,16 +5119,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B179" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D179" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5116,16 +5136,16 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B180" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D180" t="s">
-        <v>291</v>
+        <v>330</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5133,16 +5153,16 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B181" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D181" t="s">
-        <v>333</v>
+        <v>290</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5150,16 +5170,16 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B182" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D182" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5167,16 +5187,16 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B183" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D183" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5184,33 +5204,33 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B184" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D184" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E184">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B185" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D185" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E185">
         <v>2</v>
@@ -5218,16 +5238,16 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D186" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E186">
         <v>2</v>
@@ -5235,16 +5255,16 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B187" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D187" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E187">
         <v>2</v>
@@ -5252,33 +5272,33 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B188" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D188" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E188">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B189" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D189" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E189">
         <v>2</v>
@@ -5286,16 +5306,16 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B190" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D190" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E190">
         <v>2</v>
@@ -5303,16 +5323,16 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B191" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D191" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E191">
         <v>2</v>
@@ -5320,16 +5340,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B192" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D192" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="E192">
         <v>2</v>
@@ -5337,16 +5357,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B193" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D193" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E193">
         <v>2</v>
@@ -5354,16 +5374,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B194" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D194" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E194">
         <v>2</v>
@@ -5371,16 +5391,16 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B195" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D195" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E195">
         <v>2</v>
@@ -5388,67 +5408,67 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B196" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D196" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E196">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B197" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D197" t="s">
-        <v>234</v>
+        <v>345</v>
       </c>
       <c r="E197">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B198" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D198" t="s">
-        <v>348</v>
+        <v>233</v>
       </c>
       <c r="E198">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B199" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D199" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E199">
         <v>4</v>
@@ -5456,16 +5476,16 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B200" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D200" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E200">
         <v>4</v>
@@ -5473,16 +5493,16 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B201" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D201" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E201">
         <v>4</v>
@@ -5490,16 +5510,16 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B202" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D202" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="E202">
         <v>4</v>
@@ -5507,101 +5527,101 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B203" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D203" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="E203">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B204" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D204" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E204">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B205" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D205" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E205">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B206" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D206" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="E206">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B207" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D207" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E207">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B208" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D208" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E208">
         <v>10</v>
@@ -5609,33 +5629,33 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B209" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D209" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E209">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B210" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D210" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E210">
         <v>12</v>
@@ -5643,69 +5663,86 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B211" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D211" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E211">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B212" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D212" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E212">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B213" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D213" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E213">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B214" t="s">
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D214" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="E214">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5">
+      <c r="A215" t="s">
+        <v>11</v>
+      </c>
+      <c r="B215" t="s">
+        <v>41</v>
+      </c>
+      <c r="C215" t="s">
+        <v>213</v>
+      </c>
+      <c r="D215" t="s">
+        <v>361</v>
+      </c>
+      <c r="E215">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/07/2026 16:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1107,16 +1107,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1132,7 +1124,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1140,30 +1132,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1462,22 +1436,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2092,19 +2066,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/07/2026 20:41)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -191,15 +191,15 @@
     <t>quantidade_faltante</t>
   </si>
   <si>
+    <t>066-3046-07</t>
+  </si>
+  <si>
+    <t>3044000</t>
+  </si>
+  <si>
     <t>C145-00-46</t>
   </si>
   <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
-    <t>3044000</t>
-  </si>
-  <si>
     <t>C611008-0101</t>
   </si>
   <si>
@@ -218,6 +218,9 @@
     <t>2651022-20-1</t>
   </si>
   <si>
+    <t>2641014-5</t>
+  </si>
+  <si>
     <t>2641011-5</t>
   </si>
   <si>
@@ -251,6 +254,9 @@
     <t>2621013-2</t>
   </si>
   <si>
+    <t>067-06300</t>
+  </si>
+  <si>
     <t>M81934/2-32C032</t>
   </si>
   <si>
@@ -347,9 +353,6 @@
     <t>A1635-133</t>
   </si>
   <si>
-    <t>2641014-5</t>
-  </si>
-  <si>
     <t>MS24392-10</t>
   </si>
   <si>
@@ -656,18 +659,15 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>067-06300</t>
+    <t>CONTROL,INDICATOR</t>
+  </si>
+  <si>
+    <t>ENGINE PT6A-114A</t>
   </si>
   <si>
     <t>TRANSMISSION ASSY</t>
   </si>
   <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
-    <t>ENGINE PT6A-114A</t>
-  </si>
-  <si>
     <t>ALTERNATOR CONTROL UNIT ASSY</t>
   </si>
   <si>
@@ -686,6 +686,9 @@
     <t>RING ASSY ENGI</t>
   </si>
   <si>
+    <t>SPRING-MAIN GEAR CEN</t>
+  </si>
+  <si>
     <t>AXLE-MAIN GEAR</t>
   </si>
   <si>
@@ -719,6 +722,9 @@
     <t>SPACER</t>
   </si>
   <si>
+    <t>SPACER MAIN GE</t>
+  </si>
+  <si>
     <t>BEARING,SLEEVE</t>
   </si>
   <si>
@@ -812,9 +818,6 @@
     <t>SCREW</t>
   </si>
   <si>
-    <t>SPRING-MAIN GEAR CEN</t>
-  </si>
-  <si>
     <t>NIPPLE,TUBE</t>
   </si>
   <si>
@@ -1098,9 +1101,6 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
-  </si>
-  <si>
-    <t>SPACER MAIN GE</t>
   </si>
 </sst>
 </file>
@@ -2101,16 +2101,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2118,10 +2118,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
         <v>59</v>
@@ -2135,16 +2135,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2152,16 +2152,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2169,16 +2169,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2186,16 +2186,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2203,16 +2203,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2220,10 +2220,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
         <v>60</v>
@@ -2594,10 +2594,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C32" t="s">
         <v>67</v>
@@ -2606,21 +2606,21 @@
         <v>223</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2634,10 +2634,10 @@
         <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2645,19 +2645,19 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2668,10 +2668,10 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2685,38 +2685,38 @@
         <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E38">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
@@ -2725,21 +2725,21 @@
         <v>228</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2747,10 +2747,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C41" t="s">
         <v>73</v>
@@ -2759,7 +2759,7 @@
         <v>229</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2793,7 +2793,7 @@
         <v>229</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2827,7 +2827,7 @@
         <v>230</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2844,7 +2844,7 @@
         <v>230</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2866,10 +2866,10 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C48" t="s">
         <v>75</v>
@@ -2878,21 +2878,21 @@
         <v>231</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D49" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2906,10 +2906,10 @@
         <v>41</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D50" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -2917,36 +2917,36 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D51" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D52" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E52">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2957,38 +2957,38 @@
         <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D53" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D54" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C55" t="s">
         <v>80</v>
@@ -2997,15 +2997,15 @@
         <v>236</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
         <v>80</v>
@@ -3014,24 +3014,24 @@
         <v>236</v>
       </c>
       <c r="E56">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D57" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3042,10 +3042,10 @@
         <v>42</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D58" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3059,10 +3059,10 @@
         <v>42</v>
       </c>
       <c r="C59" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3076,10 +3076,10 @@
         <v>42</v>
       </c>
       <c r="C60" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D60" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3087,10 +3087,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B61" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
         <v>82</v>
@@ -3104,16 +3104,16 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
         <v>42</v>
       </c>
       <c r="C62" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D62" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3121,7 +3121,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B63" t="s">
         <v>42</v>
@@ -3133,12 +3133,12 @@
         <v>239</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
         <v>42</v>
@@ -3150,41 +3150,41 @@
         <v>239</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
         <v>42</v>
       </c>
       <c r="C65" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D65" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D66" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E66">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3195,10 +3195,10 @@
         <v>42</v>
       </c>
       <c r="C67" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D67" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3212,10 +3212,10 @@
         <v>42</v>
       </c>
       <c r="C68" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D68" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3229,10 +3229,10 @@
         <v>42</v>
       </c>
       <c r="C69" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D69" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3240,10 +3240,10 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B70" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
         <v>85</v>
@@ -3257,16 +3257,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B71" t="s">
         <v>42</v>
       </c>
       <c r="C71" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D71" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3274,36 +3274,36 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B72" t="s">
         <v>42</v>
       </c>
       <c r="C72" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D72" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C73" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D73" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E73">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3314,13 +3314,13 @@
         <v>42</v>
       </c>
       <c r="C74" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D74" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E74">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3337,7 +3337,7 @@
         <v>243</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3354,7 +3354,7 @@
         <v>243</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3371,12 +3371,12 @@
         <v>243</v>
       </c>
       <c r="E77">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
         <v>42</v>
@@ -3385,24 +3385,24 @@
         <v>88</v>
       </c>
       <c r="D78" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B79" t="s">
         <v>42</v>
       </c>
       <c r="C79" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D79" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3410,33 +3410,33 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C80" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D80" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B81" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
         <v>89</v>
       </c>
       <c r="D81" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3444,16 +3444,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B82" t="s">
         <v>42</v>
       </c>
       <c r="C82" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D82" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3461,7 +3461,7 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
         <v>42</v>
@@ -3470,7 +3470,7 @@
         <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3478,19 +3478,19 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B84" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
         <v>90</v>
       </c>
       <c r="D84" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3512,10 +3512,10 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C86" t="s">
         <v>91</v>
@@ -3546,10 +3546,10 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C88" t="s">
         <v>92</v>
@@ -3580,16 +3580,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B90" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D90" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3603,10 +3603,10 @@
         <v>42</v>
       </c>
       <c r="C91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D91" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3614,16 +3614,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B92" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D92" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3637,10 +3637,10 @@
         <v>42</v>
       </c>
       <c r="C93" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D93" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3654,10 +3654,10 @@
         <v>42</v>
       </c>
       <c r="C94" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3671,10 +3671,10 @@
         <v>42</v>
       </c>
       <c r="C95" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D95" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3688,10 +3688,10 @@
         <v>42</v>
       </c>
       <c r="C96" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D96" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3705,38 +3705,38 @@
         <v>42</v>
       </c>
       <c r="C97" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D97" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E97">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
         <v>42</v>
       </c>
       <c r="C98" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D98" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E98">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C99" t="s">
         <v>101</v>
@@ -3745,7 +3745,7 @@
         <v>256</v>
       </c>
       <c r="E99">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -3762,21 +3762,21 @@
         <v>257</v>
       </c>
       <c r="E100">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B101" t="s">
         <v>42</v>
       </c>
       <c r="C101" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D101" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E101">
         <v>2</v>
@@ -3784,7 +3784,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B102" t="s">
         <v>42</v>
@@ -3801,16 +3801,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B103" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E103">
         <v>2</v>
@@ -3824,10 +3824,10 @@
         <v>42</v>
       </c>
       <c r="C104" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D104" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E104">
         <v>2</v>
@@ -3835,16 +3835,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B105" t="s">
         <v>42</v>
       </c>
       <c r="C105" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D105" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -3858,13 +3858,13 @@
         <v>42</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D106" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E106">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -3875,13 +3875,13 @@
         <v>42</v>
       </c>
       <c r="C107" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D107" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E107">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -3892,52 +3892,52 @@
         <v>42</v>
       </c>
       <c r="C108" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D108" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E108">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B109" t="s">
         <v>42</v>
       </c>
       <c r="C109" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D109" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E109">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C110" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B111" t="s">
         <v>42</v>
@@ -3949,24 +3949,24 @@
         <v>265</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B112" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C112" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -3983,7 +3983,7 @@
         <v>266</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -4218,7 +4218,7 @@
         <v>125</v>
       </c>
       <c r="D127" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4235,7 +4235,7 @@
         <v>126</v>
       </c>
       <c r="D128" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4456,10 +4456,10 @@
         <v>139</v>
       </c>
       <c r="D141" t="s">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="E141">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -4473,7 +4473,7 @@
         <v>140</v>
       </c>
       <c r="D142" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="E142">
         <v>2</v>
@@ -4561,7 +4561,7 @@
         <v>298</v>
       </c>
       <c r="E147">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -4578,7 +4578,7 @@
         <v>299</v>
       </c>
       <c r="E148">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -4612,15 +4612,15 @@
         <v>301</v>
       </c>
       <c r="E150">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B151" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C151" t="s">
         <v>149</v>
@@ -4629,7 +4629,7 @@
         <v>302</v>
       </c>
       <c r="E151">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -4728,7 +4728,7 @@
         <v>155</v>
       </c>
       <c r="D157" t="s">
-        <v>233</v>
+        <v>308</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4745,7 +4745,7 @@
         <v>156</v>
       </c>
       <c r="D158" t="s">
-        <v>308</v>
+        <v>234</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -5136,7 +5136,7 @@
         <v>179</v>
       </c>
       <c r="D181" t="s">
-        <v>290</v>
+        <v>331</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5153,7 +5153,7 @@
         <v>180</v>
       </c>
       <c r="D182" t="s">
-        <v>331</v>
+        <v>291</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5207,7 +5207,7 @@
         <v>334</v>
       </c>
       <c r="E185">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -5357,7 +5357,7 @@
         <v>192</v>
       </c>
       <c r="D194" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E194">
         <v>2</v>
@@ -5411,7 +5411,7 @@
         <v>345</v>
       </c>
       <c r="E197">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -5425,7 +5425,7 @@
         <v>196</v>
       </c>
       <c r="D198" t="s">
-        <v>233</v>
+        <v>346</v>
       </c>
       <c r="E198">
         <v>3</v>
@@ -5442,10 +5442,10 @@
         <v>197</v>
       </c>
       <c r="D199" t="s">
-        <v>346</v>
+        <v>234</v>
       </c>
       <c r="E199">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5530,7 +5530,7 @@
         <v>351</v>
       </c>
       <c r="E204">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5564,7 +5564,7 @@
         <v>353</v>
       </c>
       <c r="E206">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5581,7 +5581,7 @@
         <v>354</v>
       </c>
       <c r="E207">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5598,7 +5598,7 @@
         <v>355</v>
       </c>
       <c r="E208">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5612,7 +5612,7 @@
         <v>207</v>
       </c>
       <c r="D209" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E209">
         <v>10</v>
@@ -5632,7 +5632,7 @@
         <v>356</v>
       </c>
       <c r="E210">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5666,7 +5666,7 @@
         <v>358</v>
       </c>
       <c r="E212">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5683,7 +5683,7 @@
         <v>359</v>
       </c>
       <c r="E213">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5700,15 +5700,15 @@
         <v>360</v>
       </c>
       <c r="E214">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B215" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C215" t="s">
         <v>213</v>
@@ -5717,7 +5717,7 @@
         <v>361</v>
       </c>
       <c r="E215">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (16/07/2026 16:03)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="362">
   <si>
     <t>matricula</t>
   </si>
@@ -1483,16 +1483,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1652,7 +1652,7 @@
         <v>82</v>
       </c>
       <c r="F11">
-        <v>231</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2062,7 +2062,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E214"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2237,10 +2237,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
         <v>61</v>
@@ -2254,16 +2254,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2271,10 +2271,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
         <v>62</v>
@@ -2288,16 +2288,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2305,10 +2305,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
         <v>63</v>
@@ -2322,7 +2322,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
         <v>42</v>
@@ -2339,7 +2339,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
         <v>42</v>
@@ -2356,10 +2356,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
         <v>63</v>
@@ -2373,16 +2373,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2390,10 +2390,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
         <v>64</v>
@@ -2407,7 +2407,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
         <v>42</v>
@@ -2424,7 +2424,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
         <v>42</v>
@@ -2441,16 +2441,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D23" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2458,10 +2458,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s">
         <v>65</v>
@@ -2475,7 +2475,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
         <v>42</v>
@@ -2492,7 +2492,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
@@ -2509,16 +2509,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D27" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2526,10 +2526,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C28" t="s">
         <v>66</v>
@@ -2543,10 +2543,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
         <v>66</v>
@@ -2560,16 +2560,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2577,10 +2577,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C31" t="s">
         <v>67</v>
@@ -2594,10 +2594,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C32" t="s">
         <v>67</v>
@@ -2611,16 +2611,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2628,10 +2628,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
         <v>68</v>
@@ -2640,24 +2640,24 @@
         <v>224</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2668,10 +2668,10 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2685,10 +2685,10 @@
         <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2702,10 +2702,10 @@
         <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2719,21 +2719,21 @@
         <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C40" t="s">
         <v>73</v>
@@ -2742,12 +2742,12 @@
         <v>229</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
         <v>42</v>
@@ -2759,15 +2759,15 @@
         <v>229</v>
       </c>
       <c r="E41">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
         <v>73</v>
@@ -2781,16 +2781,16 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2798,10 +2798,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
@@ -2815,10 +2815,10 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
         <v>74</v>
@@ -2827,32 +2827,32 @@
         <v>230</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C47" t="s">
         <v>75</v>
@@ -2861,15 +2861,15 @@
         <v>231</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
         <v>75</v>
@@ -2878,21 +2878,21 @@
         <v>231</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D49" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2900,10 +2900,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50" t="s">
         <v>76</v>
@@ -2912,24 +2912,24 @@
         <v>232</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D51" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2940,10 +2940,10 @@
         <v>41</v>
       </c>
       <c r="C52" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D52" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -2957,10 +2957,10 @@
         <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D53" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -2974,21 +2974,21 @@
         <v>41</v>
       </c>
       <c r="C54" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D54" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
         <v>80</v>
@@ -3002,16 +3002,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D56" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E56">
         <v>4</v>
@@ -3019,24 +3019,24 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E57">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B58" t="s">
         <v>42</v>
@@ -3053,7 +3053,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B59" t="s">
         <v>42</v>
@@ -3070,10 +3070,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B60" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C60" t="s">
         <v>82</v>
@@ -3087,16 +3087,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C61" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D61" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3104,7 +3104,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B62" t="s">
         <v>42</v>
@@ -3121,7 +3121,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B63" t="s">
         <v>42</v>
@@ -3138,16 +3138,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
         <v>42</v>
       </c>
       <c r="C64" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D64" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3155,7 +3155,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B65" t="s">
         <v>42</v>
@@ -3172,24 +3172,24 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B66" t="s">
         <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D66" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B67" t="s">
         <v>42</v>
@@ -3206,7 +3206,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
         <v>42</v>
@@ -3223,10 +3223,10 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B69" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
         <v>85</v>
@@ -3240,16 +3240,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C70" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D70" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3257,7 +3257,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B71" t="s">
         <v>42</v>
@@ -3274,7 +3274,7 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
         <v>42</v>
@@ -3291,16 +3291,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
         <v>42</v>
       </c>
       <c r="C73" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D73" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3308,7 +3308,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B74" t="s">
         <v>42</v>
@@ -3325,7 +3325,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
         <v>42</v>
@@ -3337,15 +3337,15 @@
         <v>243</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B76" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
         <v>87</v>
@@ -3359,41 +3359,41 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C77" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D77" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E77">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
         <v>42</v>
       </c>
       <c r="C78" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D78" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E78">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
         <v>42</v>
@@ -3410,10 +3410,10 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
         <v>89</v>
@@ -3427,16 +3427,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C81" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3444,7 +3444,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
         <v>42</v>
@@ -3461,10 +3461,10 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B83" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
         <v>90</v>
@@ -3473,29 +3473,29 @@
         <v>243</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D84" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E84">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
         <v>42</v>
@@ -3512,16 +3512,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B86" t="s">
         <v>42</v>
       </c>
       <c r="C86" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D86" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3529,7 +3529,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
         <v>42</v>
@@ -3546,16 +3546,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B88" t="s">
         <v>42</v>
       </c>
       <c r="C88" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3563,10 +3563,10 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B89" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C89" t="s">
         <v>93</v>
@@ -3580,16 +3580,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C90" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3597,10 +3597,10 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B91" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C91" t="s">
         <v>94</v>
@@ -3614,16 +3614,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C92" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3637,10 +3637,10 @@
         <v>42</v>
       </c>
       <c r="C93" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D93" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3654,10 +3654,10 @@
         <v>42</v>
       </c>
       <c r="C94" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D94" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3671,10 +3671,10 @@
         <v>42</v>
       </c>
       <c r="C95" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D95" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3688,10 +3688,10 @@
         <v>42</v>
       </c>
       <c r="C96" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D96" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3705,10 +3705,10 @@
         <v>42</v>
       </c>
       <c r="C97" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3722,10 +3722,10 @@
         <v>42</v>
       </c>
       <c r="C98" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D98" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3739,10 +3739,10 @@
         <v>42</v>
       </c>
       <c r="C99" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D99" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3756,18 +3756,18 @@
         <v>42</v>
       </c>
       <c r="C100" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D100" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E100">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
         <v>42</v>
@@ -3784,10 +3784,10 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B102" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C102" t="s">
         <v>103</v>
@@ -3801,16 +3801,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B103" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C103" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E103">
         <v>2</v>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B104" t="s">
         <v>42</v>
@@ -3835,16 +3835,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B105" t="s">
         <v>42</v>
       </c>
       <c r="C105" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D105" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -3858,10 +3858,10 @@
         <v>42</v>
       </c>
       <c r="C106" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D106" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E106">
         <v>2</v>
@@ -3875,10 +3875,10 @@
         <v>42</v>
       </c>
       <c r="C107" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D107" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -3892,10 +3892,10 @@
         <v>42</v>
       </c>
       <c r="C108" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D108" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -3909,13 +3909,13 @@
         <v>42</v>
       </c>
       <c r="C109" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D109" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E109">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -3926,13 +3926,13 @@
         <v>42</v>
       </c>
       <c r="C110" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D110" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E110">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -3943,18 +3943,18 @@
         <v>42</v>
       </c>
       <c r="C111" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D111" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E111">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B112" t="s">
         <v>42</v>
@@ -3977,13 +3977,13 @@
         <v>42</v>
       </c>
       <c r="C113" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D113" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E113">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -3994,10 +3994,10 @@
         <v>42</v>
       </c>
       <c r="C114" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D114" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E114">
         <v>1</v>
@@ -4011,10 +4011,10 @@
         <v>42</v>
       </c>
       <c r="C115" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D115" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E115">
         <v>1</v>
@@ -4028,10 +4028,10 @@
         <v>42</v>
       </c>
       <c r="C116" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D116" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E116">
         <v>1</v>
@@ -4045,10 +4045,10 @@
         <v>42</v>
       </c>
       <c r="C117" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D117" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E117">
         <v>1</v>
@@ -4062,10 +4062,10 @@
         <v>42</v>
       </c>
       <c r="C118" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D118" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E118">
         <v>1</v>
@@ -4079,10 +4079,10 @@
         <v>42</v>
       </c>
       <c r="C119" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D119" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E119">
         <v>1</v>
@@ -4096,10 +4096,10 @@
         <v>42</v>
       </c>
       <c r="C120" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D120" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E120">
         <v>1</v>
@@ -4113,10 +4113,10 @@
         <v>42</v>
       </c>
       <c r="C121" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D121" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E121">
         <v>1</v>
@@ -4130,10 +4130,10 @@
         <v>42</v>
       </c>
       <c r="C122" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D122" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E122">
         <v>1</v>
@@ -4147,10 +4147,10 @@
         <v>42</v>
       </c>
       <c r="C123" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D123" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4164,10 +4164,10 @@
         <v>42</v>
       </c>
       <c r="C124" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D124" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4181,10 +4181,10 @@
         <v>42</v>
       </c>
       <c r="C125" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D125" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4198,10 +4198,10 @@
         <v>42</v>
       </c>
       <c r="C126" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D126" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4215,10 +4215,10 @@
         <v>42</v>
       </c>
       <c r="C127" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D127" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4232,10 +4232,10 @@
         <v>42</v>
       </c>
       <c r="C128" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D128" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4249,10 +4249,10 @@
         <v>42</v>
       </c>
       <c r="C129" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D129" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4266,10 +4266,10 @@
         <v>42</v>
       </c>
       <c r="C130" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D130" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4283,10 +4283,10 @@
         <v>42</v>
       </c>
       <c r="C131" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4300,10 +4300,10 @@
         <v>42</v>
       </c>
       <c r="C132" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4317,10 +4317,10 @@
         <v>42</v>
       </c>
       <c r="C133" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4334,10 +4334,10 @@
         <v>42</v>
       </c>
       <c r="C134" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4351,10 +4351,10 @@
         <v>42</v>
       </c>
       <c r="C135" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4368,10 +4368,10 @@
         <v>42</v>
       </c>
       <c r="C136" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4385,10 +4385,10 @@
         <v>42</v>
       </c>
       <c r="C137" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4402,10 +4402,10 @@
         <v>42</v>
       </c>
       <c r="C138" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4419,10 +4419,10 @@
         <v>42</v>
       </c>
       <c r="C139" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4436,10 +4436,10 @@
         <v>42</v>
       </c>
       <c r="C140" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4453,13 +4453,13 @@
         <v>42</v>
       </c>
       <c r="C141" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="E141">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -4470,10 +4470,10 @@
         <v>42</v>
       </c>
       <c r="C142" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="E142">
         <v>2</v>
@@ -4487,10 +4487,10 @@
         <v>42</v>
       </c>
       <c r="C143" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E143">
         <v>2</v>
@@ -4504,10 +4504,10 @@
         <v>42</v>
       </c>
       <c r="C144" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E144">
         <v>2</v>
@@ -4521,10 +4521,10 @@
         <v>42</v>
       </c>
       <c r="C145" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E145">
         <v>2</v>
@@ -4538,10 +4538,10 @@
         <v>42</v>
       </c>
       <c r="C146" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E146">
         <v>2</v>
@@ -4555,13 +4555,13 @@
         <v>42</v>
       </c>
       <c r="C147" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E147">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -4572,13 +4572,13 @@
         <v>42</v>
       </c>
       <c r="C148" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E148">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -4589,10 +4589,10 @@
         <v>42</v>
       </c>
       <c r="C149" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E149">
         <v>8</v>
@@ -4606,30 +4606,30 @@
         <v>42</v>
       </c>
       <c r="C150" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E150">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B151" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E151">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -4640,10 +4640,10 @@
         <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4657,10 +4657,10 @@
         <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4674,10 +4674,10 @@
         <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4691,10 +4691,10 @@
         <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4708,10 +4708,10 @@
         <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4725,10 +4725,10 @@
         <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>308</v>
+        <v>234</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4742,10 +4742,10 @@
         <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>234</v>
+        <v>309</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4759,10 +4759,10 @@
         <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4776,10 +4776,10 @@
         <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D160" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4793,10 +4793,10 @@
         <v>40</v>
       </c>
       <c r="C161" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4810,10 +4810,10 @@
         <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4827,10 +4827,10 @@
         <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4844,10 +4844,10 @@
         <v>40</v>
       </c>
       <c r="C164" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4861,10 +4861,10 @@
         <v>40</v>
       </c>
       <c r="C165" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4878,10 +4878,10 @@
         <v>40</v>
       </c>
       <c r="C166" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D166" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4895,10 +4895,10 @@
         <v>40</v>
       </c>
       <c r="C167" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4912,10 +4912,10 @@
         <v>40</v>
       </c>
       <c r="C168" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D168" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4929,10 +4929,10 @@
         <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4946,10 +4946,10 @@
         <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D170" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4963,10 +4963,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4980,10 +4980,10 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -4997,10 +4997,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5014,10 +5014,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5031,13 +5031,13 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E175">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -5048,10 +5048,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D176" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5065,10 +5065,10 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5082,10 +5082,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5099,10 +5099,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5116,10 +5116,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D180" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5133,10 +5133,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D181" t="s">
-        <v>331</v>
+        <v>291</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5150,10 +5150,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D182" t="s">
-        <v>291</v>
+        <v>332</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5167,10 +5167,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D183" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5184,10 +5184,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D184" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5201,13 +5201,13 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D185" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E185">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -5218,10 +5218,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D186" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E186">
         <v>2</v>
@@ -5235,10 +5235,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D187" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E187">
         <v>2</v>
@@ -5252,10 +5252,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D188" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E188">
         <v>2</v>
@@ -5269,13 +5269,13 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D189" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E189">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -5286,10 +5286,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D190" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E190">
         <v>2</v>
@@ -5303,10 +5303,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D191" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E191">
         <v>2</v>
@@ -5320,10 +5320,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D192" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E192">
         <v>2</v>
@@ -5337,10 +5337,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D193" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E193">
         <v>2</v>
@@ -5354,7 +5354,7 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D194" t="s">
         <v>343</v>
@@ -5371,10 +5371,10 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D195" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E195">
         <v>2</v>
@@ -5388,10 +5388,10 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D196" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E196">
         <v>2</v>
@@ -5405,13 +5405,13 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D197" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E197">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -5422,13 +5422,13 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D198" t="s">
-        <v>346</v>
+        <v>234</v>
       </c>
       <c r="E198">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -5439,13 +5439,13 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D199" t="s">
-        <v>234</v>
+        <v>347</v>
       </c>
       <c r="E199">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5456,10 +5456,10 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D200" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E200">
         <v>4</v>
@@ -5473,10 +5473,10 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D201" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E201">
         <v>4</v>
@@ -5490,10 +5490,10 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D202" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E202">
         <v>4</v>
@@ -5507,10 +5507,10 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D203" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E203">
         <v>4</v>
@@ -5524,13 +5524,13 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D204" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E204">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5541,13 +5541,13 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D205" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E205">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5558,13 +5558,13 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D206" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E206">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5575,13 +5575,13 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D207" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E207">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5592,13 +5592,13 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D208" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E208">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5609,7 +5609,7 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D209" t="s">
         <v>356</v>
@@ -5626,13 +5626,13 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D210" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E210">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5643,10 +5643,10 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D211" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E211">
         <v>12</v>
@@ -5660,13 +5660,13 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D212" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E212">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5677,13 +5677,13 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D213" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E213">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5694,29 +5694,12 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D214" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E214">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="215" spans="1:5">
-      <c r="A215" t="s">
-        <v>15</v>
-      </c>
-      <c r="B215" t="s">
-        <v>40</v>
-      </c>
-      <c r="C215" t="s">
-        <v>213</v>
-      </c>
-      <c r="D215" t="s">
-        <v>361</v>
-      </c>
-      <c r="E215">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (17/07/2026 16:03)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="380">
   <si>
     <t>matricula</t>
   </si>
@@ -665,6 +665,27 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>ADAS-C-031-1</t>
+  </si>
+  <si>
+    <t>540-1407-4</t>
+  </si>
+  <si>
+    <t>5319026-1</t>
+  </si>
+  <si>
+    <t>066-3114-00</t>
+  </si>
+  <si>
+    <t>2601264-1</t>
+  </si>
+  <si>
+    <t>2613472-11</t>
+  </si>
+  <si>
+    <t>2601189-11</t>
+  </si>
+  <si>
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
@@ -1113,6 +1134,27 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>PORT ASSY DOWNLOAD</t>
+  </si>
+  <si>
+    <t>VALVE,COMPRESSOR BLEED</t>
+  </si>
+  <si>
+    <t>HANDLE,DOOR</t>
+  </si>
+  <si>
+    <t>IND RDR 2000</t>
+  </si>
+  <si>
+    <t>COMPRESSOR SUPPORT</t>
+  </si>
+  <si>
+    <t>ANGLE ASSY-GLARESHIELD ATTACH</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
   </si>
 </sst>
 </file>
@@ -1501,10 +1543,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1621,10 +1663,10 @@
         <v>53</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1638,13 +1680,13 @@
         <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E10">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F10">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1658,13 +1700,13 @@
         <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F11">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1678,13 +1720,13 @@
         <v>50</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E12">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F12">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1698,13 +1740,13 @@
         <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E13">
         <v>82</v>
       </c>
       <c r="F13">
-        <v>242</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2074,7 +2116,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2105,7 +2147,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2122,7 +2164,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2139,7 +2181,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2156,7 +2198,7 @@
         <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2173,7 +2215,7 @@
         <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2190,7 +2232,7 @@
         <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2207,7 +2249,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2224,7 +2266,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2241,7 +2283,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2258,7 +2300,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2275,7 +2317,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2283,16 +2325,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2300,16 +2342,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2317,16 +2359,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2334,16 +2376,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2351,16 +2393,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
         <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2368,7 +2410,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
         <v>43</v>
@@ -2377,7 +2419,7 @@
         <v>64</v>
       </c>
       <c r="D18" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2385,7 +2427,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
         <v>43</v>
@@ -2394,7 +2436,7 @@
         <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2402,16 +2444,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
         <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2419,16 +2461,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2436,16 +2478,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2453,7 +2495,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
         <v>43</v>
@@ -2462,7 +2504,7 @@
         <v>65</v>
       </c>
       <c r="D23" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2470,7 +2512,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
         <v>43</v>
@@ -2479,7 +2521,7 @@
         <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2487,16 +2529,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2504,16 +2546,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
         <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2521,7 +2563,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
         <v>43</v>
@@ -2530,7 +2572,7 @@
         <v>66</v>
       </c>
       <c r="D27" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2538,7 +2580,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" t="s">
         <v>43</v>
@@ -2547,7 +2589,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2555,16 +2597,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2572,16 +2614,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" t="s">
         <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2589,16 +2631,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C31" t="s">
         <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2606,16 +2648,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2623,16 +2665,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" t="s">
         <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2640,16 +2682,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C34" t="s">
         <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2657,16 +2699,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2674,36 +2716,36 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C36" t="s">
         <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2714,10 +2756,10 @@
         <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D38" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2731,10 +2773,10 @@
         <v>42</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2748,10 +2790,10 @@
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2765,35 +2807,35 @@
         <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C42" t="s">
         <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="E42">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
         <v>43</v>
@@ -2802,24 +2844,24 @@
         <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2827,16 +2869,16 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2844,16 +2886,16 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C46" t="s">
         <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2861,84 +2903,84 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B47" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C47" t="s">
         <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C49" t="s">
         <v>76</v>
       </c>
       <c r="D49" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C50" t="s">
         <v>76</v>
       </c>
       <c r="D50" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B51" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D51" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -2946,36 +2988,36 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C52" t="s">
         <v>77</v>
       </c>
       <c r="D52" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B53" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D53" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2986,10 +3028,10 @@
         <v>42</v>
       </c>
       <c r="C54" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D54" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="E54">
         <v>2</v>
@@ -3003,10 +3045,10 @@
         <v>42</v>
       </c>
       <c r="C55" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3020,27 +3062,27 @@
         <v>42</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D56" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="E56">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C57" t="s">
         <v>81</v>
       </c>
       <c r="D57" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E57">
         <v>4</v>
@@ -3048,16 +3090,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B58" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E58">
         <v>4</v>
@@ -3065,33 +3107,33 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
         <v>42</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3099,7 +3141,7 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
         <v>43</v>
@@ -3108,7 +3150,7 @@
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3116,7 +3158,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B62" t="s">
         <v>43</v>
@@ -3125,7 +3167,7 @@
         <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3133,16 +3175,16 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B63" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C63" t="s">
         <v>84</v>
       </c>
       <c r="D63" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3150,16 +3192,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D64" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3167,7 +3209,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B65" t="s">
         <v>43</v>
@@ -3176,7 +3218,7 @@
         <v>85</v>
       </c>
       <c r="D65" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3184,7 +3226,7 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B66" t="s">
         <v>43</v>
@@ -3193,7 +3235,7 @@
         <v>85</v>
       </c>
       <c r="D66" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3201,16 +3243,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B67" t="s">
         <v>43</v>
       </c>
       <c r="C67" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D67" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3218,7 +3260,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
         <v>43</v>
@@ -3227,7 +3269,7 @@
         <v>86</v>
       </c>
       <c r="D68" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -3235,24 +3277,24 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
         <v>43</v>
       </c>
       <c r="C69" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D69" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E69">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B70" t="s">
         <v>43</v>
@@ -3261,7 +3303,7 @@
         <v>87</v>
       </c>
       <c r="D70" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3269,7 +3311,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B71" t="s">
         <v>43</v>
@@ -3278,7 +3320,7 @@
         <v>87</v>
       </c>
       <c r="D71" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3286,16 +3328,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C72" t="s">
         <v>87</v>
       </c>
       <c r="D72" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3303,16 +3345,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B73" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D73" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3320,7 +3362,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
         <v>43</v>
@@ -3329,7 +3371,7 @@
         <v>88</v>
       </c>
       <c r="D74" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3337,7 +3379,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B75" t="s">
         <v>43</v>
@@ -3346,7 +3388,7 @@
         <v>88</v>
       </c>
       <c r="D75" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3354,16 +3396,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B76" t="s">
         <v>43</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D76" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3371,7 +3413,7 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
         <v>43</v>
@@ -3380,7 +3422,7 @@
         <v>89</v>
       </c>
       <c r="D77" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3388,7 +3430,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B78" t="s">
         <v>43</v>
@@ -3397,24 +3439,24 @@
         <v>89</v>
       </c>
       <c r="D78" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C79" t="s">
         <v>89</v>
       </c>
       <c r="D79" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E79">
         <v>4</v>
@@ -3422,41 +3464,41 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B80" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D80" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="E80">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B81" t="s">
         <v>43</v>
       </c>
       <c r="C81" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B82" t="s">
         <v>43</v>
@@ -3465,7 +3507,7 @@
         <v>91</v>
       </c>
       <c r="D82" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3473,16 +3515,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B83" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C83" t="s">
         <v>91</v>
       </c>
       <c r="D83" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3490,16 +3532,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B84" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D84" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3507,7 +3549,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B85" t="s">
         <v>43</v>
@@ -3516,7 +3558,7 @@
         <v>92</v>
       </c>
       <c r="D85" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3524,41 +3566,41 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C86" t="s">
         <v>92</v>
       </c>
       <c r="D86" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B87" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D87" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B88" t="s">
         <v>43</v>
@@ -3567,7 +3609,7 @@
         <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3575,16 +3617,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
         <v>43</v>
       </c>
       <c r="C89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D89" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3592,7 +3634,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B90" t="s">
         <v>43</v>
@@ -3601,7 +3643,7 @@
         <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3609,16 +3651,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B91" t="s">
         <v>43</v>
       </c>
       <c r="C91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D91" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3626,16 +3668,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C92" t="s">
         <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3643,16 +3685,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B93" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D93" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3660,16 +3702,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B94" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C94" t="s">
         <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3677,16 +3719,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B95" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D95" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3700,10 +3742,10 @@
         <v>43</v>
       </c>
       <c r="C96" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D96" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3717,10 +3759,10 @@
         <v>43</v>
       </c>
       <c r="C97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D97" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3734,10 +3776,10 @@
         <v>43</v>
       </c>
       <c r="C98" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D98" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3751,10 +3793,10 @@
         <v>43</v>
       </c>
       <c r="C99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D99" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3768,10 +3810,10 @@
         <v>43</v>
       </c>
       <c r="C100" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D100" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3779,16 +3821,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B101" t="s">
         <v>43</v>
       </c>
       <c r="C101" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D101" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3802,10 +3844,10 @@
         <v>43</v>
       </c>
       <c r="C102" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D102" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3819,13 +3861,13 @@
         <v>43</v>
       </c>
       <c r="C103" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D103" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="E103">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -3836,44 +3878,44 @@
         <v>43</v>
       </c>
       <c r="C104" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D104" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="E104">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B105" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C105" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D105" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="E105">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B106" t="s">
         <v>43</v>
       </c>
       <c r="C106" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D106" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E106">
         <v>2</v>
@@ -3881,16 +3923,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B107" t="s">
         <v>43</v>
       </c>
       <c r="C107" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D107" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -3898,16 +3940,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B108" t="s">
         <v>43</v>
       </c>
       <c r="C108" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D108" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -3915,16 +3957,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B109" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D109" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -3938,10 +3980,10 @@
         <v>43</v>
       </c>
       <c r="C110" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D110" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -3949,16 +3991,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B111" t="s">
         <v>43</v>
       </c>
       <c r="C111" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D111" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -3972,13 +4014,13 @@
         <v>43</v>
       </c>
       <c r="C112" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D112" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E112">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -3989,115 +4031,115 @@
         <v>43</v>
       </c>
       <c r="C113" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D113" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E113">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B114" t="s">
         <v>43</v>
       </c>
       <c r="C114" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D114" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E114">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B115" t="s">
         <v>43</v>
       </c>
       <c r="C115" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D115" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E115">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B116" t="s">
         <v>43</v>
       </c>
       <c r="C116" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D116" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E116">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B117" t="s">
         <v>43</v>
       </c>
       <c r="C117" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D117" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E117">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B118" t="s">
         <v>43</v>
       </c>
       <c r="C118" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D118" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E118">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B119" t="s">
         <v>43</v>
       </c>
       <c r="C119" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D119" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E119">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4108,13 +4150,13 @@
         <v>43</v>
       </c>
       <c r="C120" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D120" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E120">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4125,10 +4167,10 @@
         <v>43</v>
       </c>
       <c r="C121" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D121" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E121">
         <v>1</v>
@@ -4142,10 +4184,10 @@
         <v>43</v>
       </c>
       <c r="C122" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D122" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E122">
         <v>1</v>
@@ -4159,10 +4201,10 @@
         <v>43</v>
       </c>
       <c r="C123" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D123" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4176,10 +4218,10 @@
         <v>43</v>
       </c>
       <c r="C124" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4193,10 +4235,10 @@
         <v>43</v>
       </c>
       <c r="C125" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4210,10 +4252,10 @@
         <v>43</v>
       </c>
       <c r="C126" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D126" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4227,10 +4269,10 @@
         <v>43</v>
       </c>
       <c r="C127" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D127" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4244,10 +4286,10 @@
         <v>43</v>
       </c>
       <c r="C128" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D128" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4261,10 +4303,10 @@
         <v>43</v>
       </c>
       <c r="C129" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D129" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4278,10 +4320,10 @@
         <v>43</v>
       </c>
       <c r="C130" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D130" t="s">
-        <v>264</v>
+        <v>287</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4295,10 +4337,10 @@
         <v>43</v>
       </c>
       <c r="C131" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D131" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4312,10 +4354,10 @@
         <v>43</v>
       </c>
       <c r="C132" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4329,10 +4371,10 @@
         <v>43</v>
       </c>
       <c r="C133" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D133" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4346,10 +4388,10 @@
         <v>43</v>
       </c>
       <c r="C134" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D134" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4357,16 +4399,16 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B135" t="s">
         <v>43</v>
       </c>
       <c r="C135" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D135" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4380,10 +4422,10 @@
         <v>43</v>
       </c>
       <c r="C136" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D136" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4397,10 +4439,10 @@
         <v>43</v>
       </c>
       <c r="C137" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D137" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4408,16 +4450,16 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B138" t="s">
         <v>43</v>
       </c>
       <c r="C138" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D138" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4431,7 +4473,7 @@
         <v>43</v>
       </c>
       <c r="C139" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D139" t="s">
         <v>293</v>
@@ -4448,7 +4490,7 @@
         <v>43</v>
       </c>
       <c r="C140" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D140" t="s">
         <v>294</v>
@@ -4465,7 +4507,7 @@
         <v>43</v>
       </c>
       <c r="C141" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D141" t="s">
         <v>295</v>
@@ -4482,7 +4524,7 @@
         <v>43</v>
       </c>
       <c r="C142" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D142" t="s">
         <v>296</v>
@@ -4499,7 +4541,7 @@
         <v>43</v>
       </c>
       <c r="C143" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D143" t="s">
         <v>297</v>
@@ -4516,13 +4558,13 @@
         <v>43</v>
       </c>
       <c r="C144" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D144" t="s">
-        <v>283</v>
+        <v>298</v>
       </c>
       <c r="E144">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -4533,13 +4575,13 @@
         <v>43</v>
       </c>
       <c r="C145" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D145" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E145">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -4550,13 +4592,13 @@
         <v>43</v>
       </c>
       <c r="C146" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="D146" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E146">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -4567,13 +4609,13 @@
         <v>43</v>
       </c>
       <c r="C147" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D147" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E147">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -4584,13 +4626,13 @@
         <v>43</v>
       </c>
       <c r="C148" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D148" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E148">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -4601,13 +4643,13 @@
         <v>43</v>
       </c>
       <c r="C149" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D149" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E149">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -4618,13 +4660,13 @@
         <v>43</v>
       </c>
       <c r="C150" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D150" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E150">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -4635,13 +4677,13 @@
         <v>43</v>
       </c>
       <c r="C151" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D151" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="E151">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -4652,166 +4694,166 @@
         <v>43</v>
       </c>
       <c r="C152" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D152" t="s">
         <v>305</v>
       </c>
       <c r="E152">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B153" t="s">
         <v>43</v>
       </c>
       <c r="C153" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D153" t="s">
         <v>306</v>
       </c>
       <c r="E153">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B154" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C154" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D154" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E154">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B155" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C155" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D155" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E155">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B156" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C156" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="D156" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E156">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B157" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C157" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D157" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E157">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B158" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C158" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D158" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E158">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B159" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C159" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D159" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E159">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B160" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C160" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D160" t="s">
-        <v>237</v>
+        <v>312</v>
       </c>
       <c r="E160">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B161" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C161" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D161" t="s">
         <v>313</v>
       </c>
       <c r="E161">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4822,7 +4864,7 @@
         <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D162" t="s">
         <v>314</v>
@@ -4839,7 +4881,7 @@
         <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D163" t="s">
         <v>315</v>
@@ -4856,7 +4898,7 @@
         <v>40</v>
       </c>
       <c r="C164" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D164" t="s">
         <v>316</v>
@@ -4867,13 +4909,13 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B165" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C165" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D165" t="s">
         <v>317</v>
@@ -4890,10 +4932,10 @@
         <v>40</v>
       </c>
       <c r="C166" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="D166" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4907,10 +4949,10 @@
         <v>40</v>
       </c>
       <c r="C167" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D167" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4924,10 +4966,10 @@
         <v>40</v>
       </c>
       <c r="C168" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="D168" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4941,10 +4983,10 @@
         <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D169" t="s">
-        <v>321</v>
+        <v>244</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4958,10 +5000,10 @@
         <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D170" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4975,10 +5017,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D171" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4992,10 +5034,10 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="D172" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5009,10 +5051,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="D173" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5026,10 +5068,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D174" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5043,10 +5085,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D175" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5060,10 +5102,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="D176" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5077,10 +5119,10 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="D177" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5094,10 +5136,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="D178" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5111,10 +5153,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="D179" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5128,10 +5170,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D180" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5145,10 +5187,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="D181" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5162,10 +5204,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="D182" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5179,10 +5221,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="D183" t="s">
-        <v>295</v>
+        <v>333</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5196,10 +5238,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D184" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5213,10 +5255,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="D185" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5230,10 +5272,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D186" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5247,13 +5289,13 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="D187" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E187">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -5264,13 +5306,13 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D188" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E188">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -5281,13 +5323,13 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D189" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E189">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -5298,13 +5340,13 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D190" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E190">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -5315,13 +5357,13 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="D191" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E191">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -5332,13 +5374,13 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="D192" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="E192">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -5349,13 +5391,13 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="D193" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E193">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -5366,13 +5408,13 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="D194" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E194">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -5383,13 +5425,13 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="D195" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E195">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -5400,13 +5442,13 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="D196" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E196">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -5417,10 +5459,10 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="D197" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -5434,10 +5476,10 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="D198" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5451,13 +5493,13 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="D199" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E199">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5468,13 +5510,13 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D200" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E200">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -5485,13 +5527,13 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D201" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E201">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5502,13 +5544,13 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="D202" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E202">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -5519,13 +5561,13 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="D203" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E203">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -5536,13 +5578,13 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="D204" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E204">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5553,13 +5595,13 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="D205" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E205">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5570,13 +5612,13 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="D206" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E206">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5587,13 +5629,13 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D207" t="s">
-        <v>237</v>
+        <v>355</v>
       </c>
       <c r="E207">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5604,13 +5646,13 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="D208" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E208">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5621,13 +5663,13 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="D209" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E209">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5638,13 +5680,13 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="D210" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E210">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5655,13 +5697,13 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="D211" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E211">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5672,13 +5714,13 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="D212" t="s">
         <v>360</v>
       </c>
       <c r="E212">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5689,13 +5731,13 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D213" t="s">
         <v>361</v>
       </c>
       <c r="E213">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5706,13 +5748,13 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="D214" t="s">
         <v>362</v>
       </c>
       <c r="E214">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5723,13 +5765,13 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="D215" t="s">
         <v>363</v>
       </c>
       <c r="E215">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5740,13 +5782,13 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="D216" t="s">
-        <v>364</v>
+        <v>244</v>
       </c>
       <c r="E216">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5757,13 +5799,285 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
+        <v>206</v>
+      </c>
+      <c r="D217" t="s">
+        <v>364</v>
+      </c>
+      <c r="E217">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5">
+      <c r="A218" t="s">
+        <v>17</v>
+      </c>
+      <c r="B218" t="s">
+        <v>40</v>
+      </c>
+      <c r="C218" t="s">
+        <v>207</v>
+      </c>
+      <c r="D218" t="s">
+        <v>365</v>
+      </c>
+      <c r="E218">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5">
+      <c r="A219" t="s">
+        <v>17</v>
+      </c>
+      <c r="B219" t="s">
+        <v>40</v>
+      </c>
+      <c r="C219" t="s">
+        <v>208</v>
+      </c>
+      <c r="D219" t="s">
+        <v>366</v>
+      </c>
+      <c r="E219">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5">
+      <c r="A220" t="s">
+        <v>17</v>
+      </c>
+      <c r="B220" t="s">
+        <v>40</v>
+      </c>
+      <c r="C220" t="s">
+        <v>209</v>
+      </c>
+      <c r="D220" t="s">
+        <v>367</v>
+      </c>
+      <c r="E220">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5">
+      <c r="A221" t="s">
+        <v>17</v>
+      </c>
+      <c r="B221" t="s">
+        <v>40</v>
+      </c>
+      <c r="C221" t="s">
+        <v>210</v>
+      </c>
+      <c r="D221" t="s">
+        <v>367</v>
+      </c>
+      <c r="E221">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5">
+      <c r="A222" t="s">
+        <v>17</v>
+      </c>
+      <c r="B222" t="s">
+        <v>40</v>
+      </c>
+      <c r="C222" t="s">
+        <v>211</v>
+      </c>
+      <c r="D222" t="s">
+        <v>368</v>
+      </c>
+      <c r="E222">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5">
+      <c r="A223" t="s">
+        <v>17</v>
+      </c>
+      <c r="B223" t="s">
+        <v>40</v>
+      </c>
+      <c r="C223" t="s">
+        <v>212</v>
+      </c>
+      <c r="D223" t="s">
+        <v>369</v>
+      </c>
+      <c r="E223">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5">
+      <c r="A224" t="s">
+        <v>17</v>
+      </c>
+      <c r="B224" t="s">
+        <v>40</v>
+      </c>
+      <c r="C224" t="s">
+        <v>213</v>
+      </c>
+      <c r="D224" t="s">
+        <v>370</v>
+      </c>
+      <c r="E224">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5">
+      <c r="A225" t="s">
+        <v>17</v>
+      </c>
+      <c r="B225" t="s">
+        <v>40</v>
+      </c>
+      <c r="C225" t="s">
+        <v>214</v>
+      </c>
+      <c r="D225" t="s">
+        <v>371</v>
+      </c>
+      <c r="E225">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
+      <c r="A226" t="s">
+        <v>17</v>
+      </c>
+      <c r="B226" t="s">
+        <v>40</v>
+      </c>
+      <c r="C226" t="s">
         <v>215</v>
       </c>
-      <c r="D217" t="s">
-        <v>365</v>
-      </c>
-      <c r="E217">
+      <c r="D226" t="s">
+        <v>372</v>
+      </c>
+      <c r="E226">
         <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
+      <c r="A227" t="s">
+        <v>16</v>
+      </c>
+      <c r="B227" t="s">
+        <v>43</v>
+      </c>
+      <c r="C227" t="s">
+        <v>216</v>
+      </c>
+      <c r="D227" t="s">
+        <v>373</v>
+      </c>
+      <c r="E227">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
+      <c r="A228" t="s">
+        <v>13</v>
+      </c>
+      <c r="B228" t="s">
+        <v>42</v>
+      </c>
+      <c r="C228" t="s">
+        <v>217</v>
+      </c>
+      <c r="D228" t="s">
+        <v>374</v>
+      </c>
+      <c r="E228">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5">
+      <c r="A229" t="s">
+        <v>16</v>
+      </c>
+      <c r="B229" t="s">
+        <v>43</v>
+      </c>
+      <c r="C229" t="s">
+        <v>218</v>
+      </c>
+      <c r="D229" t="s">
+        <v>375</v>
+      </c>
+      <c r="E229">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
+      <c r="A230" t="s">
+        <v>7</v>
+      </c>
+      <c r="B230" t="s">
+        <v>37</v>
+      </c>
+      <c r="C230" t="s">
+        <v>219</v>
+      </c>
+      <c r="D230" t="s">
+        <v>376</v>
+      </c>
+      <c r="E230">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5">
+      <c r="A231" t="s">
+        <v>16</v>
+      </c>
+      <c r="B231" t="s">
+        <v>43</v>
+      </c>
+      <c r="C231" t="s">
+        <v>220</v>
+      </c>
+      <c r="D231" t="s">
+        <v>377</v>
+      </c>
+      <c r="E231">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5">
+      <c r="A232" t="s">
+        <v>16</v>
+      </c>
+      <c r="B232" t="s">
+        <v>43</v>
+      </c>
+      <c r="C232" t="s">
+        <v>221</v>
+      </c>
+      <c r="D232" t="s">
+        <v>378</v>
+      </c>
+      <c r="E232">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5">
+      <c r="A233" t="s">
+        <v>14</v>
+      </c>
+      <c r="B233" t="s">
+        <v>43</v>
+      </c>
+      <c r="C233" t="s">
+        <v>222</v>
+      </c>
+      <c r="D233" t="s">
+        <v>379</v>
+      </c>
+      <c r="E233">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (22/07/2026 12:01)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="372">
   <si>
     <t>matricula</t>
   </si>
@@ -203,15 +203,9 @@
     <t>C611008-0101</t>
   </si>
   <si>
-    <t>066-3114-00</t>
-  </si>
-  <si>
     <t>3122678-04</t>
   </si>
   <si>
-    <t>850C86-2</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -452,9 +446,6 @@
     <t>2650032-4</t>
   </si>
   <si>
-    <t>011-00883-20</t>
-  </si>
-  <si>
     <t>ADAS-C-031-1</t>
   </si>
   <si>
@@ -695,15 +686,9 @@
     <t>ALTERNATOR CONTROL UNIT ASSY</t>
   </si>
   <si>
-    <t>IND RDR 2000</t>
-  </si>
-  <si>
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
-    <t>PNEU PRINCIPAL 8.50-10 08PR TT FCIII MLG</t>
-  </si>
-  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
@@ -936,9 +921,6 @@
   </si>
   <si>
     <t>BRACKET</t>
-  </si>
-  <si>
-    <t>RADAR GWX 68 WEATHER</t>
   </si>
   <si>
     <t>PORT ASSY DOWNLOAD</t>
@@ -1155,8 +1137,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1172,7 +1162,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1180,12 +1170,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1484,22 +1492,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1517,10 +1525,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1531,16 +1539,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1591,16 +1599,16 @@
         <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
         <v>53</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1717,10 +1725,10 @@
         <v>54</v>
       </c>
       <c r="E12">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F12">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1737,10 +1745,10 @@
         <v>54</v>
       </c>
       <c r="E13">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F13">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2110,23 +2118,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2141,7 +2149,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2158,7 +2166,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2175,7 +2183,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2192,7 +2200,7 @@
         <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2209,7 +2217,7 @@
         <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2226,7 +2234,7 @@
         <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2243,7 +2251,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2260,7 +2268,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2277,7 +2285,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2285,16 +2293,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2302,16 +2310,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2319,16 +2327,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2336,16 +2344,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2353,16 +2361,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
         <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2370,16 +2378,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2387,16 +2395,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2404,16 +2412,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D18" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2421,16 +2429,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B19" t="s">
         <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2438,16 +2446,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2455,16 +2463,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2472,16 +2480,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2489,16 +2497,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
         <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2506,16 +2514,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2523,16 +2531,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2540,16 +2548,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2557,16 +2565,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2574,16 +2582,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
         <v>43</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2591,16 +2599,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2608,16 +2616,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B30" t="s">
         <v>43</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2625,16 +2633,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2642,16 +2650,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2659,16 +2667,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2676,16 +2684,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D34" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2693,16 +2701,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2716,13 +2724,13 @@
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2733,10 +2741,10 @@
         <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2744,19 +2752,19 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s">
         <v>70</v>
       </c>
       <c r="D38" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2770,7 +2778,7 @@
         <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2787,7 +2795,7 @@
         <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2804,41 +2812,41 @@
         <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2846,33 +2854,33 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2880,16 +2888,16 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2897,33 +2905,33 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D47" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B48" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2931,33 +2939,33 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B49" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D49" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D50" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -2965,19 +2973,19 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D51" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2988,13 +2996,13 @@
         <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D52" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3005,10 +3013,10 @@
         <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D53" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -3016,19 +3024,19 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
         <v>78</v>
       </c>
       <c r="D54" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3042,7 +3050,7 @@
         <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3059,27 +3067,27 @@
         <v>80</v>
       </c>
       <c r="D56" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D57" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3090,10 +3098,10 @@
         <v>41</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="E58">
         <v>4</v>
@@ -3101,24 +3109,24 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C59" t="s">
         <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E59">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
         <v>41</v>
@@ -3127,24 +3135,24 @@
         <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C61" t="s">
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3152,16 +3160,16 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3169,16 +3177,16 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B63" t="s">
         <v>43</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D63" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3186,16 +3194,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
         <v>43</v>
       </c>
       <c r="C64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3203,16 +3211,16 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B65" t="s">
         <v>43</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D65" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3220,16 +3228,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B66" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D66" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3243,10 +3251,10 @@
         <v>43</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3254,16 +3262,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B68" t="s">
         <v>43</v>
       </c>
       <c r="C68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D68" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -3271,7 +3279,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
         <v>43</v>
@@ -3280,7 +3288,7 @@
         <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -3288,16 +3296,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B70" t="s">
         <v>43</v>
       </c>
       <c r="C70" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D70" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -3305,7 +3313,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B71" t="s">
         <v>43</v>
@@ -3314,7 +3322,7 @@
         <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3331,15 +3339,15 @@
         <v>89</v>
       </c>
       <c r="D72" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E72">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B73" t="s">
         <v>43</v>
@@ -3348,41 +3356,41 @@
         <v>89</v>
       </c>
       <c r="D73" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B74" t="s">
         <v>43</v>
       </c>
       <c r="C74" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B75" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3390,16 +3398,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
         <v>43</v>
       </c>
       <c r="C76" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3407,16 +3415,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B77" t="s">
         <v>43</v>
       </c>
       <c r="C77" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3424,16 +3432,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C78" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3441,16 +3449,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B79" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E79">
         <v>2</v>
@@ -3458,16 +3466,16 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
         <v>43</v>
       </c>
       <c r="C80" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D80" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3475,16 +3483,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B81" t="s">
         <v>43</v>
       </c>
       <c r="C81" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D81" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E81">
         <v>2</v>
@@ -3492,16 +3500,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B82" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C82" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D82" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E82">
         <v>2</v>
@@ -3515,10 +3523,10 @@
         <v>43</v>
       </c>
       <c r="C83" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D83" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E83">
         <v>2</v>
@@ -3532,10 +3540,10 @@
         <v>43</v>
       </c>
       <c r="C84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D84" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E84">
         <v>2</v>
@@ -3549,52 +3557,52 @@
         <v>43</v>
       </c>
       <c r="C85" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D85" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E85">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B86" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D86" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
         <v>43</v>
       </c>
       <c r="C87" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D87" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B88" t="s">
         <v>43</v>
@@ -3603,44 +3611,44 @@
         <v>94</v>
       </c>
       <c r="D88" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E88">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C89" t="s">
         <v>94</v>
       </c>
       <c r="D89" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E89">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B90" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="E90">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -3651,10 +3659,10 @@
         <v>43</v>
       </c>
       <c r="C91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D91" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3668,10 +3676,10 @@
         <v>43</v>
       </c>
       <c r="C92" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3685,13 +3693,13 @@
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D93" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E93">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3702,10 +3710,10 @@
         <v>43</v>
       </c>
       <c r="C94" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3719,10 +3727,10 @@
         <v>43</v>
       </c>
       <c r="C95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D95" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3730,33 +3738,33 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B96" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C96" t="s">
         <v>97</v>
       </c>
       <c r="D96" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E96">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B97" t="s">
         <v>43</v>
       </c>
       <c r="C97" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D97" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3764,7 +3772,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B98" t="s">
         <v>43</v>
@@ -3773,7 +3781,7 @@
         <v>98</v>
       </c>
       <c r="D98" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3781,16 +3789,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B99" t="s">
         <v>43</v>
       </c>
       <c r="C99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D99" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3798,7 +3806,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B100" t="s">
         <v>43</v>
@@ -3807,7 +3815,7 @@
         <v>99</v>
       </c>
       <c r="D100" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3815,16 +3823,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B101" t="s">
         <v>43</v>
       </c>
       <c r="C101" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D101" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3832,7 +3840,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B102" t="s">
         <v>43</v>
@@ -3841,7 +3849,7 @@
         <v>100</v>
       </c>
       <c r="D102" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3849,16 +3857,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B103" t="s">
         <v>43</v>
       </c>
       <c r="C103" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D103" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3866,7 +3874,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B104" t="s">
         <v>43</v>
@@ -3875,7 +3883,7 @@
         <v>101</v>
       </c>
       <c r="D104" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3883,16 +3891,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
         <v>43</v>
       </c>
       <c r="C105" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D105" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3900,7 +3908,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B106" t="s">
         <v>43</v>
@@ -3909,7 +3917,7 @@
         <v>102</v>
       </c>
       <c r="D106" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3917,16 +3925,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B107" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D107" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3934,7 +3942,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B108" t="s">
         <v>43</v>
@@ -3943,7 +3951,7 @@
         <v>103</v>
       </c>
       <c r="D108" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3951,16 +3959,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B109" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D109" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3968,16 +3976,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B110" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C110" t="s">
         <v>104</v>
       </c>
       <c r="D110" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3994,7 +4002,7 @@
         <v>105</v>
       </c>
       <c r="D111" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4002,16 +4010,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B112" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C112" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D112" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4025,10 +4033,10 @@
         <v>43</v>
       </c>
       <c r="C113" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D113" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E113">
         <v>1</v>
@@ -4042,10 +4050,10 @@
         <v>43</v>
       </c>
       <c r="C114" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D114" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E114">
         <v>1</v>
@@ -4059,10 +4067,10 @@
         <v>43</v>
       </c>
       <c r="C115" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D115" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E115">
         <v>1</v>
@@ -4076,18 +4084,18 @@
         <v>43</v>
       </c>
       <c r="C116" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D116" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E116">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B117" t="s">
         <v>43</v>
@@ -4096,7 +4104,7 @@
         <v>110</v>
       </c>
       <c r="D117" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E117">
         <v>1</v>
@@ -4113,24 +4121,24 @@
         <v>111</v>
       </c>
       <c r="D118" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E118">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B119" t="s">
         <v>43</v>
       </c>
       <c r="C119" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D119" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4138,7 +4146,7 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B120" t="s">
         <v>43</v>
@@ -4147,32 +4155,32 @@
         <v>112</v>
       </c>
       <c r="D120" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E120">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B121" t="s">
         <v>43</v>
       </c>
       <c r="C121" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D121" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B122" t="s">
         <v>43</v>
@@ -4181,7 +4189,7 @@
         <v>113</v>
       </c>
       <c r="D122" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4198,7 +4206,7 @@
         <v>114</v>
       </c>
       <c r="D123" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4206,19 +4214,19 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B124" t="s">
         <v>43</v>
       </c>
       <c r="C124" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D124" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E124">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4229,13 +4237,13 @@
         <v>43</v>
       </c>
       <c r="C125" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D125" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4246,13 +4254,13 @@
         <v>43</v>
       </c>
       <c r="C126" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D126" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E126">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4263,18 +4271,18 @@
         <v>43</v>
       </c>
       <c r="C127" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D127" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E127">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B128" t="s">
         <v>43</v>
@@ -4283,15 +4291,15 @@
         <v>118</v>
       </c>
       <c r="D128" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E128">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B129" t="s">
         <v>43</v>
@@ -4300,27 +4308,27 @@
         <v>119</v>
       </c>
       <c r="D129" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E129">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B130" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C130" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D130" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E130">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -4334,10 +4342,10 @@
         <v>120</v>
       </c>
       <c r="D131" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -4351,7 +4359,7 @@
         <v>121</v>
       </c>
       <c r="D132" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4359,16 +4367,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B133" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C133" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D133" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4382,10 +4390,10 @@
         <v>43</v>
       </c>
       <c r="C134" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D134" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4399,10 +4407,10 @@
         <v>43</v>
       </c>
       <c r="C135" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D135" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4416,10 +4424,10 @@
         <v>43</v>
       </c>
       <c r="C136" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D136" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4433,10 +4441,10 @@
         <v>43</v>
       </c>
       <c r="C137" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D137" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4450,10 +4458,10 @@
         <v>43</v>
       </c>
       <c r="C138" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D138" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4467,10 +4475,10 @@
         <v>43</v>
       </c>
       <c r="C139" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D139" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4484,10 +4492,10 @@
         <v>43</v>
       </c>
       <c r="C140" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D140" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4501,10 +4509,10 @@
         <v>43</v>
       </c>
       <c r="C141" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D141" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4518,10 +4526,10 @@
         <v>43</v>
       </c>
       <c r="C142" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D142" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4535,10 +4543,10 @@
         <v>43</v>
       </c>
       <c r="C143" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D143" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4552,10 +4560,10 @@
         <v>43</v>
       </c>
       <c r="C144" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D144" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4569,10 +4577,10 @@
         <v>43</v>
       </c>
       <c r="C145" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D145" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4586,10 +4594,10 @@
         <v>43</v>
       </c>
       <c r="C146" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D146" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4603,10 +4611,10 @@
         <v>43</v>
       </c>
       <c r="C147" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D147" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4620,10 +4628,10 @@
         <v>43</v>
       </c>
       <c r="C148" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D148" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4637,10 +4645,10 @@
         <v>43</v>
       </c>
       <c r="C149" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D149" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4654,10 +4662,10 @@
         <v>43</v>
       </c>
       <c r="C150" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D150" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4671,10 +4679,10 @@
         <v>43</v>
       </c>
       <c r="C151" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D151" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4688,10 +4696,10 @@
         <v>43</v>
       </c>
       <c r="C152" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D152" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4705,10 +4713,10 @@
         <v>43</v>
       </c>
       <c r="C153" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D153" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4722,10 +4730,10 @@
         <v>43</v>
       </c>
       <c r="C154" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D154" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4739,10 +4747,10 @@
         <v>43</v>
       </c>
       <c r="C155" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D155" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4756,10 +4764,10 @@
         <v>43</v>
       </c>
       <c r="C156" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D156" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4773,10 +4781,10 @@
         <v>43</v>
       </c>
       <c r="C157" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D157" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4790,13 +4798,13 @@
         <v>43</v>
       </c>
       <c r="C158" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D158" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="E158">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -4807,13 +4815,13 @@
         <v>43</v>
       </c>
       <c r="C159" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D159" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E159">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4824,13 +4832,13 @@
         <v>43</v>
       </c>
       <c r="C160" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D160" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E160">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4841,13 +4849,13 @@
         <v>43</v>
       </c>
       <c r="C161" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D161" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E161">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4858,10 +4866,10 @@
         <v>43</v>
       </c>
       <c r="C162" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D162" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4875,13 +4883,13 @@
         <v>43</v>
       </c>
       <c r="C163" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D163" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E163">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4892,13 +4900,13 @@
         <v>43</v>
       </c>
       <c r="C164" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D164" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E164">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4909,13 +4917,13 @@
         <v>43</v>
       </c>
       <c r="C165" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D165" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="E165">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4926,81 +4934,81 @@
         <v>43</v>
       </c>
       <c r="C166" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D166" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E166">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B167" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D167" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E167">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B168" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D168" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E168">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B169" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D169" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E169">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B170" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D170" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E170">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5011,10 +5019,10 @@
         <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D171" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5028,10 +5036,10 @@
         <v>39</v>
       </c>
       <c r="C172" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D172" t="s">
-        <v>321</v>
+        <v>239</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5045,10 +5053,10 @@
         <v>39</v>
       </c>
       <c r="C173" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D173" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5062,10 +5070,10 @@
         <v>39</v>
       </c>
       <c r="C174" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D174" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5079,10 +5087,10 @@
         <v>39</v>
       </c>
       <c r="C175" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D175" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5096,10 +5104,10 @@
         <v>39</v>
       </c>
       <c r="C176" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D176" t="s">
-        <v>244</v>
+        <v>322</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5113,10 +5121,10 @@
         <v>39</v>
       </c>
       <c r="C177" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D177" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5130,10 +5138,10 @@
         <v>39</v>
       </c>
       <c r="C178" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D178" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5147,10 +5155,10 @@
         <v>39</v>
       </c>
       <c r="C179" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D179" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5164,10 +5172,10 @@
         <v>39</v>
       </c>
       <c r="C180" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D180" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5181,10 +5189,10 @@
         <v>39</v>
       </c>
       <c r="C181" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D181" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5198,10 +5206,10 @@
         <v>39</v>
       </c>
       <c r="C182" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D182" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5215,10 +5223,10 @@
         <v>39</v>
       </c>
       <c r="C183" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5232,10 +5240,10 @@
         <v>39</v>
       </c>
       <c r="C184" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D184" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5249,10 +5257,10 @@
         <v>39</v>
       </c>
       <c r="C185" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D185" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5266,10 +5274,10 @@
         <v>39</v>
       </c>
       <c r="C186" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D186" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5283,10 +5291,10 @@
         <v>39</v>
       </c>
       <c r="C187" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D187" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5300,10 +5308,10 @@
         <v>39</v>
       </c>
       <c r="C188" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D188" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5317,10 +5325,10 @@
         <v>39</v>
       </c>
       <c r="C189" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D189" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5334,10 +5342,10 @@
         <v>39</v>
       </c>
       <c r="C190" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D190" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5351,10 +5359,10 @@
         <v>39</v>
       </c>
       <c r="C191" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D191" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5368,10 +5376,10 @@
         <v>39</v>
       </c>
       <c r="C192" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D192" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5385,10 +5393,10 @@
         <v>39</v>
       </c>
       <c r="C193" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D193" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5402,10 +5410,10 @@
         <v>39</v>
       </c>
       <c r="C194" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D194" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5419,10 +5427,10 @@
         <v>39</v>
       </c>
       <c r="C195" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D195" t="s">
-        <v>343</v>
+        <v>301</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5436,10 +5444,10 @@
         <v>39</v>
       </c>
       <c r="C196" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D196" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5453,10 +5461,10 @@
         <v>39</v>
       </c>
       <c r="C197" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D197" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5470,10 +5478,10 @@
         <v>39</v>
       </c>
       <c r="C198" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D198" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5487,10 +5495,10 @@
         <v>39</v>
       </c>
       <c r="C199" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D199" t="s">
-        <v>306</v>
+        <v>344</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5504,13 +5512,13 @@
         <v>39</v>
       </c>
       <c r="C200" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D200" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="E200">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -5521,13 +5529,13 @@
         <v>39</v>
       </c>
       <c r="C201" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D201" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E201">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5538,13 +5546,13 @@
         <v>39</v>
       </c>
       <c r="C202" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D202" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E202">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -5555,13 +5563,13 @@
         <v>39</v>
       </c>
       <c r="C203" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D203" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E203">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -5572,10 +5580,10 @@
         <v>39</v>
       </c>
       <c r="C204" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D204" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5589,10 +5597,10 @@
         <v>39</v>
       </c>
       <c r="C205" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D205" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5606,10 +5614,10 @@
         <v>39</v>
       </c>
       <c r="C206" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D206" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5623,10 +5631,10 @@
         <v>39</v>
       </c>
       <c r="C207" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D207" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5640,10 +5648,10 @@
         <v>39</v>
       </c>
       <c r="C208" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D208" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5657,10 +5665,10 @@
         <v>39</v>
       </c>
       <c r="C209" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D209" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5674,10 +5682,10 @@
         <v>39</v>
       </c>
       <c r="C210" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D210" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5691,10 +5699,10 @@
         <v>39</v>
       </c>
       <c r="C211" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D211" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5708,13 +5716,13 @@
         <v>39</v>
       </c>
       <c r="C212" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D212" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E212">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5725,13 +5733,13 @@
         <v>39</v>
       </c>
       <c r="C213" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D213" t="s">
-        <v>359</v>
+        <v>239</v>
       </c>
       <c r="E213">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5742,13 +5750,13 @@
         <v>39</v>
       </c>
       <c r="C214" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D214" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E214">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5759,13 +5767,13 @@
         <v>39</v>
       </c>
       <c r="C215" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D215" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E215">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5776,13 +5784,13 @@
         <v>39</v>
       </c>
       <c r="C216" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D216" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E216">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5793,13 +5801,13 @@
         <v>39</v>
       </c>
       <c r="C217" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D217" t="s">
-        <v>244</v>
+        <v>360</v>
       </c>
       <c r="E217">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5810,10 +5818,10 @@
         <v>39</v>
       </c>
       <c r="C218" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D218" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -5827,13 +5835,13 @@
         <v>39</v>
       </c>
       <c r="C219" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D219" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E219">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5844,13 +5852,13 @@
         <v>39</v>
       </c>
       <c r="C220" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D220" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E220">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5861,13 +5869,13 @@
         <v>39</v>
       </c>
       <c r="C221" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D221" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E221">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5878,13 +5886,13 @@
         <v>39</v>
       </c>
       <c r="C222" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D222" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E222">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5895,13 +5903,13 @@
         <v>39</v>
       </c>
       <c r="C223" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D223" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E223">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5912,13 +5920,13 @@
         <v>39</v>
       </c>
       <c r="C224" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D224" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="E224">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5929,13 +5937,13 @@
         <v>39</v>
       </c>
       <c r="C225" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D225" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="E225">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5946,13 +5954,13 @@
         <v>39</v>
       </c>
       <c r="C226" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D226" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E226">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -5963,13 +5971,13 @@
         <v>39</v>
       </c>
       <c r="C227" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D227" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="E227">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -5980,13 +5988,13 @@
         <v>39</v>
       </c>
       <c r="C228" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D228" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E228">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -5997,80 +6005,12 @@
         <v>39</v>
       </c>
       <c r="C229" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D229" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="E229">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="230" spans="1:5">
-      <c r="A230" t="s">
-        <v>17</v>
-      </c>
-      <c r="B230" t="s">
-        <v>39</v>
-      </c>
-      <c r="C230" t="s">
-        <v>218</v>
-      </c>
-      <c r="D230" t="s">
-        <v>374</v>
-      </c>
-      <c r="E230">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="231" spans="1:5">
-      <c r="A231" t="s">
-        <v>17</v>
-      </c>
-      <c r="B231" t="s">
-        <v>39</v>
-      </c>
-      <c r="C231" t="s">
-        <v>219</v>
-      </c>
-      <c r="D231" t="s">
-        <v>375</v>
-      </c>
-      <c r="E231">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="232" spans="1:5">
-      <c r="A232" t="s">
-        <v>17</v>
-      </c>
-      <c r="B232" t="s">
-        <v>39</v>
-      </c>
-      <c r="C232" t="s">
-        <v>220</v>
-      </c>
-      <c r="D232" t="s">
-        <v>376</v>
-      </c>
-      <c r="E232">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="233" spans="1:5">
-      <c r="A233" t="s">
-        <v>17</v>
-      </c>
-      <c r="B233" t="s">
-        <v>39</v>
-      </c>
-      <c r="C233" t="s">
-        <v>221</v>
-      </c>
-      <c r="D233" t="s">
-        <v>377</v>
-      </c>
-      <c r="E233">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -38,60 +38,60 @@
     <t>2721</t>
   </si>
   <si>
+    <t>2723</t>
+  </si>
+  <si>
+    <t>2733</t>
+  </si>
+  <si>
+    <t>2728</t>
+  </si>
+  <si>
+    <t>2729</t>
+  </si>
+  <si>
+    <t>2741</t>
+  </si>
+  <si>
+    <t>2732</t>
+  </si>
+  <si>
+    <t>2730</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>2726</t>
+  </si>
+  <si>
+    <t>2702</t>
+  </si>
+  <si>
+    <t>2703</t>
+  </si>
+  <si>
+    <t>2704</t>
+  </si>
+  <si>
+    <t>2708</t>
+  </si>
+  <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>2719</t>
+  </si>
+  <si>
+    <t>2720</t>
+  </si>
+  <si>
     <t>2722</t>
   </si>
   <si>
-    <t>2723</t>
-  </si>
-  <si>
-    <t>2733</t>
-  </si>
-  <si>
     <t>2727</t>
   </si>
   <si>
-    <t>2728</t>
-  </si>
-  <si>
-    <t>2729</t>
-  </si>
-  <si>
-    <t>2741</t>
-  </si>
-  <si>
-    <t>2732</t>
-  </si>
-  <si>
-    <t>2730</t>
-  </si>
-  <si>
-    <t>2734</t>
-  </si>
-  <si>
-    <t>2726</t>
-  </si>
-  <si>
-    <t>2702</t>
-  </si>
-  <si>
-    <t>2703</t>
-  </si>
-  <si>
-    <t>2704</t>
-  </si>
-  <si>
-    <t>2708</t>
-  </si>
-  <si>
-    <t>2709</t>
-  </si>
-  <si>
-    <t>2719</t>
-  </si>
-  <si>
-    <t>2720</t>
-  </si>
-  <si>
     <t>2731</t>
   </si>
   <si>
@@ -128,33 +128,33 @@
     <t>6º ETA</t>
   </si>
   <si>
+    <t>CLA</t>
+  </si>
+  <si>
+    <t>1º ETA</t>
+  </si>
+  <si>
+    <t>1º/5º GAV</t>
+  </si>
+  <si>
+    <t>BABV</t>
+  </si>
+  <si>
+    <t>7º ETA</t>
+  </si>
+  <si>
+    <t>EPCAR</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
     <t>2ª ETA</t>
   </si>
   <si>
-    <t>CLA</t>
-  </si>
-  <si>
-    <t>1º ETA</t>
-  </si>
-  <si>
     <t>1/15 GAV</t>
   </si>
   <si>
-    <t>1º/5º GAV</t>
-  </si>
-  <si>
-    <t>BABV</t>
-  </si>
-  <si>
-    <t>7º ETA</t>
-  </si>
-  <si>
-    <t>EPCAR</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
     <t>1ª ETA</t>
   </si>
   <si>
@@ -194,75 +194,75 @@
     <t>066-3046-07</t>
   </si>
   <si>
+    <t>C611505-0201</t>
+  </si>
+  <si>
     <t>3044000</t>
   </si>
   <si>
     <t>C145-00-46</t>
   </si>
   <si>
+    <t>3122678-04</t>
+  </si>
+  <si>
+    <t>P7036368-01</t>
+  </si>
+  <si>
+    <t>2643007-1</t>
+  </si>
+  <si>
+    <t>2651022-20-1</t>
+  </si>
+  <si>
+    <t>2641014-5</t>
+  </si>
+  <si>
+    <t>2641011-5</t>
+  </si>
+  <si>
+    <t>2643100-206</t>
+  </si>
+  <si>
+    <t>162-10700</t>
+  </si>
+  <si>
+    <t>D20B-14489-KA</t>
+  </si>
+  <si>
+    <t>400454</t>
+  </si>
+  <si>
+    <t>AE3663163K0600</t>
+  </si>
+  <si>
+    <t>2641013-6</t>
+  </si>
+  <si>
+    <t>2611112-2</t>
+  </si>
+  <si>
+    <t>2601119-1</t>
+  </si>
+  <si>
+    <t>154-03000</t>
+  </si>
+  <si>
+    <t>2621013-2</t>
+  </si>
+  <si>
+    <t>067-06300</t>
+  </si>
+  <si>
+    <t>M81934/2-32C032</t>
+  </si>
+  <si>
+    <t>2611137-7</t>
+  </si>
+  <si>
     <t>C611008-0101</t>
   </si>
   <si>
-    <t>3122678-04</t>
-  </si>
-  <si>
-    <t>C611505-0201</t>
-  </si>
-  <si>
-    <t>P7036368-01</t>
-  </si>
-  <si>
-    <t>2643007-1</t>
-  </si>
-  <si>
-    <t>2651022-20-1</t>
-  </si>
-  <si>
-    <t>2641014-5</t>
-  </si>
-  <si>
-    <t>2641011-5</t>
-  </si>
-  <si>
-    <t>2643100-206</t>
-  </si>
-  <si>
-    <t>162-10700</t>
-  </si>
-  <si>
-    <t>D20B-14489-KA</t>
-  </si>
-  <si>
-    <t>400454</t>
-  </si>
-  <si>
-    <t>AE3663163K0600</t>
-  </si>
-  <si>
-    <t>2641013-6</t>
-  </si>
-  <si>
-    <t>2611112-2</t>
-  </si>
-  <si>
-    <t>2601119-1</t>
-  </si>
-  <si>
-    <t>154-03000</t>
-  </si>
-  <si>
-    <t>2621013-2</t>
-  </si>
-  <si>
-    <t>067-06300</t>
-  </si>
-  <si>
-    <t>M81934/2-32C032</t>
-  </si>
-  <si>
-    <t>2611137-7</t>
-  </si>
-  <si>
     <t>3011755</t>
   </si>
   <si>
@@ -677,73 +677,73 @@
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
+    <t>ALTERNATOR</t>
+  </si>
+  <si>
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
     <t>TRANSMISSION ASSY</t>
   </si>
   <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>PROPELLER ASSEMBLY</t>
+  </si>
+  <si>
+    <t>SHIMMY DAMP AS</t>
+  </si>
+  <si>
+    <t>RING ASSY ENGI</t>
+  </si>
+  <si>
+    <t>SPRING-MAIN GEAR CEN</t>
+  </si>
+  <si>
+    <t>AXLE-MAIN GEAR</t>
+  </si>
+  <si>
+    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+  </si>
+  <si>
+    <t>OUTER WHEEL HALF ASSY</t>
+  </si>
+  <si>
+    <t>SLEEVE</t>
+  </si>
+  <si>
+    <t>SEAL,PLAIN ENCASED</t>
+  </si>
+  <si>
+    <t>HOSE ASSY</t>
+  </si>
+  <si>
+    <t>SPRING-MAIN GEAR LH &amp; RH</t>
+  </si>
+  <si>
+    <t>STRAP</t>
+  </si>
+  <si>
+    <t>JACK PAD LH</t>
+  </si>
+  <si>
+    <t>SEAL MOLDED</t>
+  </si>
+  <si>
+    <t>SPACER</t>
+  </si>
+  <si>
+    <t>SPACER MAIN GE</t>
+  </si>
+  <si>
+    <t>BEARING,SLEEVE</t>
+  </si>
+  <si>
+    <t>CAP MAIN LAND</t>
+  </si>
+  <si>
     <t>ALTERNATOR CONTROL UNIT ASSY</t>
-  </si>
-  <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
-    <t>ALTERNATOR</t>
-  </si>
-  <si>
-    <t>PROPELLER ASSEMBLY</t>
-  </si>
-  <si>
-    <t>SHIMMY DAMP AS</t>
-  </si>
-  <si>
-    <t>RING ASSY ENGI</t>
-  </si>
-  <si>
-    <t>SPRING-MAIN GEAR CEN</t>
-  </si>
-  <si>
-    <t>AXLE-MAIN GEAR</t>
-  </si>
-  <si>
-    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
-  </si>
-  <si>
-    <t>OUTER WHEEL HALF ASSY</t>
-  </si>
-  <si>
-    <t>SLEEVE</t>
-  </si>
-  <si>
-    <t>SEAL,PLAIN ENCASED</t>
-  </si>
-  <si>
-    <t>HOSE ASSY</t>
-  </si>
-  <si>
-    <t>SPRING-MAIN GEAR LH &amp; RH</t>
-  </si>
-  <si>
-    <t>STRAP</t>
-  </si>
-  <si>
-    <t>JACK PAD LH</t>
-  </si>
-  <si>
-    <t>SEAL MOLDED</t>
-  </si>
-  <si>
-    <t>SPACER</t>
-  </si>
-  <si>
-    <t>SPACER MAIN GE</t>
-  </si>
-  <si>
-    <t>BEARING,SLEEVE</t>
-  </si>
-  <si>
-    <t>CAP MAIN LAND</t>
   </si>
   <si>
     <t>INSULATION BLANKET,T</t>
@@ -1137,16 +1137,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1162,7 +1154,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1170,30 +1162,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1492,22 +1466,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1539,16 +1513,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1565,10 +1539,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1585,10 +1559,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1596,19 +1570,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
         <v>53</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1616,7 +1590,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
@@ -1625,10 +1599,10 @@
         <v>53</v>
       </c>
       <c r="E7">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1642,13 +1616,13 @@
         <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1656,19 +1630,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1676,7 +1650,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>50</v>
@@ -1685,10 +1659,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="F10">
-        <v>27</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1696,7 +1670,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
         <v>50</v>
@@ -1705,10 +1679,10 @@
         <v>54</v>
       </c>
       <c r="E11">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="F11">
-        <v>91</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1716,19 +1690,19 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>144</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1739,16 +1713,16 @@
         <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E13">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1756,7 +1730,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1776,7 +1750,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1796,7 +1770,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1816,7 +1790,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1856,7 +1830,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1876,7 +1850,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1916,7 +1890,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
@@ -1936,7 +1910,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
         <v>51</v>
@@ -1976,7 +1950,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -1996,7 +1970,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
         <v>51</v>
@@ -2056,7 +2030,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
@@ -2076,7 +2050,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
@@ -2096,7 +2070,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C31" t="s">
         <v>52</v>
@@ -2122,19 +2096,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2157,10 +2131,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
         <v>58</v>
@@ -2191,10 +2165,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>59</v>
@@ -2208,10 +2182,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
         <v>59</v>
@@ -2225,10 +2199,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
         <v>59</v>
@@ -2242,10 +2216,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
@@ -2259,10 +2233,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>59</v>
@@ -2293,16 +2267,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2310,16 +2284,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2327,16 +2301,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2344,16 +2318,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2361,16 +2335,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2378,16 +2352,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2395,16 +2369,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2412,16 +2386,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2429,10 +2403,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
         <v>63</v>
@@ -2446,16 +2420,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
         <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2463,16 +2437,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2480,16 +2454,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2497,16 +2471,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2514,7 +2488,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
         <v>39</v>
@@ -2531,16 +2505,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>41</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2548,16 +2522,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2565,16 +2539,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2582,10 +2556,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C28" t="s">
         <v>65</v>
@@ -2599,16 +2573,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
         <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D29" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2619,13 +2593,13 @@
         <v>15</v>
       </c>
       <c r="B30" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D30" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2633,7 +2607,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B31" t="s">
         <v>39</v>
@@ -2650,16 +2624,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s">
         <v>41</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2667,16 +2641,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2684,7 +2658,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
         <v>39</v>
@@ -2701,24 +2675,24 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D35" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
@@ -2730,15 +2704,15 @@
         <v>229</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
         <v>69</v>
@@ -2752,10 +2726,10 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
         <v>70</v>
@@ -2769,10 +2743,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>71</v>
@@ -2786,10 +2760,10 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
         <v>72</v>
@@ -2798,55 +2772,55 @@
         <v>233</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
         <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E42">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D43" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2854,7 +2828,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B44" t="s">
         <v>39</v>
@@ -2871,16 +2845,16 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
         <v>41</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2888,24 +2862,24 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D46" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B47" t="s">
         <v>39</v>
@@ -2917,46 +2891,46 @@
         <v>235</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
         <v>41</v>
       </c>
       <c r="C48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D48" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D49" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B50" t="s">
         <v>39</v>
@@ -2973,24 +2947,24 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D51" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B52" t="s">
         <v>39</v>
@@ -3002,15 +2976,15 @@
         <v>237</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
         <v>77</v>
@@ -3024,10 +2998,10 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C54" t="s">
         <v>78</v>
@@ -3041,10 +3015,10 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C55" t="s">
         <v>79</v>
@@ -3053,21 +3027,21 @@
         <v>240</v>
       </c>
       <c r="E55">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E56">
         <v>4</v>
@@ -3075,7 +3049,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
@@ -3092,10 +3066,10 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
         <v>81</v>
@@ -3104,15 +3078,15 @@
         <v>242</v>
       </c>
       <c r="E58">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C59" t="s">
         <v>82</v>
@@ -3126,10 +3100,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
         <v>83</v>
@@ -3143,10 +3117,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C61" t="s">
         <v>84</v>
@@ -3160,10 +3134,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B62" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C62" t="s">
         <v>84</v>
@@ -3177,10 +3151,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C63" t="s">
         <v>84</v>
@@ -3194,10 +3168,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C64" t="s">
         <v>85</v>
@@ -3211,10 +3185,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B65" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C65" t="s">
         <v>85</v>
@@ -3228,10 +3202,10 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C66" t="s">
         <v>85</v>
@@ -3245,10 +3219,10 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C67" t="s">
         <v>86</v>
@@ -3262,10 +3236,10 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B68" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C68" t="s">
         <v>86</v>
@@ -3279,10 +3253,10 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C69" t="s">
         <v>87</v>
@@ -3296,10 +3270,10 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B70" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C70" t="s">
         <v>87</v>
@@ -3313,10 +3287,10 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B71" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C71" t="s">
         <v>88</v>
@@ -3330,10 +3304,10 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C72" t="s">
         <v>89</v>
@@ -3347,10 +3321,10 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C73" t="s">
         <v>89</v>
@@ -3364,10 +3338,10 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C74" t="s">
         <v>89</v>
@@ -3381,10 +3355,10 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B75" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C75" t="s">
         <v>89</v>
@@ -3398,10 +3372,10 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C76" t="s">
         <v>90</v>
@@ -3415,10 +3389,10 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B77" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C77" t="s">
         <v>90</v>
@@ -3432,10 +3406,10 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C78" t="s">
         <v>90</v>
@@ -3449,10 +3423,10 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B79" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C79" t="s">
         <v>90</v>
@@ -3466,10 +3440,10 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C80" t="s">
         <v>91</v>
@@ -3483,10 +3457,10 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C81" t="s">
         <v>91</v>
@@ -3500,10 +3474,10 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
         <v>91</v>
@@ -3517,10 +3491,10 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C83" t="s">
         <v>92</v>
@@ -3534,10 +3508,10 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C84" t="s">
         <v>92</v>
@@ -3551,10 +3525,10 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
         <v>92</v>
@@ -3568,10 +3542,10 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B86" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C86" t="s">
         <v>92</v>
@@ -3585,10 +3559,10 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C87" t="s">
         <v>93</v>
@@ -3602,10 +3576,10 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B88" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C88" t="s">
         <v>94</v>
@@ -3619,10 +3593,10 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B89" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C89" t="s">
         <v>94</v>
@@ -3636,10 +3610,10 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B90" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C90" t="s">
         <v>94</v>
@@ -3653,10 +3627,10 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C91" t="s">
         <v>95</v>
@@ -3670,10 +3644,10 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B92" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C92" t="s">
         <v>95</v>
@@ -3687,10 +3661,10 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B93" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C93" t="s">
         <v>95</v>
@@ -3704,10 +3678,10 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C94" t="s">
         <v>96</v>
@@ -3721,10 +3695,10 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B95" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
         <v>96</v>
@@ -3738,10 +3712,10 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C96" t="s">
         <v>97</v>
@@ -3755,10 +3729,10 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B97" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C97" t="s">
         <v>97</v>
@@ -3772,10 +3746,10 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C98" t="s">
         <v>98</v>
@@ -3789,10 +3763,10 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B99" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C99" t="s">
         <v>98</v>
@@ -3806,10 +3780,10 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B100" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C100" t="s">
         <v>99</v>
@@ -3823,10 +3797,10 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C101" t="s">
         <v>99</v>
@@ -3840,10 +3814,10 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C102" t="s">
         <v>100</v>
@@ -3857,10 +3831,10 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C103" t="s">
         <v>100</v>
@@ -3874,10 +3848,10 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B104" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C104" t="s">
         <v>101</v>
@@ -3891,10 +3865,10 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B105" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C105" t="s">
         <v>101</v>
@@ -3908,10 +3882,10 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B106" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C106" t="s">
         <v>102</v>
@@ -3925,10 +3899,10 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B107" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C107" t="s">
         <v>102</v>
@@ -3942,10 +3916,10 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B108" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C108" t="s">
         <v>103</v>
@@ -3959,10 +3933,10 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B109" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C109" t="s">
         <v>103</v>
@@ -3976,10 +3950,10 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C110" t="s">
         <v>104</v>
@@ -3993,10 +3967,10 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B111" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C111" t="s">
         <v>105</v>
@@ -4010,10 +3984,10 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B112" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C112" t="s">
         <v>106</v>
@@ -4027,10 +4001,10 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C113" t="s">
         <v>107</v>
@@ -4044,10 +4018,10 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C114" t="s">
         <v>108</v>
@@ -4061,10 +4035,10 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B115" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C115" t="s">
         <v>109</v>
@@ -4078,10 +4052,10 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B116" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C116" t="s">
         <v>110</v>
@@ -4095,10 +4069,10 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C117" t="s">
         <v>110</v>
@@ -4112,10 +4086,10 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B118" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C118" t="s">
         <v>111</v>
@@ -4129,10 +4103,10 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B119" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C119" t="s">
         <v>111</v>
@@ -4146,10 +4120,10 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B120" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C120" t="s">
         <v>112</v>
@@ -4163,10 +4137,10 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B121" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C121" t="s">
         <v>112</v>
@@ -4180,10 +4154,10 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C122" t="s">
         <v>113</v>
@@ -4197,10 +4171,10 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B123" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C123" t="s">
         <v>114</v>
@@ -4214,10 +4188,10 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C124" t="s">
         <v>115</v>
@@ -4231,10 +4205,10 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B125" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C125" t="s">
         <v>116</v>
@@ -4248,10 +4222,10 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B126" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C126" t="s">
         <v>117</v>
@@ -4265,10 +4239,10 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B127" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C127" t="s">
         <v>118</v>
@@ -4282,10 +4256,10 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B128" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C128" t="s">
         <v>118</v>
@@ -4299,10 +4273,10 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B129" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C129" t="s">
         <v>119</v>
@@ -4316,10 +4290,10 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B130" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C130" t="s">
         <v>119</v>
@@ -4333,10 +4307,10 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C131" t="s">
         <v>120</v>
@@ -4350,10 +4324,10 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B132" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C132" t="s">
         <v>121</v>
@@ -4367,10 +4341,10 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B133" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C133" t="s">
         <v>122</v>
@@ -4384,10 +4358,10 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B134" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C134" t="s">
         <v>123</v>
@@ -4401,10 +4375,10 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B135" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C135" t="s">
         <v>124</v>
@@ -4418,10 +4392,10 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B136" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C136" t="s">
         <v>125</v>
@@ -4435,10 +4409,10 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B137" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C137" t="s">
         <v>126</v>
@@ -4452,10 +4426,10 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B138" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C138" t="s">
         <v>127</v>
@@ -4469,10 +4443,10 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B139" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C139" t="s">
         <v>128</v>
@@ -4486,10 +4460,10 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B140" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C140" t="s">
         <v>129</v>
@@ -4503,10 +4477,10 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B141" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C141" t="s">
         <v>130</v>
@@ -4520,10 +4494,10 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B142" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C142" t="s">
         <v>131</v>
@@ -4537,10 +4511,10 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B143" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C143" t="s">
         <v>132</v>
@@ -4554,10 +4528,10 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B144" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C144" t="s">
         <v>133</v>
@@ -4571,10 +4545,10 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B145" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C145" t="s">
         <v>134</v>
@@ -4588,10 +4562,10 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B146" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C146" t="s">
         <v>135</v>
@@ -4605,10 +4579,10 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B147" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C147" t="s">
         <v>136</v>
@@ -4622,10 +4596,10 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B148" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C148" t="s">
         <v>137</v>
@@ -4639,10 +4613,10 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B149" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C149" t="s">
         <v>138</v>
@@ -4656,10 +4630,10 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B150" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C150" t="s">
         <v>139</v>
@@ -4673,10 +4647,10 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B151" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C151" t="s">
         <v>140</v>
@@ -4690,10 +4664,10 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B152" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C152" t="s">
         <v>141</v>
@@ -4707,10 +4681,10 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B153" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C153" t="s">
         <v>142</v>
@@ -4724,10 +4698,10 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B154" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C154" t="s">
         <v>143</v>
@@ -4741,10 +4715,10 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B155" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C155" t="s">
         <v>144</v>
@@ -4758,10 +4732,10 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B156" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C156" t="s">
         <v>145</v>
@@ -4775,10 +4749,10 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B157" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C157" t="s">
         <v>146</v>
@@ -4792,10 +4766,10 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B158" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C158" t="s">
         <v>147</v>
@@ -4809,10 +4783,10 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B159" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C159" t="s">
         <v>148</v>
@@ -4826,10 +4800,10 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B160" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C160" t="s">
         <v>149</v>
@@ -4843,10 +4817,10 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B161" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C161" t="s">
         <v>150</v>
@@ -4860,10 +4834,10 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B162" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C162" t="s">
         <v>151</v>
@@ -4877,10 +4851,10 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B163" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C163" t="s">
         <v>152</v>
@@ -4894,10 +4868,10 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B164" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C164" t="s">
         <v>153</v>
@@ -4911,10 +4885,10 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B165" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C165" t="s">
         <v>154</v>
@@ -4928,10 +4902,10 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B166" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C166" t="s">
         <v>155</v>
@@ -4945,10 +4919,10 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B167" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C167" t="s">
         <v>156</v>
@@ -4962,10 +4936,10 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B168" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C168" t="s">
         <v>157</v>
@@ -4979,10 +4953,10 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B169" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C169" t="s">
         <v>158</v>
@@ -4996,10 +4970,10 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C170" t="s">
         <v>159</v>
@@ -5013,10 +4987,10 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B171" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C171" t="s">
         <v>160</v>
@@ -5030,16 +5004,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B172" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C172" t="s">
         <v>161</v>
       </c>
       <c r="D172" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5047,10 +5021,10 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B173" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C173" t="s">
         <v>162</v>
@@ -5064,10 +5038,10 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B174" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C174" t="s">
         <v>163</v>
@@ -5081,10 +5055,10 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B175" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C175" t="s">
         <v>164</v>
@@ -5098,10 +5072,10 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B176" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C176" t="s">
         <v>165</v>
@@ -5115,10 +5089,10 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B177" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C177" t="s">
         <v>166</v>
@@ -5132,10 +5106,10 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B178" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C178" t="s">
         <v>167</v>
@@ -5149,10 +5123,10 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B179" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C179" t="s">
         <v>168</v>
@@ -5166,10 +5140,10 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B180" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C180" t="s">
         <v>169</v>
@@ -5183,10 +5157,10 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B181" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C181" t="s">
         <v>170</v>
@@ -5200,10 +5174,10 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B182" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C182" t="s">
         <v>171</v>
@@ -5217,10 +5191,10 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B183" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C183" t="s">
         <v>172</v>
@@ -5234,10 +5208,10 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B184" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C184" t="s">
         <v>173</v>
@@ -5251,10 +5225,10 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B185" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C185" t="s">
         <v>174</v>
@@ -5268,10 +5242,10 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B186" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C186" t="s">
         <v>175</v>
@@ -5285,10 +5259,10 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B187" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C187" t="s">
         <v>176</v>
@@ -5302,10 +5276,10 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B188" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C188" t="s">
         <v>177</v>
@@ -5319,10 +5293,10 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B189" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C189" t="s">
         <v>178</v>
@@ -5336,10 +5310,10 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B190" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C190" t="s">
         <v>179</v>
@@ -5353,10 +5327,10 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B191" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C191" t="s">
         <v>180</v>
@@ -5370,10 +5344,10 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B192" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C192" t="s">
         <v>181</v>
@@ -5387,10 +5361,10 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B193" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C193" t="s">
         <v>182</v>
@@ -5404,10 +5378,10 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B194" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C194" t="s">
         <v>183</v>
@@ -5421,10 +5395,10 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B195" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C195" t="s">
         <v>184</v>
@@ -5438,10 +5412,10 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B196" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C196" t="s">
         <v>185</v>
@@ -5455,10 +5429,10 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B197" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C197" t="s">
         <v>186</v>
@@ -5472,10 +5446,10 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B198" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C198" t="s">
         <v>187</v>
@@ -5489,10 +5463,10 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B199" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C199" t="s">
         <v>188</v>
@@ -5506,10 +5480,10 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B200" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C200" t="s">
         <v>189</v>
@@ -5523,10 +5497,10 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B201" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C201" t="s">
         <v>190</v>
@@ -5540,10 +5514,10 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B202" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C202" t="s">
         <v>191</v>
@@ -5557,10 +5531,10 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B203" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C203" t="s">
         <v>192</v>
@@ -5574,10 +5548,10 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B204" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C204" t="s">
         <v>193</v>
@@ -5591,10 +5565,10 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B205" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C205" t="s">
         <v>194</v>
@@ -5608,10 +5582,10 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B206" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C206" t="s">
         <v>195</v>
@@ -5625,10 +5599,10 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B207" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C207" t="s">
         <v>196</v>
@@ -5642,10 +5616,10 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B208" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C208" t="s">
         <v>197</v>
@@ -5659,10 +5633,10 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B209" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C209" t="s">
         <v>198</v>
@@ -5676,10 +5650,10 @@
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B210" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C210" t="s">
         <v>199</v>
@@ -5693,10 +5667,10 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B211" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C211" t="s">
         <v>200</v>
@@ -5710,10 +5684,10 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B212" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C212" t="s">
         <v>201</v>
@@ -5727,16 +5701,16 @@
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B213" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C213" t="s">
         <v>202</v>
       </c>
       <c r="D213" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E213">
         <v>3</v>
@@ -5744,10 +5718,10 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B214" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C214" t="s">
         <v>203</v>
@@ -5761,10 +5735,10 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B215" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C215" t="s">
         <v>204</v>
@@ -5778,10 +5752,10 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B216" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C216" t="s">
         <v>205</v>
@@ -5795,10 +5769,10 @@
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B217" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C217" t="s">
         <v>206</v>
@@ -5812,10 +5786,10 @@
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B218" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C218" t="s">
         <v>207</v>
@@ -5829,10 +5803,10 @@
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B219" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C219" t="s">
         <v>208</v>
@@ -5846,10 +5820,10 @@
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B220" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C220" t="s">
         <v>209</v>
@@ -5863,10 +5837,10 @@
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B221" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C221" t="s">
         <v>210</v>
@@ -5880,10 +5854,10 @@
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B222" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C222" t="s">
         <v>211</v>
@@ -5897,10 +5871,10 @@
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B223" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C223" t="s">
         <v>212</v>
@@ -5914,10 +5888,10 @@
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B224" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C224" t="s">
         <v>213</v>
@@ -5931,10 +5905,10 @@
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B225" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C225" t="s">
         <v>214</v>
@@ -5948,10 +5922,10 @@
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B226" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C226" t="s">
         <v>215</v>
@@ -5965,10 +5939,10 @@
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B227" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C227" t="s">
         <v>216</v>
@@ -5982,10 +5956,10 @@
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B228" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C228" t="s">
         <v>217</v>
@@ -5999,10 +5973,10 @@
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B229" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C229" t="s">
         <v>218</v>

</xml_diff>

<commit_message>
Atualização automática: rac (23/07/2026 11:41)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="370">
   <si>
     <t>matricula</t>
   </si>
@@ -260,9 +260,6 @@
     <t>2611137-7</t>
   </si>
   <si>
-    <t>C611008-0101</t>
-  </si>
-  <si>
     <t>3011755</t>
   </si>
   <si>
@@ -741,9 +738,6 @@
   </si>
   <si>
     <t>CAP MAIN LAND</t>
-  </si>
-  <si>
-    <t>ALTERNATOR CONTROL UNIT ASSY</t>
   </si>
   <si>
     <t>INSULATION BLANKET,T</t>
@@ -1137,8 +1131,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1154,7 +1156,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1162,12 +1164,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1466,22 +1486,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1579,10 +1599,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1619,10 +1639,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2092,23 +2112,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E227"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2123,7 +2143,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2140,7 +2160,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2157,7 +2177,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2174,7 +2194,7 @@
         <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2191,7 +2211,7 @@
         <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2208,7 +2228,7 @@
         <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2225,7 +2245,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2242,7 +2262,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2259,7 +2279,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2276,7 +2296,7 @@
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2293,7 +2313,7 @@
         <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2310,7 +2330,7 @@
         <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2327,7 +2347,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2344,7 +2364,7 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2361,7 +2381,7 @@
         <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2378,7 +2398,7 @@
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2395,7 +2415,7 @@
         <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2412,7 +2432,7 @@
         <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2429,7 +2449,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2446,7 +2466,7 @@
         <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2463,7 +2483,7 @@
         <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2480,7 +2500,7 @@
         <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2497,7 +2517,7 @@
         <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2505,7 +2525,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
         <v>41</v>
@@ -2514,7 +2534,7 @@
         <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2522,7 +2542,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>41</v>
@@ -2531,7 +2551,7 @@
         <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2539,13 +2559,13 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
         <v>225</v>
@@ -2556,16 +2576,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
         <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2573,16 +2593,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C29" t="s">
         <v>65</v>
       </c>
       <c r="D29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2590,13 +2610,13 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
         <v>226</v>
@@ -2607,16 +2627,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
         <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2624,16 +2644,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
         <v>66</v>
       </c>
       <c r="D32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2641,13 +2661,13 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
         <v>227</v>
@@ -2658,36 +2678,36 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" t="s">
         <v>67</v>
       </c>
       <c r="D34" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
         <v>228</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2698,7 +2718,7 @@
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
         <v>229</v>
@@ -2715,7 +2735,7 @@
         <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
         <v>230</v>
@@ -2732,7 +2752,7 @@
         <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
         <v>231</v>
@@ -2749,35 +2769,35 @@
         <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
         <v>232</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
         <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
         <v>41</v>
@@ -2786,24 +2806,24 @@
         <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E41">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
         <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2811,13 +2831,13 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
         <v>233</v>
@@ -2828,16 +2848,16 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C44" t="s">
         <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2845,81 +2865,81 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C45" t="s">
         <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B46" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C46" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
         <v>234</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C47" t="s">
         <v>74</v>
       </c>
       <c r="D47" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C48" t="s">
         <v>74</v>
       </c>
       <c r="D48" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B49" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C49" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D49" t="s">
         <v>235</v>
@@ -2930,36 +2950,36 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C50" t="s">
         <v>75</v>
       </c>
       <c r="D50" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D51" t="s">
         <v>236</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2970,7 +2990,7 @@
         <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D52" t="s">
         <v>237</v>
@@ -2987,7 +3007,7 @@
         <v>39</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D53" t="s">
         <v>238</v>
@@ -3004,27 +3024,27 @@
         <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D54" t="s">
         <v>239</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B55" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C55" t="s">
         <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E55">
         <v>4</v>
@@ -3032,13 +3052,13 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B56" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D56" t="s">
         <v>240</v>
@@ -3049,19 +3069,19 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D57" t="s">
         <v>241</v>
       </c>
       <c r="E57">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3072,7 +3092,7 @@
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D58" t="s">
         <v>242</v>
@@ -3083,13 +3103,13 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C59" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D59" t="s">
         <v>243</v>
@@ -3100,16 +3120,16 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C60" t="s">
         <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3117,16 +3137,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
         <v>41</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D61" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3134,7 +3154,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
         <v>41</v>
@@ -3143,7 +3163,7 @@
         <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3151,7 +3171,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B63" t="s">
         <v>41</v>
@@ -3160,7 +3180,7 @@
         <v>84</v>
       </c>
       <c r="D63" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3168,16 +3188,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
         <v>41</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D64" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3185,7 +3205,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
         <v>41</v>
@@ -3194,7 +3214,7 @@
         <v>85</v>
       </c>
       <c r="D65" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3211,7 +3231,7 @@
         <v>85</v>
       </c>
       <c r="D66" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3228,7 +3248,7 @@
         <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3245,7 +3265,7 @@
         <v>86</v>
       </c>
       <c r="D68" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -3262,7 +3282,7 @@
         <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -3270,24 +3290,24 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
         <v>41</v>
       </c>
       <c r="C70" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D70" t="s">
         <v>248</v>
       </c>
       <c r="E70">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B71" t="s">
         <v>41</v>
@@ -3296,24 +3316,24 @@
         <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E71">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
         <v>41</v>
       </c>
       <c r="C72" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D72" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3321,16 +3341,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3338,7 +3358,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B74" t="s">
         <v>41</v>
@@ -3347,7 +3367,7 @@
         <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3355,16 +3375,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B75" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C75" t="s">
         <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3372,16 +3392,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
         <v>41</v>
       </c>
       <c r="C76" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3389,16 +3409,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C77" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D77" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3406,7 +3426,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
         <v>41</v>
@@ -3415,7 +3435,7 @@
         <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3423,16 +3443,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B79" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C79" t="s">
         <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E79">
         <v>2</v>
@@ -3440,16 +3460,16 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
         <v>41</v>
       </c>
       <c r="C80" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3457,7 +3477,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
         <v>41</v>
@@ -3466,7 +3486,7 @@
         <v>91</v>
       </c>
       <c r="D81" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E81">
         <v>2</v>
@@ -3474,7 +3494,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B82" t="s">
         <v>41</v>
@@ -3483,7 +3503,7 @@
         <v>91</v>
       </c>
       <c r="D82" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E82">
         <v>2</v>
@@ -3491,41 +3511,41 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
         <v>41</v>
       </c>
       <c r="C83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D83" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B84" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D84" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E84">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
         <v>41</v>
@@ -3534,32 +3554,32 @@
         <v>92</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E85">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B86" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C86" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D86" t="s">
         <v>253</v>
       </c>
       <c r="E86">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
         <v>41</v>
@@ -3568,24 +3588,24 @@
         <v>93</v>
       </c>
       <c r="D87" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E87">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B88" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C88" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3593,7 +3613,7 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B89" t="s">
         <v>41</v>
@@ -3602,7 +3622,7 @@
         <v>94</v>
       </c>
       <c r="D89" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3610,16 +3630,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B90" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C90" t="s">
         <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3627,24 +3647,24 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B91" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D91" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E91">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
         <v>41</v>
@@ -3653,7 +3673,7 @@
         <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3661,19 +3681,19 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B93" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C93" t="s">
         <v>95</v>
       </c>
       <c r="D93" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E93">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3687,7 +3707,7 @@
         <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3704,7 +3724,7 @@
         <v>96</v>
       </c>
       <c r="D95" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3721,7 +3741,7 @@
         <v>97</v>
       </c>
       <c r="D96" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3738,7 +3758,7 @@
         <v>97</v>
       </c>
       <c r="D97" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3755,7 +3775,7 @@
         <v>98</v>
       </c>
       <c r="D98" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3772,7 +3792,7 @@
         <v>98</v>
       </c>
       <c r="D99" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3789,7 +3809,7 @@
         <v>99</v>
       </c>
       <c r="D100" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3806,7 +3826,7 @@
         <v>99</v>
       </c>
       <c r="D101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3823,7 +3843,7 @@
         <v>100</v>
       </c>
       <c r="D102" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3840,7 +3860,7 @@
         <v>100</v>
       </c>
       <c r="D103" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3857,7 +3877,7 @@
         <v>101</v>
       </c>
       <c r="D104" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3865,16 +3885,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B105" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C105" t="s">
         <v>101</v>
       </c>
       <c r="D105" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3891,7 +3911,7 @@
         <v>102</v>
       </c>
       <c r="D106" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3908,7 +3928,7 @@
         <v>102</v>
       </c>
       <c r="D107" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3925,7 +3945,7 @@
         <v>103</v>
       </c>
       <c r="D108" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3933,13 +3953,13 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B109" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C109" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D109" t="s">
         <v>263</v>
@@ -3956,7 +3976,7 @@
         <v>41</v>
       </c>
       <c r="C110" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D110" t="s">
         <v>264</v>
@@ -3973,7 +3993,7 @@
         <v>41</v>
       </c>
       <c r="C111" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D111" t="s">
         <v>265</v>
@@ -3990,7 +4010,7 @@
         <v>41</v>
       </c>
       <c r="C112" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D112" t="s">
         <v>266</v>
@@ -4007,7 +4027,7 @@
         <v>41</v>
       </c>
       <c r="C113" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D113" t="s">
         <v>267</v>
@@ -4024,18 +4044,18 @@
         <v>41</v>
       </c>
       <c r="C114" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D114" t="s">
         <v>268</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
         <v>41</v>
@@ -4044,7 +4064,7 @@
         <v>109</v>
       </c>
       <c r="D115" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E115">
         <v>1</v>
@@ -4061,7 +4081,7 @@
         <v>110</v>
       </c>
       <c r="D116" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4078,10 +4098,10 @@
         <v>110</v>
       </c>
       <c r="D117" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E117">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -4095,7 +4115,7 @@
         <v>111</v>
       </c>
       <c r="D118" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4112,10 +4132,10 @@
         <v>111</v>
       </c>
       <c r="D119" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4129,7 +4149,7 @@
         <v>112</v>
       </c>
       <c r="D120" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4137,19 +4157,19 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B121" t="s">
         <v>41</v>
       </c>
       <c r="C121" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D121" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4160,10 +4180,10 @@
         <v>41</v>
       </c>
       <c r="C122" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D122" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4177,13 +4197,13 @@
         <v>41</v>
       </c>
       <c r="C123" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D123" t="s">
         <v>273</v>
       </c>
       <c r="E123">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4194,13 +4214,13 @@
         <v>41</v>
       </c>
       <c r="C124" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D124" t="s">
         <v>274</v>
       </c>
       <c r="E124">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4211,18 +4231,18 @@
         <v>41</v>
       </c>
       <c r="C125" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D125" t="s">
         <v>275</v>
       </c>
       <c r="E125">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B126" t="s">
         <v>41</v>
@@ -4231,15 +4251,15 @@
         <v>117</v>
       </c>
       <c r="D126" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E126">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B127" t="s">
         <v>41</v>
@@ -4248,27 +4268,27 @@
         <v>118</v>
       </c>
       <c r="D127" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E127">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B128" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C128" t="s">
         <v>118</v>
       </c>
       <c r="D128" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E128">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -4282,7 +4302,7 @@
         <v>119</v>
       </c>
       <c r="D129" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4290,13 +4310,13 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C130" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D130" t="s">
         <v>278</v>
@@ -4313,7 +4333,7 @@
         <v>41</v>
       </c>
       <c r="C131" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D131" t="s">
         <v>279</v>
@@ -4330,7 +4350,7 @@
         <v>41</v>
       </c>
       <c r="C132" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D132" t="s">
         <v>280</v>
@@ -4347,7 +4367,7 @@
         <v>41</v>
       </c>
       <c r="C133" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D133" t="s">
         <v>281</v>
@@ -4364,7 +4384,7 @@
         <v>41</v>
       </c>
       <c r="C134" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D134" t="s">
         <v>282</v>
@@ -4381,7 +4401,7 @@
         <v>41</v>
       </c>
       <c r="C135" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D135" t="s">
         <v>283</v>
@@ -4398,7 +4418,7 @@
         <v>41</v>
       </c>
       <c r="C136" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D136" t="s">
         <v>284</v>
@@ -4415,7 +4435,7 @@
         <v>41</v>
       </c>
       <c r="C137" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D137" t="s">
         <v>285</v>
@@ -4432,7 +4452,7 @@
         <v>41</v>
       </c>
       <c r="C138" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D138" t="s">
         <v>286</v>
@@ -4449,7 +4469,7 @@
         <v>41</v>
       </c>
       <c r="C139" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D139" t="s">
         <v>287</v>
@@ -4466,7 +4486,7 @@
         <v>41</v>
       </c>
       <c r="C140" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D140" t="s">
         <v>288</v>
@@ -4483,7 +4503,7 @@
         <v>41</v>
       </c>
       <c r="C141" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D141" t="s">
         <v>289</v>
@@ -4500,7 +4520,7 @@
         <v>41</v>
       </c>
       <c r="C142" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D142" t="s">
         <v>290</v>
@@ -4517,7 +4537,7 @@
         <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D143" t="s">
         <v>291</v>
@@ -4534,7 +4554,7 @@
         <v>41</v>
       </c>
       <c r="C144" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D144" t="s">
         <v>292</v>
@@ -4551,7 +4571,7 @@
         <v>41</v>
       </c>
       <c r="C145" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D145" t="s">
         <v>293</v>
@@ -4568,7 +4588,7 @@
         <v>41</v>
       </c>
       <c r="C146" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D146" t="s">
         <v>294</v>
@@ -4585,7 +4605,7 @@
         <v>41</v>
       </c>
       <c r="C147" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D147" t="s">
         <v>295</v>
@@ -4602,7 +4622,7 @@
         <v>41</v>
       </c>
       <c r="C148" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D148" t="s">
         <v>296</v>
@@ -4619,7 +4639,7 @@
         <v>41</v>
       </c>
       <c r="C149" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D149" t="s">
         <v>297</v>
@@ -4636,7 +4656,7 @@
         <v>41</v>
       </c>
       <c r="C150" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D150" t="s">
         <v>298</v>
@@ -4653,7 +4673,7 @@
         <v>41</v>
       </c>
       <c r="C151" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D151" t="s">
         <v>299</v>
@@ -4670,7 +4690,7 @@
         <v>41</v>
       </c>
       <c r="C152" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D152" t="s">
         <v>300</v>
@@ -4687,7 +4707,7 @@
         <v>41</v>
       </c>
       <c r="C153" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D153" t="s">
         <v>301</v>
@@ -4704,7 +4724,7 @@
         <v>41</v>
       </c>
       <c r="C154" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D154" t="s">
         <v>302</v>
@@ -4721,7 +4741,7 @@
         <v>41</v>
       </c>
       <c r="C155" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D155" t="s">
         <v>303</v>
@@ -4738,13 +4758,13 @@
         <v>41</v>
       </c>
       <c r="C156" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D156" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="E156">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -4755,13 +4775,13 @@
         <v>41</v>
       </c>
       <c r="C157" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D157" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E157">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -4772,10 +4792,10 @@
         <v>41</v>
       </c>
       <c r="C158" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D158" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4789,7 +4809,7 @@
         <v>41</v>
       </c>
       <c r="C159" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D159" t="s">
         <v>306</v>
@@ -4806,7 +4826,7 @@
         <v>41</v>
       </c>
       <c r="C160" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D160" t="s">
         <v>307</v>
@@ -4823,13 +4843,13 @@
         <v>41</v>
       </c>
       <c r="C161" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D161" t="s">
         <v>308</v>
       </c>
       <c r="E161">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4840,13 +4860,13 @@
         <v>41</v>
       </c>
       <c r="C162" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D162" t="s">
         <v>309</v>
       </c>
       <c r="E162">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4857,13 +4877,13 @@
         <v>41</v>
       </c>
       <c r="C163" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D163" t="s">
         <v>310</v>
       </c>
       <c r="E163">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4874,47 +4894,47 @@
         <v>41</v>
       </c>
       <c r="C164" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D164" t="s">
         <v>311</v>
       </c>
       <c r="E164">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B165" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C165" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D165" t="s">
         <v>312</v>
       </c>
       <c r="E165">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B166" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C166" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D166" t="s">
         <v>313</v>
       </c>
       <c r="E166">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -4925,7 +4945,7 @@
         <v>38</v>
       </c>
       <c r="C167" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D167" t="s">
         <v>314</v>
@@ -4942,7 +4962,7 @@
         <v>38</v>
       </c>
       <c r="C168" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D168" t="s">
         <v>315</v>
@@ -4959,7 +4979,7 @@
         <v>38</v>
       </c>
       <c r="C169" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D169" t="s">
         <v>316</v>
@@ -4976,10 +4996,10 @@
         <v>38</v>
       </c>
       <c r="C170" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D170" t="s">
-        <v>317</v>
+        <v>237</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4993,10 +5013,10 @@
         <v>38</v>
       </c>
       <c r="C171" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D171" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5010,10 +5030,10 @@
         <v>38</v>
       </c>
       <c r="C172" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D172" t="s">
-        <v>238</v>
+        <v>318</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5027,7 +5047,7 @@
         <v>38</v>
       </c>
       <c r="C173" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D173" t="s">
         <v>319</v>
@@ -5044,7 +5064,7 @@
         <v>38</v>
       </c>
       <c r="C174" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D174" t="s">
         <v>320</v>
@@ -5061,7 +5081,7 @@
         <v>38</v>
       </c>
       <c r="C175" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D175" t="s">
         <v>321</v>
@@ -5078,7 +5098,7 @@
         <v>38</v>
       </c>
       <c r="C176" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D176" t="s">
         <v>322</v>
@@ -5095,7 +5115,7 @@
         <v>38</v>
       </c>
       <c r="C177" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D177" t="s">
         <v>323</v>
@@ -5112,7 +5132,7 @@
         <v>38</v>
       </c>
       <c r="C178" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D178" t="s">
         <v>324</v>
@@ -5129,7 +5149,7 @@
         <v>38</v>
       </c>
       <c r="C179" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D179" t="s">
         <v>325</v>
@@ -5146,7 +5166,7 @@
         <v>38</v>
       </c>
       <c r="C180" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D180" t="s">
         <v>326</v>
@@ -5163,7 +5183,7 @@
         <v>38</v>
       </c>
       <c r="C181" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D181" t="s">
         <v>327</v>
@@ -5180,7 +5200,7 @@
         <v>38</v>
       </c>
       <c r="C182" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D182" t="s">
         <v>328</v>
@@ -5197,7 +5217,7 @@
         <v>38</v>
       </c>
       <c r="C183" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D183" t="s">
         <v>329</v>
@@ -5214,7 +5234,7 @@
         <v>38</v>
       </c>
       <c r="C184" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D184" t="s">
         <v>330</v>
@@ -5231,7 +5251,7 @@
         <v>38</v>
       </c>
       <c r="C185" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D185" t="s">
         <v>331</v>
@@ -5248,7 +5268,7 @@
         <v>38</v>
       </c>
       <c r="C186" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D186" t="s">
         <v>332</v>
@@ -5265,7 +5285,7 @@
         <v>38</v>
       </c>
       <c r="C187" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D187" t="s">
         <v>333</v>
@@ -5282,7 +5302,7 @@
         <v>38</v>
       </c>
       <c r="C188" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D188" t="s">
         <v>334</v>
@@ -5299,7 +5319,7 @@
         <v>38</v>
       </c>
       <c r="C189" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D189" t="s">
         <v>335</v>
@@ -5316,7 +5336,7 @@
         <v>38</v>
       </c>
       <c r="C190" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D190" t="s">
         <v>336</v>
@@ -5333,7 +5353,7 @@
         <v>38</v>
       </c>
       <c r="C191" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D191" t="s">
         <v>337</v>
@@ -5350,7 +5370,7 @@
         <v>38</v>
       </c>
       <c r="C192" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D192" t="s">
         <v>338</v>
@@ -5367,10 +5387,10 @@
         <v>38</v>
       </c>
       <c r="C193" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D193" t="s">
-        <v>339</v>
+        <v>299</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5384,10 +5404,10 @@
         <v>38</v>
       </c>
       <c r="C194" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D194" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5401,10 +5421,10 @@
         <v>38</v>
       </c>
       <c r="C195" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D195" t="s">
-        <v>301</v>
+        <v>340</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5418,7 +5438,7 @@
         <v>38</v>
       </c>
       <c r="C196" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D196" t="s">
         <v>341</v>
@@ -5435,7 +5455,7 @@
         <v>38</v>
       </c>
       <c r="C197" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D197" t="s">
         <v>342</v>
@@ -5452,13 +5472,13 @@
         <v>38</v>
       </c>
       <c r="C198" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D198" t="s">
         <v>343</v>
       </c>
       <c r="E198">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -5469,13 +5489,13 @@
         <v>38</v>
       </c>
       <c r="C199" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D199" t="s">
         <v>344</v>
       </c>
       <c r="E199">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5486,7 +5506,7 @@
         <v>38</v>
       </c>
       <c r="C200" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D200" t="s">
         <v>345</v>
@@ -5503,7 +5523,7 @@
         <v>38</v>
       </c>
       <c r="C201" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D201" t="s">
         <v>346</v>
@@ -5520,7 +5540,7 @@
         <v>38</v>
       </c>
       <c r="C202" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D202" t="s">
         <v>347</v>
@@ -5537,7 +5557,7 @@
         <v>38</v>
       </c>
       <c r="C203" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D203" t="s">
         <v>348</v>
@@ -5554,7 +5574,7 @@
         <v>38</v>
       </c>
       <c r="C204" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D204" t="s">
         <v>349</v>
@@ -5571,7 +5591,7 @@
         <v>38</v>
       </c>
       <c r="C205" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D205" t="s">
         <v>350</v>
@@ -5588,10 +5608,10 @@
         <v>38</v>
       </c>
       <c r="C206" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D206" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5605,10 +5625,10 @@
         <v>38</v>
       </c>
       <c r="C207" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D207" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5622,7 +5642,7 @@
         <v>38</v>
       </c>
       <c r="C208" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D208" t="s">
         <v>352</v>
@@ -5639,7 +5659,7 @@
         <v>38</v>
       </c>
       <c r="C209" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D209" t="s">
         <v>353</v>
@@ -5656,13 +5676,13 @@
         <v>38</v>
       </c>
       <c r="C210" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D210" t="s">
         <v>354</v>
       </c>
       <c r="E210">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5673,13 +5693,13 @@
         <v>38</v>
       </c>
       <c r="C211" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D211" t="s">
-        <v>355</v>
+        <v>237</v>
       </c>
       <c r="E211">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5690,13 +5710,13 @@
         <v>38</v>
       </c>
       <c r="C212" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D212" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E212">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5707,13 +5727,13 @@
         <v>38</v>
       </c>
       <c r="C213" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D213" t="s">
-        <v>238</v>
+        <v>356</v>
       </c>
       <c r="E213">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5724,7 +5744,7 @@
         <v>38</v>
       </c>
       <c r="C214" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D214" t="s">
         <v>357</v>
@@ -5741,7 +5761,7 @@
         <v>38</v>
       </c>
       <c r="C215" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D215" t="s">
         <v>358</v>
@@ -5758,7 +5778,7 @@
         <v>38</v>
       </c>
       <c r="C216" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D216" t="s">
         <v>359</v>
@@ -5775,13 +5795,13 @@
         <v>38</v>
       </c>
       <c r="C217" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D217" t="s">
         <v>360</v>
       </c>
       <c r="E217">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5792,13 +5812,13 @@
         <v>38</v>
       </c>
       <c r="C218" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D218" t="s">
         <v>361</v>
       </c>
       <c r="E218">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5809,13 +5829,13 @@
         <v>38</v>
       </c>
       <c r="C219" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D219" t="s">
         <v>362</v>
       </c>
       <c r="E219">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5826,13 +5846,13 @@
         <v>38</v>
       </c>
       <c r="C220" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D220" t="s">
         <v>363</v>
       </c>
       <c r="E220">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5843,13 +5863,13 @@
         <v>38</v>
       </c>
       <c r="C221" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D221" t="s">
         <v>364</v>
       </c>
       <c r="E221">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5860,13 +5880,13 @@
         <v>38</v>
       </c>
       <c r="C222" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D222" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E222">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5877,13 +5897,13 @@
         <v>38</v>
       </c>
       <c r="C223" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D223" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E223">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5894,13 +5914,13 @@
         <v>38</v>
       </c>
       <c r="C224" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D224" t="s">
         <v>366</v>
       </c>
       <c r="E224">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5911,13 +5931,13 @@
         <v>38</v>
       </c>
       <c r="C225" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D225" t="s">
         <v>367</v>
       </c>
       <c r="E225">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5928,13 +5948,13 @@
         <v>38</v>
       </c>
       <c r="C226" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D226" t="s">
         <v>368</v>
       </c>
       <c r="E226">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -5945,46 +5965,12 @@
         <v>38</v>
       </c>
       <c r="C227" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D227" t="s">
         <v>369</v>
       </c>
       <c r="E227">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="228" spans="1:5">
-      <c r="A228" t="s">
-        <v>15</v>
-      </c>
-      <c r="B228" t="s">
-        <v>38</v>
-      </c>
-      <c r="C228" t="s">
-        <v>217</v>
-      </c>
-      <c r="D228" t="s">
-        <v>370</v>
-      </c>
-      <c r="E228">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="229" spans="1:5">
-      <c r="A229" t="s">
-        <v>15</v>
-      </c>
-      <c r="B229" t="s">
-        <v>38</v>
-      </c>
-      <c r="C229" t="s">
-        <v>218</v>
-      </c>
-      <c r="D229" t="s">
-        <v>371</v>
-      </c>
-      <c r="E229">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (23/07/2026 16:16)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="370">
   <si>
     <t>matricula</t>
   </si>
@@ -41,60 +41,60 @@
     <t>2723</t>
   </si>
   <si>
+    <t>2728</t>
+  </si>
+  <si>
+    <t>2729</t>
+  </si>
+  <si>
+    <t>2741</t>
+  </si>
+  <si>
+    <t>2732</t>
+  </si>
+  <si>
+    <t>2730</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>2726</t>
+  </si>
+  <si>
+    <t>2702</t>
+  </si>
+  <si>
+    <t>2703</t>
+  </si>
+  <si>
+    <t>2704</t>
+  </si>
+  <si>
+    <t>2708</t>
+  </si>
+  <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>2719</t>
+  </si>
+  <si>
+    <t>2720</t>
+  </si>
+  <si>
+    <t>2722</t>
+  </si>
+  <si>
+    <t>2727</t>
+  </si>
+  <si>
+    <t>2731</t>
+  </si>
+  <si>
     <t>2733</t>
   </si>
   <si>
-    <t>2728</t>
-  </si>
-  <si>
-    <t>2729</t>
-  </si>
-  <si>
-    <t>2741</t>
-  </si>
-  <si>
-    <t>2732</t>
-  </si>
-  <si>
-    <t>2730</t>
-  </si>
-  <si>
-    <t>2734</t>
-  </si>
-  <si>
-    <t>2726</t>
-  </si>
-  <si>
-    <t>2702</t>
-  </si>
-  <si>
-    <t>2703</t>
-  </si>
-  <si>
-    <t>2704</t>
-  </si>
-  <si>
-    <t>2708</t>
-  </si>
-  <si>
-    <t>2709</t>
-  </si>
-  <si>
-    <t>2719</t>
-  </si>
-  <si>
-    <t>2720</t>
-  </si>
-  <si>
-    <t>2722</t>
-  </si>
-  <si>
-    <t>2727</t>
-  </si>
-  <si>
-    <t>2731</t>
-  </si>
-  <si>
     <t>2736</t>
   </si>
   <si>
@@ -131,16 +131,16 @@
     <t>CLA</t>
   </si>
   <si>
+    <t>1º/5º GAV</t>
+  </si>
+  <si>
+    <t>BABV</t>
+  </si>
+  <si>
+    <t>7º ETA</t>
+  </si>
+  <si>
     <t>1º ETA</t>
-  </si>
-  <si>
-    <t>1º/5º GAV</t>
-  </si>
-  <si>
-    <t>BABV</t>
-  </si>
-  <si>
-    <t>7º ETA</t>
   </si>
   <si>
     <t>EPCAR</t>
@@ -1131,16 +1131,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1156,7 +1148,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1164,30 +1156,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1486,22 +1460,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1559,10 +1533,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1570,7 +1544,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1579,10 +1553,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1599,10 +1573,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1616,13 +1590,13 @@
         <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1630,7 +1604,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1639,10 +1613,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F8">
-        <v>26</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1650,7 +1624,7 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
@@ -1659,10 +1633,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="F9">
-        <v>91</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1679,10 +1653,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="F10">
-        <v>144</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1690,19 +1664,19 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E11">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1710,7 +1684,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1730,7 +1704,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1750,7 +1724,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1770,7 +1744,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1790,7 +1764,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1810,7 +1784,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1830,7 +1804,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1850,7 +1824,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1870,7 +1844,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1890,7 +1864,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
         <v>51</v>
@@ -1910,7 +1884,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
@@ -1930,7 +1904,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
         <v>51</v>
@@ -1970,7 +1944,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -1990,7 +1964,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
         <v>51</v>
@@ -2090,7 +2064,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
         <v>52</v>
@@ -2112,23 +2086,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2185,10 +2159,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>59</v>
@@ -2202,10 +2176,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>59</v>
@@ -2219,10 +2193,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
         <v>59</v>
@@ -2236,10 +2210,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
@@ -2253,10 +2227,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>59</v>
@@ -2287,10 +2261,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
         <v>60</v>
@@ -2304,10 +2278,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
         <v>60</v>
@@ -2321,10 +2295,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
         <v>60</v>
@@ -2338,10 +2312,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
         <v>60</v>
@@ -2355,10 +2329,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
         <v>60</v>
@@ -2412,10 +2386,10 @@
         <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2423,10 +2397,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
         <v>63</v>
@@ -2443,7 +2417,7 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
         <v>63</v>
@@ -2460,7 +2434,7 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
         <v>63</v>
@@ -2491,16 +2465,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
         <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2508,10 +2482,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>64</v>
@@ -2528,7 +2502,7 @@
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
         <v>64</v>
@@ -2542,16 +2516,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2559,10 +2533,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
         <v>65</v>
@@ -2576,7 +2550,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
         <v>41</v>
@@ -2593,16 +2567,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2610,10 +2584,10 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C30" t="s">
         <v>66</v>
@@ -2644,16 +2618,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B32" t="s">
         <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2661,10 +2635,10 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C33" t="s">
         <v>67</v>
@@ -2673,38 +2647,38 @@
         <v>227</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2712,16 +2686,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2729,16 +2703,16 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2746,27 +2720,27 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
@@ -2775,7 +2749,7 @@
         <v>232</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2783,7 +2757,7 @@
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
         <v>72</v>
@@ -2792,7 +2766,7 @@
         <v>232</v>
       </c>
       <c r="E40">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2814,16 +2788,16 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B42" t="s">
         <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2831,10 +2805,10 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>73</v>
@@ -2860,32 +2834,32 @@
         <v>233</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
         <v>38</v>
       </c>
       <c r="C45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
         <v>74</v>
@@ -2894,7 +2868,7 @@
         <v>234</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2911,21 +2885,21 @@
         <v>234</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
         <v>38</v>
       </c>
       <c r="C48" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2933,10 +2907,10 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C49" t="s">
         <v>75</v>
@@ -2945,38 +2919,38 @@
         <v>235</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
         <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D50" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D51" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -2984,16 +2958,16 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D52" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3001,27 +2975,27 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B53" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D53" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
         <v>79</v>
@@ -3035,16 +3009,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B55" t="s">
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D55" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E55">
         <v>4</v>
@@ -3055,30 +3029,30 @@
         <v>9</v>
       </c>
       <c r="B56" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D56" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E56">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3086,16 +3060,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3106,7 +3080,7 @@
         <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C59" t="s">
         <v>83</v>
@@ -3123,7 +3097,7 @@
         <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C60" t="s">
         <v>83</v>
@@ -3137,16 +3111,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3157,7 +3131,7 @@
         <v>12</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
         <v>84</v>
@@ -3174,7 +3148,7 @@
         <v>13</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C63" t="s">
         <v>84</v>
@@ -3188,16 +3162,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C64" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3205,10 +3179,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B65" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C65" t="s">
         <v>85</v>
@@ -3222,16 +3196,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D66" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3239,10 +3213,10 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C67" t="s">
         <v>86</v>
@@ -3256,16 +3230,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C68" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D68" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -3273,19 +3247,19 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D69" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E69">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3293,7 +3267,7 @@
         <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
         <v>88</v>
@@ -3310,7 +3284,7 @@
         <v>13</v>
       </c>
       <c r="B71" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
         <v>88</v>
@@ -3341,16 +3315,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D73" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3361,7 +3335,7 @@
         <v>12</v>
       </c>
       <c r="B74" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C74" t="s">
         <v>89</v>
@@ -3378,7 +3352,7 @@
         <v>13</v>
       </c>
       <c r="B75" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C75" t="s">
         <v>89</v>
@@ -3409,16 +3383,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3429,7 +3403,7 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
         <v>90</v>
@@ -3446,7 +3420,7 @@
         <v>13</v>
       </c>
       <c r="B79" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
         <v>90</v>
@@ -3460,16 +3434,16 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D80" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3480,7 +3454,7 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
         <v>91</v>
@@ -3497,7 +3471,7 @@
         <v>13</v>
       </c>
       <c r="B82" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C82" t="s">
         <v>91</v>
@@ -3506,7 +3480,7 @@
         <v>251</v>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3528,19 +3502,19 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B84" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D84" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E84">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3548,16 +3522,16 @@
         <v>12</v>
       </c>
       <c r="B85" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C85" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D85" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E85">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3565,7 +3539,7 @@
         <v>13</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C86" t="s">
         <v>93</v>
@@ -3596,16 +3570,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B88" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D88" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3616,7 +3590,7 @@
         <v>13</v>
       </c>
       <c r="B89" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C89" t="s">
         <v>94</v>
@@ -3642,24 +3616,24 @@
         <v>251</v>
       </c>
       <c r="E90">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D91" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E91">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -3667,7 +3641,7 @@
         <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
         <v>95</v>
@@ -3681,16 +3655,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D93" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3701,7 +3675,7 @@
         <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C94" t="s">
         <v>96</v>
@@ -3715,16 +3689,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D95" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3735,7 +3709,7 @@
         <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C96" t="s">
         <v>97</v>
@@ -3749,16 +3723,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D97" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3769,7 +3743,7 @@
         <v>13</v>
       </c>
       <c r="B98" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C98" t="s">
         <v>98</v>
@@ -3783,16 +3757,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C99" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D99" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3803,7 +3777,7 @@
         <v>13</v>
       </c>
       <c r="B100" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C100" t="s">
         <v>99</v>
@@ -3817,16 +3791,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D101" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3837,7 +3811,7 @@
         <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C102" t="s">
         <v>100</v>
@@ -3851,16 +3825,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D103" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3868,7 +3842,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B104" t="s">
         <v>41</v>
@@ -3885,16 +3859,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B105" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D105" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3902,7 +3876,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B106" t="s">
         <v>41</v>
@@ -3919,16 +3893,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C107" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D107" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3936,16 +3910,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B108" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D108" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3953,16 +3927,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D109" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3970,16 +3944,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B110" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C110" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D110" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3987,16 +3961,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B111" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D111" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4004,16 +3978,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D112" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4021,19 +3995,19 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D113" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -4041,7 +4015,7 @@
         <v>13</v>
       </c>
       <c r="B114" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C114" t="s">
         <v>109</v>
@@ -4050,24 +4024,24 @@
         <v>268</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C115" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E115">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -4075,7 +4049,7 @@
         <v>13</v>
       </c>
       <c r="B116" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C116" t="s">
         <v>110</v>
@@ -4089,16 +4063,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C117" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D117" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4109,7 +4083,7 @@
         <v>13</v>
       </c>
       <c r="B118" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C118" t="s">
         <v>111</v>
@@ -4118,38 +4092,38 @@
         <v>270</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B119" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C119" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D119" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B120" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C120" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D120" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4157,16 +4131,16 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B121" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C121" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D121" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4174,53 +4148,53 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C122" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D122" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E122">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D123" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E123">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B124" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C124" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E124">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4228,7 +4202,7 @@
         <v>13</v>
       </c>
       <c r="B125" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C125" t="s">
         <v>117</v>
@@ -4242,19 +4216,19 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B126" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C126" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D126" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E126">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4276,16 +4250,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B128" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D128" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4293,16 +4267,16 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C129" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D129" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4310,16 +4284,16 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D130" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4327,16 +4301,16 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B131" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C131" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D131" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4344,16 +4318,16 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B132" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C132" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D132" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4361,16 +4335,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B133" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C133" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D133" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4378,16 +4352,16 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C134" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D134" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4395,16 +4369,16 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B135" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C135" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D135" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4412,16 +4386,16 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B136" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C136" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D136" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4429,16 +4403,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B137" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C137" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D137" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4446,16 +4420,16 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B138" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C138" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D138" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4463,16 +4437,16 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B139" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C139" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D139" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4480,16 +4454,16 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B140" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C140" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D140" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4497,16 +4471,16 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C141" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D141" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4514,16 +4488,16 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B142" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C142" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D142" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4531,16 +4505,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B143" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C143" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D143" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4548,16 +4522,16 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B144" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C144" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D144" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4565,16 +4539,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B145" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C145" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D145" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4582,16 +4556,16 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B146" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C146" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D146" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4599,16 +4573,16 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B147" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C147" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D147" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4616,16 +4590,16 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B148" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C148" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D148" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4633,16 +4607,16 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B149" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C149" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D149" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4650,16 +4624,16 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B150" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C150" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D150" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4667,16 +4641,16 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B151" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D151" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4684,16 +4658,16 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B152" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D152" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4701,16 +4675,16 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B153" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D153" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4718,16 +4692,16 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B154" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D154" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4735,33 +4709,33 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B155" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D155" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="E155">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B156" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D156" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="E156">
         <v>2</v>
@@ -4769,16 +4743,16 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B157" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D157" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4786,16 +4760,16 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B158" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D158" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4803,16 +4777,16 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B159" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D159" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E159">
         <v>2</v>
@@ -4820,50 +4794,50 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B160" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D160" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E160">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B161" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C161" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D161" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E161">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B162" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D162" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E162">
         <v>8</v>
@@ -4871,19 +4845,19 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B163" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D163" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E163">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4894,27 +4868,27 @@
         <v>41</v>
       </c>
       <c r="C164" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D164" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E164">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B165" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C165" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D165" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4922,16 +4896,16 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B166" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C166" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D166" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4939,16 +4913,16 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B167" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C167" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D167" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4956,16 +4930,16 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B168" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C168" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D168" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4973,16 +4947,16 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B169" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C169" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D169" t="s">
-        <v>316</v>
+        <v>237</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4990,16 +4964,16 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B170" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C170" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D170" t="s">
-        <v>237</v>
+        <v>317</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5007,16 +4981,16 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B171" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C171" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D171" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5024,16 +4998,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B172" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C172" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D172" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5041,16 +5015,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B173" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C173" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D173" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5058,16 +5032,16 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B174" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C174" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D174" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5075,16 +5049,16 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B175" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C175" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D175" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5092,16 +5066,16 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B176" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C176" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D176" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5109,16 +5083,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B177" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C177" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D177" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5126,16 +5100,16 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B178" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C178" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D178" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5143,16 +5117,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B179" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C179" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D179" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5160,16 +5134,16 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B180" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C180" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D180" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5177,16 +5151,16 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B181" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C181" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D181" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5194,16 +5168,16 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B182" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C182" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D182" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5211,16 +5185,16 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B183" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C183" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D183" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5228,16 +5202,16 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B184" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C184" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D184" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5245,16 +5219,16 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B185" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C185" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D185" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5262,16 +5236,16 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B186" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C186" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D186" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5279,16 +5253,16 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B187" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C187" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D187" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5296,16 +5270,16 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B188" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C188" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D188" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5313,16 +5287,16 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B189" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C189" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D189" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5330,16 +5304,16 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B190" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C190" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D190" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5347,16 +5321,16 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B191" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C191" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D191" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5364,16 +5338,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B192" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C192" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D192" t="s">
-        <v>338</v>
+        <v>299</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5381,16 +5355,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B193" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C193" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D193" t="s">
-        <v>299</v>
+        <v>339</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5398,16 +5372,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B194" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C194" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D194" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5415,16 +5389,16 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B195" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C195" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D195" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5432,16 +5406,16 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B196" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C196" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D196" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5449,33 +5423,33 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B197" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C197" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D197" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E197">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B198" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C198" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D198" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5483,16 +5457,16 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B199" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C199" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D199" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5500,16 +5474,16 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B200" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C200" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D200" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5517,16 +5491,16 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B201" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C201" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D201" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5534,16 +5508,16 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B202" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C202" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D202" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5551,16 +5525,16 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B203" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C203" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D203" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5568,16 +5542,16 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B204" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C204" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D204" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5585,13 +5559,13 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B205" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C205" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D205" t="s">
         <v>350</v>
@@ -5602,16 +5576,16 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B206" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C206" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D206" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5619,16 +5593,16 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B207" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C207" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D207" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5636,16 +5610,16 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B208" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C208" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D208" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5653,33 +5627,33 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B209" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C209" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D209" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E209">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B210" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C210" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D210" t="s">
-        <v>354</v>
+        <v>237</v>
       </c>
       <c r="E210">
         <v>3</v>
@@ -5687,33 +5661,33 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B211" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C211" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D211" t="s">
-        <v>237</v>
+        <v>355</v>
       </c>
       <c r="E211">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B212" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C212" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D212" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E212">
         <v>4</v>
@@ -5721,16 +5695,16 @@
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B213" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C213" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D213" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E213">
         <v>4</v>
@@ -5738,16 +5712,16 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B214" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C214" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D214" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E214">
         <v>4</v>
@@ -5755,16 +5729,16 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B215" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C215" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D215" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5772,33 +5746,33 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B216" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C216" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D216" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E216">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B217" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C217" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D217" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E217">
         <v>5</v>
@@ -5806,64 +5780,64 @@
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B218" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C218" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D218" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E218">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B219" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C219" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D219" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E219">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B220" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C220" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D220" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E220">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B221" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C221" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D221" t="s">
         <v>364</v>
@@ -5874,33 +5848,33 @@
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B222" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C222" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D222" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E222">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B223" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C223" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D223" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E223">
         <v>12</v>
@@ -5908,69 +5882,52 @@
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B224" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C224" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D224" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E224">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
+        <v>14</v>
+      </c>
+      <c r="B225" t="s">
+        <v>41</v>
+      </c>
+      <c r="C225" t="s">
+        <v>216</v>
+      </c>
+      <c r="D225" t="s">
+        <v>368</v>
+      </c>
+      <c r="E225">
         <v>15</v>
-      </c>
-      <c r="B225" t="s">
-        <v>38</v>
-      </c>
-      <c r="C225" t="s">
-        <v>215</v>
-      </c>
-      <c r="D225" t="s">
-        <v>367</v>
-      </c>
-      <c r="E225">
-        <v>14</v>
       </c>
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B226" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C226" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D226" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E226">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="227" spans="1:5">
-      <c r="A227" t="s">
-        <v>15</v>
-      </c>
-      <c r="B227" t="s">
-        <v>38</v>
-      </c>
-      <c r="C227" t="s">
-        <v>217</v>
-      </c>
-      <c r="D227" t="s">
-        <v>369</v>
-      </c>
-      <c r="E227">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (24/07/2026 17:52)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="366">
   <si>
     <t>matricula</t>
   </si>
@@ -191,9 +191,6 @@
     <t>quantidade_faltante</t>
   </si>
   <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -575,9 +572,6 @@
     <t>C622010-0102</t>
   </si>
   <si>
-    <t>060-0015-00</t>
-  </si>
-  <si>
     <t>2615018-1</t>
   </si>
   <si>
@@ -671,9 +665,6 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
@@ -1038,9 +1029,6 @@
   </si>
   <si>
     <t>LIGHT STROBE RH</t>
-  </si>
-  <si>
-    <t>CONTROL,DIRECTIONAL</t>
   </si>
   <si>
     <t>MOLDING-WINDOW</t>
@@ -1493,10 +1481,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1513,10 +1501,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1653,10 +1641,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F10">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2086,7 +2074,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E222"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2108,16 +2096,16 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2125,16 +2113,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2142,16 +2130,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2159,16 +2147,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2176,16 +2164,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2193,16 +2181,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
         <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2210,16 +2198,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2227,7 +2215,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
         <v>40</v>
@@ -2236,7 +2224,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2244,16 +2232,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2261,16 +2249,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2278,16 +2266,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2295,16 +2283,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
         <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2312,16 +2300,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2329,13 +2317,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
         <v>220</v>
@@ -2346,16 +2334,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2363,16 +2351,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2380,16 +2368,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2397,16 +2385,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2414,16 +2402,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2431,7 +2419,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
         <v>40</v>
@@ -2440,7 +2428,7 @@
         <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2448,16 +2436,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
         <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2474,7 +2462,7 @@
         <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2491,7 +2479,7 @@
         <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2499,16 +2487,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
         <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2525,7 +2513,7 @@
         <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2533,7 +2521,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
@@ -2542,7 +2530,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2559,7 +2547,7 @@
         <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2576,7 +2564,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2584,33 +2572,33 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C30" t="s">
         <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2624,10 +2612,10 @@
         <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2635,19 +2623,19 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D33" t="s">
         <v>227</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2658,7 +2646,7 @@
         <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
         <v>228</v>
@@ -2675,61 +2663,61 @@
         <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
         <v>229</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
         <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -2737,19 +2725,19 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E39">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2763,7 +2751,7 @@
         <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2780,10 +2768,10 @@
         <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2797,7 +2785,7 @@
         <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2814,10 +2802,10 @@
         <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2831,10 +2819,10 @@
         <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2848,7 +2836,7 @@
         <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2856,33 +2844,33 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C46" t="s">
         <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E46">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C47" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2896,10 +2884,10 @@
         <v>38</v>
       </c>
       <c r="C48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2907,19 +2895,19 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D49" t="s">
         <v>235</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2930,30 +2918,30 @@
         <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D50" t="s">
         <v>236</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D51" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2964,78 +2952,78 @@
         <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D52" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D53" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D54" t="s">
         <v>239</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D55" t="s">
         <v>240</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3043,16 +3031,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
         <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3069,7 +3057,7 @@
         <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3086,7 +3074,7 @@
         <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3103,7 +3091,7 @@
         <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3120,7 +3108,7 @@
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3128,7 +3116,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B62" t="s">
         <v>40</v>
@@ -3137,7 +3125,7 @@
         <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3145,16 +3133,16 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B63" t="s">
         <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3162,7 +3150,7 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B64" t="s">
         <v>40</v>
@@ -3171,7 +3159,7 @@
         <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3179,16 +3167,16 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
         <v>40</v>
       </c>
       <c r="C65" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D65" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3202,35 +3190,35 @@
         <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D66" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
         <v>40</v>
       </c>
       <c r="C67" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B68" t="s">
         <v>40</v>
@@ -3239,24 +3227,24 @@
         <v>87</v>
       </c>
       <c r="D68" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E68">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C69" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3264,7 +3252,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
         <v>40</v>
@@ -3273,7 +3261,7 @@
         <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3281,7 +3269,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B71" t="s">
         <v>40</v>
@@ -3290,7 +3278,7 @@
         <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3298,16 +3286,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B72" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
         <v>88</v>
       </c>
       <c r="D72" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3315,16 +3303,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3332,7 +3320,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
         <v>40</v>
@@ -3341,7 +3329,7 @@
         <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3349,7 +3337,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
         <v>40</v>
@@ -3358,7 +3346,7 @@
         <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3366,16 +3354,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
         <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3392,7 +3380,7 @@
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3409,7 +3397,7 @@
         <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3426,32 +3414,32 @@
         <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E79">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C80" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
         <v>40</v>
@@ -3460,61 +3448,61 @@
         <v>91</v>
       </c>
       <c r="D81" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E81">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
         <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E82">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B83" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D83" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E83">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C84" t="s">
         <v>92</v>
       </c>
       <c r="D84" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E84">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3528,7 +3516,7 @@
         <v>93</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3545,7 +3533,7 @@
         <v>93</v>
       </c>
       <c r="D86" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3562,10 +3550,10 @@
         <v>93</v>
       </c>
       <c r="D87" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3604,24 +3592,24 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B90" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D90" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E90">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
         <v>40</v>
@@ -3630,7 +3618,7 @@
         <v>95</v>
       </c>
       <c r="D91" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3638,16 +3626,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B92" t="s">
         <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D92" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3655,7 +3643,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
         <v>40</v>
@@ -3664,7 +3652,7 @@
         <v>96</v>
       </c>
       <c r="D93" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3672,16 +3660,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B94" t="s">
         <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D94" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3689,7 +3677,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
         <v>40</v>
@@ -3698,7 +3686,7 @@
         <v>97</v>
       </c>
       <c r="D95" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3706,16 +3694,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B96" t="s">
         <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D96" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3723,7 +3711,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B97" t="s">
         <v>40</v>
@@ -3732,7 +3720,7 @@
         <v>98</v>
       </c>
       <c r="D97" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3740,16 +3728,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B98" t="s">
         <v>40</v>
       </c>
       <c r="C98" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D98" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3757,7 +3745,7 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
         <v>40</v>
@@ -3766,7 +3754,7 @@
         <v>99</v>
       </c>
       <c r="D99" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3774,16 +3762,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B100" t="s">
         <v>40</v>
       </c>
       <c r="C100" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D100" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3791,16 +3779,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C101" t="s">
         <v>100</v>
       </c>
       <c r="D101" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3808,16 +3796,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B102" t="s">
         <v>40</v>
       </c>
       <c r="C102" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D102" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3825,16 +3813,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C103" t="s">
         <v>101</v>
       </c>
       <c r="D103" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3842,16 +3830,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C104" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D104" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3865,10 +3853,10 @@
         <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D105" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3876,13 +3864,13 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B106" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C106" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D106" t="s">
         <v>261</v>
@@ -3899,7 +3887,7 @@
         <v>40</v>
       </c>
       <c r="C107" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D107" t="s">
         <v>262</v>
@@ -3916,7 +3904,7 @@
         <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D108" t="s">
         <v>263</v>
@@ -3933,7 +3921,7 @@
         <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D109" t="s">
         <v>264</v>
@@ -3950,27 +3938,27 @@
         <v>40</v>
       </c>
       <c r="C110" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D110" t="s">
         <v>265</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B111" t="s">
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D111" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -3984,18 +3972,18 @@
         <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D112" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
         <v>40</v>
@@ -4004,7 +3992,7 @@
         <v>109</v>
       </c>
       <c r="D113" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4012,24 +4000,24 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
       </c>
       <c r="C114" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D114" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
@@ -4038,24 +4026,24 @@
         <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B116" t="s">
         <v>40</v>
       </c>
       <c r="C116" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D116" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4069,10 +4057,10 @@
         <v>40</v>
       </c>
       <c r="C117" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D117" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4080,19 +4068,19 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B118" t="s">
         <v>40</v>
       </c>
       <c r="C118" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D118" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E118">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -4103,13 +4091,13 @@
         <v>40</v>
       </c>
       <c r="C119" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D119" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4120,13 +4108,13 @@
         <v>40</v>
       </c>
       <c r="C120" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D120" t="s">
         <v>271</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4137,64 +4125,64 @@
         <v>40</v>
       </c>
       <c r="C121" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D121" t="s">
         <v>272</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
         <v>40</v>
       </c>
       <c r="C122" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D122" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E122">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B123" t="s">
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D123" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E123">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B124" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C124" t="s">
         <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E124">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4205,13 +4193,13 @@
         <v>40</v>
       </c>
       <c r="C125" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E125">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4222,10 +4210,10 @@
         <v>40</v>
       </c>
       <c r="C126" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D126" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4233,13 +4221,13 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B127" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C127" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D127" t="s">
         <v>276</v>
@@ -4256,7 +4244,7 @@
         <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D128" t="s">
         <v>277</v>
@@ -4273,7 +4261,7 @@
         <v>40</v>
       </c>
       <c r="C129" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D129" t="s">
         <v>278</v>
@@ -4290,7 +4278,7 @@
         <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D130" t="s">
         <v>279</v>
@@ -4307,7 +4295,7 @@
         <v>40</v>
       </c>
       <c r="C131" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D131" t="s">
         <v>280</v>
@@ -4324,7 +4312,7 @@
         <v>40</v>
       </c>
       <c r="C132" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D132" t="s">
         <v>281</v>
@@ -4341,7 +4329,7 @@
         <v>40</v>
       </c>
       <c r="C133" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D133" t="s">
         <v>282</v>
@@ -4358,7 +4346,7 @@
         <v>40</v>
       </c>
       <c r="C134" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D134" t="s">
         <v>283</v>
@@ -4375,7 +4363,7 @@
         <v>40</v>
       </c>
       <c r="C135" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D135" t="s">
         <v>284</v>
@@ -4392,7 +4380,7 @@
         <v>40</v>
       </c>
       <c r="C136" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D136" t="s">
         <v>285</v>
@@ -4409,7 +4397,7 @@
         <v>40</v>
       </c>
       <c r="C137" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D137" t="s">
         <v>286</v>
@@ -4426,7 +4414,7 @@
         <v>40</v>
       </c>
       <c r="C138" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D138" t="s">
         <v>287</v>
@@ -4443,7 +4431,7 @@
         <v>40</v>
       </c>
       <c r="C139" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D139" t="s">
         <v>288</v>
@@ -4460,7 +4448,7 @@
         <v>40</v>
       </c>
       <c r="C140" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D140" t="s">
         <v>289</v>
@@ -4477,7 +4465,7 @@
         <v>40</v>
       </c>
       <c r="C141" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D141" t="s">
         <v>290</v>
@@ -4494,7 +4482,7 @@
         <v>40</v>
       </c>
       <c r="C142" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D142" t="s">
         <v>291</v>
@@ -4511,7 +4499,7 @@
         <v>40</v>
       </c>
       <c r="C143" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D143" t="s">
         <v>292</v>
@@ -4528,7 +4516,7 @@
         <v>40</v>
       </c>
       <c r="C144" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D144" t="s">
         <v>293</v>
@@ -4545,7 +4533,7 @@
         <v>40</v>
       </c>
       <c r="C145" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D145" t="s">
         <v>294</v>
@@ -4562,7 +4550,7 @@
         <v>40</v>
       </c>
       <c r="C146" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D146" t="s">
         <v>295</v>
@@ -4579,7 +4567,7 @@
         <v>40</v>
       </c>
       <c r="C147" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D147" t="s">
         <v>296</v>
@@ -4596,7 +4584,7 @@
         <v>40</v>
       </c>
       <c r="C148" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D148" t="s">
         <v>297</v>
@@ -4613,7 +4601,7 @@
         <v>40</v>
       </c>
       <c r="C149" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D149" t="s">
         <v>298</v>
@@ -4630,7 +4618,7 @@
         <v>40</v>
       </c>
       <c r="C150" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D150" t="s">
         <v>299</v>
@@ -4647,7 +4635,7 @@
         <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D151" t="s">
         <v>300</v>
@@ -4664,13 +4652,13 @@
         <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>301</v>
+        <v>286</v>
       </c>
       <c r="E152">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -4681,13 +4669,13 @@
         <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E153">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -4698,13 +4686,13 @@
         <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E154">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -4715,10 +4703,10 @@
         <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="E155">
         <v>2</v>
@@ -4732,7 +4720,7 @@
         <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D156" t="s">
         <v>304</v>
@@ -4749,13 +4737,13 @@
         <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D157" t="s">
         <v>305</v>
       </c>
       <c r="E157">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -4766,13 +4754,13 @@
         <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D158" t="s">
         <v>306</v>
       </c>
       <c r="E158">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -4783,13 +4771,13 @@
         <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D159" t="s">
         <v>307</v>
       </c>
       <c r="E159">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4800,64 +4788,64 @@
         <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D160" t="s">
         <v>308</v>
       </c>
       <c r="E160">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B161" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C161" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D161" t="s">
         <v>309</v>
       </c>
       <c r="E161">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B162" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C162" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D162" t="s">
         <v>310</v>
       </c>
       <c r="E162">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B163" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C163" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D163" t="s">
         <v>311</v>
       </c>
       <c r="E163">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4868,7 +4856,7 @@
         <v>41</v>
       </c>
       <c r="C164" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D164" t="s">
         <v>312</v>
@@ -4885,7 +4873,7 @@
         <v>41</v>
       </c>
       <c r="C165" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D165" t="s">
         <v>313</v>
@@ -4902,10 +4890,10 @@
         <v>41</v>
       </c>
       <c r="C166" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>314</v>
+        <v>234</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4919,10 +4907,10 @@
         <v>41</v>
       </c>
       <c r="C167" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4936,10 +4924,10 @@
         <v>41</v>
       </c>
       <c r="C168" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4953,10 +4941,10 @@
         <v>41</v>
       </c>
       <c r="C169" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>237</v>
+        <v>316</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4970,7 +4958,7 @@
         <v>41</v>
       </c>
       <c r="C170" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D170" t="s">
         <v>317</v>
@@ -4987,7 +4975,7 @@
         <v>41</v>
       </c>
       <c r="C171" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D171" t="s">
         <v>318</v>
@@ -5004,7 +4992,7 @@
         <v>41</v>
       </c>
       <c r="C172" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D172" t="s">
         <v>319</v>
@@ -5021,7 +5009,7 @@
         <v>41</v>
       </c>
       <c r="C173" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D173" t="s">
         <v>320</v>
@@ -5038,7 +5026,7 @@
         <v>41</v>
       </c>
       <c r="C174" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D174" t="s">
         <v>321</v>
@@ -5055,7 +5043,7 @@
         <v>41</v>
       </c>
       <c r="C175" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D175" t="s">
         <v>322</v>
@@ -5072,7 +5060,7 @@
         <v>41</v>
       </c>
       <c r="C176" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D176" t="s">
         <v>323</v>
@@ -5089,7 +5077,7 @@
         <v>41</v>
       </c>
       <c r="C177" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D177" t="s">
         <v>324</v>
@@ -5106,7 +5094,7 @@
         <v>41</v>
       </c>
       <c r="C178" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D178" t="s">
         <v>325</v>
@@ -5123,7 +5111,7 @@
         <v>41</v>
       </c>
       <c r="C179" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D179" t="s">
         <v>326</v>
@@ -5140,7 +5128,7 @@
         <v>41</v>
       </c>
       <c r="C180" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D180" t="s">
         <v>327</v>
@@ -5157,7 +5145,7 @@
         <v>41</v>
       </c>
       <c r="C181" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D181" t="s">
         <v>328</v>
@@ -5174,7 +5162,7 @@
         <v>41</v>
       </c>
       <c r="C182" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D182" t="s">
         <v>329</v>
@@ -5191,7 +5179,7 @@
         <v>41</v>
       </c>
       <c r="C183" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D183" t="s">
         <v>330</v>
@@ -5208,7 +5196,7 @@
         <v>41</v>
       </c>
       <c r="C184" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D184" t="s">
         <v>331</v>
@@ -5225,7 +5213,7 @@
         <v>41</v>
       </c>
       <c r="C185" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D185" t="s">
         <v>332</v>
@@ -5242,7 +5230,7 @@
         <v>41</v>
       </c>
       <c r="C186" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D186" t="s">
         <v>333</v>
@@ -5259,7 +5247,7 @@
         <v>41</v>
       </c>
       <c r="C187" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D187" t="s">
         <v>334</v>
@@ -5276,7 +5264,7 @@
         <v>41</v>
       </c>
       <c r="C188" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D188" t="s">
         <v>335</v>
@@ -5293,10 +5281,10 @@
         <v>41</v>
       </c>
       <c r="C189" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D189" t="s">
-        <v>336</v>
+        <v>296</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5310,10 +5298,10 @@
         <v>41</v>
       </c>
       <c r="C190" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D190" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5327,10 +5315,10 @@
         <v>41</v>
       </c>
       <c r="C191" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D191" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5344,10 +5332,10 @@
         <v>41</v>
       </c>
       <c r="C192" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D192" t="s">
-        <v>299</v>
+        <v>338</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5361,13 +5349,13 @@
         <v>41</v>
       </c>
       <c r="C193" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D193" t="s">
         <v>339</v>
       </c>
       <c r="E193">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -5378,13 +5366,13 @@
         <v>41</v>
       </c>
       <c r="C194" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D194" t="s">
         <v>340</v>
       </c>
       <c r="E194">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -5395,13 +5383,13 @@
         <v>41</v>
       </c>
       <c r="C195" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D195" t="s">
         <v>341</v>
       </c>
       <c r="E195">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -5412,13 +5400,13 @@
         <v>41</v>
       </c>
       <c r="C196" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D196" t="s">
         <v>342</v>
       </c>
       <c r="E196">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -5429,7 +5417,7 @@
         <v>41</v>
       </c>
       <c r="C197" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D197" t="s">
         <v>343</v>
@@ -5446,7 +5434,7 @@
         <v>41</v>
       </c>
       <c r="C198" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D198" t="s">
         <v>344</v>
@@ -5463,7 +5451,7 @@
         <v>41</v>
       </c>
       <c r="C199" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D199" t="s">
         <v>345</v>
@@ -5480,7 +5468,7 @@
         <v>41</v>
       </c>
       <c r="C200" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D200" t="s">
         <v>346</v>
@@ -5497,10 +5485,10 @@
         <v>41</v>
       </c>
       <c r="C201" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D201" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5514,10 +5502,10 @@
         <v>41</v>
       </c>
       <c r="C202" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D202" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5531,10 +5519,10 @@
         <v>41</v>
       </c>
       <c r="C203" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D203" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5548,10 +5536,10 @@
         <v>41</v>
       </c>
       <c r="C204" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D204" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5565,13 +5553,13 @@
         <v>41</v>
       </c>
       <c r="C205" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D205" t="s">
         <v>350</v>
       </c>
       <c r="E205">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5582,13 +5570,13 @@
         <v>41</v>
       </c>
       <c r="C206" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D206" t="s">
-        <v>351</v>
+        <v>234</v>
       </c>
       <c r="E206">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5599,13 +5587,13 @@
         <v>41</v>
       </c>
       <c r="C207" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D207" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E207">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5616,13 +5604,13 @@
         <v>41</v>
       </c>
       <c r="C208" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D208" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E208">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5633,13 +5621,13 @@
         <v>41</v>
       </c>
       <c r="C209" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D209" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E209">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5650,13 +5638,13 @@
         <v>41</v>
       </c>
       <c r="C210" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D210" t="s">
-        <v>237</v>
+        <v>354</v>
       </c>
       <c r="E210">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5667,7 +5655,7 @@
         <v>41</v>
       </c>
       <c r="C211" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D211" t="s">
         <v>355</v>
@@ -5684,13 +5672,13 @@
         <v>41</v>
       </c>
       <c r="C212" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D212" t="s">
         <v>356</v>
       </c>
       <c r="E212">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5701,13 +5689,13 @@
         <v>41</v>
       </c>
       <c r="C213" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D213" t="s">
         <v>357</v>
       </c>
       <c r="E213">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5718,13 +5706,13 @@
         <v>41</v>
       </c>
       <c r="C214" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D214" t="s">
         <v>358</v>
       </c>
       <c r="E214">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5735,13 +5723,13 @@
         <v>41</v>
       </c>
       <c r="C215" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D215" t="s">
         <v>359</v>
       </c>
       <c r="E215">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5752,13 +5740,13 @@
         <v>41</v>
       </c>
       <c r="C216" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D216" t="s">
         <v>360</v>
       </c>
       <c r="E216">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5769,13 +5757,13 @@
         <v>41</v>
       </c>
       <c r="C217" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D217" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E217">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5786,13 +5774,13 @@
         <v>41</v>
       </c>
       <c r="C218" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D218" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E218">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5803,13 +5791,13 @@
         <v>41</v>
       </c>
       <c r="C219" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D219" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E219">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5820,13 +5808,13 @@
         <v>41</v>
       </c>
       <c r="C220" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E220">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5837,13 +5825,13 @@
         <v>41</v>
       </c>
       <c r="C221" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D221" t="s">
         <v>364</v>
       </c>
       <c r="E221">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5854,80 +5842,12 @@
         <v>41</v>
       </c>
       <c r="C222" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D222" t="s">
         <v>365</v>
       </c>
       <c r="E222">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="223" spans="1:5">
-      <c r="A223" t="s">
-        <v>14</v>
-      </c>
-      <c r="B223" t="s">
-        <v>41</v>
-      </c>
-      <c r="C223" t="s">
-        <v>214</v>
-      </c>
-      <c r="D223" t="s">
-        <v>366</v>
-      </c>
-      <c r="E223">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="224" spans="1:5">
-      <c r="A224" t="s">
-        <v>14</v>
-      </c>
-      <c r="B224" t="s">
-        <v>41</v>
-      </c>
-      <c r="C224" t="s">
-        <v>215</v>
-      </c>
-      <c r="D224" t="s">
-        <v>367</v>
-      </c>
-      <c r="E224">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="225" spans="1:5">
-      <c r="A225" t="s">
-        <v>14</v>
-      </c>
-      <c r="B225" t="s">
-        <v>41</v>
-      </c>
-      <c r="C225" t="s">
-        <v>216</v>
-      </c>
-      <c r="D225" t="s">
-        <v>368</v>
-      </c>
-      <c r="E225">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="226" spans="1:5">
-      <c r="A226" t="s">
-        <v>14</v>
-      </c>
-      <c r="B226" t="s">
-        <v>41</v>
-      </c>
-      <c r="C226" t="s">
-        <v>217</v>
-      </c>
-      <c r="D226" t="s">
-        <v>369</v>
-      </c>
-      <c r="E226">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (27/07/2026 14:22)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="382">
   <si>
     <t>matricula</t>
   </si>
@@ -41,15 +41,15 @@
     <t>2723</t>
   </si>
   <si>
+    <t>2729</t>
+  </si>
+  <si>
+    <t>2741</t>
+  </si>
+  <si>
     <t>2728</t>
   </si>
   <si>
-    <t>2729</t>
-  </si>
-  <si>
-    <t>2741</t>
-  </si>
-  <si>
     <t>2732</t>
   </si>
   <si>
@@ -191,18 +191,24 @@
     <t>quantidade_faltante</t>
   </si>
   <si>
+    <t>3044000</t>
+  </si>
+  <si>
+    <t>C145-00-46</t>
+  </si>
+  <si>
+    <t>3122678-04</t>
+  </si>
+  <si>
+    <t>3011755</t>
+  </si>
+  <si>
+    <t>540-1407-4</t>
+  </si>
+  <si>
     <t>C611505-0201</t>
   </si>
   <si>
-    <t>3044000</t>
-  </si>
-  <si>
-    <t>C145-00-46</t>
-  </si>
-  <si>
-    <t>3122678-04</t>
-  </si>
-  <si>
     <t>P7036368-01</t>
   </si>
   <si>
@@ -257,12 +263,6 @@
     <t>2611137-7</t>
   </si>
   <si>
-    <t>3011755</t>
-  </si>
-  <si>
-    <t>540-1407-4</t>
-  </si>
-  <si>
     <t>1H75-21</t>
   </si>
   <si>
@@ -572,6 +572,9 @@
     <t>C622010-0102</t>
   </si>
   <si>
+    <t>060-0015-00</t>
+  </si>
+  <si>
     <t>2615018-1</t>
   </si>
   <si>
@@ -665,18 +668,48 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>MICROB MONITOR 2</t>
+  </si>
+  <si>
+    <t>S3461-76</t>
+  </si>
+  <si>
+    <t>2622243-11</t>
+  </si>
+  <si>
+    <t>AE713797-005</t>
+  </si>
+  <si>
+    <t>S2319-64</t>
+  </si>
+  <si>
+    <t>MS24694-S135</t>
+  </si>
+  <si>
+    <t>1214134-1</t>
+  </si>
+  <si>
+    <t>CAB-33-02</t>
+  </si>
+  <si>
+    <t>ENGINE PT6A-114A</t>
+  </si>
+  <si>
+    <t>TRANSMISSION ASSY</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>INSULATION BLANKET,T</t>
+  </si>
+  <si>
+    <t>VALVE,COMPRESSOR BLEED</t>
+  </si>
+  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
-    <t>ENGINE PT6A-114A</t>
-  </si>
-  <si>
-    <t>TRANSMISSION ASSY</t>
-  </si>
-  <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
     <t>PROPELLER ASSEMBLY</t>
   </si>
   <si>
@@ -731,12 +764,6 @@
     <t>CAP MAIN LAND</t>
   </si>
   <si>
-    <t>INSULATION BLANKET,T</t>
-  </si>
-  <si>
-    <t>VALVE,COMPRESSOR BLEED</t>
-  </si>
-  <si>
     <t>PRESSURE REGULATOR</t>
   </si>
   <si>
@@ -1031,6 +1058,9 @@
     <t>LIGHT STROBE RH</t>
   </si>
   <si>
+    <t>CONTROL,DIRECTIONAL</t>
+  </si>
+  <si>
     <t>MOLDING-WINDOW</t>
   </si>
   <si>
@@ -1113,6 +1143,24 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>TEST KIT, FUEL, WORK</t>
+  </si>
+  <si>
+    <t>ECCENTRIC-WING ASSY</t>
+  </si>
+  <si>
+    <t>HOSE ASSY-SUCTION LI</t>
+  </si>
+  <si>
+    <t>GROMMET</t>
+  </si>
+  <si>
+    <t>BELLCRANK ASSY</t>
+  </si>
+  <si>
+    <t>KIT CAB-33-02</t>
   </si>
 </sst>
 </file>
@@ -1521,10 +1569,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1532,7 +1580,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1541,10 +1589,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1552,7 +1600,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1561,10 +1609,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1581,10 +1629,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1601,10 +1649,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1621,10 +1669,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F9">
-        <v>144</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1641,10 +1689,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F10">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2074,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2096,16 +2144,16 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2116,13 +2164,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2139,7 +2187,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2156,7 +2204,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2173,7 +2221,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2181,16 +2229,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2198,16 +2246,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2215,16 +2263,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2232,16 +2280,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2249,16 +2297,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2266,16 +2314,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2283,16 +2331,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2300,16 +2348,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2317,16 +2365,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2334,16 +2382,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
         <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2351,16 +2399,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2368,16 +2416,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2385,16 +2433,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2402,16 +2450,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2419,16 +2467,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2436,16 +2484,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2453,16 +2501,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D23" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2470,16 +2518,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2487,16 +2535,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2504,16 +2552,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2521,16 +2569,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D27" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2538,16 +2586,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2555,16 +2603,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2578,27 +2626,27 @@
         <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2606,24 +2654,24 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C32" t="s">
         <v>68</v>
       </c>
       <c r="D32" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>38</v>
@@ -2632,7 +2680,7 @@
         <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2640,7 +2688,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
@@ -2649,7 +2697,7 @@
         <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2657,7 +2705,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
         <v>38</v>
@@ -2666,41 +2714,41 @@
         <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D37" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2708,33 +2756,33 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2742,16 +2790,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2759,33 +2807,33 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2793,33 +2841,33 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="E43">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2827,19 +2875,19 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2850,27 +2898,27 @@
         <v>41</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B47" t="s">
         <v>38</v>
       </c>
       <c r="C47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2878,24 +2926,24 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C48" t="s">
         <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
         <v>38</v>
@@ -2904,7 +2952,7 @@
         <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2912,7 +2960,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B50" t="s">
         <v>38</v>
@@ -2921,41 +2969,41 @@
         <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D51" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B52" t="s">
         <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D52" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="E52">
         <v>4</v>
@@ -2963,24 +3011,24 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
         <v>80</v>
       </c>
       <c r="D53" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B54" t="s">
         <v>38</v>
@@ -2989,10 +3037,10 @@
         <v>81</v>
       </c>
       <c r="D54" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3006,7 +3054,7 @@
         <v>82</v>
       </c>
       <c r="D55" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3023,7 +3071,7 @@
         <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3040,7 +3088,7 @@
         <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3057,7 +3105,7 @@
         <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3074,7 +3122,7 @@
         <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3091,7 +3139,7 @@
         <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3108,7 +3156,7 @@
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3125,7 +3173,7 @@
         <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3142,7 +3190,7 @@
         <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3159,7 +3207,7 @@
         <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3176,7 +3224,7 @@
         <v>86</v>
       </c>
       <c r="D65" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3193,7 +3241,7 @@
         <v>87</v>
       </c>
       <c r="D66" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3210,7 +3258,7 @@
         <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3227,7 +3275,7 @@
         <v>87</v>
       </c>
       <c r="D68" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3244,7 +3292,7 @@
         <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3261,7 +3309,7 @@
         <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3278,7 +3326,7 @@
         <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3295,7 +3343,7 @@
         <v>88</v>
       </c>
       <c r="D72" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3312,7 +3360,7 @@
         <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3329,7 +3377,7 @@
         <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3346,7 +3394,7 @@
         <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3363,7 +3411,7 @@
         <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3380,7 +3428,7 @@
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3397,7 +3445,7 @@
         <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3414,7 +3462,7 @@
         <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E79">
         <v>4</v>
@@ -3431,7 +3479,7 @@
         <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E80">
         <v>4</v>
@@ -3448,7 +3496,7 @@
         <v>91</v>
       </c>
       <c r="D81" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="E81">
         <v>10</v>
@@ -3465,7 +3513,7 @@
         <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3482,7 +3530,7 @@
         <v>92</v>
       </c>
       <c r="D83" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3499,7 +3547,7 @@
         <v>92</v>
       </c>
       <c r="D84" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3516,7 +3564,7 @@
         <v>93</v>
       </c>
       <c r="D85" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3533,7 +3581,7 @@
         <v>93</v>
       </c>
       <c r="D86" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3550,7 +3598,7 @@
         <v>93</v>
       </c>
       <c r="D87" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E87">
         <v>2</v>
@@ -3567,7 +3615,7 @@
         <v>94</v>
       </c>
       <c r="D88" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3584,7 +3632,7 @@
         <v>94</v>
       </c>
       <c r="D89" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3601,7 +3649,7 @@
         <v>95</v>
       </c>
       <c r="D90" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3618,7 +3666,7 @@
         <v>95</v>
       </c>
       <c r="D91" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3635,7 +3683,7 @@
         <v>96</v>
       </c>
       <c r="D92" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3652,7 +3700,7 @@
         <v>96</v>
       </c>
       <c r="D93" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3669,7 +3717,7 @@
         <v>97</v>
       </c>
       <c r="D94" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3686,7 +3734,7 @@
         <v>97</v>
       </c>
       <c r="D95" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3703,7 +3751,7 @@
         <v>98</v>
       </c>
       <c r="D96" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3720,7 +3768,7 @@
         <v>98</v>
       </c>
       <c r="D97" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3737,7 +3785,7 @@
         <v>99</v>
       </c>
       <c r="D98" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3754,7 +3802,7 @@
         <v>99</v>
       </c>
       <c r="D99" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3771,7 +3819,7 @@
         <v>100</v>
       </c>
       <c r="D100" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3788,7 +3836,7 @@
         <v>100</v>
       </c>
       <c r="D101" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3805,7 +3853,7 @@
         <v>101</v>
       </c>
       <c r="D102" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3822,7 +3870,7 @@
         <v>101</v>
       </c>
       <c r="D103" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3839,7 +3887,7 @@
         <v>102</v>
       </c>
       <c r="D104" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3856,7 +3904,7 @@
         <v>103</v>
       </c>
       <c r="D105" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3873,7 +3921,7 @@
         <v>104</v>
       </c>
       <c r="D106" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3890,7 +3938,7 @@
         <v>105</v>
       </c>
       <c r="D107" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3907,7 +3955,7 @@
         <v>106</v>
       </c>
       <c r="D108" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3924,7 +3972,7 @@
         <v>107</v>
       </c>
       <c r="D109" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3941,7 +3989,7 @@
         <v>108</v>
       </c>
       <c r="D110" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -3958,7 +4006,7 @@
         <v>108</v>
       </c>
       <c r="D111" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -3975,7 +4023,7 @@
         <v>109</v>
       </c>
       <c r="D112" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -3992,7 +4040,7 @@
         <v>109</v>
       </c>
       <c r="D113" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4009,7 +4057,7 @@
         <v>110</v>
       </c>
       <c r="D114" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4026,7 +4074,7 @@
         <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="E115">
         <v>4</v>
@@ -4043,7 +4091,7 @@
         <v>111</v>
       </c>
       <c r="D116" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4060,7 +4108,7 @@
         <v>112</v>
       </c>
       <c r="D117" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4077,7 +4125,7 @@
         <v>113</v>
       </c>
       <c r="D118" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4094,7 +4142,7 @@
         <v>114</v>
       </c>
       <c r="D119" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="E119">
         <v>7</v>
@@ -4111,7 +4159,7 @@
         <v>115</v>
       </c>
       <c r="D120" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="E120">
         <v>8</v>
@@ -4128,7 +4176,7 @@
         <v>116</v>
       </c>
       <c r="D121" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="E121">
         <v>30</v>
@@ -4145,7 +4193,7 @@
         <v>116</v>
       </c>
       <c r="D122" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="E122">
         <v>30</v>
@@ -4162,7 +4210,7 @@
         <v>117</v>
       </c>
       <c r="D123" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4179,7 +4227,7 @@
         <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4196,7 +4244,7 @@
         <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4213,7 +4261,7 @@
         <v>119</v>
       </c>
       <c r="D126" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4230,7 +4278,7 @@
         <v>120</v>
       </c>
       <c r="D127" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4247,7 +4295,7 @@
         <v>121</v>
       </c>
       <c r="D128" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4264,7 +4312,7 @@
         <v>122</v>
       </c>
       <c r="D129" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4281,7 +4329,7 @@
         <v>123</v>
       </c>
       <c r="D130" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4298,7 +4346,7 @@
         <v>124</v>
       </c>
       <c r="D131" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4315,7 +4363,7 @@
         <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4332,7 +4380,7 @@
         <v>126</v>
       </c>
       <c r="D133" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4349,7 +4397,7 @@
         <v>127</v>
       </c>
       <c r="D134" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4366,7 +4414,7 @@
         <v>128</v>
       </c>
       <c r="D135" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4383,7 +4431,7 @@
         <v>129</v>
       </c>
       <c r="D136" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4400,7 +4448,7 @@
         <v>130</v>
       </c>
       <c r="D137" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4417,7 +4465,7 @@
         <v>131</v>
       </c>
       <c r="D138" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4434,7 +4482,7 @@
         <v>132</v>
       </c>
       <c r="D139" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4451,7 +4499,7 @@
         <v>133</v>
       </c>
       <c r="D140" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4468,7 +4516,7 @@
         <v>134</v>
       </c>
       <c r="D141" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4485,7 +4533,7 @@
         <v>135</v>
       </c>
       <c r="D142" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4502,7 +4550,7 @@
         <v>136</v>
       </c>
       <c r="D143" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4519,7 +4567,7 @@
         <v>137</v>
       </c>
       <c r="D144" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4536,7 +4584,7 @@
         <v>138</v>
       </c>
       <c r="D145" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4553,7 +4601,7 @@
         <v>139</v>
       </c>
       <c r="D146" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4570,7 +4618,7 @@
         <v>140</v>
       </c>
       <c r="D147" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4587,7 +4635,7 @@
         <v>141</v>
       </c>
       <c r="D148" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4604,7 +4652,7 @@
         <v>142</v>
       </c>
       <c r="D149" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4621,7 +4669,7 @@
         <v>143</v>
       </c>
       <c r="D150" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4638,7 +4686,7 @@
         <v>144</v>
       </c>
       <c r="D151" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4655,7 +4703,7 @@
         <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="E152">
         <v>2</v>
@@ -4672,7 +4720,7 @@
         <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="E153">
         <v>2</v>
@@ -4689,7 +4737,7 @@
         <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="E154">
         <v>2</v>
@@ -4706,7 +4754,7 @@
         <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="E155">
         <v>2</v>
@@ -4723,7 +4771,7 @@
         <v>149</v>
       </c>
       <c r="D156" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="E156">
         <v>2</v>
@@ -4740,7 +4788,7 @@
         <v>150</v>
       </c>
       <c r="D157" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="E157">
         <v>3</v>
@@ -4757,7 +4805,7 @@
         <v>151</v>
       </c>
       <c r="D158" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="E158">
         <v>8</v>
@@ -4774,7 +4822,7 @@
         <v>152</v>
       </c>
       <c r="D159" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="E159">
         <v>8</v>
@@ -4791,7 +4839,7 @@
         <v>153</v>
       </c>
       <c r="D160" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="E160">
         <v>15</v>
@@ -4808,7 +4856,7 @@
         <v>154</v>
       </c>
       <c r="D161" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4825,7 +4873,7 @@
         <v>155</v>
       </c>
       <c r="D162" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4842,7 +4890,7 @@
         <v>156</v>
       </c>
       <c r="D163" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4859,7 +4907,7 @@
         <v>157</v>
       </c>
       <c r="D164" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4876,7 +4924,7 @@
         <v>158</v>
       </c>
       <c r="D165" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4893,7 +4941,7 @@
         <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4910,7 +4958,7 @@
         <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4927,7 +4975,7 @@
         <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4944,7 +4992,7 @@
         <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4961,7 +5009,7 @@
         <v>163</v>
       </c>
       <c r="D170" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4978,7 +5026,7 @@
         <v>164</v>
       </c>
       <c r="D171" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4995,7 +5043,7 @@
         <v>165</v>
       </c>
       <c r="D172" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5012,7 +5060,7 @@
         <v>166</v>
       </c>
       <c r="D173" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5029,7 +5077,7 @@
         <v>167</v>
       </c>
       <c r="D174" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5046,7 +5094,7 @@
         <v>168</v>
       </c>
       <c r="D175" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5063,7 +5111,7 @@
         <v>169</v>
       </c>
       <c r="D176" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5080,7 +5128,7 @@
         <v>170</v>
       </c>
       <c r="D177" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5097,7 +5145,7 @@
         <v>171</v>
       </c>
       <c r="D178" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5114,7 +5162,7 @@
         <v>172</v>
       </c>
       <c r="D179" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5131,7 +5179,7 @@
         <v>173</v>
       </c>
       <c r="D180" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5148,7 +5196,7 @@
         <v>174</v>
       </c>
       <c r="D181" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5165,7 +5213,7 @@
         <v>175</v>
       </c>
       <c r="D182" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5182,7 +5230,7 @@
         <v>176</v>
       </c>
       <c r="D183" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5199,7 +5247,7 @@
         <v>177</v>
       </c>
       <c r="D184" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5216,7 +5264,7 @@
         <v>178</v>
       </c>
       <c r="D185" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5233,7 +5281,7 @@
         <v>179</v>
       </c>
       <c r="D186" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5250,7 +5298,7 @@
         <v>180</v>
       </c>
       <c r="D187" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5267,7 +5315,7 @@
         <v>181</v>
       </c>
       <c r="D188" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5284,7 +5332,7 @@
         <v>182</v>
       </c>
       <c r="D189" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5301,7 +5349,7 @@
         <v>183</v>
       </c>
       <c r="D190" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5318,7 +5366,7 @@
         <v>184</v>
       </c>
       <c r="D191" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5335,7 +5383,7 @@
         <v>185</v>
       </c>
       <c r="D192" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5352,10 +5400,10 @@
         <v>186</v>
       </c>
       <c r="D193" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="E193">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -5369,7 +5417,7 @@
         <v>187</v>
       </c>
       <c r="D194" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="E194">
         <v>2</v>
@@ -5386,7 +5434,7 @@
         <v>188</v>
       </c>
       <c r="D195" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="E195">
         <v>2</v>
@@ -5403,7 +5451,7 @@
         <v>189</v>
       </c>
       <c r="D196" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="E196">
         <v>2</v>
@@ -5420,7 +5468,7 @@
         <v>190</v>
       </c>
       <c r="D197" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -5437,7 +5485,7 @@
         <v>191</v>
       </c>
       <c r="D198" t="s">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5454,7 +5502,7 @@
         <v>192</v>
       </c>
       <c r="D199" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5471,7 +5519,7 @@
         <v>193</v>
       </c>
       <c r="D200" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5488,7 +5536,7 @@
         <v>194</v>
       </c>
       <c r="D201" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5505,7 +5553,7 @@
         <v>195</v>
       </c>
       <c r="D202" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5522,7 +5570,7 @@
         <v>196</v>
       </c>
       <c r="D203" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5539,7 +5587,7 @@
         <v>197</v>
       </c>
       <c r="D204" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5556,10 +5604,10 @@
         <v>198</v>
       </c>
       <c r="D205" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="E205">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5573,7 +5621,7 @@
         <v>199</v>
       </c>
       <c r="D206" t="s">
-        <v>234</v>
+        <v>360</v>
       </c>
       <c r="E206">
         <v>3</v>
@@ -5590,10 +5638,10 @@
         <v>200</v>
       </c>
       <c r="D207" t="s">
-        <v>351</v>
+        <v>245</v>
       </c>
       <c r="E207">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5607,7 +5655,7 @@
         <v>201</v>
       </c>
       <c r="D208" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="E208">
         <v>4</v>
@@ -5624,7 +5672,7 @@
         <v>202</v>
       </c>
       <c r="D209" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="E209">
         <v>4</v>
@@ -5641,7 +5689,7 @@
         <v>203</v>
       </c>
       <c r="D210" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="E210">
         <v>4</v>
@@ -5658,7 +5706,7 @@
         <v>204</v>
       </c>
       <c r="D211" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="E211">
         <v>4</v>
@@ -5675,10 +5723,10 @@
         <v>205</v>
       </c>
       <c r="D212" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="E212">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5692,7 +5740,7 @@
         <v>206</v>
       </c>
       <c r="D213" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="E213">
         <v>5</v>
@@ -5709,10 +5757,10 @@
         <v>207</v>
       </c>
       <c r="D214" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="E214">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5726,10 +5774,10 @@
         <v>208</v>
       </c>
       <c r="D215" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="E215">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5743,10 +5791,10 @@
         <v>209</v>
       </c>
       <c r="D216" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="E216">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5760,7 +5808,7 @@
         <v>210</v>
       </c>
       <c r="D217" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="E217">
         <v>10</v>
@@ -5777,10 +5825,10 @@
         <v>211</v>
       </c>
       <c r="D218" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="E218">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5794,7 +5842,7 @@
         <v>212</v>
       </c>
       <c r="D219" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="E219">
         <v>12</v>
@@ -5811,10 +5859,10 @@
         <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="E220">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5828,10 +5876,10 @@
         <v>214</v>
       </c>
       <c r="D221" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="E221">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5845,10 +5893,214 @@
         <v>215</v>
       </c>
       <c r="D222" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="E222">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5">
+      <c r="A223" t="s">
+        <v>14</v>
+      </c>
+      <c r="B223" t="s">
+        <v>41</v>
+      </c>
+      <c r="C223" t="s">
+        <v>216</v>
+      </c>
+      <c r="D223" t="s">
+        <v>375</v>
+      </c>
+      <c r="E223">
         <v>20</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5">
+      <c r="A224" t="s">
+        <v>11</v>
+      </c>
+      <c r="B224" t="s">
+        <v>40</v>
+      </c>
+      <c r="C224" t="s">
+        <v>217</v>
+      </c>
+      <c r="D224" t="s">
+        <v>376</v>
+      </c>
+      <c r="E224">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5">
+      <c r="A225" t="s">
+        <v>12</v>
+      </c>
+      <c r="B225" t="s">
+        <v>40</v>
+      </c>
+      <c r="C225" t="s">
+        <v>217</v>
+      </c>
+      <c r="D225" t="s">
+        <v>376</v>
+      </c>
+      <c r="E225">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
+      <c r="A226" t="s">
+        <v>13</v>
+      </c>
+      <c r="B226" t="s">
+        <v>40</v>
+      </c>
+      <c r="C226" t="s">
+        <v>217</v>
+      </c>
+      <c r="D226" t="s">
+        <v>376</v>
+      </c>
+      <c r="E226">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
+      <c r="A227" t="s">
+        <v>10</v>
+      </c>
+      <c r="B227" t="s">
+        <v>38</v>
+      </c>
+      <c r="C227" t="s">
+        <v>218</v>
+      </c>
+      <c r="D227" t="s">
+        <v>371</v>
+      </c>
+      <c r="E227">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
+      <c r="A228" t="s">
+        <v>10</v>
+      </c>
+      <c r="B228" t="s">
+        <v>38</v>
+      </c>
+      <c r="C228" t="s">
+        <v>219</v>
+      </c>
+      <c r="D228" t="s">
+        <v>377</v>
+      </c>
+      <c r="E228">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5">
+      <c r="A229" t="s">
+        <v>13</v>
+      </c>
+      <c r="B229" t="s">
+        <v>40</v>
+      </c>
+      <c r="C229" t="s">
+        <v>220</v>
+      </c>
+      <c r="D229" t="s">
+        <v>378</v>
+      </c>
+      <c r="E229">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
+      <c r="A230" t="s">
+        <v>13</v>
+      </c>
+      <c r="B230" t="s">
+        <v>40</v>
+      </c>
+      <c r="C230" t="s">
+        <v>221</v>
+      </c>
+      <c r="D230" t="s">
+        <v>379</v>
+      </c>
+      <c r="E230">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5">
+      <c r="A231" t="s">
+        <v>13</v>
+      </c>
+      <c r="B231" t="s">
+        <v>40</v>
+      </c>
+      <c r="C231" t="s">
+        <v>222</v>
+      </c>
+      <c r="D231" t="s">
+        <v>281</v>
+      </c>
+      <c r="E231">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5">
+      <c r="A232" t="s">
+        <v>12</v>
+      </c>
+      <c r="B232" t="s">
+        <v>40</v>
+      </c>
+      <c r="C232" t="s">
+        <v>223</v>
+      </c>
+      <c r="D232" t="s">
+        <v>380</v>
+      </c>
+      <c r="E232">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5">
+      <c r="A233" t="s">
+        <v>12</v>
+      </c>
+      <c r="B233" t="s">
+        <v>40</v>
+      </c>
+      <c r="C233" t="s">
+        <v>224</v>
+      </c>
+      <c r="D233" t="s">
+        <v>381</v>
+      </c>
+      <c r="E233">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
+      <c r="A234" t="s">
+        <v>13</v>
+      </c>
+      <c r="B234" t="s">
+        <v>40</v>
+      </c>
+      <c r="C234" t="s">
+        <v>224</v>
+      </c>
+      <c r="D234" t="s">
+        <v>381</v>
+      </c>
+      <c r="E234">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Verificação ao vivo real durante os testes (RAC/Disponibilidade Diária)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="376">
   <si>
     <t>matricula</t>
   </si>
@@ -200,12 +200,6 @@
     <t>3122678-04</t>
   </si>
   <si>
-    <t>3011755</t>
-  </si>
-  <si>
-    <t>540-1407-4</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -572,9 +566,6 @@
     <t>C622010-0102</t>
   </si>
   <si>
-    <t>060-0015-00</t>
-  </si>
-  <si>
     <t>2615018-1</t>
   </si>
   <si>
@@ -701,12 +692,6 @@
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
-    <t>INSULATION BLANKET,T</t>
-  </si>
-  <si>
-    <t>VALVE,COMPRESSOR BLEED</t>
-  </si>
-  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
@@ -1056,9 +1041,6 @@
   </si>
   <si>
     <t>LIGHT STROBE RH</t>
-  </si>
-  <si>
-    <t>CONTROL,DIRECTIONAL</t>
   </si>
   <si>
     <t>MOLDING-WINDOW</t>
@@ -1167,8 +1149,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1184,7 +1174,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1192,12 +1182,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1496,22 +1504,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1563,16 +1571,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1689,10 +1697,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F10">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2122,23 +2130,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2153,7 +2161,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2170,7 +2178,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2187,7 +2195,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2204,7 +2212,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2221,7 +2229,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2238,7 +2246,7 @@
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2255,7 +2263,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2272,7 +2280,7 @@
         <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2280,16 +2288,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2297,16 +2305,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2314,16 +2322,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2331,16 +2339,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2348,16 +2356,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2365,16 +2373,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2382,16 +2390,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
         <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2399,16 +2407,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2416,16 +2424,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2433,16 +2441,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2450,16 +2458,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2467,16 +2475,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2484,16 +2492,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2501,16 +2509,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2518,16 +2526,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2535,16 +2543,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2552,16 +2560,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2569,16 +2577,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2586,16 +2594,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2603,16 +2611,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2626,13 +2634,13 @@
         <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2643,10 +2651,10 @@
         <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2654,19 +2662,19 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
         <v>68</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2680,7 +2688,7 @@
         <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2697,7 +2705,7 @@
         <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2714,41 +2722,41 @@
         <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2756,33 +2764,33 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E38">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2790,16 +2798,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2807,33 +2815,33 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2841,33 +2849,33 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2875,19 +2883,19 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2898,13 +2906,13 @@
         <v>41</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2915,10 +2923,10 @@
         <v>38</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2926,19 +2934,19 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C48" t="s">
         <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2952,7 +2960,7 @@
         <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2969,27 +2977,27 @@
         <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D51" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3000,10 +3008,10 @@
         <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D52" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E52">
         <v>4</v>
@@ -3011,50 +3019,50 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
         <v>80</v>
       </c>
       <c r="D53" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D54" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B55" t="s">
         <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D55" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3062,16 +3070,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B56" t="s">
         <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D56" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3079,16 +3087,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
         <v>40</v>
       </c>
       <c r="C57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D57" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3096,16 +3104,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B58" t="s">
         <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3113,16 +3121,16 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
         <v>40</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3136,10 +3144,10 @@
         <v>40</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D60" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3153,10 +3161,10 @@
         <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D61" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3170,10 +3178,10 @@
         <v>40</v>
       </c>
       <c r="C62" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D62" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3187,10 +3195,10 @@
         <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D63" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3198,7 +3206,7 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
         <v>40</v>
@@ -3207,41 +3215,41 @@
         <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
         <v>40</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D65" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
         <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D66" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3249,16 +3257,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D67" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3266,16 +3274,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>40</v>
       </c>
       <c r="C68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D68" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3283,16 +3291,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D69" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3300,16 +3308,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B70" t="s">
         <v>40</v>
       </c>
       <c r="C70" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D70" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3317,16 +3325,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B71" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C71" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D71" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3334,16 +3342,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
         <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D72" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3351,16 +3359,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D73" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3368,16 +3376,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B74" t="s">
         <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D74" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3385,16 +3393,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
         <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D75" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3402,16 +3410,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
         <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D76" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3419,101 +3427,101 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B77" t="s">
         <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D77" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E77">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C78" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D78" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E78">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s">
         <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D79" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E79">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
         <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E80">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
         <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E81">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D82" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3521,16 +3529,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
         <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D83" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3538,16 +3546,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D84" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3555,33 +3563,33 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D85" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B86" t="s">
         <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D86" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3589,19 +3597,19 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D87" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3612,10 +3620,10 @@
         <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3629,10 +3637,10 @@
         <v>40</v>
       </c>
       <c r="C89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D89" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3646,10 +3654,10 @@
         <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3663,10 +3671,10 @@
         <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D91" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3680,10 +3688,10 @@
         <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3697,10 +3705,10 @@
         <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D93" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3714,10 +3722,10 @@
         <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3731,10 +3739,10 @@
         <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D95" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3748,10 +3756,10 @@
         <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D96" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3765,10 +3773,10 @@
         <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D97" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3782,10 +3790,10 @@
         <v>40</v>
       </c>
       <c r="C98" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D98" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3793,16 +3801,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B99" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D99" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3816,10 +3824,10 @@
         <v>40</v>
       </c>
       <c r="C100" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D100" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3833,10 +3841,10 @@
         <v>41</v>
       </c>
       <c r="C101" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D101" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3850,10 +3858,10 @@
         <v>40</v>
       </c>
       <c r="C102" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D102" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3861,16 +3869,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C103" t="s">
         <v>101</v>
       </c>
       <c r="D103" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3887,7 +3895,7 @@
         <v>102</v>
       </c>
       <c r="D104" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3904,7 +3912,7 @@
         <v>103</v>
       </c>
       <c r="D105" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3921,7 +3929,7 @@
         <v>104</v>
       </c>
       <c r="D106" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3938,7 +3946,7 @@
         <v>105</v>
       </c>
       <c r="D107" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3955,24 +3963,24 @@
         <v>106</v>
       </c>
       <c r="D108" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B109" t="s">
         <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D109" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3986,10 +3994,10 @@
         <v>40</v>
       </c>
       <c r="C110" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D110" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4003,13 +4011,13 @@
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D111" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -4020,10 +4028,10 @@
         <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D112" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4037,13 +4045,13 @@
         <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D113" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E113">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -4054,10 +4062,10 @@
         <v>40</v>
       </c>
       <c r="C114" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D114" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4065,7 +4073,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
@@ -4074,10 +4082,10 @@
         <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E115">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -4091,7 +4099,7 @@
         <v>111</v>
       </c>
       <c r="D116" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4108,10 +4116,10 @@
         <v>112</v>
       </c>
       <c r="D117" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -4125,10 +4133,10 @@
         <v>113</v>
       </c>
       <c r="D118" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -4142,61 +4150,61 @@
         <v>114</v>
       </c>
       <c r="D119" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E119">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B120" t="s">
         <v>40</v>
       </c>
       <c r="C120" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D120" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="E120">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B121" t="s">
         <v>40</v>
       </c>
       <c r="C121" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D121" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E121">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B122" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C122" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D122" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E122">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4207,10 +4215,10 @@
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D123" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4218,16 +4226,16 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C124" t="s">
         <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4244,7 +4252,7 @@
         <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4261,7 +4269,7 @@
         <v>119</v>
       </c>
       <c r="D126" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4278,7 +4286,7 @@
         <v>120</v>
       </c>
       <c r="D127" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4295,7 +4303,7 @@
         <v>121</v>
       </c>
       <c r="D128" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4312,7 +4320,7 @@
         <v>122</v>
       </c>
       <c r="D129" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4329,7 +4337,7 @@
         <v>123</v>
       </c>
       <c r="D130" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4346,7 +4354,7 @@
         <v>124</v>
       </c>
       <c r="D131" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4363,7 +4371,7 @@
         <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4380,7 +4388,7 @@
         <v>126</v>
       </c>
       <c r="D133" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4397,7 +4405,7 @@
         <v>127</v>
       </c>
       <c r="D134" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4414,7 +4422,7 @@
         <v>128</v>
       </c>
       <c r="D135" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4431,7 +4439,7 @@
         <v>129</v>
       </c>
       <c r="D136" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4448,7 +4456,7 @@
         <v>130</v>
       </c>
       <c r="D137" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4465,7 +4473,7 @@
         <v>131</v>
       </c>
       <c r="D138" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4482,7 +4490,7 @@
         <v>132</v>
       </c>
       <c r="D139" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4499,7 +4507,7 @@
         <v>133</v>
       </c>
       <c r="D140" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4516,7 +4524,7 @@
         <v>134</v>
       </c>
       <c r="D141" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4533,7 +4541,7 @@
         <v>135</v>
       </c>
       <c r="D142" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4550,7 +4558,7 @@
         <v>136</v>
       </c>
       <c r="D143" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4567,7 +4575,7 @@
         <v>137</v>
       </c>
       <c r="D144" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4584,7 +4592,7 @@
         <v>138</v>
       </c>
       <c r="D145" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4601,7 +4609,7 @@
         <v>139</v>
       </c>
       <c r="D146" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4618,7 +4626,7 @@
         <v>140</v>
       </c>
       <c r="D147" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4635,7 +4643,7 @@
         <v>141</v>
       </c>
       <c r="D148" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4652,7 +4660,7 @@
         <v>142</v>
       </c>
       <c r="D149" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4669,10 +4677,10 @@
         <v>143</v>
       </c>
       <c r="D150" t="s">
-        <v>308</v>
+        <v>290</v>
       </c>
       <c r="E150">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -4686,10 +4694,10 @@
         <v>144</v>
       </c>
       <c r="D151" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="E151">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -4703,7 +4711,7 @@
         <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>295</v>
+        <v>306</v>
       </c>
       <c r="E152">
         <v>2</v>
@@ -4720,7 +4728,7 @@
         <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E153">
         <v>2</v>
@@ -4737,7 +4745,7 @@
         <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E154">
         <v>2</v>
@@ -4754,10 +4762,10 @@
         <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E155">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -4771,10 +4779,10 @@
         <v>149</v>
       </c>
       <c r="D156" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E156">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -4788,10 +4796,10 @@
         <v>150</v>
       </c>
       <c r="D157" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E157">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -4805,44 +4813,44 @@
         <v>151</v>
       </c>
       <c r="D158" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E158">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B159" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C159" t="s">
         <v>152</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E159">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B160" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C160" t="s">
         <v>153</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E160">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4856,7 +4864,7 @@
         <v>154</v>
       </c>
       <c r="D161" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4873,7 +4881,7 @@
         <v>155</v>
       </c>
       <c r="D162" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4890,7 +4898,7 @@
         <v>156</v>
       </c>
       <c r="D163" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4907,7 +4915,7 @@
         <v>157</v>
       </c>
       <c r="D164" t="s">
-        <v>321</v>
+        <v>240</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4924,7 +4932,7 @@
         <v>158</v>
       </c>
       <c r="D165" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4941,7 +4949,7 @@
         <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>245</v>
+        <v>319</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4958,7 +4966,7 @@
         <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4975,7 +4983,7 @@
         <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4992,7 +5000,7 @@
         <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -5009,7 +5017,7 @@
         <v>163</v>
       </c>
       <c r="D170" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5026,7 +5034,7 @@
         <v>164</v>
       </c>
       <c r="D171" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5043,7 +5051,7 @@
         <v>165</v>
       </c>
       <c r="D172" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5060,7 +5068,7 @@
         <v>166</v>
       </c>
       <c r="D173" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5077,7 +5085,7 @@
         <v>167</v>
       </c>
       <c r="D174" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5094,7 +5102,7 @@
         <v>168</v>
       </c>
       <c r="D175" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5111,7 +5119,7 @@
         <v>169</v>
       </c>
       <c r="D176" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5128,7 +5136,7 @@
         <v>170</v>
       </c>
       <c r="D177" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5145,7 +5153,7 @@
         <v>171</v>
       </c>
       <c r="D178" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5162,7 +5170,7 @@
         <v>172</v>
       </c>
       <c r="D179" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5179,7 +5187,7 @@
         <v>173</v>
       </c>
       <c r="D180" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5196,7 +5204,7 @@
         <v>174</v>
       </c>
       <c r="D181" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5213,7 +5221,7 @@
         <v>175</v>
       </c>
       <c r="D182" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5230,7 +5238,7 @@
         <v>176</v>
       </c>
       <c r="D183" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5247,7 +5255,7 @@
         <v>177</v>
       </c>
       <c r="D184" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5264,7 +5272,7 @@
         <v>178</v>
       </c>
       <c r="D185" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5281,7 +5289,7 @@
         <v>179</v>
       </c>
       <c r="D186" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5298,7 +5306,7 @@
         <v>180</v>
       </c>
       <c r="D187" t="s">
-        <v>343</v>
+        <v>300</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5315,7 +5323,7 @@
         <v>181</v>
       </c>
       <c r="D188" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5332,7 +5340,7 @@
         <v>182</v>
       </c>
       <c r="D189" t="s">
-        <v>305</v>
+        <v>341</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5349,7 +5357,7 @@
         <v>183</v>
       </c>
       <c r="D190" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5366,10 +5374,10 @@
         <v>184</v>
       </c>
       <c r="D191" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E191">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -5383,10 +5391,10 @@
         <v>185</v>
       </c>
       <c r="D192" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E192">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -5400,10 +5408,10 @@
         <v>186</v>
       </c>
       <c r="D193" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E193">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -5417,7 +5425,7 @@
         <v>187</v>
       </c>
       <c r="D194" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E194">
         <v>2</v>
@@ -5434,7 +5442,7 @@
         <v>188</v>
       </c>
       <c r="D195" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E195">
         <v>2</v>
@@ -5451,7 +5459,7 @@
         <v>189</v>
       </c>
       <c r="D196" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E196">
         <v>2</v>
@@ -5468,7 +5476,7 @@
         <v>190</v>
       </c>
       <c r="D197" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -5485,7 +5493,7 @@
         <v>191</v>
       </c>
       <c r="D198" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5502,7 +5510,7 @@
         <v>192</v>
       </c>
       <c r="D199" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5519,7 +5527,7 @@
         <v>193</v>
       </c>
       <c r="D200" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5536,7 +5544,7 @@
         <v>194</v>
       </c>
       <c r="D201" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5553,7 +5561,7 @@
         <v>195</v>
       </c>
       <c r="D202" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5570,10 +5578,10 @@
         <v>196</v>
       </c>
       <c r="D203" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E203">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -5587,10 +5595,10 @@
         <v>197</v>
       </c>
       <c r="D204" t="s">
-        <v>358</v>
+        <v>240</v>
       </c>
       <c r="E204">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5604,10 +5612,10 @@
         <v>198</v>
       </c>
       <c r="D205" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="E205">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5621,10 +5629,10 @@
         <v>199</v>
       </c>
       <c r="D206" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="E206">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5638,10 +5646,10 @@
         <v>200</v>
       </c>
       <c r="D207" t="s">
-        <v>245</v>
+        <v>357</v>
       </c>
       <c r="E207">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5655,7 +5663,7 @@
         <v>201</v>
       </c>
       <c r="D208" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E208">
         <v>4</v>
@@ -5672,7 +5680,7 @@
         <v>202</v>
       </c>
       <c r="D209" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E209">
         <v>4</v>
@@ -5689,10 +5697,10 @@
         <v>203</v>
       </c>
       <c r="D210" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="E210">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5706,10 +5714,10 @@
         <v>204</v>
       </c>
       <c r="D211" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E211">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5723,10 +5731,10 @@
         <v>205</v>
       </c>
       <c r="D212" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E212">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5740,10 +5748,10 @@
         <v>206</v>
       </c>
       <c r="D213" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E213">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5757,10 +5765,10 @@
         <v>207</v>
       </c>
       <c r="D214" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="E214">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5774,10 +5782,10 @@
         <v>208</v>
       </c>
       <c r="D215" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="E215">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5791,10 +5799,10 @@
         <v>209</v>
       </c>
       <c r="D216" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E216">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5808,10 +5816,10 @@
         <v>210</v>
       </c>
       <c r="D217" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="E217">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5825,10 +5833,10 @@
         <v>211</v>
       </c>
       <c r="D218" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="E218">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5842,10 +5850,10 @@
         <v>212</v>
       </c>
       <c r="D219" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E219">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5859,95 +5867,95 @@
         <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="E220">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B221" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C221" t="s">
         <v>214</v>
       </c>
       <c r="D221" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E221">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D222" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="E222">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B223" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D223" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="E223">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B224" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C224" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D224" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="E224">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B225" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C225" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D225" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="E225">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5961,49 +5969,49 @@
         <v>217</v>
       </c>
       <c r="D226" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="E226">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B227" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C227" t="s">
         <v>218</v>
       </c>
       <c r="D227" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E227">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B228" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C228" t="s">
         <v>219</v>
       </c>
       <c r="D228" t="s">
-        <v>377</v>
+        <v>276</v>
       </c>
       <c r="E228">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B229" t="s">
         <v>40</v>
@@ -6012,15 +6020,15 @@
         <v>220</v>
       </c>
       <c r="D229" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="E229">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="230" spans="1:5">
       <c r="A230" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B230" t="s">
         <v>40</v>
@@ -6029,10 +6037,10 @@
         <v>221</v>
       </c>
       <c r="D230" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="E230">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6043,63 +6051,12 @@
         <v>40</v>
       </c>
       <c r="C231" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D231" t="s">
-        <v>281</v>
+        <v>375</v>
       </c>
       <c r="E231">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="232" spans="1:5">
-      <c r="A232" t="s">
-        <v>12</v>
-      </c>
-      <c r="B232" t="s">
-        <v>40</v>
-      </c>
-      <c r="C232" t="s">
-        <v>223</v>
-      </c>
-      <c r="D232" t="s">
-        <v>380</v>
-      </c>
-      <c r="E232">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="233" spans="1:5">
-      <c r="A233" t="s">
-        <v>12</v>
-      </c>
-      <c r="B233" t="s">
-        <v>40</v>
-      </c>
-      <c r="C233" t="s">
-        <v>224</v>
-      </c>
-      <c r="D233" t="s">
-        <v>381</v>
-      </c>
-      <c r="E233">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="234" spans="1:5">
-      <c r="A234" t="s">
-        <v>13</v>
-      </c>
-      <c r="B234" t="s">
-        <v>40</v>
-      </c>
-      <c r="C234" t="s">
-        <v>224</v>
-      </c>
-      <c r="D234" t="s">
-        <v>381</v>
-      </c>
-      <c r="E234">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (27/07/2026 19:40)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1149,16 +1149,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1174,7 +1166,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1182,30 +1174,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1504,22 +1478,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2134,19 +2108,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (29/07/2026 13:12)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="371">
   <si>
     <t>matricula</t>
   </si>
@@ -584,9 +584,6 @@
     <t>C622010-0102</t>
   </si>
   <si>
-    <t>2615018-1</t>
-  </si>
-  <si>
     <t>C662041-0102</t>
   </si>
   <si>
@@ -677,6 +674,9 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>2617015-15</t>
+  </si>
+  <si>
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
@@ -1050,9 +1050,6 @@
   </si>
   <si>
     <t>LIGHT STROBE RH</t>
-  </si>
-  <si>
-    <t>MOLDING-WINDOW</t>
   </si>
   <si>
     <t>INDICATOR FUEL</t>
@@ -1559,10 +1556,10 @@
         <v>54</v>
       </c>
       <c r="E5">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F5">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1599,10 +1596,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F7">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2092,7 +2089,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E227"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2437,10 +2434,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
         <v>62</v>
@@ -2454,10 +2451,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
         <v>62</v>
@@ -2471,16 +2468,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2488,10 +2485,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
         <v>63</v>
@@ -2505,10 +2502,10 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -2522,16 +2519,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2539,10 +2536,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
         <v>64</v>
@@ -2551,24 +2548,24 @@
         <v>226</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2579,10 +2576,10 @@
         <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2596,10 +2593,10 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2613,10 +2610,10 @@
         <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2630,21 +2627,21 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
         <v>69</v>
@@ -2653,12 +2650,12 @@
         <v>231</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
@@ -2670,15 +2667,15 @@
         <v>231</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
         <v>69</v>
@@ -2692,16 +2689,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E36">
         <v>2</v>
@@ -2709,10 +2706,10 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
         <v>70</v>
@@ -2726,10 +2723,10 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
         <v>70</v>
@@ -2738,32 +2735,32 @@
         <v>232</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" t="s">
         <v>71</v>
@@ -2772,15 +2769,15 @@
         <v>233</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
         <v>71</v>
@@ -2789,21 +2786,21 @@
         <v>233</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2811,10 +2808,10 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C43" t="s">
         <v>72</v>
@@ -2823,24 +2820,24 @@
         <v>234</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2851,10 +2848,10 @@
         <v>37</v>
       </c>
       <c r="C45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2868,10 +2865,10 @@
         <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2885,10 +2882,10 @@
         <v>37</v>
       </c>
       <c r="C47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2902,21 +2899,21 @@
         <v>37</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C49" t="s">
         <v>77</v>
@@ -2930,16 +2927,16 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B50" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E50">
         <v>4</v>
@@ -2953,10 +2950,10 @@
         <v>37</v>
       </c>
       <c r="C51" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D51" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -2964,24 +2961,24 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D52" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E52">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
@@ -2998,7 +2995,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B54" t="s">
         <v>38</v>
@@ -3015,16 +3012,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B55" t="s">
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D55" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3032,7 +3029,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B56" t="s">
         <v>38</v>
@@ -3049,7 +3046,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
         <v>38</v>
@@ -3066,16 +3063,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B58" t="s">
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D58" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3083,7 +3080,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B59" t="s">
         <v>38</v>
@@ -3100,16 +3097,16 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B60" t="s">
         <v>38</v>
       </c>
       <c r="C60" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3117,7 +3114,7 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B61" t="s">
         <v>38</v>
@@ -3134,16 +3131,16 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B62" t="s">
         <v>38</v>
       </c>
       <c r="C62" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3157,18 +3154,18 @@
         <v>38</v>
       </c>
       <c r="C63" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B64" t="s">
         <v>38</v>
@@ -3185,7 +3182,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B65" t="s">
         <v>38</v>
@@ -3202,10 +3199,10 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C66" t="s">
         <v>85</v>
@@ -3219,16 +3216,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B67" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C67" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3236,7 +3233,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B68" t="s">
         <v>38</v>
@@ -3253,7 +3250,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B69" t="s">
         <v>38</v>
@@ -3270,10 +3267,10 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C70" t="s">
         <v>86</v>
@@ -3287,16 +3284,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B71" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C71" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D71" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3304,7 +3301,7 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B72" t="s">
         <v>38</v>
@@ -3321,7 +3318,7 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B73" t="s">
         <v>38</v>
@@ -3338,16 +3335,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B74" t="s">
         <v>38</v>
       </c>
       <c r="C74" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D74" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3355,7 +3352,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B75" t="s">
         <v>38</v>
@@ -3372,7 +3369,7 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B76" t="s">
         <v>38</v>
@@ -3384,15 +3381,15 @@
         <v>250</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>88</v>
@@ -3406,24 +3403,24 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C78" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D78" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B79" t="s">
         <v>38</v>
@@ -3435,12 +3432,12 @@
         <v>251</v>
       </c>
       <c r="E79">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
         <v>38</v>
@@ -3457,41 +3454,41 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B81" t="s">
         <v>38</v>
       </c>
       <c r="C81" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E81">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B82" t="s">
         <v>38</v>
       </c>
       <c r="C82" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D82" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E82">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B83" t="s">
         <v>38</v>
@@ -3508,10 +3505,10 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B84" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C84" t="s">
         <v>91</v>
@@ -3525,16 +3522,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B85" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C85" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3542,7 +3539,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
         <v>38</v>
@@ -3559,10 +3556,10 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B87" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
         <v>92</v>
@@ -3571,29 +3568,29 @@
         <v>250</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B88" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C88" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B89" t="s">
         <v>38</v>
@@ -3610,16 +3607,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B90" t="s">
         <v>38</v>
       </c>
       <c r="C90" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D90" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3627,7 +3624,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B91" t="s">
         <v>38</v>
@@ -3644,16 +3641,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B92" t="s">
         <v>38</v>
       </c>
       <c r="C92" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D92" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3661,7 +3658,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B93" t="s">
         <v>38</v>
@@ -3678,16 +3675,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B94" t="s">
         <v>38</v>
       </c>
       <c r="C94" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D94" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3695,7 +3692,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B95" t="s">
         <v>38</v>
@@ -3712,16 +3709,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B96" t="s">
         <v>38</v>
       </c>
       <c r="C96" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D96" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3729,7 +3726,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B97" t="s">
         <v>38</v>
@@ -3752,10 +3749,10 @@
         <v>38</v>
       </c>
       <c r="C98" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D98" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3769,10 +3766,10 @@
         <v>38</v>
       </c>
       <c r="C99" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D99" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3786,10 +3783,10 @@
         <v>38</v>
       </c>
       <c r="C100" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D100" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3803,10 +3800,10 @@
         <v>38</v>
       </c>
       <c r="C101" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D101" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3814,16 +3811,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B102" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D102" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3837,10 +3834,10 @@
         <v>38</v>
       </c>
       <c r="C103" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D103" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3854,10 +3851,10 @@
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D104" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3871,10 +3868,10 @@
         <v>38</v>
       </c>
       <c r="C105" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D105" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3882,16 +3879,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B106" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C106" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D106" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3905,10 +3902,10 @@
         <v>38</v>
       </c>
       <c r="C107" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D107" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3922,10 +3919,10 @@
         <v>38</v>
       </c>
       <c r="C108" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D108" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3939,10 +3936,10 @@
         <v>38</v>
       </c>
       <c r="C109" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D109" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3956,10 +3953,10 @@
         <v>38</v>
       </c>
       <c r="C110" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D110" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3973,27 +3970,27 @@
         <v>38</v>
       </c>
       <c r="C111" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D111" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B112" t="s">
         <v>38</v>
       </c>
       <c r="C112" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D112" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4007,10 +4004,10 @@
         <v>38</v>
       </c>
       <c r="C113" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D113" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4024,13 +4021,13 @@
         <v>38</v>
       </c>
       <c r="C114" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D114" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -4041,10 +4038,10 @@
         <v>38</v>
       </c>
       <c r="C115" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4058,13 +4055,13 @@
         <v>38</v>
       </c>
       <c r="C116" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D116" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -4075,10 +4072,10 @@
         <v>38</v>
       </c>
       <c r="C117" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D117" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4086,19 +4083,19 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B118" t="s">
         <v>38</v>
       </c>
       <c r="C118" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D118" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E118">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -4109,10 +4106,10 @@
         <v>38</v>
       </c>
       <c r="C119" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D119" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4126,13 +4123,13 @@
         <v>38</v>
       </c>
       <c r="C120" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D120" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4143,13 +4140,13 @@
         <v>38</v>
       </c>
       <c r="C121" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D121" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4160,13 +4157,13 @@
         <v>38</v>
       </c>
       <c r="C122" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D122" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E122">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4177,64 +4174,64 @@
         <v>38</v>
       </c>
       <c r="C123" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D123" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E123">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B124" t="s">
         <v>38</v>
       </c>
       <c r="C124" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E124">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B125" t="s">
         <v>38</v>
       </c>
       <c r="C125" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E125">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B126" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D126" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E126">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4245,10 +4242,10 @@
         <v>38</v>
       </c>
       <c r="C127" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D127" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4256,16 +4253,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B128" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C128" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D128" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4279,10 +4276,10 @@
         <v>38</v>
       </c>
       <c r="C129" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D129" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4296,10 +4293,10 @@
         <v>38</v>
       </c>
       <c r="C130" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D130" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4313,10 +4310,10 @@
         <v>38</v>
       </c>
       <c r="C131" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D131" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4330,10 +4327,10 @@
         <v>38</v>
       </c>
       <c r="C132" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D132" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4347,10 +4344,10 @@
         <v>38</v>
       </c>
       <c r="C133" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D133" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4364,10 +4361,10 @@
         <v>38</v>
       </c>
       <c r="C134" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D134" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4381,10 +4378,10 @@
         <v>38</v>
       </c>
       <c r="C135" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D135" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4398,10 +4395,10 @@
         <v>38</v>
       </c>
       <c r="C136" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D136" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4415,10 +4412,10 @@
         <v>38</v>
       </c>
       <c r="C137" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D137" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4432,10 +4429,10 @@
         <v>38</v>
       </c>
       <c r="C138" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D138" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4449,10 +4446,10 @@
         <v>38</v>
       </c>
       <c r="C139" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D139" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4466,10 +4463,10 @@
         <v>38</v>
       </c>
       <c r="C140" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D140" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4483,10 +4480,10 @@
         <v>38</v>
       </c>
       <c r="C141" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D141" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4500,10 +4497,10 @@
         <v>38</v>
       </c>
       <c r="C142" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D142" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4517,10 +4514,10 @@
         <v>38</v>
       </c>
       <c r="C143" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D143" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4534,10 +4531,10 @@
         <v>38</v>
       </c>
       <c r="C144" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D144" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4551,10 +4548,10 @@
         <v>38</v>
       </c>
       <c r="C145" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D145" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4568,10 +4565,10 @@
         <v>38</v>
       </c>
       <c r="C146" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D146" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4585,10 +4582,10 @@
         <v>38</v>
       </c>
       <c r="C147" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D147" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4602,10 +4599,10 @@
         <v>38</v>
       </c>
       <c r="C148" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D148" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4619,10 +4616,10 @@
         <v>38</v>
       </c>
       <c r="C149" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D149" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4636,10 +4633,10 @@
         <v>38</v>
       </c>
       <c r="C150" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D150" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4653,10 +4650,10 @@
         <v>38</v>
       </c>
       <c r="C151" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D151" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4670,10 +4667,10 @@
         <v>38</v>
       </c>
       <c r="C152" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D152" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4687,10 +4684,10 @@
         <v>38</v>
       </c>
       <c r="C153" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D153" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4704,10 +4701,10 @@
         <v>38</v>
       </c>
       <c r="C154" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D154" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4721,13 +4718,13 @@
         <v>38</v>
       </c>
       <c r="C155" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D155" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="E155">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -4738,13 +4735,13 @@
         <v>38</v>
       </c>
       <c r="C156" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D156" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E156">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -4755,10 +4752,10 @@
         <v>38</v>
       </c>
       <c r="C157" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D157" t="s">
-        <v>291</v>
+        <v>308</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4772,10 +4769,10 @@
         <v>38</v>
       </c>
       <c r="C158" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D158" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4789,10 +4786,10 @@
         <v>38</v>
       </c>
       <c r="C159" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D159" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E159">
         <v>2</v>
@@ -4806,13 +4803,13 @@
         <v>38</v>
       </c>
       <c r="C160" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D160" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E160">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4823,13 +4820,13 @@
         <v>38</v>
       </c>
       <c r="C161" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D161" t="s">
-        <v>310</v>
+        <v>277</v>
       </c>
       <c r="E161">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4840,13 +4837,13 @@
         <v>38</v>
       </c>
       <c r="C162" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D162" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E162">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4857,13 +4854,13 @@
         <v>38</v>
       </c>
       <c r="C163" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D163" t="s">
-        <v>277</v>
+        <v>313</v>
       </c>
       <c r="E163">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4874,13 +4871,13 @@
         <v>38</v>
       </c>
       <c r="C164" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D164" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E164">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4891,47 +4888,47 @@
         <v>38</v>
       </c>
       <c r="C165" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D165" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E165">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B166" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D166" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E166">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B167" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D167" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E167">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -4942,10 +4939,10 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D168" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4959,10 +4956,10 @@
         <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D169" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4976,10 +4973,10 @@
         <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D170" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4993,10 +4990,10 @@
         <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D171" t="s">
-        <v>319</v>
+        <v>236</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5010,10 +5007,10 @@
         <v>39</v>
       </c>
       <c r="C172" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D172" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5027,10 +5024,10 @@
         <v>39</v>
       </c>
       <c r="C173" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D173" t="s">
-        <v>236</v>
+        <v>322</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5044,10 +5041,10 @@
         <v>39</v>
       </c>
       <c r="C174" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D174" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5061,10 +5058,10 @@
         <v>39</v>
       </c>
       <c r="C175" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D175" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5078,10 +5075,10 @@
         <v>39</v>
       </c>
       <c r="C176" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D176" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5095,10 +5092,10 @@
         <v>39</v>
       </c>
       <c r="C177" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D177" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5112,10 +5109,10 @@
         <v>39</v>
       </c>
       <c r="C178" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D178" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5129,10 +5126,10 @@
         <v>39</v>
       </c>
       <c r="C179" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D179" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5146,10 +5143,10 @@
         <v>39</v>
       </c>
       <c r="C180" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D180" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5163,10 +5160,10 @@
         <v>39</v>
       </c>
       <c r="C181" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D181" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5180,10 +5177,10 @@
         <v>39</v>
       </c>
       <c r="C182" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D182" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5197,10 +5194,10 @@
         <v>39</v>
       </c>
       <c r="C183" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D183" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5214,10 +5211,10 @@
         <v>39</v>
       </c>
       <c r="C184" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D184" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5231,10 +5228,10 @@
         <v>39</v>
       </c>
       <c r="C185" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D185" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5248,10 +5245,10 @@
         <v>39</v>
       </c>
       <c r="C186" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D186" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5265,10 +5262,10 @@
         <v>39</v>
       </c>
       <c r="C187" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D187" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5282,10 +5279,10 @@
         <v>39</v>
       </c>
       <c r="C188" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D188" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5299,10 +5296,10 @@
         <v>39</v>
       </c>
       <c r="C189" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D189" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5316,10 +5313,10 @@
         <v>39</v>
       </c>
       <c r="C190" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D190" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5333,10 +5330,10 @@
         <v>39</v>
       </c>
       <c r="C191" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D191" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5350,10 +5347,10 @@
         <v>39</v>
       </c>
       <c r="C192" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D192" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5367,10 +5364,10 @@
         <v>39</v>
       </c>
       <c r="C193" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D193" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5384,10 +5381,10 @@
         <v>39</v>
       </c>
       <c r="C194" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D194" t="s">
-        <v>341</v>
+        <v>301</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5401,10 +5398,10 @@
         <v>39</v>
       </c>
       <c r="C195" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D195" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5418,10 +5415,10 @@
         <v>39</v>
       </c>
       <c r="C196" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D196" t="s">
-        <v>301</v>
+        <v>344</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5435,13 +5432,13 @@
         <v>39</v>
       </c>
       <c r="C197" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D197" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E197">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -5452,13 +5449,13 @@
         <v>39</v>
       </c>
       <c r="C198" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D198" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E198">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -5469,13 +5466,13 @@
         <v>39</v>
       </c>
       <c r="C199" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D199" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E199">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5486,10 +5483,10 @@
         <v>39</v>
       </c>
       <c r="C200" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D200" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5503,10 +5500,10 @@
         <v>39</v>
       </c>
       <c r="C201" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D201" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5520,10 +5517,10 @@
         <v>39</v>
       </c>
       <c r="C202" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D202" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5537,10 +5534,10 @@
         <v>39</v>
       </c>
       <c r="C203" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D203" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5554,10 +5551,10 @@
         <v>39</v>
       </c>
       <c r="C204" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D204" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5571,10 +5568,10 @@
         <v>39</v>
       </c>
       <c r="C205" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D205" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5588,10 +5585,10 @@
         <v>39</v>
       </c>
       <c r="C206" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D206" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5605,10 +5602,10 @@
         <v>39</v>
       </c>
       <c r="C207" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D207" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5622,10 +5619,10 @@
         <v>39</v>
       </c>
       <c r="C208" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D208" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5639,13 +5636,13 @@
         <v>39</v>
       </c>
       <c r="C209" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D209" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E209">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5656,13 +5653,13 @@
         <v>39</v>
       </c>
       <c r="C210" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D210" t="s">
-        <v>355</v>
+        <v>236</v>
       </c>
       <c r="E210">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5673,13 +5670,13 @@
         <v>39</v>
       </c>
       <c r="C211" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D211" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E211">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5690,13 +5687,13 @@
         <v>39</v>
       </c>
       <c r="C212" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D212" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E212">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5707,13 +5704,13 @@
         <v>39</v>
       </c>
       <c r="C213" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D213" t="s">
-        <v>236</v>
+        <v>359</v>
       </c>
       <c r="E213">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5724,10 +5721,10 @@
         <v>39</v>
       </c>
       <c r="C214" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D214" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E214">
         <v>4</v>
@@ -5741,10 +5738,10 @@
         <v>39</v>
       </c>
       <c r="C215" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D215" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5758,13 +5755,13 @@
         <v>39</v>
       </c>
       <c r="C216" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D216" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E216">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5775,13 +5772,13 @@
         <v>39</v>
       </c>
       <c r="C217" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D217" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E217">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5792,13 +5789,13 @@
         <v>39</v>
       </c>
       <c r="C218" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D218" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E218">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5809,13 +5806,13 @@
         <v>39</v>
       </c>
       <c r="C219" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D219" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E219">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5826,13 +5823,13 @@
         <v>39</v>
       </c>
       <c r="C220" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D220" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E220">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5843,13 +5840,13 @@
         <v>39</v>
       </c>
       <c r="C221" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D221" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E221">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5860,13 +5857,13 @@
         <v>39</v>
       </c>
       <c r="C222" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D222" t="s">
-        <v>366</v>
+        <v>238</v>
       </c>
       <c r="E222">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5877,13 +5874,13 @@
         <v>39</v>
       </c>
       <c r="C223" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D223" t="s">
         <v>367</v>
       </c>
       <c r="E223">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5894,13 +5891,13 @@
         <v>39</v>
       </c>
       <c r="C224" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D224" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E224">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5911,13 +5908,13 @@
         <v>39</v>
       </c>
       <c r="C225" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D225" t="s">
-        <v>238</v>
+        <v>369</v>
       </c>
       <c r="E225">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5928,64 +5925,30 @@
         <v>39</v>
       </c>
       <c r="C226" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D226" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E226">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B227" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C227" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D227" t="s">
-        <v>369</v>
+        <v>346</v>
       </c>
       <c r="E227">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="228" spans="1:5">
-      <c r="A228" t="s">
-        <v>11</v>
-      </c>
-      <c r="B228" t="s">
-        <v>39</v>
-      </c>
-      <c r="C228" t="s">
-        <v>218</v>
-      </c>
-      <c r="D228" t="s">
-        <v>370</v>
-      </c>
-      <c r="E228">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="229" spans="1:5">
-      <c r="A229" t="s">
-        <v>11</v>
-      </c>
-      <c r="B229" t="s">
-        <v>39</v>
-      </c>
-      <c r="C229" t="s">
-        <v>219</v>
-      </c>
-      <c r="D229" t="s">
-        <v>371</v>
-      </c>
-      <c r="E229">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (30/07/2026 13:19)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="373">
   <si>
     <t>matricula</t>
   </si>
@@ -203,93 +203,96 @@
     <t>2643007-1</t>
   </si>
   <si>
+    <t>2641014-5</t>
+  </si>
+  <si>
+    <t>2641011-5</t>
+  </si>
+  <si>
+    <t>2643100-206</t>
+  </si>
+  <si>
+    <t>162-10700</t>
+  </si>
+  <si>
+    <t>D20B-14489-KA</t>
+  </si>
+  <si>
+    <t>400454</t>
+  </si>
+  <si>
+    <t>2617015-15</t>
+  </si>
+  <si>
+    <t>AE3663163K0600</t>
+  </si>
+  <si>
+    <t>2641013-6</t>
+  </si>
+  <si>
+    <t>2611112-2</t>
+  </si>
+  <si>
+    <t>2601119-1</t>
+  </si>
+  <si>
+    <t>154-03000</t>
+  </si>
+  <si>
+    <t>2621013-2</t>
+  </si>
+  <si>
+    <t>067-06300</t>
+  </si>
+  <si>
+    <t>S3461-76</t>
+  </si>
+  <si>
+    <t>M81934/2-32C032</t>
+  </si>
+  <si>
+    <t>2611137-7</t>
+  </si>
+  <si>
+    <t>2622243-11</t>
+  </si>
+  <si>
+    <t>1H75-21</t>
+  </si>
+  <si>
+    <t>2600100-7</t>
+  </si>
+  <si>
+    <t>2698010-7</t>
+  </si>
+  <si>
+    <t>S1053K22T144.00</t>
+  </si>
+  <si>
+    <t>2601189-11</t>
+  </si>
+  <si>
+    <t>030-18200</t>
+  </si>
+  <si>
+    <t>S2837-1</t>
+  </si>
+  <si>
+    <t>2115040-8</t>
+  </si>
+  <si>
+    <t>S1053K16T</t>
+  </si>
+  <si>
+    <t>MICROB MONITOR 2</t>
+  </si>
+  <si>
+    <t>42854-11</t>
+  </si>
+  <si>
     <t>2651022-20-1</t>
   </si>
   <si>
-    <t>2641014-5</t>
-  </si>
-  <si>
-    <t>2641011-5</t>
-  </si>
-  <si>
-    <t>2643100-206</t>
-  </si>
-  <si>
-    <t>162-10700</t>
-  </si>
-  <si>
-    <t>D20B-14489-KA</t>
-  </si>
-  <si>
-    <t>400454</t>
-  </si>
-  <si>
-    <t>AE3663163K0600</t>
-  </si>
-  <si>
-    <t>2641013-6</t>
-  </si>
-  <si>
-    <t>2611112-2</t>
-  </si>
-  <si>
-    <t>2601119-1</t>
-  </si>
-  <si>
-    <t>154-03000</t>
-  </si>
-  <si>
-    <t>2621013-2</t>
-  </si>
-  <si>
-    <t>067-06300</t>
-  </si>
-  <si>
-    <t>S3461-76</t>
-  </si>
-  <si>
-    <t>M81934/2-32C032</t>
-  </si>
-  <si>
-    <t>2611137-7</t>
-  </si>
-  <si>
-    <t>2622243-11</t>
-  </si>
-  <si>
-    <t>1H75-21</t>
-  </si>
-  <si>
-    <t>2600100-7</t>
-  </si>
-  <si>
-    <t>2698010-7</t>
-  </si>
-  <si>
-    <t>S1053K22T144.00</t>
-  </si>
-  <si>
-    <t>2601189-11</t>
-  </si>
-  <si>
-    <t>030-18200</t>
-  </si>
-  <si>
-    <t>S2837-1</t>
-  </si>
-  <si>
-    <t>2115040-8</t>
-  </si>
-  <si>
-    <t>S1053K16T</t>
-  </si>
-  <si>
-    <t>MICROB MONITOR 2</t>
-  </si>
-  <si>
-    <t>42854-11</t>
-  </si>
-  <si>
     <t>799-1</t>
   </si>
   <si>
@@ -674,7 +677,7 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>2617015-15</t>
+    <t>F2552-070</t>
   </si>
   <si>
     <t>ENGINE PT6A-114A</t>
@@ -689,93 +692,96 @@
     <t>SHIMMY DAMP AS</t>
   </si>
   <si>
+    <t>SPRING-MAIN GEAR CEN</t>
+  </si>
+  <si>
+    <t>AXLE-MAIN GEAR</t>
+  </si>
+  <si>
+    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+  </si>
+  <si>
+    <t>OUTER WHEEL HALF ASSY</t>
+  </si>
+  <si>
+    <t>SLEEVE</t>
+  </si>
+  <si>
+    <t>SEAL,PLAIN ENCASED</t>
+  </si>
+  <si>
+    <t>HINGE-DOOR LH</t>
+  </si>
+  <si>
+    <t>HOSE ASSY</t>
+  </si>
+  <si>
+    <t>SPRING-MAIN GEAR LH &amp; RH</t>
+  </si>
+  <si>
+    <t>STRAP</t>
+  </si>
+  <si>
+    <t>JACK PAD LH</t>
+  </si>
+  <si>
+    <t>SEAL MOLDED</t>
+  </si>
+  <si>
+    <t>SPACER</t>
+  </si>
+  <si>
+    <t>SPACER MAIN GE</t>
+  </si>
+  <si>
+    <t>BOLT</t>
+  </si>
+  <si>
+    <t>BEARING,SLEEVE</t>
+  </si>
+  <si>
+    <t>CAP MAIN LAND</t>
+  </si>
+  <si>
+    <t>ECCENTRIC-WING ASSY</t>
+  </si>
+  <si>
+    <t>PRESSURE REGULATOR</t>
+  </si>
+  <si>
+    <t>LINE ASSY-PROP</t>
+  </si>
+  <si>
+    <t>PASSENGER DOOR - LOW</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
+  </si>
+  <si>
+    <t>MAIN WHEEL BRAKE</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-PASSENGER</t>
+  </si>
+  <si>
+    <t>CYLINDER GAS S</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT</t>
+  </si>
+  <si>
+    <t>TEST KIT, FUEL, WORK</t>
+  </si>
+  <si>
+    <t>FITTING A S TR</t>
+  </si>
+  <si>
     <t>RING ASSY ENGI</t>
   </si>
   <si>
-    <t>SPRING-MAIN GEAR CEN</t>
-  </si>
-  <si>
-    <t>AXLE-MAIN GEAR</t>
-  </si>
-  <si>
-    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
-  </si>
-  <si>
-    <t>OUTER WHEEL HALF ASSY</t>
-  </si>
-  <si>
-    <t>SLEEVE</t>
-  </si>
-  <si>
-    <t>SEAL,PLAIN ENCASED</t>
-  </si>
-  <si>
-    <t>HOSE ASSY</t>
-  </si>
-  <si>
-    <t>SPRING-MAIN GEAR LH &amp; RH</t>
-  </si>
-  <si>
-    <t>STRAP</t>
-  </si>
-  <si>
-    <t>JACK PAD LH</t>
-  </si>
-  <si>
-    <t>SEAL MOLDED</t>
-  </si>
-  <si>
-    <t>SPACER</t>
-  </si>
-  <si>
-    <t>SPACER MAIN GE</t>
-  </si>
-  <si>
-    <t>BOLT</t>
-  </si>
-  <si>
-    <t>BEARING,SLEEVE</t>
-  </si>
-  <si>
-    <t>CAP MAIN LAND</t>
-  </si>
-  <si>
-    <t>ECCENTRIC-WING ASSY</t>
-  </si>
-  <si>
-    <t>PRESSURE REGULATOR</t>
-  </si>
-  <si>
-    <t>LINE ASSY-PROP</t>
-  </si>
-  <si>
-    <t>PASSENGER DOOR - LOW</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
-  </si>
-  <si>
-    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
-  </si>
-  <si>
-    <t>MAIN WHEEL BRAKE</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-PASSENGER</t>
-  </si>
-  <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT</t>
-  </si>
-  <si>
-    <t>TEST KIT, FUEL, WORK</t>
-  </si>
-  <si>
-    <t>FITTING A S TR</t>
-  </si>
-  <si>
     <t>TRANSDUCER</t>
   </si>
   <si>
@@ -1055,9 +1061,6 @@
     <t>INDICATOR FUEL</t>
   </si>
   <si>
-    <t>HINGE-DOOR LH</t>
-  </si>
-  <si>
     <t>WASHER</t>
   </si>
   <si>
@@ -1128,6 +1131,9 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>BARREL NUT</t>
   </si>
 </sst>
 </file>
@@ -1496,10 +1502,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1516,10 +1522,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1536,10 +1542,10 @@
         <v>54</v>
       </c>
       <c r="E4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F4">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2089,7 +2095,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E225"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2120,7 +2126,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2137,7 +2143,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2154,7 +2160,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2171,7 +2177,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2188,7 +2194,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2205,7 +2211,7 @@
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2213,16 +2219,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2230,16 +2236,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2247,7 +2253,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
@@ -2256,7 +2262,7 @@
         <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2264,7 +2270,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
@@ -2273,7 +2279,7 @@
         <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2281,16 +2287,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2298,16 +2304,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2315,7 +2321,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
@@ -2324,7 +2330,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2332,7 +2338,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>38</v>
@@ -2341,7 +2347,7 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2349,16 +2355,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2366,16 +2372,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2383,16 +2389,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" t="s">
         <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2400,7 +2406,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
         <v>38</v>
@@ -2409,7 +2415,7 @@
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2417,16 +2423,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2434,7 +2440,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
         <v>38</v>
@@ -2443,7 +2449,7 @@
         <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2460,7 +2466,7 @@
         <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2477,7 +2483,7 @@
         <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2485,33 +2491,33 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
         <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E24">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2525,10 +2531,10 @@
         <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2536,19 +2542,19 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D27" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2559,10 +2565,10 @@
         <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2576,10 +2582,10 @@
         <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2593,44 +2599,44 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
         <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E32">
         <v>2</v>
@@ -2638,33 +2644,33 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
         <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E33">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2672,16 +2678,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E35">
         <v>2</v>
@@ -2689,33 +2695,33 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
         <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2723,33 +2729,33 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2757,19 +2763,19 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2780,13 +2786,13 @@
         <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2797,10 +2803,10 @@
         <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -2808,19 +2814,19 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2831,10 +2837,10 @@
         <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2848,10 +2854,10 @@
         <v>37</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2865,30 +2871,30 @@
         <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D46" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2899,10 +2905,10 @@
         <v>37</v>
       </c>
       <c r="C48" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D48" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E48">
         <v>4</v>
@@ -2910,16 +2916,16 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B49" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D49" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E49">
         <v>4</v>
@@ -2927,41 +2933,41 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D50" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B52" t="s">
         <v>38</v>
@@ -2970,7 +2976,7 @@
         <v>80</v>
       </c>
       <c r="D52" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -2978,16 +2984,16 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D53" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -2995,16 +3001,16 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B54" t="s">
         <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D54" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3012,7 +3018,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B55" t="s">
         <v>38</v>
@@ -3021,7 +3027,7 @@
         <v>81</v>
       </c>
       <c r="D55" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3029,16 +3035,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B56" t="s">
         <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3052,10 +3058,10 @@
         <v>38</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3069,10 +3075,10 @@
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3086,10 +3092,10 @@
         <v>38</v>
       </c>
       <c r="C59" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3103,10 +3109,10 @@
         <v>38</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D60" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3114,41 +3120,41 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B61" t="s">
         <v>38</v>
       </c>
       <c r="C61" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B62" t="s">
         <v>38</v>
       </c>
       <c r="C62" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
         <v>38</v>
@@ -3157,7 +3163,7 @@
         <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3165,16 +3171,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C64" t="s">
         <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3182,16 +3188,16 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B65" t="s">
         <v>38</v>
       </c>
       <c r="C65" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D65" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3199,16 +3205,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C66" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D66" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3216,16 +3222,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B67" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C67" t="s">
         <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3233,16 +3239,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B68" t="s">
         <v>38</v>
       </c>
       <c r="C68" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D68" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3250,16 +3256,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B69" t="s">
         <v>38</v>
       </c>
       <c r="C69" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3267,16 +3273,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D70" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3290,10 +3296,10 @@
         <v>38</v>
       </c>
       <c r="C71" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3307,10 +3313,10 @@
         <v>38</v>
       </c>
       <c r="C72" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D72" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3324,30 +3330,30 @@
         <v>38</v>
       </c>
       <c r="C73" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
         <v>88</v>
       </c>
       <c r="D74" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3358,13 +3364,13 @@
         <v>38</v>
       </c>
       <c r="C75" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3375,112 +3381,112 @@
         <v>38</v>
       </c>
       <c r="C76" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B77" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C77" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E77">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B78" t="s">
         <v>38</v>
       </c>
       <c r="C78" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D78" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E78">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D79" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E79">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B80" t="s">
         <v>38</v>
       </c>
       <c r="C80" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B81" t="s">
         <v>38</v>
       </c>
       <c r="C81" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D81" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E81">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C82" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3488,16 +3494,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B83" t="s">
         <v>38</v>
       </c>
       <c r="C83" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D83" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3505,16 +3511,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C84" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D84" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3522,33 +3528,33 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B85" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D85" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B86" t="s">
         <v>38</v>
       </c>
       <c r="C86" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D86" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3556,19 +3562,19 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C87" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D87" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3579,10 +3585,10 @@
         <v>38</v>
       </c>
       <c r="C88" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D88" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3596,10 +3602,10 @@
         <v>38</v>
       </c>
       <c r="C89" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D89" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3613,10 +3619,10 @@
         <v>38</v>
       </c>
       <c r="C90" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D90" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3630,10 +3636,10 @@
         <v>38</v>
       </c>
       <c r="C91" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D91" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3647,10 +3653,10 @@
         <v>38</v>
       </c>
       <c r="C92" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D92" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3664,10 +3670,10 @@
         <v>38</v>
       </c>
       <c r="C93" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D93" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3681,10 +3687,10 @@
         <v>38</v>
       </c>
       <c r="C94" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D94" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3698,10 +3704,10 @@
         <v>38</v>
       </c>
       <c r="C95" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D95" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3709,16 +3715,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B96" t="s">
         <v>38</v>
       </c>
       <c r="C96" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D96" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3726,16 +3732,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B97" t="s">
         <v>38</v>
       </c>
       <c r="C97" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3749,10 +3755,10 @@
         <v>38</v>
       </c>
       <c r="C98" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D98" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3766,10 +3772,10 @@
         <v>38</v>
       </c>
       <c r="C99" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D99" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3777,16 +3783,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B100" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D100" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3800,10 +3806,10 @@
         <v>38</v>
       </c>
       <c r="C101" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D101" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3817,10 +3823,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D102" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3834,10 +3840,10 @@
         <v>38</v>
       </c>
       <c r="C103" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D103" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3845,16 +3851,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B104" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C104" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D104" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3868,10 +3874,10 @@
         <v>38</v>
       </c>
       <c r="C105" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D105" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3885,10 +3891,10 @@
         <v>38</v>
       </c>
       <c r="C106" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D106" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3902,10 +3908,10 @@
         <v>38</v>
       </c>
       <c r="C107" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D107" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3919,10 +3925,10 @@
         <v>38</v>
       </c>
       <c r="C108" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D108" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3936,27 +3942,27 @@
         <v>38</v>
       </c>
       <c r="C109" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D109" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B110" t="s">
         <v>38</v>
       </c>
       <c r="C110" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3970,10 +3976,10 @@
         <v>38</v>
       </c>
       <c r="C111" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -3987,13 +3993,13 @@
         <v>38</v>
       </c>
       <c r="C112" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D112" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -4004,10 +4010,10 @@
         <v>38</v>
       </c>
       <c r="C113" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D113" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4021,13 +4027,13 @@
         <v>38</v>
       </c>
       <c r="C114" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D114" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -4038,10 +4044,10 @@
         <v>38</v>
       </c>
       <c r="C115" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D115" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4049,19 +4055,19 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B116" t="s">
         <v>38</v>
       </c>
       <c r="C116" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D116" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E116">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -4072,10 +4078,10 @@
         <v>38</v>
       </c>
       <c r="C117" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4089,13 +4095,13 @@
         <v>38</v>
       </c>
       <c r="C118" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D118" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -4106,13 +4112,13 @@
         <v>38</v>
       </c>
       <c r="C119" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D119" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4123,13 +4129,13 @@
         <v>38</v>
       </c>
       <c r="C120" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D120" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="E120">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4140,64 +4146,64 @@
         <v>38</v>
       </c>
       <c r="C121" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D121" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="E121">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B122" t="s">
         <v>38</v>
       </c>
       <c r="C122" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E122">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B123" t="s">
         <v>38</v>
       </c>
       <c r="C123" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D123" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E123">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B124" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D124" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E124">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4208,10 +4214,10 @@
         <v>38</v>
       </c>
       <c r="C125" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D125" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4219,16 +4225,16 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B126" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C126" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D126" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4242,10 +4248,10 @@
         <v>38</v>
       </c>
       <c r="C127" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D127" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4259,10 +4265,10 @@
         <v>38</v>
       </c>
       <c r="C128" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D128" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4276,10 +4282,10 @@
         <v>38</v>
       </c>
       <c r="C129" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D129" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4293,10 +4299,10 @@
         <v>38</v>
       </c>
       <c r="C130" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D130" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4310,10 +4316,10 @@
         <v>38</v>
       </c>
       <c r="C131" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D131" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4327,10 +4333,10 @@
         <v>38</v>
       </c>
       <c r="C132" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D132" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4344,10 +4350,10 @@
         <v>38</v>
       </c>
       <c r="C133" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D133" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4361,10 +4367,10 @@
         <v>38</v>
       </c>
       <c r="C134" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D134" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4378,10 +4384,10 @@
         <v>38</v>
       </c>
       <c r="C135" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D135" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4395,10 +4401,10 @@
         <v>38</v>
       </c>
       <c r="C136" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D136" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4412,10 +4418,10 @@
         <v>38</v>
       </c>
       <c r="C137" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D137" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4429,10 +4435,10 @@
         <v>38</v>
       </c>
       <c r="C138" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D138" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4446,10 +4452,10 @@
         <v>38</v>
       </c>
       <c r="C139" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D139" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4463,10 +4469,10 @@
         <v>38</v>
       </c>
       <c r="C140" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D140" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4480,10 +4486,10 @@
         <v>38</v>
       </c>
       <c r="C141" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D141" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4497,10 +4503,10 @@
         <v>38</v>
       </c>
       <c r="C142" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D142" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4514,10 +4520,10 @@
         <v>38</v>
       </c>
       <c r="C143" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D143" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4531,10 +4537,10 @@
         <v>38</v>
       </c>
       <c r="C144" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D144" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4548,10 +4554,10 @@
         <v>38</v>
       </c>
       <c r="C145" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D145" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4565,10 +4571,10 @@
         <v>38</v>
       </c>
       <c r="C146" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D146" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4582,10 +4588,10 @@
         <v>38</v>
       </c>
       <c r="C147" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D147" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4599,10 +4605,10 @@
         <v>38</v>
       </c>
       <c r="C148" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D148" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4616,10 +4622,10 @@
         <v>38</v>
       </c>
       <c r="C149" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D149" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4633,10 +4639,10 @@
         <v>38</v>
       </c>
       <c r="C150" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D150" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4650,10 +4656,10 @@
         <v>38</v>
       </c>
       <c r="C151" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D151" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4667,10 +4673,10 @@
         <v>38</v>
       </c>
       <c r="C152" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D152" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4684,13 +4690,13 @@
         <v>38</v>
       </c>
       <c r="C153" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D153" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="E153">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -4701,13 +4707,13 @@
         <v>38</v>
       </c>
       <c r="C154" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D154" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E154">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -4718,10 +4724,10 @@
         <v>38</v>
       </c>
       <c r="C155" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D155" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="E155">
         <v>2</v>
@@ -4735,10 +4741,10 @@
         <v>38</v>
       </c>
       <c r="C156" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D156" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="E156">
         <v>2</v>
@@ -4752,10 +4758,10 @@
         <v>38</v>
       </c>
       <c r="C157" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D157" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4769,13 +4775,13 @@
         <v>38</v>
       </c>
       <c r="C158" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D158" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="E158">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -4786,13 +4792,13 @@
         <v>38</v>
       </c>
       <c r="C159" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D159" t="s">
-        <v>310</v>
+        <v>279</v>
       </c>
       <c r="E159">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4803,13 +4809,13 @@
         <v>38</v>
       </c>
       <c r="C160" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D160" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E160">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4820,13 +4826,13 @@
         <v>38</v>
       </c>
       <c r="C161" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D161" t="s">
-        <v>277</v>
+        <v>315</v>
       </c>
       <c r="E161">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4837,13 +4843,13 @@
         <v>38</v>
       </c>
       <c r="C162" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D162" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="E162">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4854,47 +4860,47 @@
         <v>38</v>
       </c>
       <c r="C163" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D163" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="E163">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B164" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D164" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E164">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B165" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D165" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E165">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4905,10 +4911,10 @@
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D166" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -4922,10 +4928,10 @@
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D167" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4939,10 +4945,10 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D168" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4956,10 +4962,10 @@
         <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D169" t="s">
-        <v>319</v>
+        <v>237</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4973,10 +4979,10 @@
         <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D170" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4990,10 +4996,10 @@
         <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D171" t="s">
-        <v>236</v>
+        <v>324</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5007,10 +5013,10 @@
         <v>39</v>
       </c>
       <c r="C172" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D172" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5024,10 +5030,10 @@
         <v>39</v>
       </c>
       <c r="C173" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D173" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5041,10 +5047,10 @@
         <v>39</v>
       </c>
       <c r="C174" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D174" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5058,10 +5064,10 @@
         <v>39</v>
       </c>
       <c r="C175" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D175" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5075,10 +5081,10 @@
         <v>39</v>
       </c>
       <c r="C176" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D176" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5092,10 +5098,10 @@
         <v>39</v>
       </c>
       <c r="C177" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D177" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5109,10 +5115,10 @@
         <v>39</v>
       </c>
       <c r="C178" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D178" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5126,10 +5132,10 @@
         <v>39</v>
       </c>
       <c r="C179" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D179" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5143,10 +5149,10 @@
         <v>39</v>
       </c>
       <c r="C180" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D180" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5160,10 +5166,10 @@
         <v>39</v>
       </c>
       <c r="C181" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D181" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5177,10 +5183,10 @@
         <v>39</v>
       </c>
       <c r="C182" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D182" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5194,10 +5200,10 @@
         <v>39</v>
       </c>
       <c r="C183" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D183" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5211,10 +5217,10 @@
         <v>39</v>
       </c>
       <c r="C184" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D184" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5228,10 +5234,10 @@
         <v>39</v>
       </c>
       <c r="C185" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D185" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5245,10 +5251,10 @@
         <v>39</v>
       </c>
       <c r="C186" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D186" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5262,10 +5268,10 @@
         <v>39</v>
       </c>
       <c r="C187" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D187" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5279,10 +5285,10 @@
         <v>39</v>
       </c>
       <c r="C188" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D188" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5296,10 +5302,10 @@
         <v>39</v>
       </c>
       <c r="C189" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D189" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5313,10 +5319,10 @@
         <v>39</v>
       </c>
       <c r="C190" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D190" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5330,10 +5336,10 @@
         <v>39</v>
       </c>
       <c r="C191" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D191" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5347,10 +5353,10 @@
         <v>39</v>
       </c>
       <c r="C192" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D192" t="s">
-        <v>341</v>
+        <v>303</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5364,10 +5370,10 @@
         <v>39</v>
       </c>
       <c r="C193" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D193" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5381,10 +5387,10 @@
         <v>39</v>
       </c>
       <c r="C194" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D194" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5398,13 +5404,13 @@
         <v>39</v>
       </c>
       <c r="C195" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D195" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E195">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -5415,13 +5421,13 @@
         <v>39</v>
       </c>
       <c r="C196" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D196" t="s">
-        <v>344</v>
+        <v>231</v>
       </c>
       <c r="E196">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -5432,10 +5438,10 @@
         <v>39</v>
       </c>
       <c r="C197" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D197" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -5449,10 +5455,10 @@
         <v>39</v>
       </c>
       <c r="C198" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D198" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5466,10 +5472,10 @@
         <v>39</v>
       </c>
       <c r="C199" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D199" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5483,10 +5489,10 @@
         <v>39</v>
       </c>
       <c r="C200" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D200" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5500,10 +5506,10 @@
         <v>39</v>
       </c>
       <c r="C201" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D201" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5517,10 +5523,10 @@
         <v>39</v>
       </c>
       <c r="C202" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D202" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5534,10 +5540,10 @@
         <v>39</v>
       </c>
       <c r="C203" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D203" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5551,10 +5557,10 @@
         <v>39</v>
       </c>
       <c r="C204" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D204" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5568,10 +5574,10 @@
         <v>39</v>
       </c>
       <c r="C205" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D205" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5585,10 +5591,10 @@
         <v>39</v>
       </c>
       <c r="C206" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D206" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5602,13 +5608,13 @@
         <v>39</v>
       </c>
       <c r="C207" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D207" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E207">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5619,13 +5625,13 @@
         <v>39</v>
       </c>
       <c r="C208" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D208" t="s">
-        <v>355</v>
+        <v>237</v>
       </c>
       <c r="E208">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5636,13 +5642,13 @@
         <v>39</v>
       </c>
       <c r="C209" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D209" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E209">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5653,13 +5659,13 @@
         <v>39</v>
       </c>
       <c r="C210" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D210" t="s">
-        <v>236</v>
+        <v>359</v>
       </c>
       <c r="E210">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5670,10 +5676,10 @@
         <v>39</v>
       </c>
       <c r="C211" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D211" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E211">
         <v>4</v>
@@ -5687,10 +5693,10 @@
         <v>39</v>
       </c>
       <c r="C212" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D212" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E212">
         <v>4</v>
@@ -5704,10 +5710,10 @@
         <v>39</v>
       </c>
       <c r="C213" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D213" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E213">
         <v>4</v>
@@ -5721,13 +5727,13 @@
         <v>39</v>
       </c>
       <c r="C214" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D214" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E214">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5738,13 +5744,13 @@
         <v>39</v>
       </c>
       <c r="C215" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D215" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E215">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5755,13 +5761,13 @@
         <v>39</v>
       </c>
       <c r="C216" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D216" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E216">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5772,13 +5778,13 @@
         <v>39</v>
       </c>
       <c r="C217" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D217" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E217">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5789,13 +5795,13 @@
         <v>39</v>
       </c>
       <c r="C218" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D218" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E218">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5806,13 +5812,13 @@
         <v>39</v>
       </c>
       <c r="C219" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D219" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E219">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5823,13 +5829,13 @@
         <v>39</v>
       </c>
       <c r="C220" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D220" t="s">
-        <v>366</v>
+        <v>239</v>
       </c>
       <c r="E220">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5840,13 +5846,13 @@
         <v>39</v>
       </c>
       <c r="C221" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D221" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E221">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5857,13 +5863,13 @@
         <v>39</v>
       </c>
       <c r="C222" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D222" t="s">
-        <v>238</v>
+        <v>369</v>
       </c>
       <c r="E222">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5874,13 +5880,13 @@
         <v>39</v>
       </c>
       <c r="C223" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D223" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E223">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5891,64 +5897,30 @@
         <v>39</v>
       </c>
       <c r="C224" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D224" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E224">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B225" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C225" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D225" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E225">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="226" spans="1:5">
-      <c r="A226" t="s">
-        <v>11</v>
-      </c>
-      <c r="B226" t="s">
-        <v>39</v>
-      </c>
-      <c r="C226" t="s">
-        <v>218</v>
-      </c>
-      <c r="D226" t="s">
-        <v>370</v>
-      </c>
-      <c r="E226">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="227" spans="1:5">
-      <c r="A227" t="s">
-        <v>7</v>
-      </c>
-      <c r="B227" t="s">
-        <v>37</v>
-      </c>
-      <c r="C227" t="s">
-        <v>219</v>
-      </c>
-      <c r="D227" t="s">
-        <v>346</v>
-      </c>
-      <c r="E227">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (03/08/2026 14:29)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="375">
   <si>
     <t>matricula</t>
   </si>
@@ -38,6 +38,9 @@
     <t>2721</t>
   </si>
   <si>
+    <t>2733</t>
+  </si>
+  <si>
     <t>2728</t>
   </si>
   <si>
@@ -89,9 +92,6 @@
     <t>2731</t>
   </si>
   <si>
-    <t>2733</t>
-  </si>
-  <si>
     <t>2736</t>
   </si>
   <si>
@@ -128,15 +128,15 @@
     <t>6º ETA</t>
   </si>
   <si>
+    <t>1º ETA</t>
+  </si>
+  <si>
     <t>1º/5º GAV</t>
   </si>
   <si>
     <t>7º ETA</t>
   </si>
   <si>
-    <t>1º ETA</t>
-  </si>
-  <si>
     <t>EPCAR</t>
   </si>
   <si>
@@ -194,12 +194,12 @@
     <t>3044000</t>
   </si>
   <si>
+    <t>P7036368-01</t>
+  </si>
+  <si>
     <t>C611505-0201</t>
   </si>
   <si>
-    <t>P7036368-01</t>
-  </si>
-  <si>
     <t>2643007-1</t>
   </si>
   <si>
@@ -254,6 +254,9 @@
     <t>2611137-7</t>
   </si>
   <si>
+    <t>2601102-1</t>
+  </si>
+  <si>
     <t>2622243-11</t>
   </si>
   <si>
@@ -269,21 +272,21 @@
     <t>S1053K22T144.00</t>
   </si>
   <si>
+    <t>030-18200</t>
+  </si>
+  <si>
+    <t>2115040-8</t>
+  </si>
+  <si>
+    <t>S1053K16T</t>
+  </si>
+  <si>
+    <t>S2837-1</t>
+  </si>
+  <si>
     <t>2601189-11</t>
   </si>
   <si>
-    <t>030-18200</t>
-  </si>
-  <si>
-    <t>S2837-1</t>
-  </si>
-  <si>
-    <t>2115040-8</t>
-  </si>
-  <si>
-    <t>S1053K16T</t>
-  </si>
-  <si>
     <t>MICROB MONITOR 2</t>
   </si>
   <si>
@@ -314,66 +317,66 @@
     <t>1134380-4</t>
   </si>
   <si>
+    <t>CAB-33-02</t>
+  </si>
+  <si>
+    <t>2601266-2</t>
+  </si>
+  <si>
+    <t>30994-001</t>
+  </si>
+  <si>
+    <t>2641018-25</t>
+  </si>
+  <si>
+    <t>2641018-26</t>
+  </si>
+  <si>
+    <t>S2814-2</t>
+  </si>
+  <si>
+    <t>S2574-1</t>
+  </si>
+  <si>
+    <t>2601188-9</t>
+  </si>
+  <si>
+    <t>2622236-6</t>
+  </si>
+  <si>
+    <t>1H101-4</t>
+  </si>
+  <si>
+    <t>S51-14</t>
+  </si>
+  <si>
+    <t>5211369-8</t>
+  </si>
+  <si>
+    <t>1134380-5</t>
+  </si>
+  <si>
+    <t>5950017-11</t>
+  </si>
+  <si>
+    <t>040-0043</t>
+  </si>
+  <si>
+    <t>1214134-1</t>
+  </si>
+  <si>
+    <t>DLS4-02303</t>
+  </si>
+  <si>
+    <t>DLS4-01786</t>
+  </si>
+  <si>
+    <t>A1635-133</t>
+  </si>
+  <si>
     <t>011-00870-00</t>
   </si>
   <si>
-    <t>CAB-33-02</t>
-  </si>
-  <si>
-    <t>2601266-2</t>
-  </si>
-  <si>
-    <t>30994-001</t>
-  </si>
-  <si>
-    <t>2641018-25</t>
-  </si>
-  <si>
-    <t>2641018-26</t>
-  </si>
-  <si>
-    <t>S2814-2</t>
-  </si>
-  <si>
-    <t>S2574-1</t>
-  </si>
-  <si>
-    <t>2601188-9</t>
-  </si>
-  <si>
-    <t>2622236-6</t>
-  </si>
-  <si>
-    <t>1H101-4</t>
-  </si>
-  <si>
-    <t>S51-14</t>
-  </si>
-  <si>
-    <t>5211369-8</t>
-  </si>
-  <si>
-    <t>1134380-5</t>
-  </si>
-  <si>
-    <t>5950017-11</t>
-  </si>
-  <si>
-    <t>040-0043</t>
-  </si>
-  <si>
-    <t>1214134-1</t>
-  </si>
-  <si>
-    <t>DLS4-02303</t>
-  </si>
-  <si>
-    <t>DLS4-01786</t>
-  </si>
-  <si>
-    <t>A1635-133</t>
-  </si>
-  <si>
     <t>1J18-10</t>
   </si>
   <si>
@@ -683,12 +686,12 @@
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
+    <t>PROPELLER ASSEMBLY</t>
+  </si>
+  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
-    <t>PROPELLER ASSEMBLY</t>
-  </si>
-  <si>
     <t>SHIMMY DAMP AS</t>
   </si>
   <si>
@@ -743,6 +746,9 @@
     <t>CAP MAIN LAND</t>
   </si>
   <si>
+    <t>HINGE-ASSY-HOISTING</t>
+  </si>
+  <si>
     <t>ECCENTRIC-WING ASSY</t>
   </si>
   <si>
@@ -758,21 +764,21 @@
     <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
   </si>
   <si>
+    <t>MAIN WHEEL BRAKE</t>
+  </si>
+  <si>
+    <t>CYLINDER GAS S</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-PASSENGER</t>
+  </si>
+  <si>
     <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
   </si>
   <si>
-    <t>MAIN WHEEL BRAKE</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-PASSENGER</t>
-  </si>
-  <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT</t>
-  </si>
-  <si>
     <t>TEST KIT, FUEL, WORK</t>
   </si>
   <si>
@@ -800,61 +806,61 @@
     <t>EVAPORATOR MODULE AS</t>
   </si>
   <si>
+    <t>KIT CAB-33-02</t>
+  </si>
+  <si>
+    <t>COUPLING-SPLINED</t>
+  </si>
+  <si>
+    <t>BATTERY-MARATHON TSP410 NICAD</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY LH</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY RH</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-DOOR PULL</t>
+  </si>
+  <si>
+    <t>NUT-DIODE ATTACH</t>
+  </si>
+  <si>
+    <t>COMPRESSOR DRIVE ASS</t>
+  </si>
+  <si>
+    <t>COVER ACCESS RH</t>
+  </si>
+  <si>
+    <t>FLOW CONTROL VALVE</t>
+  </si>
+  <si>
+    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+  </si>
+  <si>
+    <t>EXTENDER-CREW, (WHEN</t>
+  </si>
+  <si>
+    <t>REDUCER ASSEMBY</t>
+  </si>
+  <si>
+    <t>STROB TUB</t>
+  </si>
+  <si>
+    <t>BELLCRANK ASSY</t>
+  </si>
+  <si>
+    <t>IMOBILIZADOR</t>
+  </si>
+  <si>
+    <t>BLOQUEIO DA VENTILAÇ</t>
+  </si>
+  <si>
+    <t>SCREW</t>
+  </si>
+  <si>
     <t>MAGNETOMETER GMU 44</t>
-  </si>
-  <si>
-    <t>KIT CAB-33-02</t>
-  </si>
-  <si>
-    <t>COUPLING-SPLINED</t>
-  </si>
-  <si>
-    <t>BATTERY-MARATHON TSP410 NICAD</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY LH</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY RH</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-DOOR PULL</t>
-  </si>
-  <si>
-    <t>NUT-DIODE ATTACH</t>
-  </si>
-  <si>
-    <t>COMPRESSOR DRIVE ASS</t>
-  </si>
-  <si>
-    <t>COVER ACCESS RH</t>
-  </si>
-  <si>
-    <t>FLOW CONTROL VALVE</t>
-  </si>
-  <si>
-    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
-  </si>
-  <si>
-    <t>EXTENDER-CREW, (WHEN</t>
-  </si>
-  <si>
-    <t>REDUCER ASSEMBY</t>
-  </si>
-  <si>
-    <t>STROB TUB</t>
-  </si>
-  <si>
-    <t>BELLCRANK ASSY</t>
-  </si>
-  <si>
-    <t>IMOBILIZADOR</t>
-  </si>
-  <si>
-    <t>BLOQUEIO DA VENTILAÇ</t>
-  </si>
-  <si>
-    <t>SCREW</t>
   </si>
   <si>
     <t>FUEL FILTER ASSY</t>
@@ -1522,10 +1528,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>41</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1539,13 +1545,13 @@
         <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F4">
-        <v>24</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1553,7 +1559,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1562,10 +1568,10 @@
         <v>54</v>
       </c>
       <c r="E5">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F5">
-        <v>100</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1573,7 +1579,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1582,10 +1588,10 @@
         <v>54</v>
       </c>
       <c r="E6">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="F6">
-        <v>166</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1602,10 +1608,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="F7">
-        <v>228</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1613,19 +1619,19 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1633,7 +1639,7 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>51</v>
@@ -1653,7 +1659,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>51</v>
@@ -1673,7 +1679,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
         <v>51</v>
@@ -1693,7 +1699,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1713,7 +1719,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1733,7 +1739,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1753,7 +1759,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1773,7 +1779,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1793,7 +1799,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1813,7 +1819,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1833,7 +1839,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1853,7 +1859,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1873,7 +1879,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>51</v>
@@ -1893,7 +1899,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
@@ -1933,7 +1939,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
@@ -1953,7 +1959,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -2095,7 +2101,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E225"/>
+  <dimension ref="A1:E227"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2126,7 +2132,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2134,16 +2140,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2151,16 +2157,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2168,16 +2174,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2185,16 +2191,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2202,16 +2208,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2228,7 +2234,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2245,7 +2251,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2256,13 +2262,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
         <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2273,13 +2279,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2287,13 +2293,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
         <v>223</v>
@@ -2304,13 +2310,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D13" t="s">
         <v>223</v>
@@ -2321,7 +2327,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
@@ -2330,7 +2336,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2338,16 +2344,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2355,7 +2361,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
         <v>39</v>
@@ -2364,7 +2370,7 @@
         <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2372,13 +2378,13 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
         <v>224</v>
@@ -2389,7 +2395,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
         <v>38</v>
@@ -2398,7 +2404,7 @@
         <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2409,13 +2415,13 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2423,13 +2429,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
         <v>225</v>
@@ -2440,7 +2446,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
         <v>38</v>
@@ -2449,7 +2455,7 @@
         <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2466,7 +2472,7 @@
         <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2474,13 +2480,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
         <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D23" t="s">
         <v>226</v>
@@ -2491,47 +2497,47 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
         <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
         <v>227</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
         <v>228</v>
@@ -2542,13 +2548,13 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
         <v>229</v>
@@ -2559,13 +2565,13 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D28" t="s">
         <v>230</v>
@@ -2576,13 +2582,13 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
         <v>231</v>
@@ -2593,24 +2599,24 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
         <v>232</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
@@ -2619,10 +2625,10 @@
         <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2630,16 +2636,16 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
         <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2653,7 +2659,7 @@
         <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2661,13 +2667,13 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
         <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
         <v>233</v>
@@ -2678,7 +2684,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
         <v>38</v>
@@ -2687,7 +2693,7 @@
         <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E35">
         <v>2</v>
@@ -2704,32 +2710,32 @@
         <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
         <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
         <v>234</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
         <v>38</v>
@@ -2738,10 +2744,10 @@
         <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2755,21 +2761,21 @@
         <v>71</v>
       </c>
       <c r="D39" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
         <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
         <v>235</v>
@@ -2780,47 +2786,47 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
         <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
         <v>236</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
         <v>237</v>
@@ -2831,13 +2837,13 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D44" t="s">
         <v>238</v>
@@ -2848,13 +2854,13 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
         <v>239</v>
@@ -2865,33 +2871,33 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
         <v>240</v>
       </c>
       <c r="E46">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C47" t="s">
         <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E47">
         <v>4</v>
@@ -2899,13 +2905,13 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
         <v>37</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
         <v>241</v>
@@ -2916,13 +2922,13 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D49" t="s">
         <v>242</v>
@@ -2939,18 +2945,18 @@
         <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D50" t="s">
         <v>243</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B51" t="s">
         <v>38</v>
@@ -2959,24 +2965,24 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B52" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -2984,16 +2990,16 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
         <v>81</v>
       </c>
       <c r="D53" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -3001,16 +3007,16 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C54" t="s">
         <v>81</v>
       </c>
       <c r="D54" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3018,16 +3024,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B55" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C55" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D55" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3035,16 +3041,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
         <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3052,16 +3058,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3069,16 +3075,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B58" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
         <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3086,16 +3092,16 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C59" t="s">
         <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3103,16 +3109,16 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
         <v>84</v>
       </c>
       <c r="D60" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3120,19 +3126,19 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D61" t="s">
         <v>248</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3140,13 +3146,13 @@
         <v>9</v>
       </c>
       <c r="B62" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C62" t="s">
         <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3157,13 +3163,13 @@
         <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C63" t="s">
         <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3180,7 +3186,7 @@
         <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3188,13 +3194,13 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D65" t="s">
         <v>249</v>
@@ -3205,16 +3211,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B66" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C66" t="s">
         <v>86</v>
       </c>
       <c r="D66" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3222,7 +3228,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
@@ -3231,7 +3237,7 @@
         <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3239,13 +3245,13 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D68" t="s">
         <v>250</v>
@@ -3259,13 +3265,13 @@
         <v>9</v>
       </c>
       <c r="B69" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C69" t="s">
         <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3276,13 +3282,13 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C70" t="s">
         <v>87</v>
       </c>
       <c r="D70" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3290,36 +3296,36 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D71" t="s">
         <v>251</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C72" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D72" t="s">
         <v>251</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3327,16 +3333,16 @@
         <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
         <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E73">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3350,27 +3356,27 @@
         <v>88</v>
       </c>
       <c r="D74" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E74">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D75" t="s">
         <v>252</v>
       </c>
       <c r="E75">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3378,55 +3384,55 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C76" t="s">
         <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E76">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E77">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D78" t="s">
         <v>254</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
@@ -3435,24 +3441,24 @@
         <v>91</v>
       </c>
       <c r="D79" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E79">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C80" t="s">
         <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3460,16 +3466,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C81" t="s">
         <v>92</v>
       </c>
       <c r="D81" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3477,16 +3483,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
       </c>
       <c r="C82" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D82" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3494,16 +3500,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B83" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C83" t="s">
         <v>93</v>
       </c>
       <c r="D83" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3511,16 +3517,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C84" t="s">
         <v>93</v>
       </c>
       <c r="D84" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3528,33 +3534,33 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D85" t="s">
         <v>251</v>
       </c>
       <c r="E85">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B86" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C86" t="s">
         <v>94</v>
       </c>
       <c r="D86" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3562,33 +3568,33 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C87" t="s">
         <v>94</v>
       </c>
       <c r="D87" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C88" t="s">
         <v>95</v>
       </c>
       <c r="D88" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3596,16 +3602,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B89" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C89" t="s">
         <v>95</v>
       </c>
       <c r="D89" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3613,16 +3619,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C90" t="s">
         <v>96</v>
       </c>
       <c r="D90" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3630,16 +3636,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B91" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C91" t="s">
         <v>96</v>
       </c>
       <c r="D91" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3647,16 +3653,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B92" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C92" t="s">
         <v>97</v>
       </c>
       <c r="D92" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3664,16 +3670,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B93" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C93" t="s">
         <v>97</v>
       </c>
       <c r="D93" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3681,16 +3687,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B94" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
         <v>98</v>
       </c>
       <c r="D94" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3698,16 +3704,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B95" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C95" t="s">
         <v>98</v>
       </c>
       <c r="D95" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3718,13 +3724,13 @@
         <v>10</v>
       </c>
       <c r="B96" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C96" t="s">
         <v>99</v>
       </c>
       <c r="D96" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3732,13 +3738,13 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B97" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D97" t="s">
         <v>262</v>
@@ -3752,13 +3758,13 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C98" t="s">
         <v>100</v>
       </c>
       <c r="D98" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3766,13 +3772,13 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B99" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D99" t="s">
         <v>263</v>
@@ -3783,7 +3789,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
@@ -3792,7 +3798,7 @@
         <v>101</v>
       </c>
       <c r="D100" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3800,13 +3806,13 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C101" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D101" t="s">
         <v>264</v>
@@ -3817,7 +3823,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B102" t="s">
         <v>39</v>
@@ -3826,7 +3832,7 @@
         <v>102</v>
       </c>
       <c r="D102" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3834,13 +3840,13 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C103" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D103" t="s">
         <v>265</v>
@@ -3851,13 +3857,13 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B104" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D104" t="s">
         <v>266</v>
@@ -3868,13 +3874,13 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B105" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D105" t="s">
         <v>267</v>
@@ -3885,13 +3891,13 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B106" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D106" t="s">
         <v>268</v>
@@ -3902,13 +3908,13 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B107" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D107" t="s">
         <v>269</v>
@@ -3919,13 +3925,13 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B108" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D108" t="s">
         <v>270</v>
@@ -3936,19 +3942,19 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B109" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D109" t="s">
         <v>271</v>
       </c>
       <c r="E109">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -3956,33 +3962,33 @@
         <v>10</v>
       </c>
       <c r="B110" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C110" t="s">
         <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B111" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D111" t="s">
         <v>272</v>
       </c>
       <c r="E111">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -3990,13 +3996,13 @@
         <v>10</v>
       </c>
       <c r="B112" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C112" t="s">
         <v>110</v>
       </c>
       <c r="D112" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4004,13 +4010,13 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B113" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D113" t="s">
         <v>273</v>
@@ -4024,47 +4030,47 @@
         <v>10</v>
       </c>
       <c r="B114" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C114" t="s">
         <v>111</v>
       </c>
       <c r="D114" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E114">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B115" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D115" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B116" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D116" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4072,13 +4078,13 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B117" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C117" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D117" t="s">
         <v>275</v>
@@ -4089,70 +4095,70 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B118" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D118" t="s">
         <v>276</v>
       </c>
       <c r="E118">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B119" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D119" t="s">
         <v>277</v>
       </c>
       <c r="E119">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B120" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D120" t="s">
         <v>278</v>
       </c>
       <c r="E120">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B121" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D121" t="s">
         <v>279</v>
       </c>
       <c r="E121">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4160,13 +4166,13 @@
         <v>10</v>
       </c>
       <c r="B122" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C122" t="s">
         <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E122">
         <v>30</v>
@@ -4174,19 +4180,19 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B123" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D123" t="s">
         <v>280</v>
       </c>
       <c r="E123">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4200,7 +4206,7 @@
         <v>119</v>
       </c>
       <c r="D124" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4208,16 +4214,16 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B125" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C125" t="s">
         <v>120</v>
       </c>
       <c r="D125" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4225,13 +4231,13 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B126" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C126" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D126" t="s">
         <v>282</v>
@@ -4242,13 +4248,13 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B127" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D127" t="s">
         <v>283</v>
@@ -4259,13 +4265,13 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B128" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D128" t="s">
         <v>284</v>
@@ -4276,13 +4282,13 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B129" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C129" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D129" t="s">
         <v>285</v>
@@ -4293,13 +4299,13 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B130" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C130" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D130" t="s">
         <v>286</v>
@@ -4310,13 +4316,13 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B131" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D131" t="s">
         <v>287</v>
@@ -4327,13 +4333,13 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B132" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D132" t="s">
         <v>288</v>
@@ -4344,13 +4350,13 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B133" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D133" t="s">
         <v>289</v>
@@ -4361,13 +4367,13 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B134" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D134" t="s">
         <v>290</v>
@@ -4378,13 +4384,13 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B135" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D135" t="s">
         <v>291</v>
@@ -4395,13 +4401,13 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B136" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D136" t="s">
         <v>292</v>
@@ -4412,13 +4418,13 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B137" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D137" t="s">
         <v>293</v>
@@ -4429,13 +4435,13 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B138" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D138" t="s">
         <v>294</v>
@@ -4446,13 +4452,13 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B139" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D139" t="s">
         <v>295</v>
@@ -4463,13 +4469,13 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B140" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D140" t="s">
         <v>296</v>
@@ -4480,13 +4486,13 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B141" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D141" t="s">
         <v>297</v>
@@ -4497,13 +4503,13 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B142" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D142" t="s">
         <v>298</v>
@@ -4514,13 +4520,13 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B143" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D143" t="s">
         <v>299</v>
@@ -4531,13 +4537,13 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B144" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D144" t="s">
         <v>300</v>
@@ -4548,13 +4554,13 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B145" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D145" t="s">
         <v>301</v>
@@ -4565,13 +4571,13 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B146" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D146" t="s">
         <v>302</v>
@@ -4582,13 +4588,13 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B147" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D147" t="s">
         <v>303</v>
@@ -4599,13 +4605,13 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B148" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D148" t="s">
         <v>304</v>
@@ -4616,13 +4622,13 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B149" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D149" t="s">
         <v>305</v>
@@ -4633,13 +4639,13 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B150" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D150" t="s">
         <v>306</v>
@@ -4650,13 +4656,13 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B151" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D151" t="s">
         <v>307</v>
@@ -4667,13 +4673,13 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B152" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D152" t="s">
         <v>308</v>
@@ -4684,50 +4690,50 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B153" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="E153">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B154" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E154">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B155" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="E155">
         <v>2</v>
@@ -4735,13 +4741,13 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B156" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D156" t="s">
         <v>311</v>
@@ -4752,13 +4758,13 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B157" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D157" t="s">
         <v>312</v>
@@ -4769,104 +4775,104 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B158" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D158" t="s">
         <v>313</v>
       </c>
       <c r="E158">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B159" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>279</v>
+        <v>314</v>
       </c>
       <c r="E159">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B160" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E160">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B161" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>315</v>
+        <v>280</v>
       </c>
       <c r="E161">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B162" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D162" t="s">
         <v>316</v>
       </c>
       <c r="E162">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B163" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D163" t="s">
         <v>317</v>
       </c>
       <c r="E163">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4877,13 +4883,13 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D164" t="s">
         <v>318</v>
       </c>
       <c r="E164">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4894,24 +4900,24 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D165" t="s">
         <v>319</v>
       </c>
       <c r="E165">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C166" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D166" t="s">
         <v>320</v>
@@ -4922,13 +4928,13 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C167" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D167" t="s">
         <v>321</v>
@@ -4939,13 +4945,13 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C168" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D168" t="s">
         <v>322</v>
@@ -4956,16 +4962,16 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C169" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>237</v>
+        <v>323</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4973,16 +4979,16 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C170" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4990,16 +4996,16 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C171" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>324</v>
+        <v>238</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5007,13 +5013,13 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C172" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D172" t="s">
         <v>325</v>
@@ -5024,13 +5030,13 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C173" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D173" t="s">
         <v>326</v>
@@ -5041,13 +5047,13 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C174" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D174" t="s">
         <v>327</v>
@@ -5058,13 +5064,13 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C175" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D175" t="s">
         <v>328</v>
@@ -5075,13 +5081,13 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B176" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C176" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D176" t="s">
         <v>329</v>
@@ -5092,13 +5098,13 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B177" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C177" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D177" t="s">
         <v>330</v>
@@ -5109,13 +5115,13 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B178" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C178" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D178" t="s">
         <v>331</v>
@@ -5126,13 +5132,13 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B179" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C179" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D179" t="s">
         <v>332</v>
@@ -5143,13 +5149,13 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B180" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C180" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D180" t="s">
         <v>333</v>
@@ -5160,13 +5166,13 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B181" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C181" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D181" t="s">
         <v>334</v>
@@ -5177,13 +5183,13 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B182" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C182" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D182" t="s">
         <v>335</v>
@@ -5194,13 +5200,13 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B183" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C183" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D183" t="s">
         <v>336</v>
@@ -5211,13 +5217,13 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B184" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C184" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D184" t="s">
         <v>337</v>
@@ -5228,13 +5234,13 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C185" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D185" t="s">
         <v>338</v>
@@ -5245,13 +5251,13 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B186" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C186" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D186" t="s">
         <v>339</v>
@@ -5262,13 +5268,13 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B187" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C187" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D187" t="s">
         <v>340</v>
@@ -5279,13 +5285,13 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B188" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C188" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D188" t="s">
         <v>341</v>
@@ -5296,13 +5302,13 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B189" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C189" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D189" t="s">
         <v>342</v>
@@ -5313,13 +5319,13 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B190" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C190" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D190" t="s">
         <v>343</v>
@@ -5330,13 +5336,13 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B191" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C191" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D191" t="s">
         <v>344</v>
@@ -5347,16 +5353,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B192" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C192" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>303</v>
+        <v>345</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5364,16 +5370,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B193" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C193" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5381,16 +5387,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B194" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C194" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5398,50 +5404,50 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B195" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C195" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D195" t="s">
         <v>347</v>
       </c>
       <c r="E195">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B196" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C196" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>231</v>
+        <v>348</v>
       </c>
       <c r="E196">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B197" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C197" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -5449,16 +5455,16 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B198" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C198" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>349</v>
+        <v>232</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5466,13 +5472,13 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C199" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D199" t="s">
         <v>350</v>
@@ -5483,13 +5489,13 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C200" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D200" t="s">
         <v>351</v>
@@ -5500,13 +5506,13 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B201" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C201" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D201" t="s">
         <v>352</v>
@@ -5517,13 +5523,13 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C202" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D202" t="s">
         <v>353</v>
@@ -5534,16 +5540,16 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C203" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5551,16 +5557,16 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C204" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5568,13 +5574,13 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C205" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D205" t="s">
         <v>355</v>
@@ -5585,13 +5591,13 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B206" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C206" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D206" t="s">
         <v>356</v>
@@ -5602,81 +5608,81 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C207" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D207" t="s">
         <v>357</v>
       </c>
       <c r="E207">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C208" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>237</v>
+        <v>358</v>
       </c>
       <c r="E208">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B209" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C209" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E209">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B210" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C210" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>359</v>
+        <v>238</v>
       </c>
       <c r="E210">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B211" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C211" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D211" t="s">
         <v>360</v>
@@ -5687,13 +5693,13 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C212" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D212" t="s">
         <v>361</v>
@@ -5704,13 +5710,13 @@
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C213" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D213" t="s">
         <v>362</v>
@@ -5721,205 +5727,239 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B214" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C214" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D214" t="s">
         <v>363</v>
       </c>
       <c r="E214">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B215" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C215" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D215" t="s">
         <v>364</v>
       </c>
       <c r="E215">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C216" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D216" t="s">
         <v>365</v>
       </c>
       <c r="E216">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C217" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D217" t="s">
         <v>366</v>
       </c>
       <c r="E217">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C218" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D218" t="s">
         <v>367</v>
       </c>
       <c r="E218">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B219" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C219" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E219">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B220" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C220" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D220" t="s">
-        <v>239</v>
+        <v>369</v>
       </c>
       <c r="E220">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B221" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C221" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E221">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C222" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>369</v>
+        <v>240</v>
       </c>
       <c r="E222">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B223" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C223" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D223" t="s">
         <v>370</v>
       </c>
       <c r="E223">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C224" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D224" t="s">
         <v>371</v>
       </c>
       <c r="E224">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B225" t="s">
         <v>37</v>
       </c>
       <c r="C225" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D225" t="s">
         <v>372</v>
       </c>
       <c r="E225">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
+      <c r="A226" t="s">
+        <v>12</v>
+      </c>
+      <c r="B226" t="s">
+        <v>37</v>
+      </c>
+      <c r="C226" t="s">
+        <v>220</v>
+      </c>
+      <c r="D226" t="s">
+        <v>373</v>
+      </c>
+      <c r="E226">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
+      <c r="A227" t="s">
+        <v>8</v>
+      </c>
+      <c r="B227" t="s">
+        <v>38</v>
+      </c>
+      <c r="C227" t="s">
+        <v>221</v>
+      </c>
+      <c r="D227" t="s">
+        <v>374</v>
+      </c>
+      <c r="E227">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (04/08/2026 14:15)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="379">
   <si>
     <t>matricula</t>
   </si>
@@ -35,6 +35,12 @@
     <t>soma_unidades_faltantes</t>
   </si>
   <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>2720</t>
+  </si>
+  <si>
     <t>2721</t>
   </si>
   <si>
@@ -68,15 +74,9 @@
     <t>2708</t>
   </si>
   <si>
-    <t>2709</t>
-  </si>
-  <si>
     <t>2719</t>
   </si>
   <si>
-    <t>2720</t>
-  </si>
-  <si>
     <t>2722</t>
   </si>
   <si>
@@ -191,6 +191,12 @@
     <t>quantidade_faltante</t>
   </si>
   <si>
+    <t>068-02800</t>
+  </si>
+  <si>
+    <t>C668050-1108</t>
+  </si>
+  <si>
     <t>3044000</t>
   </si>
   <si>
@@ -681,6 +687,12 @@
   </si>
   <si>
     <t>F2552-070</t>
+  </si>
+  <si>
+    <t>INSULATOR</t>
+  </si>
+  <si>
+    <t>TRANSMITTER FUEL</t>
   </si>
   <si>
     <t>ENGINE PT6A-114A</t>
@@ -1511,7 +1523,7 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1519,7 +1531,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
         <v>50</v>
@@ -1539,7 +1551,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
         <v>50</v>
@@ -1548,10 +1560,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>43</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1559,19 +1571,19 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1579,19 +1591,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E6">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="F6">
-        <v>111</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1608,10 +1620,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>166</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1619,7 +1631,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1628,10 +1640,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="F8">
-        <v>228</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1639,19 +1651,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1659,19 +1671,19 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1679,7 +1691,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
         <v>51</v>
@@ -1719,7 +1731,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1739,7 +1751,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1759,7 +1771,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -2101,7 +2113,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2132,24 +2144,24 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2157,16 +2169,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2177,13 +2189,13 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2197,10 +2209,10 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2211,13 +2223,13 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2225,16 +2237,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2242,16 +2254,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2262,13 +2274,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2279,13 +2291,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2299,10 +2311,10 @@
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2313,13 +2325,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2327,16 +2339,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2344,16 +2356,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2364,13 +2376,13 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2384,10 +2396,10 @@
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2395,16 +2407,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2412,16 +2424,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2429,16 +2441,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2446,16 +2458,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2463,16 +2475,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2480,16 +2492,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2497,16 +2509,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2514,33 +2526,33 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
         <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2548,24 +2560,24 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" t="s">
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
@@ -2574,7 +2586,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2582,7 +2594,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
@@ -2591,7 +2603,7 @@
         <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2599,7 +2611,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B30" t="s">
         <v>38</v>
@@ -2608,7 +2620,7 @@
         <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2616,7 +2628,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
@@ -2625,10 +2637,10 @@
         <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2636,30 +2648,30 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E32">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D33" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2670,30 +2682,30 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E35">
         <v>2</v>
@@ -2701,16 +2713,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E36">
         <v>2</v>
@@ -2718,33 +2730,33 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -2752,33 +2764,33 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E39">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2786,50 +2798,50 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
         <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
         <v>38</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2837,24 +2849,24 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
         <v>38</v>
@@ -2863,7 +2875,7 @@
         <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2871,7 +2883,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B46" t="s">
         <v>38</v>
@@ -2880,7 +2892,7 @@
         <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2888,7 +2900,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B47" t="s">
         <v>38</v>
@@ -2897,41 +2909,41 @@
         <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C48" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D48" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
         <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D49" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E49">
         <v>4</v>
@@ -2939,24 +2951,24 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C50" t="s">
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
         <v>38</v>
@@ -2965,7 +2977,7 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -2973,19 +2985,19 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
         <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2993,16 +3005,16 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3013,10 +3025,10 @@
         <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3024,16 +3036,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B55" t="s">
         <v>39</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3041,16 +3053,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B56" t="s">
         <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D56" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3064,10 +3076,10 @@
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3075,16 +3087,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D58" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3092,16 +3104,16 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D59" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3109,16 +3121,16 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B60" t="s">
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D60" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3126,16 +3138,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3143,36 +3155,36 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D62" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3183,10 +3195,10 @@
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D64" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3197,13 +3209,13 @@
         <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D65" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3211,16 +3223,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
         <v>39</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D66" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3228,16 +3240,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C67" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3251,10 +3263,10 @@
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D68" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3262,16 +3274,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D69" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3279,16 +3291,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B70" t="s">
         <v>39</v>
       </c>
       <c r="C70" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3302,13 +3314,13 @@
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D71" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3316,50 +3328,50 @@
         <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C72" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D72" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
         <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D73" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C74" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3367,13 +3379,13 @@
         <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3381,75 +3393,75 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B76" t="s">
         <v>39</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C77" t="s">
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D78" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E78">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E79">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B80" t="s">
         <v>39</v>
@@ -3458,10 +3470,10 @@
         <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3469,30 +3481,30 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D81" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
       </c>
       <c r="C82" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D82" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3500,16 +3512,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C83" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3520,13 +3532,13 @@
         <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D84" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3534,16 +3546,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D85" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3551,16 +3563,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C86" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D86" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3571,30 +3583,30 @@
         <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D88" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3602,33 +3614,33 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B89" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C89" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D89" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D90" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3636,16 +3648,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D91" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3653,16 +3665,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D92" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3670,16 +3682,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D93" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3687,16 +3699,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D94" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3704,16 +3716,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D95" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3721,16 +3733,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
       </c>
       <c r="C96" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D96" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3738,16 +3750,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B97" t="s">
         <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3755,16 +3767,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B98" t="s">
         <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D98" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3772,16 +3784,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
         <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D99" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3789,16 +3801,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D100" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3806,16 +3818,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B101" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D101" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3823,16 +3835,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B102" t="s">
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D102" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3840,16 +3852,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
         <v>37</v>
       </c>
       <c r="C103" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D103" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3857,16 +3869,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D104" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3874,16 +3886,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B105" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C105" t="s">
         <v>104</v>
       </c>
       <c r="D105" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3891,7 +3903,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
@@ -3900,7 +3912,7 @@
         <v>105</v>
       </c>
       <c r="D106" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3908,7 +3920,7 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
@@ -3917,7 +3929,7 @@
         <v>106</v>
       </c>
       <c r="D107" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3925,7 +3937,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
@@ -3934,7 +3946,7 @@
         <v>107</v>
       </c>
       <c r="D108" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3942,7 +3954,7 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
@@ -3951,7 +3963,7 @@
         <v>108</v>
       </c>
       <c r="D109" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3959,7 +3971,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
@@ -3968,24 +3980,24 @@
         <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -3993,16 +4005,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4010,33 +4022,33 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D113" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E113">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D114" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4044,33 +4056,33 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D115" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E115">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D116" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4078,7 +4090,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4087,15 +4099,15 @@
         <v>113</v>
       </c>
       <c r="D117" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
@@ -4104,7 +4116,7 @@
         <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4112,7 +4124,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
@@ -4121,15 +4133,15 @@
         <v>115</v>
       </c>
       <c r="D119" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B120" t="s">
         <v>39</v>
@@ -4138,15 +4150,15 @@
         <v>116</v>
       </c>
       <c r="D120" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E120">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B121" t="s">
         <v>39</v>
@@ -4155,15 +4167,15 @@
         <v>117</v>
       </c>
       <c r="D121" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E121">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
@@ -4172,49 +4184,49 @@
         <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E122">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D123" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E123">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D124" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E124">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
@@ -4223,24 +4235,24 @@
         <v>120</v>
       </c>
       <c r="D125" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E125">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B126" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D126" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4248,16 +4260,16 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D127" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4265,16 +4277,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B128" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C128" t="s">
         <v>122</v>
       </c>
       <c r="D128" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4282,7 +4294,7 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
         <v>39</v>
@@ -4291,7 +4303,7 @@
         <v>123</v>
       </c>
       <c r="D129" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4299,7 +4311,7 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
         <v>39</v>
@@ -4308,7 +4320,7 @@
         <v>124</v>
       </c>
       <c r="D130" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4316,7 +4328,7 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
@@ -4325,7 +4337,7 @@
         <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4333,7 +4345,7 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B132" t="s">
         <v>39</v>
@@ -4342,7 +4354,7 @@
         <v>126</v>
       </c>
       <c r="D132" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4350,7 +4362,7 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B133" t="s">
         <v>39</v>
@@ -4359,7 +4371,7 @@
         <v>127</v>
       </c>
       <c r="D133" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4367,7 +4379,7 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
         <v>39</v>
@@ -4376,7 +4388,7 @@
         <v>128</v>
       </c>
       <c r="D134" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4384,7 +4396,7 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B135" t="s">
         <v>39</v>
@@ -4393,7 +4405,7 @@
         <v>129</v>
       </c>
       <c r="D135" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4401,7 +4413,7 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B136" t="s">
         <v>39</v>
@@ -4410,7 +4422,7 @@
         <v>130</v>
       </c>
       <c r="D136" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4418,7 +4430,7 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B137" t="s">
         <v>39</v>
@@ -4427,7 +4439,7 @@
         <v>131</v>
       </c>
       <c r="D137" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4435,7 +4447,7 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B138" t="s">
         <v>39</v>
@@ -4444,7 +4456,7 @@
         <v>132</v>
       </c>
       <c r="D138" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4452,7 +4464,7 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B139" t="s">
         <v>39</v>
@@ -4461,7 +4473,7 @@
         <v>133</v>
       </c>
       <c r="D139" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4469,7 +4481,7 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B140" t="s">
         <v>39</v>
@@ -4478,7 +4490,7 @@
         <v>134</v>
       </c>
       <c r="D140" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4486,7 +4498,7 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
         <v>39</v>
@@ -4495,7 +4507,7 @@
         <v>135</v>
       </c>
       <c r="D141" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4503,7 +4515,7 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B142" t="s">
         <v>39</v>
@@ -4512,7 +4524,7 @@
         <v>136</v>
       </c>
       <c r="D142" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4520,7 +4532,7 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B143" t="s">
         <v>39</v>
@@ -4529,7 +4541,7 @@
         <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4537,7 +4549,7 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B144" t="s">
         <v>39</v>
@@ -4546,7 +4558,7 @@
         <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4554,7 +4566,7 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B145" t="s">
         <v>39</v>
@@ -4563,7 +4575,7 @@
         <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4571,7 +4583,7 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B146" t="s">
         <v>39</v>
@@ -4580,7 +4592,7 @@
         <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4588,7 +4600,7 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B147" t="s">
         <v>39</v>
@@ -4597,7 +4609,7 @@
         <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4605,7 +4617,7 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B148" t="s">
         <v>39</v>
@@ -4614,7 +4626,7 @@
         <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4622,7 +4634,7 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B149" t="s">
         <v>39</v>
@@ -4631,7 +4643,7 @@
         <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4639,7 +4651,7 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B150" t="s">
         <v>39</v>
@@ -4648,7 +4660,7 @@
         <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4656,7 +4668,7 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B151" t="s">
         <v>39</v>
@@ -4665,7 +4677,7 @@
         <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4673,7 +4685,7 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B152" t="s">
         <v>39</v>
@@ -4682,7 +4694,7 @@
         <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4690,7 +4702,7 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B153" t="s">
         <v>39</v>
@@ -4699,7 +4711,7 @@
         <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4707,7 +4719,7 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B154" t="s">
         <v>39</v>
@@ -4716,7 +4728,7 @@
         <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4724,7 +4736,7 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B155" t="s">
         <v>39</v>
@@ -4733,15 +4745,15 @@
         <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="E155">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B156" t="s">
         <v>39</v>
@@ -4750,15 +4762,15 @@
         <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E156">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B157" t="s">
         <v>39</v>
@@ -4767,7 +4779,7 @@
         <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4775,7 +4787,7 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B158" t="s">
         <v>39</v>
@@ -4784,7 +4796,7 @@
         <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4792,7 +4804,7 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B159" t="s">
         <v>39</v>
@@ -4801,7 +4813,7 @@
         <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E159">
         <v>2</v>
@@ -4809,7 +4821,7 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B160" t="s">
         <v>39</v>
@@ -4818,15 +4830,15 @@
         <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E160">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B161" t="s">
         <v>39</v>
@@ -4835,15 +4847,15 @@
         <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>280</v>
+        <v>318</v>
       </c>
       <c r="E161">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B162" t="s">
         <v>39</v>
@@ -4852,15 +4864,15 @@
         <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E162">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B163" t="s">
         <v>39</v>
@@ -4869,15 +4881,15 @@
         <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>317</v>
+        <v>284</v>
       </c>
       <c r="E163">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B164" t="s">
         <v>39</v>
@@ -4886,15 +4898,15 @@
         <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E164">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B165" t="s">
         <v>39</v>
@@ -4903,49 +4915,49 @@
         <v>159</v>
       </c>
       <c r="D165" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E165">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B166" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C166" t="s">
         <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E166">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B167" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C167" t="s">
         <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E167">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B168" t="s">
         <v>37</v>
@@ -4954,7 +4966,7 @@
         <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4962,7 +4974,7 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B169" t="s">
         <v>37</v>
@@ -4971,7 +4983,7 @@
         <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4979,7 +4991,7 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B170" t="s">
         <v>37</v>
@@ -4988,7 +5000,7 @@
         <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -4996,7 +5008,7 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B171" t="s">
         <v>37</v>
@@ -5005,7 +5017,7 @@
         <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>238</v>
+        <v>327</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5013,7 +5025,7 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B172" t="s">
         <v>37</v>
@@ -5022,7 +5034,7 @@
         <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5030,7 +5042,7 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B173" t="s">
         <v>37</v>
@@ -5039,7 +5051,7 @@
         <v>167</v>
       </c>
       <c r="D173" t="s">
-        <v>326</v>
+        <v>242</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5047,7 +5059,7 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B174" t="s">
         <v>37</v>
@@ -5056,7 +5068,7 @@
         <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5064,7 +5076,7 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B175" t="s">
         <v>37</v>
@@ -5073,7 +5085,7 @@
         <v>169</v>
       </c>
       <c r="D175" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5081,7 +5093,7 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B176" t="s">
         <v>37</v>
@@ -5090,7 +5102,7 @@
         <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5098,7 +5110,7 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B177" t="s">
         <v>37</v>
@@ -5107,7 +5119,7 @@
         <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5115,7 +5127,7 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B178" t="s">
         <v>37</v>
@@ -5124,7 +5136,7 @@
         <v>172</v>
       </c>
       <c r="D178" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5132,7 +5144,7 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B179" t="s">
         <v>37</v>
@@ -5141,7 +5153,7 @@
         <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5149,7 +5161,7 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B180" t="s">
         <v>37</v>
@@ -5158,7 +5170,7 @@
         <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5166,7 +5178,7 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B181" t="s">
         <v>37</v>
@@ -5175,7 +5187,7 @@
         <v>175</v>
       </c>
       <c r="D181" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5183,7 +5195,7 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B182" t="s">
         <v>37</v>
@@ -5192,7 +5204,7 @@
         <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5200,7 +5212,7 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B183" t="s">
         <v>37</v>
@@ -5209,7 +5221,7 @@
         <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5217,7 +5229,7 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B184" t="s">
         <v>37</v>
@@ -5226,7 +5238,7 @@
         <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5234,7 +5246,7 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B185" t="s">
         <v>37</v>
@@ -5243,7 +5255,7 @@
         <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5251,7 +5263,7 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B186" t="s">
         <v>37</v>
@@ -5260,7 +5272,7 @@
         <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5268,7 +5280,7 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B187" t="s">
         <v>37</v>
@@ -5277,7 +5289,7 @@
         <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5285,7 +5297,7 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B188" t="s">
         <v>37</v>
@@ -5294,7 +5306,7 @@
         <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5302,7 +5314,7 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B189" t="s">
         <v>37</v>
@@ -5311,7 +5323,7 @@
         <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5319,7 +5331,7 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B190" t="s">
         <v>37</v>
@@ -5328,7 +5340,7 @@
         <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5336,7 +5348,7 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B191" t="s">
         <v>37</v>
@@ -5345,7 +5357,7 @@
         <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5353,7 +5365,7 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B192" t="s">
         <v>37</v>
@@ -5362,7 +5374,7 @@
         <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5370,7 +5382,7 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B193" t="s">
         <v>37</v>
@@ -5379,7 +5391,7 @@
         <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5387,7 +5399,7 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B194" t="s">
         <v>37</v>
@@ -5396,7 +5408,7 @@
         <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>305</v>
+        <v>349</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5404,7 +5416,7 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B195" t="s">
         <v>37</v>
@@ -5413,7 +5425,7 @@
         <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5421,7 +5433,7 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B196" t="s">
         <v>37</v>
@@ -5430,7 +5442,7 @@
         <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>348</v>
+        <v>309</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5438,7 +5450,7 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B197" t="s">
         <v>37</v>
@@ -5447,15 +5459,15 @@
         <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E197">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B198" t="s">
         <v>37</v>
@@ -5464,15 +5476,15 @@
         <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>232</v>
+        <v>352</v>
       </c>
       <c r="E198">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B199" t="s">
         <v>37</v>
@@ -5481,7 +5493,7 @@
         <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5489,7 +5501,7 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B200" t="s">
         <v>37</v>
@@ -5498,7 +5510,7 @@
         <v>194</v>
       </c>
       <c r="D200" t="s">
-        <v>351</v>
+        <v>236</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5506,7 +5518,7 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B201" t="s">
         <v>37</v>
@@ -5515,7 +5527,7 @@
         <v>195</v>
       </c>
       <c r="D201" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5523,7 +5535,7 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B202" t="s">
         <v>37</v>
@@ -5532,7 +5544,7 @@
         <v>196</v>
       </c>
       <c r="D202" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5540,7 +5552,7 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B203" t="s">
         <v>37</v>
@@ -5549,7 +5561,7 @@
         <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5557,7 +5569,7 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B204" t="s">
         <v>37</v>
@@ -5566,7 +5578,7 @@
         <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5574,7 +5586,7 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B205" t="s">
         <v>37</v>
@@ -5583,7 +5595,7 @@
         <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5591,7 +5603,7 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B206" t="s">
         <v>37</v>
@@ -5600,7 +5612,7 @@
         <v>200</v>
       </c>
       <c r="D206" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5608,7 +5620,7 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B207" t="s">
         <v>37</v>
@@ -5617,7 +5629,7 @@
         <v>201</v>
       </c>
       <c r="D207" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5625,7 +5637,7 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B208" t="s">
         <v>37</v>
@@ -5634,7 +5646,7 @@
         <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5642,7 +5654,7 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B209" t="s">
         <v>37</v>
@@ -5651,15 +5663,15 @@
         <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E209">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B210" t="s">
         <v>37</v>
@@ -5668,15 +5680,15 @@
         <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>238</v>
+        <v>362</v>
       </c>
       <c r="E210">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B211" t="s">
         <v>37</v>
@@ -5685,15 +5697,15 @@
         <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E211">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B212" t="s">
         <v>37</v>
@@ -5702,15 +5714,15 @@
         <v>206</v>
       </c>
       <c r="D212" t="s">
-        <v>361</v>
+        <v>242</v>
       </c>
       <c r="E212">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B213" t="s">
         <v>37</v>
@@ -5719,7 +5731,7 @@
         <v>207</v>
       </c>
       <c r="D213" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E213">
         <v>4</v>
@@ -5727,7 +5739,7 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B214" t="s">
         <v>37</v>
@@ -5736,7 +5748,7 @@
         <v>208</v>
       </c>
       <c r="D214" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E214">
         <v>4</v>
@@ -5744,7 +5756,7 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B215" t="s">
         <v>37</v>
@@ -5753,7 +5765,7 @@
         <v>209</v>
       </c>
       <c r="D215" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5761,7 +5773,7 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B216" t="s">
         <v>37</v>
@@ -5770,15 +5782,15 @@
         <v>210</v>
       </c>
       <c r="D216" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E216">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B217" t="s">
         <v>37</v>
@@ -5787,15 +5799,15 @@
         <v>211</v>
       </c>
       <c r="D217" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E217">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B218" t="s">
         <v>37</v>
@@ -5804,15 +5816,15 @@
         <v>212</v>
       </c>
       <c r="D218" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E218">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B219" t="s">
         <v>37</v>
@@ -5821,15 +5833,15 @@
         <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E219">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B220" t="s">
         <v>37</v>
@@ -5838,15 +5850,15 @@
         <v>214</v>
       </c>
       <c r="D220" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E220">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B221" t="s">
         <v>37</v>
@@ -5855,15 +5867,15 @@
         <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E221">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B222" t="s">
         <v>37</v>
@@ -5872,15 +5884,15 @@
         <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>240</v>
+        <v>373</v>
       </c>
       <c r="E222">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B223" t="s">
         <v>37</v>
@@ -5889,15 +5901,15 @@
         <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E223">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B224" t="s">
         <v>37</v>
@@ -5906,15 +5918,15 @@
         <v>218</v>
       </c>
       <c r="D224" t="s">
-        <v>371</v>
+        <v>244</v>
       </c>
       <c r="E224">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B225" t="s">
         <v>37</v>
@@ -5923,15 +5935,15 @@
         <v>219</v>
       </c>
       <c r="D225" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E225">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B226" t="s">
         <v>37</v>
@@ -5940,26 +5952,60 @@
         <v>220</v>
       </c>
       <c r="D226" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E226">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B227" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C227" t="s">
         <v>221</v>
       </c>
       <c r="D227" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E227">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
+      <c r="A228" t="s">
+        <v>14</v>
+      </c>
+      <c r="B228" t="s">
+        <v>37</v>
+      </c>
+      <c r="C228" t="s">
+        <v>222</v>
+      </c>
+      <c r="D228" t="s">
+        <v>377</v>
+      </c>
+      <c r="E228">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5">
+      <c r="A229" t="s">
+        <v>10</v>
+      </c>
+      <c r="B229" t="s">
+        <v>38</v>
+      </c>
+      <c r="C229" t="s">
+        <v>223</v>
+      </c>
+      <c r="D229" t="s">
+        <v>378</v>
+      </c>
+      <c r="E229">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (05/08/2026 12:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="381">
   <si>
     <t>matricula</t>
   </si>
@@ -35,63 +35,63 @@
     <t>soma_unidades_faltantes</t>
   </si>
   <si>
+    <t>2721</t>
+  </si>
+  <si>
+    <t>2731</t>
+  </si>
+  <si>
+    <t>2728</t>
+  </si>
+  <si>
+    <t>2732</t>
+  </si>
+  <si>
+    <t>2730</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>2726</t>
+  </si>
+  <si>
+    <t>2702</t>
+  </si>
+  <si>
+    <t>2703</t>
+  </si>
+  <si>
+    <t>2704</t>
+  </si>
+  <si>
+    <t>2708</t>
+  </si>
+  <si>
     <t>2709</t>
   </si>
   <si>
+    <t>2719</t>
+  </si>
+  <si>
     <t>2720</t>
   </si>
   <si>
-    <t>2721</t>
+    <t>2722</t>
+  </si>
+  <si>
+    <t>2723</t>
+  </si>
+  <si>
+    <t>2727</t>
+  </si>
+  <si>
+    <t>2729</t>
   </si>
   <si>
     <t>2733</t>
   </si>
   <si>
-    <t>2728</t>
-  </si>
-  <si>
-    <t>2732</t>
-  </si>
-  <si>
-    <t>2730</t>
-  </si>
-  <si>
-    <t>2734</t>
-  </si>
-  <si>
-    <t>2726</t>
-  </si>
-  <si>
-    <t>2702</t>
-  </si>
-  <si>
-    <t>2703</t>
-  </si>
-  <si>
-    <t>2704</t>
-  </si>
-  <si>
-    <t>2708</t>
-  </si>
-  <si>
-    <t>2719</t>
-  </si>
-  <si>
-    <t>2722</t>
-  </si>
-  <si>
-    <t>2723</t>
-  </si>
-  <si>
-    <t>2727</t>
-  </si>
-  <si>
-    <t>2729</t>
-  </si>
-  <si>
-    <t>2731</t>
-  </si>
-  <si>
     <t>2736</t>
   </si>
   <si>
@@ -128,15 +128,18 @@
     <t>6º ETA</t>
   </si>
   <si>
+    <t>1ª ETA</t>
+  </si>
+  <si>
+    <t>1º/5º GAV</t>
+  </si>
+  <si>
+    <t>7º ETA</t>
+  </si>
+  <si>
     <t>1º ETA</t>
   </si>
   <si>
-    <t>1º/5º GAV</t>
-  </si>
-  <si>
-    <t>7º ETA</t>
-  </si>
-  <si>
     <t>EPCAR</t>
   </si>
   <si>
@@ -152,9 +155,6 @@
     <t>1/15 GAV</t>
   </si>
   <si>
-    <t>1ª ETA</t>
-  </si>
-  <si>
     <t>BAPV</t>
   </si>
   <si>
@@ -191,12 +191,6 @@
     <t>quantidade_faltante</t>
   </si>
   <si>
-    <t>068-02800</t>
-  </si>
-  <si>
-    <t>C668050-1108</t>
-  </si>
-  <si>
     <t>3044000</t>
   </si>
   <si>
@@ -266,6 +260,9 @@
     <t>2622243-11</t>
   </si>
   <si>
+    <t>MS28778-4</t>
+  </si>
+  <si>
     <t>1H75-21</t>
   </si>
   <si>
@@ -686,13 +683,13 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>NAS147-84</t>
+  </si>
+  <si>
     <t>F2552-070</t>
   </si>
   <si>
-    <t>INSULATOR</t>
-  </si>
-  <si>
-    <t>TRANSMITTER FUEL</t>
+    <t>MS29512-5</t>
   </si>
   <si>
     <t>ENGINE PT6A-114A</t>
@@ -764,6 +761,9 @@
     <t>ECCENTRIC-WING ASSY</t>
   </si>
   <si>
+    <t>RETAINER-PACKING BACKUP</t>
+  </si>
+  <si>
     <t>PRESSURE REGULATOR</t>
   </si>
   <si>
@@ -1151,7 +1151,13 @@
     <t>POST LIGHT ASS</t>
   </si>
   <si>
+    <t>BOLT,INTERNAL WRENCHING</t>
+  </si>
+  <si>
     <t>BARREL NUT</t>
+  </si>
+  <si>
+    <t>O-RING</t>
   </si>
 </sst>
 </file>
@@ -1523,7 +1529,7 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1531,7 +1537,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
         <v>50</v>
@@ -1551,7 +1557,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
         <v>50</v>
@@ -1560,10 +1566,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1571,19 +1577,19 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1591,19 +1597,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="F6">
-        <v>43</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1620,10 +1626,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="F7">
-        <v>13</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1631,7 +1637,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1640,10 +1646,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="F8">
-        <v>111</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1651,19 +1657,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E9">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>166</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1671,19 +1677,19 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E10">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>228</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1691,7 +1697,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
         <v>51</v>
@@ -1731,7 +1737,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1751,7 +1757,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1771,7 +1777,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1791,7 +1797,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1811,7 +1817,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1831,7 +1837,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1871,7 +1877,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1951,7 +1957,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
@@ -2051,7 +2057,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
@@ -2071,7 +2077,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
@@ -2113,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2144,21 +2150,21 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
         <v>225</v>
@@ -2169,16 +2175,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2189,13 +2195,13 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2209,10 +2215,10 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2223,13 +2229,13 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2237,13 +2243,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
         <v>226</v>
@@ -2254,13 +2260,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
         <v>226</v>
@@ -2274,13 +2280,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2291,13 +2297,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2311,10 +2317,10 @@
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2325,13 +2331,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2339,13 +2345,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
         <v>227</v>
@@ -2356,13 +2362,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
         <v>227</v>
@@ -2376,13 +2382,13 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2396,10 +2402,10 @@
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2407,13 +2413,13 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
         <v>228</v>
@@ -2424,13 +2430,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
         <v>228</v>
@@ -2441,16 +2447,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2458,13 +2464,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
         <v>229</v>
@@ -2475,13 +2481,13 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D22" t="s">
         <v>229</v>
@@ -2492,16 +2498,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2509,13 +2515,13 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D24" t="s">
         <v>230</v>
@@ -2526,30 +2532,30 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
         <v>230</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
         <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D26" t="s">
         <v>231</v>
@@ -2560,24 +2566,24 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C27" t="s">
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
@@ -2586,7 +2592,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2594,7 +2600,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
@@ -2603,7 +2609,7 @@
         <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2611,7 +2617,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B30" t="s">
         <v>38</v>
@@ -2620,7 +2626,7 @@
         <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2628,7 +2634,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
@@ -2637,10 +2643,10 @@
         <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2648,30 +2654,30 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
         <v>236</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2682,27 +2688,27 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
         <v>237</v>
@@ -2713,13 +2719,13 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
         <v>237</v>
@@ -2730,30 +2736,30 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
         <v>238</v>
@@ -2764,33 +2770,33 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D39" t="s">
         <v>238</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2798,47 +2804,47 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
         <v>239</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
         <v>239</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B43" t="s">
         <v>38</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
         <v>240</v>
@@ -2849,24 +2855,24 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
         <v>38</v>
@@ -2875,7 +2881,7 @@
         <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2883,7 +2889,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
         <v>38</v>
@@ -2892,7 +2898,7 @@
         <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2900,7 +2906,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
         <v>38</v>
@@ -2909,38 +2915,38 @@
         <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
         <v>244</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
         <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D49" t="s">
         <v>245</v>
@@ -2951,24 +2957,24 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C50" t="s">
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B51" t="s">
         <v>38</v>
@@ -2977,7 +2983,7 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -2985,7 +2991,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
         <v>38</v>
@@ -2994,38 +3000,38 @@
         <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
         <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B54" t="s">
         <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
         <v>249</v>
@@ -3036,13 +3042,13 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
         <v>39</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D55" t="s">
         <v>249</v>
@@ -3053,7 +3059,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B56" t="s">
         <v>39</v>
@@ -3062,7 +3068,7 @@
         <v>83</v>
       </c>
       <c r="D56" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3070,13 +3076,13 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D57" t="s">
         <v>250</v>
@@ -3087,13 +3093,13 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D58" t="s">
         <v>250</v>
@@ -3104,7 +3110,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
@@ -3113,7 +3119,7 @@
         <v>84</v>
       </c>
       <c r="D59" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3127,7 +3133,7 @@
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D60" t="s">
         <v>251</v>
@@ -3138,7 +3144,7 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
@@ -3147,7 +3153,7 @@
         <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3161,7 +3167,7 @@
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D62" t="s">
         <v>252</v>
@@ -3172,7 +3178,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
@@ -3181,21 +3187,21 @@
         <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D64" t="s">
         <v>253</v>
@@ -3206,13 +3212,13 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D65" t="s">
         <v>253</v>
@@ -3223,13 +3229,13 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B66" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D66" t="s">
         <v>253</v>
@@ -3240,16 +3246,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B67" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C67" t="s">
         <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3257,13 +3263,13 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D68" t="s">
         <v>254</v>
@@ -3274,13 +3280,13 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D69" t="s">
         <v>254</v>
@@ -3291,7 +3297,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B70" t="s">
         <v>39</v>
@@ -3300,7 +3306,7 @@
         <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3308,13 +3314,13 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D71" t="s">
         <v>255</v>
@@ -3325,30 +3331,30 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
         <v>39</v>
       </c>
       <c r="C72" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D72" t="s">
         <v>255</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
         <v>255</v>
@@ -3359,30 +3365,30 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
         <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E74">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
         <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D75" t="s">
         <v>256</v>
@@ -3393,13 +3399,13 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D76" t="s">
         <v>256</v>
@@ -3410,24 +3416,24 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E77">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
@@ -3436,21 +3442,21 @@
         <v>91</v>
       </c>
       <c r="D78" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D79" t="s">
         <v>258</v>
@@ -3461,7 +3467,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
         <v>39</v>
@@ -3470,15 +3476,15 @@
         <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B81" t="s">
         <v>39</v>
@@ -3487,10 +3493,10 @@
         <v>93</v>
       </c>
       <c r="D81" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E81">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3498,10 +3504,10 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D82" t="s">
         <v>260</v>
@@ -3512,16 +3518,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C83" t="s">
         <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3529,13 +3535,13 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D84" t="s">
         <v>261</v>
@@ -3546,13 +3552,13 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D85" t="s">
         <v>261</v>
@@ -3563,16 +3569,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C86" t="s">
         <v>95</v>
       </c>
       <c r="D86" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3580,13 +3586,13 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D87" t="s">
         <v>255</v>
@@ -3597,47 +3603,47 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B88" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D88" t="s">
         <v>255</v>
       </c>
       <c r="E88">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B89" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C89" t="s">
         <v>96</v>
       </c>
       <c r="D89" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="E89">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D90" t="s">
         <v>262</v>
@@ -3648,7 +3654,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
@@ -3657,7 +3663,7 @@
         <v>97</v>
       </c>
       <c r="D91" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3665,13 +3671,13 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D92" t="s">
         <v>263</v>
@@ -3682,7 +3688,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
@@ -3691,7 +3697,7 @@
         <v>98</v>
       </c>
       <c r="D93" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3699,13 +3705,13 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D94" t="s">
         <v>264</v>
@@ -3716,7 +3722,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
@@ -3725,7 +3731,7 @@
         <v>99</v>
       </c>
       <c r="D95" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3733,13 +3739,13 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
       </c>
       <c r="C96" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D96" t="s">
         <v>265</v>
@@ -3750,7 +3756,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B97" t="s">
         <v>39</v>
@@ -3759,7 +3765,7 @@
         <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3767,13 +3773,13 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B98" t="s">
         <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D98" t="s">
         <v>266</v>
@@ -3784,7 +3790,7 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B99" t="s">
         <v>39</v>
@@ -3793,7 +3799,7 @@
         <v>101</v>
       </c>
       <c r="D99" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3801,13 +3807,13 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D100" t="s">
         <v>267</v>
@@ -3818,7 +3824,7 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B101" t="s">
         <v>39</v>
@@ -3827,7 +3833,7 @@
         <v>102</v>
       </c>
       <c r="D101" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3838,10 +3844,10 @@
         <v>12</v>
       </c>
       <c r="B102" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C102" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D102" t="s">
         <v>268</v>
@@ -3852,16 +3858,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C103" t="s">
         <v>103</v>
       </c>
       <c r="D103" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3872,10 +3878,10 @@
         <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C104" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D104" t="s">
         <v>269</v>
@@ -3886,16 +3892,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B105" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C105" t="s">
         <v>104</v>
       </c>
       <c r="D105" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3903,7 +3909,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
@@ -3912,7 +3918,7 @@
         <v>105</v>
       </c>
       <c r="D106" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3920,7 +3926,7 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
@@ -3929,7 +3935,7 @@
         <v>106</v>
       </c>
       <c r="D107" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3937,7 +3943,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
@@ -3946,7 +3952,7 @@
         <v>107</v>
       </c>
       <c r="D108" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3954,7 +3960,7 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
@@ -3963,7 +3969,7 @@
         <v>108</v>
       </c>
       <c r="D109" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3971,7 +3977,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
@@ -3980,7 +3986,7 @@
         <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3988,7 +3994,7 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
@@ -3997,32 +4003,32 @@
         <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D112" t="s">
         <v>276</v>
       </c>
       <c r="E112">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
@@ -4031,21 +4037,21 @@
         <v>111</v>
       </c>
       <c r="D113" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D114" t="s">
         <v>277</v>
@@ -4056,7 +4062,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
@@ -4065,7 +4071,7 @@
         <v>112</v>
       </c>
       <c r="D115" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4073,24 +4079,24 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D116" t="s">
         <v>278</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4099,15 +4105,15 @@
         <v>113</v>
       </c>
       <c r="D117" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
@@ -4116,7 +4122,7 @@
         <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4124,7 +4130,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
@@ -4133,7 +4139,7 @@
         <v>115</v>
       </c>
       <c r="D119" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4141,7 +4147,7 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B120" t="s">
         <v>39</v>
@@ -4150,15 +4156,15 @@
         <v>116</v>
       </c>
       <c r="D120" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B121" t="s">
         <v>39</v>
@@ -4167,15 +4173,15 @@
         <v>117</v>
       </c>
       <c r="D121" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
@@ -4184,15 +4190,15 @@
         <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E122">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
@@ -4201,21 +4207,21 @@
         <v>119</v>
       </c>
       <c r="D123" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E123">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D124" t="s">
         <v>284</v>
@@ -4226,7 +4232,7 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
@@ -4235,15 +4241,15 @@
         <v>120</v>
       </c>
       <c r="D125" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E125">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B126" t="s">
         <v>39</v>
@@ -4252,7 +4258,7 @@
         <v>121</v>
       </c>
       <c r="D126" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4260,13 +4266,13 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C127" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D127" t="s">
         <v>286</v>
@@ -4277,16 +4283,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B128" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C128" t="s">
         <v>122</v>
       </c>
       <c r="D128" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4294,7 +4300,7 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B129" t="s">
         <v>39</v>
@@ -4303,7 +4309,7 @@
         <v>123</v>
       </c>
       <c r="D129" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4311,7 +4317,7 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B130" t="s">
         <v>39</v>
@@ -4320,7 +4326,7 @@
         <v>124</v>
       </c>
       <c r="D130" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4328,7 +4334,7 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
@@ -4337,7 +4343,7 @@
         <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4345,7 +4351,7 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B132" t="s">
         <v>39</v>
@@ -4354,7 +4360,7 @@
         <v>126</v>
       </c>
       <c r="D132" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4362,7 +4368,7 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B133" t="s">
         <v>39</v>
@@ -4371,7 +4377,7 @@
         <v>127</v>
       </c>
       <c r="D133" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4379,7 +4385,7 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B134" t="s">
         <v>39</v>
@@ -4388,7 +4394,7 @@
         <v>128</v>
       </c>
       <c r="D134" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4396,7 +4402,7 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B135" t="s">
         <v>39</v>
@@ -4405,7 +4411,7 @@
         <v>129</v>
       </c>
       <c r="D135" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4413,7 +4419,7 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B136" t="s">
         <v>39</v>
@@ -4422,7 +4428,7 @@
         <v>130</v>
       </c>
       <c r="D136" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4430,7 +4436,7 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B137" t="s">
         <v>39</v>
@@ -4439,7 +4445,7 @@
         <v>131</v>
       </c>
       <c r="D137" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4447,7 +4453,7 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B138" t="s">
         <v>39</v>
@@ -4456,7 +4462,7 @@
         <v>132</v>
       </c>
       <c r="D138" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4464,7 +4470,7 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B139" t="s">
         <v>39</v>
@@ -4473,7 +4479,7 @@
         <v>133</v>
       </c>
       <c r="D139" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4481,7 +4487,7 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B140" t="s">
         <v>39</v>
@@ -4490,7 +4496,7 @@
         <v>134</v>
       </c>
       <c r="D140" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4498,7 +4504,7 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B141" t="s">
         <v>39</v>
@@ -4507,7 +4513,7 @@
         <v>135</v>
       </c>
       <c r="D141" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4515,7 +4521,7 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B142" t="s">
         <v>39</v>
@@ -4524,7 +4530,7 @@
         <v>136</v>
       </c>
       <c r="D142" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4532,7 +4538,7 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B143" t="s">
         <v>39</v>
@@ -4541,7 +4547,7 @@
         <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4549,7 +4555,7 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B144" t="s">
         <v>39</v>
@@ -4558,7 +4564,7 @@
         <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4566,7 +4572,7 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B145" t="s">
         <v>39</v>
@@ -4575,7 +4581,7 @@
         <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4583,7 +4589,7 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B146" t="s">
         <v>39</v>
@@ -4592,7 +4598,7 @@
         <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4600,7 +4606,7 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B147" t="s">
         <v>39</v>
@@ -4609,7 +4615,7 @@
         <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4617,7 +4623,7 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B148" t="s">
         <v>39</v>
@@ -4626,7 +4632,7 @@
         <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4634,7 +4640,7 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B149" t="s">
         <v>39</v>
@@ -4643,7 +4649,7 @@
         <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4651,7 +4657,7 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B150" t="s">
         <v>39</v>
@@ -4660,7 +4666,7 @@
         <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4668,7 +4674,7 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B151" t="s">
         <v>39</v>
@@ -4677,7 +4683,7 @@
         <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4685,7 +4691,7 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B152" t="s">
         <v>39</v>
@@ -4694,7 +4700,7 @@
         <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4702,7 +4708,7 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B153" t="s">
         <v>39</v>
@@ -4711,7 +4717,7 @@
         <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4719,7 +4725,7 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B154" t="s">
         <v>39</v>
@@ -4728,7 +4734,7 @@
         <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4736,7 +4742,7 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B155" t="s">
         <v>39</v>
@@ -4745,7 +4751,7 @@
         <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4753,7 +4759,7 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B156" t="s">
         <v>39</v>
@@ -4762,15 +4768,15 @@
         <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="E156">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B157" t="s">
         <v>39</v>
@@ -4779,7 +4785,7 @@
         <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4787,7 +4793,7 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B158" t="s">
         <v>39</v>
@@ -4796,7 +4802,7 @@
         <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4804,7 +4810,7 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B159" t="s">
         <v>39</v>
@@ -4813,7 +4819,7 @@
         <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E159">
         <v>2</v>
@@ -4821,7 +4827,7 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B160" t="s">
         <v>39</v>
@@ -4830,7 +4836,7 @@
         <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E160">
         <v>2</v>
@@ -4838,7 +4844,7 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B161" t="s">
         <v>39</v>
@@ -4847,15 +4853,15 @@
         <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E161">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B162" t="s">
         <v>39</v>
@@ -4864,15 +4870,15 @@
         <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>319</v>
+        <v>284</v>
       </c>
       <c r="E162">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B163" t="s">
         <v>39</v>
@@ -4881,15 +4887,15 @@
         <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>284</v>
+        <v>320</v>
       </c>
       <c r="E163">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B164" t="s">
         <v>39</v>
@@ -4898,7 +4904,7 @@
         <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E164">
         <v>8</v>
@@ -4906,7 +4912,7 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B165" t="s">
         <v>39</v>
@@ -4915,15 +4921,15 @@
         <v>159</v>
       </c>
       <c r="D165" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E165">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B166" t="s">
         <v>39</v>
@@ -4932,41 +4938,41 @@
         <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E166">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C167" t="s">
         <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E167">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C168" t="s">
         <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4974,16 +4980,16 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B169" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C169" t="s">
         <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -4991,16 +4997,16 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C170" t="s">
         <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5008,16 +5014,16 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B171" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C171" t="s">
         <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5025,16 +5031,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C172" t="s">
         <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>328</v>
+        <v>241</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5042,16 +5048,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C173" t="s">
         <v>167</v>
       </c>
       <c r="D173" t="s">
-        <v>242</v>
+        <v>329</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5059,16 +5065,16 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C174" t="s">
         <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5076,16 +5082,16 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C175" t="s">
         <v>169</v>
       </c>
       <c r="D175" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5093,16 +5099,16 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B176" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C176" t="s">
         <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5110,16 +5116,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B177" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C177" t="s">
         <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5127,16 +5133,16 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B178" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C178" t="s">
         <v>172</v>
       </c>
       <c r="D178" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5144,16 +5150,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B179" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C179" t="s">
         <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5161,16 +5167,16 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B180" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C180" t="s">
         <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5178,16 +5184,16 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B181" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C181" t="s">
         <v>175</v>
       </c>
       <c r="D181" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5195,16 +5201,16 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B182" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C182" t="s">
         <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5212,16 +5218,16 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B183" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C183" t="s">
         <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5229,16 +5235,16 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B184" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C184" t="s">
         <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5246,16 +5252,16 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C185" t="s">
         <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5263,16 +5269,16 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B186" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C186" t="s">
         <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5280,16 +5286,16 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B187" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C187" t="s">
         <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5297,16 +5303,16 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B188" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C188" t="s">
         <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5314,16 +5320,16 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B189" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C189" t="s">
         <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5331,16 +5337,16 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B190" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C190" t="s">
         <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5348,16 +5354,16 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B191" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C191" t="s">
         <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5365,16 +5371,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B192" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C192" t="s">
         <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5382,16 +5388,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B193" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C193" t="s">
         <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5399,16 +5405,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B194" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C194" t="s">
         <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5416,16 +5422,16 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B195" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C195" t="s">
         <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5433,16 +5439,16 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B196" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C196" t="s">
         <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>309</v>
+        <v>351</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5450,16 +5456,16 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B197" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C197" t="s">
         <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5467,33 +5473,33 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B198" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C198" t="s">
         <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E198">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C199" t="s">
         <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>353</v>
+        <v>235</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5501,16 +5507,16 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C200" t="s">
         <v>194</v>
       </c>
       <c r="D200" t="s">
-        <v>236</v>
+        <v>354</v>
       </c>
       <c r="E200">
         <v>2</v>
@@ -5518,16 +5524,16 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B201" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C201" t="s">
         <v>195</v>
       </c>
       <c r="D201" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E201">
         <v>2</v>
@@ -5535,16 +5541,16 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C202" t="s">
         <v>196</v>
       </c>
       <c r="D202" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5552,16 +5558,16 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C203" t="s">
         <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5569,16 +5575,16 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C204" t="s">
         <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5586,16 +5592,16 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C205" t="s">
         <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5603,10 +5609,10 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B206" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C206" t="s">
         <v>200</v>
@@ -5620,16 +5626,16 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C207" t="s">
         <v>201</v>
       </c>
       <c r="D207" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5637,16 +5643,16 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B208" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C208" t="s">
         <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5654,16 +5660,16 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B209" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C209" t="s">
         <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5671,33 +5677,33 @@
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B210" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C210" t="s">
         <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E210">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B211" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C211" t="s">
         <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>363</v>
+        <v>241</v>
       </c>
       <c r="E211">
         <v>3</v>
@@ -5705,33 +5711,33 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C212" t="s">
         <v>206</v>
       </c>
       <c r="D212" t="s">
-        <v>242</v>
+        <v>364</v>
       </c>
       <c r="E212">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C213" t="s">
         <v>207</v>
       </c>
       <c r="D213" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E213">
         <v>4</v>
@@ -5739,16 +5745,16 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B214" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C214" t="s">
         <v>208</v>
       </c>
       <c r="D214" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E214">
         <v>4</v>
@@ -5756,16 +5762,16 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B215" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C215" t="s">
         <v>209</v>
       </c>
       <c r="D215" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5773,16 +5779,16 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C216" t="s">
         <v>210</v>
       </c>
       <c r="D216" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E216">
         <v>4</v>
@@ -5790,33 +5796,33 @@
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B217" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C217" t="s">
         <v>211</v>
       </c>
       <c r="D217" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E217">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C218" t="s">
         <v>212</v>
       </c>
       <c r="D218" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E218">
         <v>5</v>
@@ -5824,61 +5830,61 @@
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B219" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C219" t="s">
         <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E219">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B220" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C220" t="s">
         <v>214</v>
       </c>
       <c r="D220" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E220">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B221" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C221" t="s">
         <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E221">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C222" t="s">
         <v>216</v>
@@ -5892,33 +5898,33 @@
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B223" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C223" t="s">
         <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>373</v>
+        <v>243</v>
       </c>
       <c r="E223">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C224" t="s">
         <v>218</v>
       </c>
       <c r="D224" t="s">
-        <v>244</v>
+        <v>374</v>
       </c>
       <c r="E224">
         <v>12</v>
@@ -5926,75 +5932,75 @@
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B225" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C225" t="s">
         <v>219</v>
       </c>
       <c r="D225" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E225">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B226" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C226" t="s">
         <v>220</v>
       </c>
       <c r="D226" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E226">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B227" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C227" t="s">
         <v>221</v>
       </c>
       <c r="D227" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E227">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B228" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C228" t="s">
         <v>222</v>
       </c>
       <c r="D228" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E228">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B229" t="s">
         <v>38</v>
@@ -6003,10 +6009,27 @@
         <v>223</v>
       </c>
       <c r="D229" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E229">
         <v>2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
+      <c r="A230" t="s">
+        <v>8</v>
+      </c>
+      <c r="B230" t="s">
+        <v>38</v>
+      </c>
+      <c r="C230" t="s">
+        <v>224</v>
+      </c>
+      <c r="D230" t="s">
+        <v>380</v>
+      </c>
+      <c r="E230">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (07/08/2026 11:16)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="380">
   <si>
     <t>matricula</t>
   </si>
@@ -221,9 +221,6 @@
     <t>400454</t>
   </si>
   <si>
-    <t>2617015-15</t>
-  </si>
-  <si>
     <t>AE3663163K0600</t>
   </si>
   <si>
@@ -722,361 +719,361 @@
     <t>SEAL,PLAIN ENCASED</t>
   </si>
   <si>
+    <t>HOSE ASSY</t>
+  </si>
+  <si>
+    <t>SPRING-MAIN GEAR LH &amp; RH</t>
+  </si>
+  <si>
+    <t>STRAP</t>
+  </si>
+  <si>
+    <t>JACK PAD LH</t>
+  </si>
+  <si>
+    <t>SEAL MOLDED</t>
+  </si>
+  <si>
+    <t>SPACER</t>
+  </si>
+  <si>
+    <t>SPACER MAIN GE</t>
+  </si>
+  <si>
+    <t>BOLT</t>
+  </si>
+  <si>
+    <t>BEARING,SLEEVE</t>
+  </si>
+  <si>
+    <t>CAP MAIN LAND</t>
+  </si>
+  <si>
+    <t>HINGE-ASSY-HOISTING</t>
+  </si>
+  <si>
+    <t>ECCENTRIC-WING ASSY</t>
+  </si>
+  <si>
+    <t>RETAINER-PACKING BACKUP</t>
+  </si>
+  <si>
+    <t>PRESSURE REGULATOR</t>
+  </si>
+  <si>
+    <t>LINE ASSY-PROP</t>
+  </si>
+  <si>
+    <t>PASSENGER DOOR - LOW</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
+  </si>
+  <si>
+    <t>MAIN WHEEL BRAKE</t>
+  </si>
+  <si>
+    <t>CYLINDER GAS S</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-PASSENGER</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
+  </si>
+  <si>
+    <t>TEST KIT, FUEL, WORK</t>
+  </si>
+  <si>
+    <t>FITTING A S TR</t>
+  </si>
+  <si>
+    <t>RING ASSY ENGI</t>
+  </si>
+  <si>
+    <t>TRANSDUCER</t>
+  </si>
+  <si>
+    <t>EXTINGUISHER,FIRE</t>
+  </si>
+  <si>
+    <t>CAP,TUBE</t>
+  </si>
+  <si>
+    <t>SUPORT PLATE</t>
+  </si>
+  <si>
+    <t>ADJUSTER PLATE</t>
+  </si>
+  <si>
+    <t>EVAPORATOR MODULE AS</t>
+  </si>
+  <si>
+    <t>KIT CAB-33-02</t>
+  </si>
+  <si>
+    <t>COUPLING-SPLINED</t>
+  </si>
+  <si>
+    <t>BATTERY-MARATHON TSP410 NICAD</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY LH</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY RH</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-DOOR PULL</t>
+  </si>
+  <si>
+    <t>NUT-DIODE ATTACH</t>
+  </si>
+  <si>
+    <t>COMPRESSOR DRIVE ASS</t>
+  </si>
+  <si>
+    <t>COVER ACCESS RH</t>
+  </si>
+  <si>
+    <t>FLOW CONTROL VALVE</t>
+  </si>
+  <si>
+    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+  </si>
+  <si>
+    <t>EXTENDER-CREW, (WHEN</t>
+  </si>
+  <si>
+    <t>REDUCER ASSEMBY</t>
+  </si>
+  <si>
+    <t>STROB TUB</t>
+  </si>
+  <si>
+    <t>BELLCRANK ASSY</t>
+  </si>
+  <si>
+    <t>IMOBILIZADOR</t>
+  </si>
+  <si>
+    <t>BLOQUEIO DA VENTILAÇ</t>
+  </si>
+  <si>
+    <t>SCREW</t>
+  </si>
+  <si>
+    <t>MAGNETOMETER GMU 44</t>
+  </si>
+  <si>
+    <t>FUEL FILTER ASSY</t>
+  </si>
+  <si>
+    <t>NIPPLE,TUBE</t>
+  </si>
+  <si>
+    <t>REDUCER, TUBE</t>
+  </si>
+  <si>
+    <t>COUPLING,CLAMP,GROOV</t>
+  </si>
+  <si>
+    <t>CONNECTOR</t>
+  </si>
+  <si>
+    <t>TEE,TUBE</t>
+  </si>
+  <si>
+    <t>BEACON,DISTRESS</t>
+  </si>
+  <si>
+    <t>HOSE ASSY BRAKE CYL</t>
+  </si>
+  <si>
+    <t>HOSE ASSY BRAK</t>
+  </si>
+  <si>
+    <t>CONNECTOR BODY,RECEP</t>
+  </si>
+  <si>
+    <t>CONTROL UNIT,GENERA</t>
+  </si>
+  <si>
+    <t>ANEL-O</t>
+  </si>
+  <si>
+    <t>BUNGEE ASSY</t>
+  </si>
+  <si>
+    <t>GASKET</t>
+  </si>
+  <si>
+    <t>DRIVE PULLEY</t>
+  </si>
+  <si>
+    <t>DOOR ASSY COWL LH</t>
+  </si>
+  <si>
+    <t>CAPACITOR-6.0 MF 150</t>
+  </si>
+  <si>
+    <t>SEAT ASSEMBLY - BENCH</t>
+  </si>
+  <si>
+    <t>GSA-80 TORQUE SERVO</t>
+  </si>
+  <si>
+    <t>GSA-81 TORQUE SERVO</t>
+  </si>
+  <si>
+    <t>AFCS MODE CONTROLLER</t>
+  </si>
+  <si>
+    <t>CLIP</t>
+  </si>
+  <si>
+    <t>AIRSPEED INDICATOR</t>
+  </si>
+  <si>
+    <t>BRACKET</t>
+  </si>
+  <si>
+    <t>PORT ASSY DOWNLOAD</t>
+  </si>
+  <si>
+    <t>HANDLE,DOOR</t>
+  </si>
+  <si>
+    <t>COMPRESSOR SUPPORT</t>
+  </si>
+  <si>
+    <t>ANGLE ASSY-GLARESHIELD ATTACH</t>
+  </si>
+  <si>
+    <t>HOSE ASSY-SUCTION LI</t>
+  </si>
+  <si>
+    <t>GAS SPRING</t>
+  </si>
+  <si>
+    <t>RETAINING RING</t>
+  </si>
+  <si>
+    <t>TUBE MAIN 850X10</t>
+  </si>
+  <si>
+    <t>DIMMING ASSY,SPEC</t>
+  </si>
+  <si>
+    <t>CAP</t>
+  </si>
+  <si>
+    <t>WASHER, FLAT</t>
+  </si>
+  <si>
+    <t>BOLT,MACHINE</t>
+  </si>
+  <si>
+    <t>GROMMET</t>
+  </si>
+  <si>
+    <t>STATIC WICK</t>
+  </si>
+  <si>
+    <t>TRUNNION ASSY-RH-MAI</t>
+  </si>
+  <si>
+    <t>VANT,BREATHER</t>
+  </si>
+  <si>
+    <t>HOSE ASSY TEE</t>
+  </si>
+  <si>
+    <t>TRANSMITER FUEL</t>
+  </si>
+  <si>
+    <t>ENGINE MOUNT ASSEMBL</t>
+  </si>
+  <si>
+    <t>TRANSMITTER,RATE OF FLOW</t>
+  </si>
+  <si>
+    <t>WHEEL HALF ASSY-OUTER</t>
+  </si>
+  <si>
+    <t>CABLE FIRE DET</t>
+  </si>
+  <si>
+    <t>HINGE BKT INBD</t>
+  </si>
+  <si>
+    <t>RESTRAINT ASSY</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY AFT NOSE GEAR</t>
+  </si>
+  <si>
+    <t>COVER</t>
+  </si>
+  <si>
+    <t>SHIELD</t>
+  </si>
+  <si>
+    <t>RESERVOIR ASSY-BRAKE</t>
+  </si>
+  <si>
+    <t>STRUT ASSY-RH WING</t>
+  </si>
+  <si>
+    <t>TUBE ASSY-LONG</t>
+  </si>
+  <si>
+    <t>SCREW INTERNAL</t>
+  </si>
+  <si>
+    <t>RIB ASSY-RH-AILERON</t>
+  </si>
+  <si>
+    <t>LOCKNUT,TUBE F</t>
+  </si>
+  <si>
+    <t>BOOT N G STEER</t>
+  </si>
+  <si>
+    <t>HOSE ASSY ELBOW</t>
+  </si>
+  <si>
+    <t>HINGE DOOR LH</t>
+  </si>
+  <si>
+    <t>SCUFF PLATE-LH CREW</t>
+  </si>
+  <si>
+    <t>SCUFF PLATE-RH CREW</t>
+  </si>
+  <si>
+    <t>PLATE - COVER</t>
+  </si>
+  <si>
+    <t>WINDOW MOLDING</t>
+  </si>
+  <si>
+    <t>TRUNNION ASSY</t>
+  </si>
+  <si>
+    <t>BRACKET ASSY-95 AMP</t>
+  </si>
+  <si>
+    <t>LIGHT STROBE RH</t>
+  </si>
+  <si>
+    <t>INDICATOR FUEL</t>
+  </si>
+  <si>
     <t>HINGE-DOOR LH</t>
-  </si>
-  <si>
-    <t>HOSE ASSY</t>
-  </si>
-  <si>
-    <t>SPRING-MAIN GEAR LH &amp; RH</t>
-  </si>
-  <si>
-    <t>STRAP</t>
-  </si>
-  <si>
-    <t>JACK PAD LH</t>
-  </si>
-  <si>
-    <t>SEAL MOLDED</t>
-  </si>
-  <si>
-    <t>SPACER</t>
-  </si>
-  <si>
-    <t>SPACER MAIN GE</t>
-  </si>
-  <si>
-    <t>BOLT</t>
-  </si>
-  <si>
-    <t>BEARING,SLEEVE</t>
-  </si>
-  <si>
-    <t>CAP MAIN LAND</t>
-  </si>
-  <si>
-    <t>HINGE-ASSY-HOISTING</t>
-  </si>
-  <si>
-    <t>ECCENTRIC-WING ASSY</t>
-  </si>
-  <si>
-    <t>RETAINER-PACKING BACKUP</t>
-  </si>
-  <si>
-    <t>PRESSURE REGULATOR</t>
-  </si>
-  <si>
-    <t>LINE ASSY-PROP</t>
-  </si>
-  <si>
-    <t>PASSENGER DOOR - LOW</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
-  </si>
-  <si>
-    <t>MAIN WHEEL BRAKE</t>
-  </si>
-  <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-PASSENGER</t>
-  </si>
-  <si>
-    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
-  </si>
-  <si>
-    <t>TEST KIT, FUEL, WORK</t>
-  </si>
-  <si>
-    <t>FITTING A S TR</t>
-  </si>
-  <si>
-    <t>RING ASSY ENGI</t>
-  </si>
-  <si>
-    <t>TRANSDUCER</t>
-  </si>
-  <si>
-    <t>EXTINGUISHER,FIRE</t>
-  </si>
-  <si>
-    <t>CAP,TUBE</t>
-  </si>
-  <si>
-    <t>SUPORT PLATE</t>
-  </si>
-  <si>
-    <t>ADJUSTER PLATE</t>
-  </si>
-  <si>
-    <t>EVAPORATOR MODULE AS</t>
-  </si>
-  <si>
-    <t>KIT CAB-33-02</t>
-  </si>
-  <si>
-    <t>COUPLING-SPLINED</t>
-  </si>
-  <si>
-    <t>BATTERY-MARATHON TSP410 NICAD</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY LH</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY RH</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-DOOR PULL</t>
-  </si>
-  <si>
-    <t>NUT-DIODE ATTACH</t>
-  </si>
-  <si>
-    <t>COMPRESSOR DRIVE ASS</t>
-  </si>
-  <si>
-    <t>COVER ACCESS RH</t>
-  </si>
-  <si>
-    <t>FLOW CONTROL VALVE</t>
-  </si>
-  <si>
-    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
-  </si>
-  <si>
-    <t>EXTENDER-CREW, (WHEN</t>
-  </si>
-  <si>
-    <t>REDUCER ASSEMBY</t>
-  </si>
-  <si>
-    <t>STROB TUB</t>
-  </si>
-  <si>
-    <t>BELLCRANK ASSY</t>
-  </si>
-  <si>
-    <t>IMOBILIZADOR</t>
-  </si>
-  <si>
-    <t>BLOQUEIO DA VENTILAÇ</t>
-  </si>
-  <si>
-    <t>SCREW</t>
-  </si>
-  <si>
-    <t>MAGNETOMETER GMU 44</t>
-  </si>
-  <si>
-    <t>FUEL FILTER ASSY</t>
-  </si>
-  <si>
-    <t>NIPPLE,TUBE</t>
-  </si>
-  <si>
-    <t>REDUCER, TUBE</t>
-  </si>
-  <si>
-    <t>COUPLING,CLAMP,GROOV</t>
-  </si>
-  <si>
-    <t>CONNECTOR</t>
-  </si>
-  <si>
-    <t>TEE,TUBE</t>
-  </si>
-  <si>
-    <t>BEACON,DISTRESS</t>
-  </si>
-  <si>
-    <t>HOSE ASSY BRAKE CYL</t>
-  </si>
-  <si>
-    <t>HOSE ASSY BRAK</t>
-  </si>
-  <si>
-    <t>CONNECTOR BODY,RECEP</t>
-  </si>
-  <si>
-    <t>CONTROL UNIT,GENERA</t>
-  </si>
-  <si>
-    <t>ANEL-O</t>
-  </si>
-  <si>
-    <t>BUNGEE ASSY</t>
-  </si>
-  <si>
-    <t>GASKET</t>
-  </si>
-  <si>
-    <t>DRIVE PULLEY</t>
-  </si>
-  <si>
-    <t>DOOR ASSY COWL LH</t>
-  </si>
-  <si>
-    <t>CAPACITOR-6.0 MF 150</t>
-  </si>
-  <si>
-    <t>SEAT ASSEMBLY - BENCH</t>
-  </si>
-  <si>
-    <t>GSA-80 TORQUE SERVO</t>
-  </si>
-  <si>
-    <t>GSA-81 TORQUE SERVO</t>
-  </si>
-  <si>
-    <t>AFCS MODE CONTROLLER</t>
-  </si>
-  <si>
-    <t>CLIP</t>
-  </si>
-  <si>
-    <t>AIRSPEED INDICATOR</t>
-  </si>
-  <si>
-    <t>BRACKET</t>
-  </si>
-  <si>
-    <t>PORT ASSY DOWNLOAD</t>
-  </si>
-  <si>
-    <t>HANDLE,DOOR</t>
-  </si>
-  <si>
-    <t>COMPRESSOR SUPPORT</t>
-  </si>
-  <si>
-    <t>ANGLE ASSY-GLARESHIELD ATTACH</t>
-  </si>
-  <si>
-    <t>HOSE ASSY-SUCTION LI</t>
-  </si>
-  <si>
-    <t>GAS SPRING</t>
-  </si>
-  <si>
-    <t>RETAINING RING</t>
-  </si>
-  <si>
-    <t>TUBE MAIN 850X10</t>
-  </si>
-  <si>
-    <t>DIMMING ASSY,SPEC</t>
-  </si>
-  <si>
-    <t>CAP</t>
-  </si>
-  <si>
-    <t>WASHER, FLAT</t>
-  </si>
-  <si>
-    <t>BOLT,MACHINE</t>
-  </si>
-  <si>
-    <t>GROMMET</t>
-  </si>
-  <si>
-    <t>STATIC WICK</t>
-  </si>
-  <si>
-    <t>TRUNNION ASSY-RH-MAI</t>
-  </si>
-  <si>
-    <t>VANT,BREATHER</t>
-  </si>
-  <si>
-    <t>HOSE ASSY TEE</t>
-  </si>
-  <si>
-    <t>TRANSMITER FUEL</t>
-  </si>
-  <si>
-    <t>ENGINE MOUNT ASSEMBL</t>
-  </si>
-  <si>
-    <t>TRANSMITTER,RATE OF FLOW</t>
-  </si>
-  <si>
-    <t>WHEEL HALF ASSY-OUTER</t>
-  </si>
-  <si>
-    <t>CABLE FIRE DET</t>
-  </si>
-  <si>
-    <t>HINGE BKT INBD</t>
-  </si>
-  <si>
-    <t>RESTRAINT ASSY</t>
-  </si>
-  <si>
-    <t>SUPPORT ASSY AFT NOSE GEAR</t>
-  </si>
-  <si>
-    <t>COVER</t>
-  </si>
-  <si>
-    <t>SHIELD</t>
-  </si>
-  <si>
-    <t>RESERVOIR ASSY-BRAKE</t>
-  </si>
-  <si>
-    <t>STRUT ASSY-RH WING</t>
-  </si>
-  <si>
-    <t>TUBE ASSY-LONG</t>
-  </si>
-  <si>
-    <t>SCREW INTERNAL</t>
-  </si>
-  <si>
-    <t>RIB ASSY-RH-AILERON</t>
-  </si>
-  <si>
-    <t>LOCKNUT,TUBE F</t>
-  </si>
-  <si>
-    <t>BOOT N G STEER</t>
-  </si>
-  <si>
-    <t>HOSE ASSY ELBOW</t>
-  </si>
-  <si>
-    <t>HINGE DOOR LH</t>
-  </si>
-  <si>
-    <t>SCUFF PLATE-LH CREW</t>
-  </si>
-  <si>
-    <t>SCUFF PLATE-RH CREW</t>
-  </si>
-  <si>
-    <t>PLATE - COVER</t>
-  </si>
-  <si>
-    <t>WINDOW MOLDING</t>
-  </si>
-  <si>
-    <t>TRUNNION ASSY</t>
-  </si>
-  <si>
-    <t>BRACKET ASSY-95 AMP</t>
-  </si>
-  <si>
-    <t>LIGHT STROBE RH</t>
-  </si>
-  <si>
-    <t>INDICATOR FUEL</t>
   </si>
   <si>
     <t>WASHER</t>
@@ -1566,10 +1563,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F4">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2119,7 +2116,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2150,7 +2147,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2167,7 +2164,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2184,7 +2181,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2201,7 +2198,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2218,7 +2215,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2235,7 +2232,7 @@
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2252,7 +2249,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2269,7 +2266,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2286,7 +2283,7 @@
         <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2303,7 +2300,7 @@
         <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2320,7 +2317,7 @@
         <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2337,7 +2334,7 @@
         <v>59</v>
       </c>
       <c r="D13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2354,7 +2351,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2371,7 +2368,7 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2388,7 +2385,7 @@
         <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2405,7 +2402,7 @@
         <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2422,7 +2419,7 @@
         <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2439,7 +2436,7 @@
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2456,7 +2453,7 @@
         <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2473,7 +2470,7 @@
         <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2490,7 +2487,7 @@
         <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2507,7 +2504,7 @@
         <v>62</v>
       </c>
       <c r="D23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2524,7 +2521,7 @@
         <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2541,7 +2538,7 @@
         <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E25">
         <v>2</v>
@@ -2558,7 +2555,7 @@
         <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2575,7 +2572,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2592,7 +2589,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2609,7 +2606,7 @@
         <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2626,58 +2623,58 @@
         <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D32" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E32">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2685,16 +2682,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C34" t="s">
         <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2702,16 +2699,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E35">
         <v>2</v>
@@ -2719,84 +2716,84 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
         <v>70</v>
       </c>
       <c r="D37" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D38" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E39">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C40" t="s">
         <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -2804,36 +2801,36 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
         <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2847,7 +2844,7 @@
         <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2864,7 +2861,7 @@
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2881,7 +2878,7 @@
         <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2898,24 +2895,24 @@
         <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E47">
         <v>4</v>
@@ -2923,16 +2920,16 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C48" t="s">
         <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E48">
         <v>4</v>
@@ -2949,10 +2946,10 @@
         <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2966,10 +2963,10 @@
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2983,24 +2980,24 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B52" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C52" t="s">
         <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3008,16 +3005,16 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B53" t="s">
         <v>39</v>
       </c>
       <c r="C53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D53" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -3025,16 +3022,16 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
         <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D54" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3042,7 +3039,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B55" t="s">
         <v>39</v>
@@ -3051,7 +3048,7 @@
         <v>82</v>
       </c>
       <c r="D55" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3059,16 +3056,16 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B56" t="s">
         <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3076,16 +3073,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D57" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3093,7 +3090,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
@@ -3102,7 +3099,7 @@
         <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3110,16 +3107,16 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D59" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3127,7 +3124,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B60" t="s">
         <v>39</v>
@@ -3136,7 +3133,7 @@
         <v>84</v>
       </c>
       <c r="D60" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3144,16 +3141,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3161,7 +3158,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B62" t="s">
         <v>39</v>
@@ -3170,24 +3167,24 @@
         <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3195,16 +3192,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3212,16 +3209,16 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D65" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3229,16 +3226,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C66" t="s">
         <v>86</v>
       </c>
       <c r="D66" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3246,16 +3243,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D67" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3263,16 +3260,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D68" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3280,7 +3277,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
@@ -3289,7 +3286,7 @@
         <v>87</v>
       </c>
       <c r="D69" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3297,16 +3294,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B70" t="s">
         <v>39</v>
       </c>
       <c r="C70" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D70" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3314,33 +3311,33 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D71" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D72" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E72">
         <v>4</v>
@@ -3348,33 +3345,33 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
         <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E73">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
         <v>39</v>
       </c>
       <c r="C74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D74" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3382,16 +3379,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D75" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3399,19 +3396,19 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C76" t="s">
         <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3425,24 +3422,24 @@
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E77">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E78">
         <v>5</v>
@@ -3450,7 +3447,7 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
@@ -3459,10 +3456,10 @@
         <v>91</v>
       </c>
       <c r="D79" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E79">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3476,24 +3473,24 @@
         <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E80">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D81" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3501,16 +3498,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C82" t="s">
         <v>93</v>
       </c>
       <c r="D82" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3518,16 +3515,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D83" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3535,16 +3532,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D84" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3552,16 +3549,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C85" t="s">
         <v>94</v>
       </c>
       <c r="D85" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3569,16 +3566,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D86" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3586,50 +3583,50 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D87" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B88" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C88" t="s">
         <v>95</v>
       </c>
       <c r="D88" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D89" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3637,7 +3634,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
@@ -3646,7 +3643,7 @@
         <v>96</v>
       </c>
       <c r="D90" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3654,16 +3651,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D91" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3671,7 +3668,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
@@ -3680,7 +3677,7 @@
         <v>97</v>
       </c>
       <c r="D92" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3688,16 +3685,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D93" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3705,7 +3702,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
@@ -3714,7 +3711,7 @@
         <v>98</v>
       </c>
       <c r="D94" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3722,16 +3719,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D95" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3739,7 +3736,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
@@ -3748,7 +3745,7 @@
         <v>99</v>
       </c>
       <c r="D96" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3756,16 +3753,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B97" t="s">
         <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D97" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3773,7 +3770,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B98" t="s">
         <v>39</v>
@@ -3782,7 +3779,7 @@
         <v>100</v>
       </c>
       <c r="D98" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3790,16 +3787,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B99" t="s">
         <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D99" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3807,7 +3804,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
@@ -3816,7 +3813,7 @@
         <v>101</v>
       </c>
       <c r="D100" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3824,16 +3821,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D101" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3841,16 +3838,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B102" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C102" t="s">
         <v>102</v>
       </c>
       <c r="D102" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3858,16 +3855,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D103" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3875,16 +3872,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B104" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C104" t="s">
         <v>103</v>
       </c>
       <c r="D104" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3901,7 +3898,7 @@
         <v>104</v>
       </c>
       <c r="D105" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3918,7 +3915,7 @@
         <v>105</v>
       </c>
       <c r="D106" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3935,7 +3932,7 @@
         <v>106</v>
       </c>
       <c r="D107" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3952,7 +3949,7 @@
         <v>107</v>
       </c>
       <c r="D108" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3969,7 +3966,7 @@
         <v>108</v>
       </c>
       <c r="D109" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3986,32 +3983,32 @@
         <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D111" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E111">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
@@ -4020,24 +4017,24 @@
         <v>110</v>
       </c>
       <c r="D112" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D113" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4045,7 +4042,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
@@ -4054,7 +4051,7 @@
         <v>111</v>
       </c>
       <c r="D114" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4062,24 +4059,24 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D115" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
@@ -4088,10 +4085,10 @@
         <v>112</v>
       </c>
       <c r="D116" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="E116">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -4105,7 +4102,7 @@
         <v>113</v>
       </c>
       <c r="D117" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4122,7 +4119,7 @@
         <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4139,10 +4136,10 @@
         <v>115</v>
       </c>
       <c r="D119" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4156,10 +4153,10 @@
         <v>116</v>
       </c>
       <c r="D120" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E120">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4173,10 +4170,10 @@
         <v>117</v>
       </c>
       <c r="D121" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E121">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4190,24 +4187,24 @@
         <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E122">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D123" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E123">
         <v>30</v>
@@ -4224,10 +4221,10 @@
         <v>119</v>
       </c>
       <c r="D124" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E124">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4241,7 +4238,7 @@
         <v>120</v>
       </c>
       <c r="D125" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4249,16 +4246,16 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B126" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C126" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D126" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E126">
         <v>1</v>
@@ -4266,16 +4263,16 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B127" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C127" t="s">
         <v>121</v>
       </c>
       <c r="D127" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E127">
         <v>1</v>
@@ -4292,7 +4289,7 @@
         <v>122</v>
       </c>
       <c r="D128" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E128">
         <v>1</v>
@@ -4309,7 +4306,7 @@
         <v>123</v>
       </c>
       <c r="D129" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4326,7 +4323,7 @@
         <v>124</v>
       </c>
       <c r="D130" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4343,7 +4340,7 @@
         <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4360,7 +4357,7 @@
         <v>126</v>
       </c>
       <c r="D132" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4377,7 +4374,7 @@
         <v>127</v>
       </c>
       <c r="D133" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4394,7 +4391,7 @@
         <v>128</v>
       </c>
       <c r="D134" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4411,7 +4408,7 @@
         <v>129</v>
       </c>
       <c r="D135" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4428,7 +4425,7 @@
         <v>130</v>
       </c>
       <c r="D136" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4445,7 +4442,7 @@
         <v>131</v>
       </c>
       <c r="D137" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4462,7 +4459,7 @@
         <v>132</v>
       </c>
       <c r="D138" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4479,7 +4476,7 @@
         <v>133</v>
       </c>
       <c r="D139" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4496,7 +4493,7 @@
         <v>134</v>
       </c>
       <c r="D140" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4513,7 +4510,7 @@
         <v>135</v>
       </c>
       <c r="D141" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4530,7 +4527,7 @@
         <v>136</v>
       </c>
       <c r="D142" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4547,7 +4544,7 @@
         <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4564,7 +4561,7 @@
         <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4581,7 +4578,7 @@
         <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4598,7 +4595,7 @@
         <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4615,7 +4612,7 @@
         <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4632,7 +4629,7 @@
         <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4649,7 +4646,7 @@
         <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4666,7 +4663,7 @@
         <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4683,7 +4680,7 @@
         <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4700,7 +4697,7 @@
         <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4717,7 +4714,7 @@
         <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4734,7 +4731,7 @@
         <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4751,10 +4748,10 @@
         <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>314</v>
+        <v>297</v>
       </c>
       <c r="E155">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -4768,7 +4765,7 @@
         <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="E156">
         <v>2</v>
@@ -4785,7 +4782,7 @@
         <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E157">
         <v>2</v>
@@ -4802,7 +4799,7 @@
         <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -4819,7 +4816,7 @@
         <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E159">
         <v>2</v>
@@ -4836,10 +4833,10 @@
         <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E160">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4853,10 +4850,10 @@
         <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>319</v>
+        <v>282</v>
       </c>
       <c r="E161">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4870,10 +4867,10 @@
         <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>284</v>
+        <v>318</v>
       </c>
       <c r="E162">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4887,7 +4884,7 @@
         <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E163">
         <v>8</v>
@@ -4904,10 +4901,10 @@
         <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E164">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4921,27 +4918,27 @@
         <v>159</v>
       </c>
       <c r="D165" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E165">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C166" t="s">
         <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E166">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -4955,7 +4952,7 @@
         <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -4972,7 +4969,7 @@
         <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -4989,7 +4986,7 @@
         <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -5006,7 +5003,7 @@
         <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5023,7 +5020,7 @@
         <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>328</v>
+        <v>239</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5040,7 +5037,7 @@
         <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>241</v>
+        <v>327</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5057,7 +5054,7 @@
         <v>167</v>
       </c>
       <c r="D173" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5074,7 +5071,7 @@
         <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5091,7 +5088,7 @@
         <v>169</v>
       </c>
       <c r="D175" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5108,7 +5105,7 @@
         <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5125,7 +5122,7 @@
         <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5142,7 +5139,7 @@
         <v>172</v>
       </c>
       <c r="D178" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5159,7 +5156,7 @@
         <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5176,7 +5173,7 @@
         <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5193,7 +5190,7 @@
         <v>175</v>
       </c>
       <c r="D181" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5210,7 +5207,7 @@
         <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5227,7 +5224,7 @@
         <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5244,7 +5241,7 @@
         <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5261,7 +5258,7 @@
         <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5278,7 +5275,7 @@
         <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5295,7 +5292,7 @@
         <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5312,7 +5309,7 @@
         <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5329,7 +5326,7 @@
         <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5346,7 +5343,7 @@
         <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5363,7 +5360,7 @@
         <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5380,7 +5377,7 @@
         <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5397,7 +5394,7 @@
         <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5414,7 +5411,7 @@
         <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>350</v>
+        <v>307</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5431,7 +5428,7 @@
         <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>309</v>
+        <v>349</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5448,7 +5445,7 @@
         <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5465,10 +5462,10 @@
         <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E197">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -5482,7 +5479,7 @@
         <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E198">
         <v>2</v>
@@ -5499,7 +5496,7 @@
         <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>235</v>
+        <v>353</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -5601,7 +5598,7 @@
         <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5672,7 +5669,7 @@
         <v>362</v>
       </c>
       <c r="E209">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5686,7 +5683,7 @@
         <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>363</v>
+        <v>239</v>
       </c>
       <c r="E210">
         <v>3</v>
@@ -5703,10 +5700,10 @@
         <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>241</v>
+        <v>363</v>
       </c>
       <c r="E211">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5791,7 +5788,7 @@
         <v>368</v>
       </c>
       <c r="E216">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5825,7 +5822,7 @@
         <v>370</v>
       </c>
       <c r="E218">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5842,7 +5839,7 @@
         <v>371</v>
       </c>
       <c r="E219">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5859,7 +5856,7 @@
         <v>372</v>
       </c>
       <c r="E220">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5873,7 +5870,7 @@
         <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E221">
         <v>10</v>
@@ -5890,10 +5887,10 @@
         <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>373</v>
+        <v>241</v>
       </c>
       <c r="E222">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5907,7 +5904,7 @@
         <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>243</v>
+        <v>373</v>
       </c>
       <c r="E223">
         <v>12</v>
@@ -5927,7 +5924,7 @@
         <v>374</v>
       </c>
       <c r="E224">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5944,7 +5941,7 @@
         <v>375</v>
       </c>
       <c r="E225">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5961,15 +5958,15 @@
         <v>376</v>
       </c>
       <c r="E226">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B227" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C227" t="s">
         <v>221</v>
@@ -5978,7 +5975,7 @@
         <v>377</v>
       </c>
       <c r="E227">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6012,23 +6009,6 @@
         <v>379</v>
       </c>
       <c r="E229">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="230" spans="1:5">
-      <c r="A230" t="s">
-        <v>8</v>
-      </c>
-      <c r="B230" t="s">
-        <v>38</v>
-      </c>
-      <c r="C230" t="s">
-        <v>224</v>
-      </c>
-      <c r="D230" t="s">
-        <v>380</v>
-      </c>
-      <c r="E230">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (07/08/2026 13:02)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="380">
   <si>
     <t>matricula</t>
   </si>
@@ -194,6 +194,9 @@
     <t>3044000</t>
   </si>
   <si>
+    <t>C662041-0102</t>
+  </si>
+  <si>
     <t>P7036368-01</t>
   </si>
   <si>
@@ -221,6 +224,12 @@
     <t>400454</t>
   </si>
   <si>
+    <t>MS28778-4</t>
+  </si>
+  <si>
+    <t>MS29512-5</t>
+  </si>
+  <si>
     <t>AE3663163K0600</t>
   </si>
   <si>
@@ -245,21 +254,24 @@
     <t>S3461-76</t>
   </si>
   <si>
+    <t>2601102-1</t>
+  </si>
+  <si>
+    <t>NAS147-84</t>
+  </si>
+  <si>
+    <t>F2552-070</t>
+  </si>
+  <si>
     <t>M81934/2-32C032</t>
   </si>
   <si>
     <t>2611137-7</t>
   </si>
   <si>
-    <t>2601102-1</t>
-  </si>
-  <si>
     <t>2622243-11</t>
   </si>
   <si>
-    <t>MS28778-4</t>
-  </si>
-  <si>
     <t>1H75-21</t>
   </si>
   <si>
@@ -281,105 +293,105 @@
     <t>S1053K16T</t>
   </si>
   <si>
+    <t>799-1</t>
+  </si>
+  <si>
+    <t>S1053K24T</t>
+  </si>
+  <si>
+    <t>C352TS</t>
+  </si>
+  <si>
+    <t>AN929-4W</t>
+  </si>
+  <si>
+    <t>2601393-1</t>
+  </si>
+  <si>
+    <t>2601392-1</t>
+  </si>
+  <si>
+    <t>1134380-4</t>
+  </si>
+  <si>
+    <t>CAB-33-02</t>
+  </si>
+  <si>
+    <t>2651022-20-1</t>
+  </si>
+  <si>
+    <t>2601266-2</t>
+  </si>
+  <si>
+    <t>30994-001</t>
+  </si>
+  <si>
+    <t>2601189-11</t>
+  </si>
+  <si>
+    <t>2641018-25</t>
+  </si>
+  <si>
+    <t>2641018-26</t>
+  </si>
+  <si>
+    <t>S2814-2</t>
+  </si>
+  <si>
+    <t>S2574-1</t>
+  </si>
+  <si>
+    <t>2601188-9</t>
+  </si>
+  <si>
+    <t>2622236-6</t>
+  </si>
+  <si>
+    <t>1H101-4</t>
+  </si>
+  <si>
     <t>S2837-1</t>
   </si>
   <si>
-    <t>2601189-11</t>
+    <t>S51-14</t>
+  </si>
+  <si>
+    <t>5211369-8</t>
+  </si>
+  <si>
+    <t>1134380-5</t>
+  </si>
+  <si>
+    <t>5950017-11</t>
+  </si>
+  <si>
+    <t>040-0043</t>
+  </si>
+  <si>
+    <t>1214134-1</t>
   </si>
   <si>
     <t>MICROB MONITOR 2</t>
   </si>
   <si>
+    <t>DLS4-02303</t>
+  </si>
+  <si>
+    <t>DLS4-01786</t>
+  </si>
+  <si>
     <t>42854-11</t>
   </si>
   <si>
-    <t>2651022-20-1</t>
-  </si>
-  <si>
-    <t>799-1</t>
-  </si>
-  <si>
-    <t>S1053K24T</t>
-  </si>
-  <si>
-    <t>C352TS</t>
-  </si>
-  <si>
-    <t>AN929-4W</t>
-  </si>
-  <si>
-    <t>2601393-1</t>
-  </si>
-  <si>
-    <t>2601392-1</t>
-  </si>
-  <si>
-    <t>1134380-4</t>
-  </si>
-  <si>
-    <t>CAB-33-02</t>
-  </si>
-  <si>
-    <t>2601266-2</t>
-  </si>
-  <si>
-    <t>30994-001</t>
-  </si>
-  <si>
-    <t>2641018-25</t>
-  </si>
-  <si>
-    <t>2641018-26</t>
-  </si>
-  <si>
-    <t>S2814-2</t>
-  </si>
-  <si>
-    <t>S2574-1</t>
-  </si>
-  <si>
-    <t>2601188-9</t>
-  </si>
-  <si>
-    <t>2622236-6</t>
-  </si>
-  <si>
-    <t>1H101-4</t>
-  </si>
-  <si>
-    <t>S51-14</t>
-  </si>
-  <si>
-    <t>5211369-8</t>
-  </si>
-  <si>
-    <t>1134380-5</t>
-  </si>
-  <si>
-    <t>5950017-11</t>
-  </si>
-  <si>
-    <t>040-0043</t>
-  </si>
-  <si>
-    <t>1214134-1</t>
-  </si>
-  <si>
-    <t>DLS4-02303</t>
-  </si>
-  <si>
-    <t>DLS4-01786</t>
-  </si>
-  <si>
     <t>A1635-133</t>
   </si>
   <si>
+    <t>1J18-10</t>
+  </si>
+  <si>
     <t>011-00870-00</t>
   </si>
   <si>
-    <t>1J18-10</t>
-  </si>
-  <si>
     <t>MS24392-10</t>
   </si>
   <si>
@@ -590,9 +602,6 @@
     <t>C622010-0102</t>
   </si>
   <si>
-    <t>C662041-0102</t>
-  </si>
-  <si>
     <t>2617015-22</t>
   </si>
   <si>
@@ -680,18 +689,12 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>NAS147-84</t>
-  </si>
-  <si>
-    <t>F2552-070</t>
-  </si>
-  <si>
-    <t>MS29512-5</t>
-  </si>
-  <si>
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
+    <t>INDICATOR FUEL</t>
+  </si>
+  <si>
     <t>PROPELLER ASSEMBLY</t>
   </si>
   <si>
@@ -719,6 +722,12 @@
     <t>SEAL,PLAIN ENCASED</t>
   </si>
   <si>
+    <t>RETAINER-PACKING BACKUP</t>
+  </si>
+  <si>
+    <t>O-RING</t>
+  </si>
+  <si>
     <t>HOSE ASSY</t>
   </si>
   <si>
@@ -743,21 +752,24 @@
     <t>BOLT</t>
   </si>
   <si>
+    <t>HINGE-ASSY-HOISTING</t>
+  </si>
+  <si>
+    <t>BOLT,INTERNAL WRENCHING</t>
+  </si>
+  <si>
+    <t>BARREL NUT</t>
+  </si>
+  <si>
     <t>BEARING,SLEEVE</t>
   </si>
   <si>
     <t>CAP MAIN LAND</t>
   </si>
   <si>
-    <t>HINGE-ASSY-HOISTING</t>
-  </si>
-  <si>
     <t>ECCENTRIC-WING ASSY</t>
   </si>
   <si>
-    <t>RETAINER-PACKING BACKUP</t>
-  </si>
-  <si>
     <t>PRESSURE REGULATOR</t>
   </si>
   <si>
@@ -779,99 +791,99 @@
     <t>HOSE,AIR DUCT</t>
   </si>
   <si>
+    <t>TRANSDUCER</t>
+  </si>
+  <si>
+    <t>EXTINGUISHER,FIRE</t>
+  </si>
+  <si>
+    <t>CAP,TUBE</t>
+  </si>
+  <si>
+    <t>SUPORT PLATE</t>
+  </si>
+  <si>
+    <t>ADJUSTER PLATE</t>
+  </si>
+  <si>
+    <t>EVAPORATOR MODULE AS</t>
+  </si>
+  <si>
+    <t>KIT CAB-33-02</t>
+  </si>
+  <si>
+    <t>RING ASSY ENGI</t>
+  </si>
+  <si>
+    <t>COUPLING-SPLINED</t>
+  </si>
+  <si>
+    <t>BATTERY-MARATHON TSP410 NICAD</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY LH</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY RH</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-DOOR PULL</t>
+  </si>
+  <si>
+    <t>NUT-DIODE ATTACH</t>
+  </si>
+  <si>
+    <t>COMPRESSOR DRIVE ASS</t>
+  </si>
+  <si>
+    <t>COVER ACCESS RH</t>
+  </si>
+  <si>
+    <t>FLOW CONTROL VALVE</t>
+  </si>
+  <si>
     <t>CABLE ASSY-PASSENGER</t>
   </si>
   <si>
-    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
+    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
+  </si>
+  <si>
+    <t>EXTENDER-CREW, (WHEN</t>
+  </si>
+  <si>
+    <t>REDUCER ASSEMBY</t>
+  </si>
+  <si>
+    <t>STROB TUB</t>
+  </si>
+  <si>
+    <t>BELLCRANK ASSY</t>
   </si>
   <si>
     <t>TEST KIT, FUEL, WORK</t>
   </si>
   <si>
+    <t>IMOBILIZADOR</t>
+  </si>
+  <si>
+    <t>BLOQUEIO DA VENTILAÇ</t>
+  </si>
+  <si>
     <t>FITTING A S TR</t>
   </si>
   <si>
-    <t>RING ASSY ENGI</t>
-  </si>
-  <si>
-    <t>TRANSDUCER</t>
-  </si>
-  <si>
-    <t>EXTINGUISHER,FIRE</t>
-  </si>
-  <si>
-    <t>CAP,TUBE</t>
-  </si>
-  <si>
-    <t>SUPORT PLATE</t>
-  </si>
-  <si>
-    <t>ADJUSTER PLATE</t>
-  </si>
-  <si>
-    <t>EVAPORATOR MODULE AS</t>
-  </si>
-  <si>
-    <t>KIT CAB-33-02</t>
-  </si>
-  <si>
-    <t>COUPLING-SPLINED</t>
-  </si>
-  <si>
-    <t>BATTERY-MARATHON TSP410 NICAD</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY LH</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY RH</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-DOOR PULL</t>
-  </si>
-  <si>
-    <t>NUT-DIODE ATTACH</t>
-  </si>
-  <si>
-    <t>COMPRESSOR DRIVE ASS</t>
-  </si>
-  <si>
-    <t>COVER ACCESS RH</t>
-  </si>
-  <si>
-    <t>FLOW CONTROL VALVE</t>
-  </si>
-  <si>
-    <t>HOSE-OVERBOAD OIL BREATHER 12.50 IN</t>
-  </si>
-  <si>
-    <t>EXTENDER-CREW, (WHEN</t>
-  </si>
-  <si>
-    <t>REDUCER ASSEMBY</t>
-  </si>
-  <si>
-    <t>STROB TUB</t>
-  </si>
-  <si>
-    <t>BELLCRANK ASSY</t>
-  </si>
-  <si>
-    <t>IMOBILIZADOR</t>
-  </si>
-  <si>
-    <t>BLOQUEIO DA VENTILAÇ</t>
-  </si>
-  <si>
     <t>SCREW</t>
   </si>
   <si>
+    <t>FUEL FILTER ASSY</t>
+  </si>
+  <si>
     <t>MAGNETOMETER GMU 44</t>
   </si>
   <si>
-    <t>FUEL FILTER ASSY</t>
-  </si>
-  <si>
     <t>NIPPLE,TUBE</t>
   </si>
   <si>
@@ -1070,9 +1082,6 @@
     <t>LIGHT STROBE RH</t>
   </si>
   <si>
-    <t>INDICATOR FUEL</t>
-  </si>
-  <si>
     <t>HINGE-DOOR LH</t>
   </si>
   <si>
@@ -1146,15 +1155,6 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
-  </si>
-  <si>
-    <t>BOLT,INTERNAL WRENCHING</t>
-  </si>
-  <si>
-    <t>BARREL NUT</t>
-  </si>
-  <si>
-    <t>O-RING</t>
   </si>
 </sst>
 </file>
@@ -1523,10 +1523,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2116,7 +2116,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E230"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2240,10 +2240,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>59</v>
@@ -2252,15 +2252,15 @@
         <v>225</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>59</v>
@@ -2269,21 +2269,21 @@
         <v>225</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2291,16 +2291,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2308,16 +2308,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2325,16 +2325,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2342,10 +2342,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>60</v>
@@ -2359,10 +2359,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
         <v>60</v>
@@ -2376,16 +2376,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2393,16 +2393,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2410,10 +2410,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
         <v>61</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
@@ -2444,16 +2444,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2461,10 +2461,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>62</v>
@@ -2495,16 +2495,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2512,10 +2512,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
         <v>63</v>
@@ -2541,7 +2541,7 @@
         <v>229</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2563,19 +2563,19 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2586,10 +2586,10 @@
         <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2603,10 +2603,10 @@
         <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2620,21 +2620,21 @@
         <v>38</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
         <v>68</v>
@@ -2643,41 +2643,41 @@
         <v>234</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2688,10 +2688,10 @@
         <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2699,50 +2699,50 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
         <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2750,33 +2750,33 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2784,61 +2784,61 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
         <v>73</v>
@@ -2869,19 +2869,19 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2892,21 +2892,21 @@
         <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E46">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C47" t="s">
         <v>76</v>
@@ -2915,7 +2915,7 @@
         <v>242</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2932,7 +2932,7 @@
         <v>243</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2966,7 +2966,7 @@
         <v>245</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2983,15 +2983,15 @@
         <v>246</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
         <v>81</v>
@@ -3000,89 +3000,89 @@
         <v>247</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B53" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B55" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B56" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D56" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E56">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D57" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3090,16 +3090,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D58" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3113,10 +3113,10 @@
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D59" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3130,10 +3130,10 @@
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D60" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3141,16 +3141,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D61" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3158,36 +3158,36 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D62" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D63" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3198,61 +3198,61 @@
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D64" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B65" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
         <v>39</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E66">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
       </c>
       <c r="C67" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3260,16 +3260,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D68" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3277,16 +3277,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D69" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3294,16 +3294,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D70" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3311,50 +3311,50 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D71" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C72" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
         <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D73" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3362,16 +3362,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B74" t="s">
         <v>39</v>
       </c>
       <c r="C74" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D74" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3379,16 +3379,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D75" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3396,78 +3396,78 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
         <v>39</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D76" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D77" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D78" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E78">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E79">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
         <v>92</v>
@@ -3481,16 +3481,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D81" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3498,7 +3498,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
@@ -3507,7 +3507,7 @@
         <v>93</v>
       </c>
       <c r="D82" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3515,30 +3515,30 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
         <v>93</v>
       </c>
       <c r="D83" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D84" t="s">
         <v>259</v>
@@ -3549,7 +3549,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
@@ -3558,7 +3558,7 @@
         <v>94</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3566,16 +3566,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D86" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3583,19 +3583,19 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B87" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D87" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3606,10 +3606,10 @@
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D88" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3623,10 +3623,10 @@
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D89" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3640,10 +3640,10 @@
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D90" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3657,10 +3657,10 @@
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D91" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3674,10 +3674,10 @@
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D92" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3691,10 +3691,10 @@
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D93" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3708,10 +3708,10 @@
         <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D94" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3725,10 +3725,10 @@
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D95" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3742,10 +3742,10 @@
         <v>39</v>
       </c>
       <c r="C96" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D96" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3753,16 +3753,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D97" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3776,10 +3776,10 @@
         <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D98" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3787,16 +3787,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C99" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D99" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3810,10 +3810,10 @@
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D100" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3827,10 +3827,10 @@
         <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D101" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3844,10 +3844,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D102" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3855,16 +3855,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B103" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3878,10 +3878,10 @@
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D104" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3895,10 +3895,10 @@
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D105" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3912,10 +3912,10 @@
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D106" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3929,10 +3929,10 @@
         <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D107" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3946,10 +3946,10 @@
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D108" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3963,61 +3963,61 @@
         <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D109" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
       </c>
       <c r="C110" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D110" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D111" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4025,16 +4025,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D113" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4048,10 +4048,10 @@
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D114" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4065,13 +4065,13 @@
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D115" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E115">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -4082,10 +4082,10 @@
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D116" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4093,7 +4093,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4102,10 +4102,10 @@
         <v>113</v>
       </c>
       <c r="D117" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -4119,7 +4119,7 @@
         <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4139,7 +4139,7 @@
         <v>279</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4156,7 +4156,7 @@
         <v>280</v>
       </c>
       <c r="E120">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4173,7 +4173,7 @@
         <v>281</v>
       </c>
       <c r="E121">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4190,7 +4190,7 @@
         <v>282</v>
       </c>
       <c r="E122">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4207,12 +4207,12 @@
         <v>282</v>
       </c>
       <c r="E123">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
@@ -4224,12 +4224,12 @@
         <v>283</v>
       </c>
       <c r="E124">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
@@ -4241,41 +4241,41 @@
         <v>284</v>
       </c>
       <c r="E125">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B126" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D126" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E126">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D127" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E127">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -4292,7 +4292,7 @@
         <v>286</v>
       </c>
       <c r="E128">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -4314,16 +4314,16 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B130" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D130" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4337,10 +4337,10 @@
         <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D131" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4354,10 +4354,10 @@
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4371,10 +4371,10 @@
         <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D133" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4388,10 +4388,10 @@
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D134" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4405,10 +4405,10 @@
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D135" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4422,10 +4422,10 @@
         <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D136" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4439,10 +4439,10 @@
         <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D137" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4456,10 +4456,10 @@
         <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D138" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4473,10 +4473,10 @@
         <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D139" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4490,10 +4490,10 @@
         <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D140" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4507,10 +4507,10 @@
         <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D141" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4524,10 +4524,10 @@
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D142" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4541,10 +4541,10 @@
         <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D143" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4558,10 +4558,10 @@
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D144" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4575,10 +4575,10 @@
         <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D145" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4592,10 +4592,10 @@
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D146" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4609,10 +4609,10 @@
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D147" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4626,10 +4626,10 @@
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D148" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4643,10 +4643,10 @@
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D149" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4660,10 +4660,10 @@
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D150" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4677,10 +4677,10 @@
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D151" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4694,10 +4694,10 @@
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4711,10 +4711,10 @@
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4728,10 +4728,10 @@
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4745,13 +4745,13 @@
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="E155">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -4762,13 +4762,13 @@
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D156" t="s">
         <v>313</v>
       </c>
       <c r="E156">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -4779,13 +4779,13 @@
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D157" t="s">
         <v>314</v>
       </c>
       <c r="E157">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -4796,13 +4796,13 @@
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D158" t="s">
         <v>315</v>
       </c>
       <c r="E158">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -4813,13 +4813,13 @@
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D159" t="s">
         <v>316</v>
       </c>
       <c r="E159">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4830,13 +4830,13 @@
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>301</v>
       </c>
       <c r="E160">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4847,13 +4847,13 @@
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D161" t="s">
-        <v>282</v>
+        <v>317</v>
       </c>
       <c r="E161">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4864,13 +4864,13 @@
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D162" t="s">
         <v>318</v>
       </c>
       <c r="E162">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4881,13 +4881,13 @@
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D163" t="s">
         <v>319</v>
       </c>
       <c r="E163">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4898,13 +4898,13 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D164" t="s">
         <v>320</v>
       </c>
       <c r="E164">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4915,98 +4915,98 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D165" t="s">
         <v>321</v>
       </c>
       <c r="E165">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B166" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>322</v>
+        <v>286</v>
       </c>
       <c r="E166">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B167" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E167">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B168" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E168">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B169" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E169">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B170" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D170" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E170">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5017,10 +5017,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D171" t="s">
-        <v>239</v>
+        <v>326</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5034,7 +5034,7 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D172" t="s">
         <v>327</v>
@@ -5051,7 +5051,7 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D173" t="s">
         <v>328</v>
@@ -5068,7 +5068,7 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D174" t="s">
         <v>329</v>
@@ -5085,7 +5085,7 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D175" t="s">
         <v>330</v>
@@ -5102,10 +5102,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D176" t="s">
-        <v>331</v>
+        <v>242</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5119,10 +5119,10 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D177" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5136,10 +5136,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D178" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5153,10 +5153,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D179" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5170,10 +5170,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D180" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5187,10 +5187,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D181" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5204,10 +5204,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D182" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5221,10 +5221,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D183" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5238,10 +5238,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D184" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5255,10 +5255,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D185" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5272,10 +5272,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D186" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5289,10 +5289,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D187" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5306,10 +5306,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D188" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5323,10 +5323,10 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D189" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5340,10 +5340,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D190" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5357,10 +5357,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D191" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5374,10 +5374,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D192" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5391,10 +5391,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D193" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5408,10 +5408,10 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D194" t="s">
-        <v>307</v>
+        <v>348</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5425,7 +5425,7 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D195" t="s">
         <v>349</v>
@@ -5442,7 +5442,7 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D196" t="s">
         <v>350</v>
@@ -5459,13 +5459,13 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D197" t="s">
         <v>351</v>
       </c>
       <c r="E197">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -5476,13 +5476,13 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D198" t="s">
         <v>352</v>
       </c>
       <c r="E198">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -5493,13 +5493,13 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D199" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="E199">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -5510,13 +5510,13 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D200" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E200">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -5527,13 +5527,13 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D201" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E201">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5544,10 +5544,10 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D202" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5561,10 +5561,10 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D203" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5578,10 +5578,10 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D204" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5595,7 +5595,7 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D205" t="s">
         <v>358</v>
@@ -5612,7 +5612,7 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D206" t="s">
         <v>359</v>
@@ -5629,7 +5629,7 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D207" t="s">
         <v>360</v>
@@ -5646,7 +5646,7 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D208" t="s">
         <v>361</v>
@@ -5663,13 +5663,13 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D209" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E209">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5680,13 +5680,13 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D210" t="s">
-        <v>239</v>
+        <v>362</v>
       </c>
       <c r="E210">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5697,13 +5697,13 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D211" t="s">
         <v>363</v>
       </c>
       <c r="E211">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5714,13 +5714,13 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D212" t="s">
         <v>364</v>
       </c>
       <c r="E212">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5731,13 +5731,13 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D213" t="s">
         <v>365</v>
       </c>
       <c r="E213">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5748,13 +5748,13 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D214" t="s">
-        <v>366</v>
+        <v>242</v>
       </c>
       <c r="E214">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5765,10 +5765,10 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D215" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5782,13 +5782,13 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D216" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E216">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5799,13 +5799,13 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D217" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E217">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5816,13 +5816,13 @@
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D218" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E218">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5833,13 +5833,13 @@
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D219" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E219">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5850,13 +5850,13 @@
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E220">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5867,13 +5867,13 @@
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D221" t="s">
         <v>372</v>
       </c>
       <c r="E221">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5884,13 +5884,13 @@
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D222" t="s">
-        <v>241</v>
+        <v>373</v>
       </c>
       <c r="E222">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5901,13 +5901,13 @@
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D223" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E223">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5918,13 +5918,13 @@
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D224" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E224">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5935,13 +5935,13 @@
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D225" t="s">
         <v>375</v>
       </c>
       <c r="E225">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5952,64 +5952,81 @@
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D226" t="s">
-        <v>376</v>
+        <v>244</v>
       </c>
       <c r="E226">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B227" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D227" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E227">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D228" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E228">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B229" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C229" t="s">
+        <v>222</v>
+      </c>
+      <c r="D229" t="s">
+        <v>378</v>
+      </c>
+      <c r="E229">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
+      <c r="A230" t="s">
+        <v>12</v>
+      </c>
+      <c r="B230" t="s">
+        <v>40</v>
+      </c>
+      <c r="C230" t="s">
         <v>223</v>
       </c>
-      <c r="D229" t="s">
+      <c r="D230" t="s">
         <v>379</v>
       </c>
-      <c r="E229">
-        <v>1</v>
+      <c r="E230">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (10/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1626,7 +1626,7 @@
         <v>70</v>
       </c>
       <c r="F7">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1646,7 +1646,7 @@
         <v>79</v>
       </c>
       <c r="F8">
-        <v>228</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -4309,7 +4309,7 @@
         <v>287</v>
       </c>
       <c r="E129">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -5720,7 +5720,7 @@
         <v>364</v>
       </c>
       <c r="E212">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5754,7 +5754,7 @@
         <v>242</v>
       </c>
       <c r="E214">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5873,7 +5873,7 @@
         <v>372</v>
       </c>
       <c r="E221">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="222" spans="1:5">

</xml_diff>

<commit_message>
Atualização automática: rac (10/08/2026 13:05)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="382">
   <si>
     <t>matricula</t>
   </si>
@@ -41,6 +41,9 @@
     <t>2731</t>
   </si>
   <si>
+    <t>2729</t>
+  </si>
+  <si>
     <t>2728</t>
   </si>
   <si>
@@ -86,9 +89,6 @@
     <t>2727</t>
   </si>
   <si>
-    <t>2729</t>
-  </si>
-  <si>
     <t>2733</t>
   </si>
   <si>
@@ -200,6 +200,9 @@
     <t>P7036368-01</t>
   </si>
   <si>
+    <t>2641010-3</t>
+  </si>
+  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -696,6 +699,9 @@
   </si>
   <si>
     <t>PROPELLER ASSEMBLY</t>
+  </si>
+  <si>
+    <t>AXLE FITTING</t>
   </si>
   <si>
     <t>ALTERNATOR</t>
@@ -1563,10 +1569,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>46</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1574,19 +1580,19 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1603,10 +1609,10 @@
         <v>54</v>
       </c>
       <c r="E6">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>111</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1623,10 +1629,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="F7">
-        <v>167</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1634,7 +1640,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1643,10 +1649,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="F8">
-        <v>238</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1654,19 +1660,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1674,7 +1680,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>51</v>
@@ -1694,7 +1700,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
         <v>51</v>
@@ -1714,7 +1720,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1734,7 +1740,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1754,7 +1760,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1774,7 +1780,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1794,7 +1800,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1814,7 +1820,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1834,7 +1840,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1854,7 +1860,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -2147,7 +2153,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2155,7 +2161,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
@@ -2164,7 +2170,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2172,7 +2178,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>39</v>
@@ -2181,7 +2187,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2189,7 +2195,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
         <v>39</v>
@@ -2198,7 +2204,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2206,7 +2212,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
@@ -2215,7 +2221,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2223,7 +2229,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -2232,7 +2238,7 @@
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2249,7 +2255,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -2257,7 +2263,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
         <v>40</v>
@@ -2266,7 +2272,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -2283,7 +2289,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2291,7 +2297,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
@@ -2300,7 +2306,7 @@
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2308,7 +2314,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
@@ -2317,7 +2323,7 @@
         <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2325,7 +2331,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
@@ -2334,7 +2340,7 @@
         <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2342,7 +2348,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
@@ -2351,7 +2357,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2359,7 +2365,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>40</v>
@@ -2368,7 +2374,7 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2385,7 +2391,7 @@
         <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2396,13 +2402,13 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2416,10 +2422,10 @@
         <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2433,10 +2439,10 @@
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2444,16 +2450,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2461,16 +2467,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2484,10 +2490,10 @@
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2495,16 +2501,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
         <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2512,16 +2518,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2532,13 +2538,13 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D25" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2546,16 +2552,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
         <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2563,41 +2569,41 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C28" t="s">
         <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
@@ -2606,7 +2612,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2614,7 +2620,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
         <v>38</v>
@@ -2623,7 +2629,7 @@
         <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2631,7 +2637,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
@@ -2640,7 +2646,7 @@
         <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2648,7 +2654,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32" t="s">
         <v>38</v>
@@ -2657,7 +2663,7 @@
         <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2665,7 +2671,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" t="s">
         <v>38</v>
@@ -2674,7 +2680,7 @@
         <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2682,7 +2688,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
@@ -2691,27 +2697,27 @@
         <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D35" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E35">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2722,13 +2728,13 @@
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2736,13 +2742,13 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2750,16 +2756,16 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -2767,16 +2773,16 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2787,50 +2793,50 @@
         <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C41" t="s">
         <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E42">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2838,30 +2844,30 @@
         <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2869,41 +2875,41 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
         <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B47" t="s">
         <v>38</v>
@@ -2912,7 +2918,7 @@
         <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2920,7 +2926,7 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B48" t="s">
         <v>38</v>
@@ -2929,7 +2935,7 @@
         <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2937,7 +2943,7 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B49" t="s">
         <v>38</v>
@@ -2946,7 +2952,7 @@
         <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2954,7 +2960,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B50" t="s">
         <v>38</v>
@@ -2963,7 +2969,7 @@
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -2971,7 +2977,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B51" t="s">
         <v>38</v>
@@ -2980,7 +2986,7 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -2988,7 +2994,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B52" t="s">
         <v>38</v>
@@ -2997,7 +3003,7 @@
         <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3005,7 +3011,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
@@ -3014,24 +3020,24 @@
         <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B54" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E54">
         <v>4</v>
@@ -3039,16 +3045,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E55">
         <v>4</v>
@@ -3056,7 +3062,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B56" t="s">
         <v>38</v>
@@ -3065,7 +3071,7 @@
         <v>84</v>
       </c>
       <c r="D56" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E56">
         <v>4</v>
@@ -3076,16 +3082,16 @@
         <v>9</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C57" t="s">
         <v>85</v>
       </c>
       <c r="D57" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3096,10 +3102,10 @@
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D58" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3113,10 +3119,10 @@
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3124,7 +3130,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
         <v>39</v>
@@ -3133,7 +3139,7 @@
         <v>86</v>
       </c>
       <c r="D60" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3147,10 +3153,10 @@
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D61" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3164,10 +3170,10 @@
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D62" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3175,7 +3181,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
@@ -3184,7 +3190,7 @@
         <v>87</v>
       </c>
       <c r="D63" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3192,16 +3198,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D64" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3209,7 +3215,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
@@ -3218,7 +3224,7 @@
         <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3226,16 +3232,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B66" t="s">
         <v>39</v>
       </c>
       <c r="C66" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D66" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3243,7 +3249,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
@@ -3252,24 +3258,24 @@
         <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3277,16 +3283,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3294,16 +3300,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B70" t="s">
         <v>40</v>
       </c>
       <c r="C70" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3311,16 +3317,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D71" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3328,16 +3334,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
         <v>39</v>
       </c>
       <c r="C72" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D72" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3345,16 +3351,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
         <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D73" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3362,16 +3368,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B74" t="s">
         <v>39</v>
       </c>
       <c r="C74" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D74" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3379,16 +3385,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
         <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D75" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3396,16 +3402,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
         <v>39</v>
       </c>
       <c r="C76" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D76" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3413,16 +3419,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B77" t="s">
         <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D77" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E77">
         <v>4</v>
@@ -3430,16 +3436,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D78" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3447,16 +3453,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D79" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3464,16 +3470,16 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B80" t="s">
         <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D80" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3481,16 +3487,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
         <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D81" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3498,16 +3504,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
       </c>
       <c r="C82" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D82" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3515,16 +3521,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B83" t="s">
         <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E83">
         <v>2</v>
@@ -3532,16 +3538,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D84" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3549,16 +3555,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D85" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3566,16 +3572,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D86" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3583,16 +3589,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3600,16 +3606,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D88" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3617,16 +3623,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D89" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3634,16 +3640,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D90" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3651,16 +3657,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D91" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3668,16 +3674,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D92" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3685,16 +3691,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D93" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3702,16 +3708,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D94" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3719,16 +3725,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D95" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3736,16 +3742,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
       </c>
       <c r="C96" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D96" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3753,16 +3759,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B97" t="s">
         <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D97" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3770,16 +3776,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B98" t="s">
         <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D98" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3787,16 +3793,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
         <v>40</v>
       </c>
       <c r="C99" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D99" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3804,16 +3810,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D100" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3821,16 +3827,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B101" t="s">
         <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D101" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3838,16 +3844,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B102" t="s">
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D102" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3855,16 +3861,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B103" t="s">
         <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D103" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3872,16 +3878,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D104" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3889,16 +3895,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B105" t="s">
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D105" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3906,16 +3912,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D106" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3923,16 +3929,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D107" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3940,16 +3946,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D108" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3957,16 +3963,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D109" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -3974,16 +3980,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
       </c>
       <c r="C110" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D110" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -3991,16 +3997,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D111" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4008,16 +4014,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D112" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4025,16 +4031,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
         <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D113" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4042,16 +4048,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D114" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4059,16 +4065,16 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D115" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4076,16 +4082,16 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D116" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4093,16 +4099,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
       </c>
       <c r="C117" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E117">
         <v>4</v>
@@ -4110,16 +4116,16 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D118" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4127,16 +4133,16 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D119" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4144,16 +4150,16 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B120" t="s">
         <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D120" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4161,16 +4167,16 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B121" t="s">
         <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D121" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E121">
         <v>4</v>
@@ -4178,16 +4184,16 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D122" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E122">
         <v>5</v>
@@ -4195,16 +4201,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D123" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E123">
         <v>5</v>
@@ -4212,16 +4218,16 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D124" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E124">
         <v>7</v>
@@ -4229,16 +4235,16 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
       </c>
       <c r="C125" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D125" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E125">
         <v>8</v>
@@ -4246,16 +4252,16 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B126" t="s">
         <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D126" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E126">
         <v>10</v>
@@ -4263,16 +4269,16 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D127" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E127">
         <v>30</v>
@@ -4280,16 +4286,16 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B128" t="s">
         <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D128" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E128">
         <v>30</v>
@@ -4297,33 +4303,33 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B129" t="s">
         <v>39</v>
       </c>
       <c r="C129" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D129" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E129">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
         <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D130" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4331,16 +4337,16 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4348,16 +4354,16 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B132" t="s">
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D132" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4365,16 +4371,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B133" t="s">
         <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D133" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4382,16 +4388,16 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B134" t="s">
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D134" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4399,16 +4405,16 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B135" t="s">
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D135" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4416,16 +4422,16 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B136" t="s">
         <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D136" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4433,16 +4439,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B137" t="s">
         <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D137" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4450,16 +4456,16 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B138" t="s">
         <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D138" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4467,16 +4473,16 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B139" t="s">
         <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D139" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4484,16 +4490,16 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B140" t="s">
         <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D140" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4501,16 +4507,16 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B141" t="s">
         <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D141" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4518,16 +4524,16 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B142" t="s">
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D142" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4535,16 +4541,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B143" t="s">
         <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4552,16 +4558,16 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B144" t="s">
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4569,16 +4575,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B145" t="s">
         <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4586,16 +4592,16 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B146" t="s">
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4603,16 +4609,16 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B147" t="s">
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4620,16 +4626,16 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B148" t="s">
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4637,16 +4643,16 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B149" t="s">
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4654,16 +4660,16 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B150" t="s">
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4671,16 +4677,16 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B151" t="s">
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4688,16 +4694,16 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B152" t="s">
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4705,16 +4711,16 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B153" t="s">
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4722,16 +4728,16 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B154" t="s">
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4739,16 +4745,16 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B155" t="s">
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4756,16 +4762,16 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B156" t="s">
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4773,16 +4779,16 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B157" t="s">
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4790,16 +4796,16 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B158" t="s">
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4807,16 +4813,16 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B159" t="s">
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4824,16 +4830,16 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B160" t="s">
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E160">
         <v>2</v>
@@ -4841,16 +4847,16 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B161" t="s">
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E161">
         <v>2</v>
@@ -4858,16 +4864,16 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B162" t="s">
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4875,16 +4881,16 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B163" t="s">
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4892,16 +4898,16 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B164" t="s">
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E164">
         <v>2</v>
@@ -4909,16 +4915,16 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B165" t="s">
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D165" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E165">
         <v>3</v>
@@ -4926,16 +4932,16 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B166" t="s">
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E166">
         <v>5</v>
@@ -4943,16 +4949,16 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B167" t="s">
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E167">
         <v>8</v>
@@ -4960,16 +4966,16 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B168" t="s">
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E168">
         <v>8</v>
@@ -4977,16 +4983,16 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B169" t="s">
         <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E169">
         <v>10</v>
@@ -4994,16 +5000,16 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B170" t="s">
         <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E170">
         <v>15</v>
@@ -5011,16 +5017,16 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B171" t="s">
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5028,16 +5034,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B172" t="s">
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5045,16 +5051,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B173" t="s">
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D173" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5062,16 +5068,16 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B174" t="s">
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5079,16 +5085,16 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B175" t="s">
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D175" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5096,16 +5102,16 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B176" t="s">
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5113,16 +5119,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B177" t="s">
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5130,16 +5136,16 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B178" t="s">
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D178" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5147,16 +5153,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B179" t="s">
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5164,16 +5170,16 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B180" t="s">
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5181,16 +5187,16 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B181" t="s">
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D181" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5198,16 +5204,16 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B182" t="s">
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5215,16 +5221,16 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B183" t="s">
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5232,16 +5238,16 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B184" t="s">
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5249,16 +5255,16 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B185" t="s">
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5266,16 +5272,16 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B186" t="s">
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5283,16 +5289,16 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B187" t="s">
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5300,16 +5306,16 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B188" t="s">
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5317,16 +5323,16 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B189" t="s">
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5334,16 +5340,16 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B190" t="s">
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5351,16 +5357,16 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B191" t="s">
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5368,16 +5374,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B192" t="s">
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5385,16 +5391,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B193" t="s">
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5402,16 +5408,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B194" t="s">
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5419,16 +5425,16 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B195" t="s">
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5436,16 +5442,16 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B196" t="s">
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5453,16 +5459,16 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B197" t="s">
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5470,16 +5476,16 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B198" t="s">
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5487,16 +5493,16 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B199" t="s">
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5504,16 +5510,16 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B200" t="s">
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D200" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5521,16 +5527,16 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B201" t="s">
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D201" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5538,16 +5544,16 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B202" t="s">
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D202" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5555,16 +5561,16 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B203" t="s">
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5572,16 +5578,16 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B204" t="s">
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5589,16 +5595,16 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B205" t="s">
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5606,16 +5612,16 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B206" t="s">
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D206" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5623,16 +5629,16 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B207" t="s">
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D207" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5640,16 +5646,16 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B208" t="s">
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5657,16 +5663,16 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B209" t="s">
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5674,16 +5680,16 @@
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B210" t="s">
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5691,16 +5697,16 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B211" t="s">
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5708,33 +5714,33 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B212" t="s">
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D212" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E212">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B213" t="s">
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D213" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E213">
         <v>3</v>
@@ -5742,33 +5748,33 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B214" t="s">
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D214" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E214">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B215" t="s">
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D215" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5776,16 +5782,16 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B216" t="s">
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D216" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E216">
         <v>4</v>
@@ -5793,16 +5799,16 @@
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B217" t="s">
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D217" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E217">
         <v>4</v>
@@ -5810,16 +5816,16 @@
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B218" t="s">
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D218" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -5827,16 +5833,16 @@
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B219" t="s">
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E219">
         <v>4</v>
@@ -5844,16 +5850,16 @@
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B220" t="s">
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D220" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E220">
         <v>5</v>
@@ -5861,33 +5867,33 @@
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B221" t="s">
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E221">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B222" t="s">
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E222">
         <v>6</v>
@@ -5895,16 +5901,16 @@
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B223" t="s">
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E223">
         <v>8</v>
@@ -5912,16 +5918,16 @@
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B224" t="s">
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D224" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E224">
         <v>10</v>
@@ -5929,16 +5935,16 @@
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B225" t="s">
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D225" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E225">
         <v>10</v>
@@ -5946,16 +5952,16 @@
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B226" t="s">
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D226" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E226">
         <v>12</v>
@@ -5963,16 +5969,16 @@
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B227" t="s">
         <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D227" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E227">
         <v>12</v>
@@ -5980,16 +5986,16 @@
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B228" t="s">
         <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D228" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E228">
         <v>14</v>
@@ -5997,16 +6003,16 @@
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B229" t="s">
         <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D229" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E229">
         <v>15</v>
@@ -6014,16 +6020,16 @@
     </row>
     <row r="230" spans="1:5">
       <c r="A230" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B230" t="s">
         <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D230" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E230">
         <v>20</v>

</xml_diff>

<commit_message>
Atualização automática: rac (10/08/2026 14:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -287,72 +287,72 @@
     <t>S1053K22T144.00</t>
   </si>
   <si>
+    <t>2115040-8</t>
+  </si>
+  <si>
+    <t>S1053K16T</t>
+  </si>
+  <si>
+    <t>799-1</t>
+  </si>
+  <si>
+    <t>S1053K24T</t>
+  </si>
+  <si>
+    <t>C352TS</t>
+  </si>
+  <si>
+    <t>AN929-4W</t>
+  </si>
+  <si>
+    <t>2601393-1</t>
+  </si>
+  <si>
+    <t>2601392-1</t>
+  </si>
+  <si>
+    <t>1134380-4</t>
+  </si>
+  <si>
+    <t>CAB-33-02</t>
+  </si>
+  <si>
+    <t>2651022-20-1</t>
+  </si>
+  <si>
+    <t>2601266-2</t>
+  </si>
+  <si>
+    <t>30994-001</t>
+  </si>
+  <si>
+    <t>2601189-11</t>
+  </si>
+  <si>
+    <t>2641018-25</t>
+  </si>
+  <si>
+    <t>2641018-26</t>
+  </si>
+  <si>
+    <t>S2814-2</t>
+  </si>
+  <si>
+    <t>S2574-1</t>
+  </si>
+  <si>
+    <t>2601188-9</t>
+  </si>
+  <si>
+    <t>2622236-6</t>
+  </si>
+  <si>
+    <t>1H101-4</t>
+  </si>
+  <si>
     <t>030-18200</t>
   </si>
   <si>
-    <t>2115040-8</t>
-  </si>
-  <si>
-    <t>S1053K16T</t>
-  </si>
-  <si>
-    <t>799-1</t>
-  </si>
-  <si>
-    <t>S1053K24T</t>
-  </si>
-  <si>
-    <t>C352TS</t>
-  </si>
-  <si>
-    <t>AN929-4W</t>
-  </si>
-  <si>
-    <t>2601393-1</t>
-  </si>
-  <si>
-    <t>2601392-1</t>
-  </si>
-  <si>
-    <t>1134380-4</t>
-  </si>
-  <si>
-    <t>CAB-33-02</t>
-  </si>
-  <si>
-    <t>2651022-20-1</t>
-  </si>
-  <si>
-    <t>2601266-2</t>
-  </si>
-  <si>
-    <t>30994-001</t>
-  </si>
-  <si>
-    <t>2601189-11</t>
-  </si>
-  <si>
-    <t>2641018-25</t>
-  </si>
-  <si>
-    <t>2641018-26</t>
-  </si>
-  <si>
-    <t>S2814-2</t>
-  </si>
-  <si>
-    <t>S2574-1</t>
-  </si>
-  <si>
-    <t>2601188-9</t>
-  </si>
-  <si>
-    <t>2622236-6</t>
-  </si>
-  <si>
-    <t>1H101-4</t>
-  </si>
-  <si>
     <t>S2837-1</t>
   </si>
   <si>
@@ -788,67 +788,67 @@
     <t>HOSE,AIR DUCT, INSIDE DIA, 2-3/4 IN, LENGTH, 144 IN, MATERIAL FIBERGLASS, RUBBER BUTYL AND SILICONE</t>
   </si>
   <si>
+    <t>CYLINDER GAS S</t>
+  </si>
+  <si>
+    <t>HOSE,AIR DUCT</t>
+  </si>
+  <si>
+    <t>TRANSDUCER</t>
+  </si>
+  <si>
+    <t>EXTINGUISHER,FIRE</t>
+  </si>
+  <si>
+    <t>CAP,TUBE</t>
+  </si>
+  <si>
+    <t>SUPORT PLATE</t>
+  </si>
+  <si>
+    <t>ADJUSTER PLATE</t>
+  </si>
+  <si>
+    <t>EVAPORATOR MODULE AS</t>
+  </si>
+  <si>
+    <t>KIT CAB-33-02</t>
+  </si>
+  <si>
+    <t>RING ASSY ENGI</t>
+  </si>
+  <si>
+    <t>COUPLING-SPLINED</t>
+  </si>
+  <si>
+    <t>BATTERY-MARATHON TSP410 NICAD</t>
+  </si>
+  <si>
+    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY LH</t>
+  </si>
+  <si>
+    <t>FAIRING ASSY RH</t>
+  </si>
+  <si>
+    <t>CABLE ASSY-DOOR PULL</t>
+  </si>
+  <si>
+    <t>NUT-DIODE ATTACH</t>
+  </si>
+  <si>
+    <t>COMPRESSOR DRIVE ASS</t>
+  </si>
+  <si>
+    <t>COVER ACCESS RH</t>
+  </si>
+  <si>
+    <t>FLOW CONTROL VALVE</t>
+  </si>
+  <si>
     <t>MAIN WHEEL BRAKE</t>
-  </si>
-  <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
-    <t>HOSE,AIR DUCT</t>
-  </si>
-  <si>
-    <t>TRANSDUCER</t>
-  </si>
-  <si>
-    <t>EXTINGUISHER,FIRE</t>
-  </si>
-  <si>
-    <t>CAP,TUBE</t>
-  </si>
-  <si>
-    <t>SUPORT PLATE</t>
-  </si>
-  <si>
-    <t>ADJUSTER PLATE</t>
-  </si>
-  <si>
-    <t>EVAPORATOR MODULE AS</t>
-  </si>
-  <si>
-    <t>KIT CAB-33-02</t>
-  </si>
-  <si>
-    <t>RING ASSY ENGI</t>
-  </si>
-  <si>
-    <t>COUPLING-SPLINED</t>
-  </si>
-  <si>
-    <t>BATTERY-MARATHON TSP410 NICAD</t>
-  </si>
-  <si>
-    <t>SUPPORT ASSY COMPRESSOR DRIVE</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY LH</t>
-  </si>
-  <si>
-    <t>FAIRING ASSY RH</t>
-  </si>
-  <si>
-    <t>CABLE ASSY-DOOR PULL</t>
-  </si>
-  <si>
-    <t>NUT-DIODE ATTACH</t>
-  </si>
-  <si>
-    <t>COMPRESSOR DRIVE ASS</t>
-  </si>
-  <si>
-    <t>COVER ACCESS RH</t>
-  </si>
-  <si>
-    <t>FLOW CONTROL VALVE</t>
   </si>
   <si>
     <t>CABLE ASSY-PASSENGER</t>
@@ -3266,7 +3266,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
@@ -3283,7 +3283,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
@@ -3300,10 +3300,10 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C70" t="s">
         <v>90</v>
@@ -3363,24 +3363,24 @@
         <v>258</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B74" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D74" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3397,7 +3397,7 @@
         <v>259</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3414,7 +3414,7 @@
         <v>259</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3431,7 +3431,7 @@
         <v>259</v>
       </c>
       <c r="E77">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3445,7 +3445,7 @@
         <v>93</v>
       </c>
       <c r="D78" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3462,7 +3462,7 @@
         <v>93</v>
       </c>
       <c r="D79" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3479,10 +3479,10 @@
         <v>93</v>
       </c>
       <c r="D80" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3496,7 +3496,7 @@
         <v>94</v>
       </c>
       <c r="D81" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3513,7 +3513,7 @@
         <v>94</v>
       </c>
       <c r="D82" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3521,24 +3521,24 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B83" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D83" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
@@ -3555,16 +3555,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D85" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3572,7 +3572,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
@@ -3589,16 +3589,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D87" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3606,7 +3606,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
@@ -3623,16 +3623,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D89" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3640,7 +3640,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
@@ -3657,16 +3657,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D91" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3674,7 +3674,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
@@ -3691,16 +3691,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D93" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3708,10 +3708,10 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C94" t="s">
         <v>100</v>
@@ -3725,16 +3725,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D95" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3742,10 +3742,10 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C96" t="s">
         <v>101</v>
@@ -3759,16 +3759,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B97" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D97" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3776,10 +3776,10 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C98" t="s">
         <v>102</v>
@@ -3793,16 +3793,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B99" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D99" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3816,10 +3816,10 @@
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D100" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3827,16 +3827,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B101" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D101" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3850,10 +3850,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D102" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3867,10 +3867,10 @@
         <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D103" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3884,10 +3884,10 @@
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D104" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3901,10 +3901,10 @@
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D105" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3918,27 +3918,27 @@
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D106" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D107" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3952,18 +3952,18 @@
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D108" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
@@ -3980,10 +3980,10 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C110" t="s">
         <v>111</v>
@@ -3992,7 +3992,7 @@
         <v>277</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -4125,7 +4125,7 @@
         <v>115</v>
       </c>
       <c r="D118" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E118">
         <v>2</v>

</xml_diff>

<commit_message>
Atualização automática: rac (11/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="380">
   <si>
     <t>matricula</t>
   </si>
@@ -200,9 +200,6 @@
     <t>P7036368-01</t>
   </si>
   <si>
-    <t>2641010-3</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -699,9 +696,6 @@
   </si>
   <si>
     <t>PROPELLER ASSEMBLY</t>
-  </si>
-  <si>
-    <t>AXLE FITTING</t>
   </si>
   <si>
     <t>ALTERNATOR</t>
@@ -1563,16 +1557,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2122,7 +2116,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2153,7 +2147,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2170,7 +2164,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2187,7 +2181,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2204,7 +2198,7 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2221,7 +2215,7 @@
         <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2238,7 +2232,7 @@
         <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2255,7 +2249,7 @@
         <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -2272,7 +2266,7 @@
         <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -2289,7 +2283,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2306,7 +2300,7 @@
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2323,7 +2317,7 @@
         <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2340,7 +2334,7 @@
         <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2357,7 +2351,7 @@
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2374,7 +2368,7 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2382,7 +2376,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
         <v>38</v>
@@ -2391,7 +2385,7 @@
         <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2399,16 +2393,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2416,16 +2410,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
         <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2433,16 +2427,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2450,16 +2444,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2467,16 +2461,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2484,16 +2478,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
         <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D22" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2501,16 +2495,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
         <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2518,16 +2512,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2535,16 +2529,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2552,16 +2546,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
         <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2569,36 +2563,36 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
         <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2612,7 +2606,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2629,7 +2623,7 @@
         <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2646,7 +2640,7 @@
         <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2663,7 +2657,7 @@
         <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2680,7 +2674,7 @@
         <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2697,58 +2691,58 @@
         <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2756,16 +2750,16 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -2773,16 +2767,16 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -2790,84 +2784,84 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C41" t="s">
         <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E43">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -2875,36 +2869,36 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C46" t="s">
         <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2918,7 +2912,7 @@
         <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2935,7 +2929,7 @@
         <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2952,7 +2946,7 @@
         <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2969,7 +2963,7 @@
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -2986,7 +2980,7 @@
         <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -3003,7 +2997,7 @@
         <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3020,24 +3014,24 @@
         <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E54">
         <v>4</v>
@@ -3045,16 +3039,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B55" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E55">
         <v>4</v>
@@ -3071,7 +3065,7 @@
         <v>84</v>
       </c>
       <c r="D56" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E56">
         <v>4</v>
@@ -3079,33 +3073,33 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>85</v>
       </c>
       <c r="D57" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E57">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D58" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3113,16 +3107,16 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D59" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -3130,7 +3124,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
         <v>39</v>
@@ -3139,7 +3133,7 @@
         <v>86</v>
       </c>
       <c r="D60" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3147,16 +3141,16 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D61" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -3164,16 +3158,16 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B62" t="s">
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D62" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3181,7 +3175,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
@@ -3190,7 +3184,7 @@
         <v>87</v>
       </c>
       <c r="D63" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -3198,16 +3192,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
       </c>
       <c r="C64" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D64" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -3215,7 +3209,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
@@ -3224,7 +3218,7 @@
         <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3232,16 +3226,16 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B66" t="s">
         <v>39</v>
       </c>
       <c r="C66" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3249,7 +3243,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
@@ -3258,24 +3252,24 @@
         <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D68" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3283,16 +3277,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D69" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3300,7 +3294,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B70" t="s">
         <v>39</v>
@@ -3309,7 +3303,7 @@
         <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3317,16 +3311,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D71" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3334,33 +3328,33 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
         <v>39</v>
       </c>
       <c r="C72" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D73" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3368,33 +3362,33 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
         <v>91</v>
       </c>
       <c r="D74" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E74">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
         <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D75" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3402,16 +3396,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B76" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D76" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E76">
         <v>1</v>
@@ -3419,16 +3413,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>92</v>
       </c>
       <c r="D77" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3436,16 +3430,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D78" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3453,27 +3447,27 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B79" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E79">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C80" t="s">
         <v>93</v>
@@ -3482,21 +3476,21 @@
         <v>258</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
         <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D81" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3504,7 +3498,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
@@ -3513,7 +3507,7 @@
         <v>94</v>
       </c>
       <c r="D82" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3521,16 +3515,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3538,7 +3532,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
@@ -3547,7 +3541,7 @@
         <v>95</v>
       </c>
       <c r="D84" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3555,16 +3549,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D85" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3572,7 +3566,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
@@ -3581,7 +3575,7 @@
         <v>96</v>
       </c>
       <c r="D86" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3589,16 +3583,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D87" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3606,7 +3600,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
@@ -3615,7 +3609,7 @@
         <v>97</v>
       </c>
       <c r="D88" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3623,16 +3617,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D89" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3640,7 +3634,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
@@ -3649,7 +3643,7 @@
         <v>98</v>
       </c>
       <c r="D90" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3657,16 +3651,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D91" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3674,7 +3668,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
@@ -3683,7 +3677,7 @@
         <v>99</v>
       </c>
       <c r="D92" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3691,16 +3685,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D93" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3708,16 +3702,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B94" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
         <v>100</v>
       </c>
       <c r="D94" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3725,16 +3719,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D95" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3742,16 +3736,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B96" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C96" t="s">
         <v>101</v>
       </c>
       <c r="D96" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3759,16 +3753,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B97" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D97" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3776,16 +3770,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B98" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C98" t="s">
         <v>102</v>
       </c>
       <c r="D98" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3802,7 +3796,7 @@
         <v>103</v>
       </c>
       <c r="D99" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3819,7 +3813,7 @@
         <v>104</v>
       </c>
       <c r="D100" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3836,7 +3830,7 @@
         <v>105</v>
       </c>
       <c r="D101" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3853,7 +3847,7 @@
         <v>106</v>
       </c>
       <c r="D102" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3870,7 +3864,7 @@
         <v>107</v>
       </c>
       <c r="D103" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3887,7 +3881,7 @@
         <v>108</v>
       </c>
       <c r="D104" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3904,32 +3898,32 @@
         <v>109</v>
       </c>
       <c r="D105" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E105">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D106" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E106">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
@@ -3938,24 +3932,24 @@
         <v>110</v>
       </c>
       <c r="D107" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E107">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D108" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -3963,16 +3957,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B109" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D109" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -3980,16 +3974,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C110" t="s">
         <v>111</v>
       </c>
       <c r="D110" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -3997,16 +3991,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D111" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4014,16 +4008,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B112" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4031,16 +4025,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B113" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C113" t="s">
         <v>112</v>
       </c>
       <c r="D113" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4048,16 +4042,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D114" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4065,7 +4059,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
@@ -4074,7 +4068,7 @@
         <v>113</v>
       </c>
       <c r="D115" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4082,24 +4076,24 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D116" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4108,10 +4102,10 @@
         <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -4125,7 +4119,7 @@
         <v>115</v>
       </c>
       <c r="D118" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4142,7 +4136,7 @@
         <v>116</v>
       </c>
       <c r="D119" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4159,10 +4153,10 @@
         <v>117</v>
       </c>
       <c r="D120" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4176,24 +4170,24 @@
         <v>118</v>
       </c>
       <c r="D121" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D122" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E122">
         <v>5</v>
@@ -4201,7 +4195,7 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
@@ -4210,10 +4204,10 @@
         <v>119</v>
       </c>
       <c r="D123" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E123">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4227,10 +4221,10 @@
         <v>120</v>
       </c>
       <c r="D124" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E124">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4244,10 +4238,10 @@
         <v>121</v>
       </c>
       <c r="D125" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E125">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4261,24 +4255,24 @@
         <v>122</v>
       </c>
       <c r="D126" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E126">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D127" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E127">
         <v>30</v>
@@ -4295,24 +4289,24 @@
         <v>123</v>
       </c>
       <c r="D128" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E128">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C129" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D129" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4320,16 +4314,16 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B130" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C130" t="s">
         <v>124</v>
       </c>
       <c r="D130" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4346,7 +4340,7 @@
         <v>125</v>
       </c>
       <c r="D131" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4363,7 +4357,7 @@
         <v>126</v>
       </c>
       <c r="D132" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4380,7 +4374,7 @@
         <v>127</v>
       </c>
       <c r="D133" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4397,7 +4391,7 @@
         <v>128</v>
       </c>
       <c r="D134" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4414,7 +4408,7 @@
         <v>129</v>
       </c>
       <c r="D135" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4431,7 +4425,7 @@
         <v>130</v>
       </c>
       <c r="D136" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4448,7 +4442,7 @@
         <v>131</v>
       </c>
       <c r="D137" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4465,7 +4459,7 @@
         <v>132</v>
       </c>
       <c r="D138" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4482,7 +4476,7 @@
         <v>133</v>
       </c>
       <c r="D139" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4499,7 +4493,7 @@
         <v>134</v>
       </c>
       <c r="D140" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4516,7 +4510,7 @@
         <v>135</v>
       </c>
       <c r="D141" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4533,7 +4527,7 @@
         <v>136</v>
       </c>
       <c r="D142" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4550,7 +4544,7 @@
         <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4567,7 +4561,7 @@
         <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4584,7 +4578,7 @@
         <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4601,7 +4595,7 @@
         <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4618,7 +4612,7 @@
         <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4635,7 +4629,7 @@
         <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4652,7 +4646,7 @@
         <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4669,7 +4663,7 @@
         <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4686,7 +4680,7 @@
         <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4703,7 +4697,7 @@
         <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4720,7 +4714,7 @@
         <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4737,7 +4731,7 @@
         <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4754,7 +4748,7 @@
         <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4771,7 +4765,7 @@
         <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4788,7 +4782,7 @@
         <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4805,7 +4799,7 @@
         <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4822,10 +4816,10 @@
         <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>318</v>
+        <v>301</v>
       </c>
       <c r="E159">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4839,7 +4833,7 @@
         <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
       <c r="E160">
         <v>2</v>
@@ -4856,7 +4850,7 @@
         <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E161">
         <v>2</v>
@@ -4873,7 +4867,7 @@
         <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4890,7 +4884,7 @@
         <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4907,10 +4901,10 @@
         <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E164">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4924,10 +4918,10 @@
         <v>159</v>
       </c>
       <c r="D165" t="s">
-        <v>323</v>
+        <v>286</v>
       </c>
       <c r="E165">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4941,10 +4935,10 @@
         <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>288</v>
+        <v>322</v>
       </c>
       <c r="E166">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -4958,7 +4952,7 @@
         <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E167">
         <v>8</v>
@@ -4975,10 +4969,10 @@
         <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E168">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -4992,27 +4986,27 @@
         <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E169">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C170" t="s">
         <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E170">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5026,7 +5020,7 @@
         <v>165</v>
       </c>
       <c r="D171" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5043,7 +5037,7 @@
         <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5060,7 +5054,7 @@
         <v>167</v>
       </c>
       <c r="D173" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5077,7 +5071,7 @@
         <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5094,7 +5088,7 @@
         <v>169</v>
       </c>
       <c r="D175" t="s">
-        <v>332</v>
+        <v>242</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5111,7 +5105,7 @@
         <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>244</v>
+        <v>331</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5128,7 +5122,7 @@
         <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5145,7 +5139,7 @@
         <v>172</v>
       </c>
       <c r="D178" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5162,7 +5156,7 @@
         <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5179,7 +5173,7 @@
         <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5196,7 +5190,7 @@
         <v>175</v>
       </c>
       <c r="D181" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5213,7 +5207,7 @@
         <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5230,7 +5224,7 @@
         <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5247,7 +5241,7 @@
         <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5264,7 +5258,7 @@
         <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5281,7 +5275,7 @@
         <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5298,7 +5292,7 @@
         <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5315,7 +5309,7 @@
         <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5332,7 +5326,7 @@
         <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5349,7 +5343,7 @@
         <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5366,7 +5360,7 @@
         <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5383,7 +5377,7 @@
         <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5400,7 +5394,7 @@
         <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5417,7 +5411,7 @@
         <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5434,7 +5428,7 @@
         <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5451,7 +5445,7 @@
         <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5468,7 +5462,7 @@
         <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5485,7 +5479,7 @@
         <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>354</v>
+        <v>311</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5502,7 +5496,7 @@
         <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>313</v>
+        <v>353</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5519,7 +5513,7 @@
         <v>194</v>
       </c>
       <c r="D200" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5536,10 +5530,10 @@
         <v>195</v>
       </c>
       <c r="D201" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E201">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5553,7 +5547,7 @@
         <v>196</v>
       </c>
       <c r="D202" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5570,7 +5564,7 @@
         <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5587,7 +5581,7 @@
         <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5604,7 +5598,7 @@
         <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5621,7 +5615,7 @@
         <v>200</v>
       </c>
       <c r="D206" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5638,7 +5632,7 @@
         <v>201</v>
       </c>
       <c r="D207" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5655,7 +5649,7 @@
         <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5672,7 +5666,7 @@
         <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5689,7 +5683,7 @@
         <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5706,7 +5700,7 @@
         <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5723,10 +5717,10 @@
         <v>206</v>
       </c>
       <c r="D212" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E212">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5740,7 +5734,7 @@
         <v>207</v>
       </c>
       <c r="D213" t="s">
-        <v>367</v>
+        <v>242</v>
       </c>
       <c r="E213">
         <v>3</v>
@@ -5757,10 +5751,10 @@
         <v>208</v>
       </c>
       <c r="D214" t="s">
-        <v>244</v>
+        <v>366</v>
       </c>
       <c r="E214">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5774,7 +5768,7 @@
         <v>209</v>
       </c>
       <c r="D215" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E215">
         <v>4</v>
@@ -5791,7 +5785,7 @@
         <v>210</v>
       </c>
       <c r="D216" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E216">
         <v>4</v>
@@ -5808,7 +5802,7 @@
         <v>211</v>
       </c>
       <c r="D217" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E217">
         <v>4</v>
@@ -5825,7 +5819,7 @@
         <v>212</v>
       </c>
       <c r="D218" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -5842,10 +5836,10 @@
         <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E219">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5859,7 +5853,7 @@
         <v>214</v>
       </c>
       <c r="D220" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E220">
         <v>5</v>
@@ -5876,10 +5870,10 @@
         <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E221">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5893,10 +5887,10 @@
         <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E222">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5910,10 +5904,10 @@
         <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E223">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5927,7 +5921,7 @@
         <v>218</v>
       </c>
       <c r="D224" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E224">
         <v>10</v>
@@ -5944,10 +5938,10 @@
         <v>219</v>
       </c>
       <c r="D225" t="s">
-        <v>377</v>
+        <v>244</v>
       </c>
       <c r="E225">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5961,7 +5955,7 @@
         <v>220</v>
       </c>
       <c r="D226" t="s">
-        <v>246</v>
+        <v>376</v>
       </c>
       <c r="E226">
         <v>12</v>
@@ -5978,10 +5972,10 @@
         <v>221</v>
       </c>
       <c r="D227" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E227">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -5995,10 +5989,10 @@
         <v>222</v>
       </c>
       <c r="D228" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E228">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6012,26 +6006,9 @@
         <v>223</v>
       </c>
       <c r="D229" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E229">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="230" spans="1:5">
-      <c r="A230" t="s">
-        <v>13</v>
-      </c>
-      <c r="B230" t="s">
-        <v>40</v>
-      </c>
-      <c r="C230" t="s">
-        <v>224</v>
-      </c>
-      <c r="D230" t="s">
-        <v>381</v>
-      </c>
-      <c r="E230">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (11/08/2026 15:01)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -41,52 +41,52 @@
     <t>2731</t>
   </si>
   <si>
+    <t>2728</t>
+  </si>
+  <si>
+    <t>2732</t>
+  </si>
+  <si>
+    <t>2730</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>2726</t>
+  </si>
+  <si>
+    <t>2702</t>
+  </si>
+  <si>
+    <t>2703</t>
+  </si>
+  <si>
+    <t>2704</t>
+  </si>
+  <si>
+    <t>2708</t>
+  </si>
+  <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>2719</t>
+  </si>
+  <si>
+    <t>2720</t>
+  </si>
+  <si>
+    <t>2722</t>
+  </si>
+  <si>
+    <t>2723</t>
+  </si>
+  <si>
+    <t>2727</t>
+  </si>
+  <si>
     <t>2729</t>
-  </si>
-  <si>
-    <t>2728</t>
-  </si>
-  <si>
-    <t>2732</t>
-  </si>
-  <si>
-    <t>2730</t>
-  </si>
-  <si>
-    <t>2734</t>
-  </si>
-  <si>
-    <t>2726</t>
-  </si>
-  <si>
-    <t>2702</t>
-  </si>
-  <si>
-    <t>2703</t>
-  </si>
-  <si>
-    <t>2704</t>
-  </si>
-  <si>
-    <t>2708</t>
-  </si>
-  <si>
-    <t>2709</t>
-  </si>
-  <si>
-    <t>2719</t>
-  </si>
-  <si>
-    <t>2720</t>
-  </si>
-  <si>
-    <t>2722</t>
-  </si>
-  <si>
-    <t>2723</t>
-  </si>
-  <si>
-    <t>2727</t>
   </si>
   <si>
     <t>2733</t>
@@ -1557,16 +1557,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1574,19 +1574,19 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E5">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F5">
-        <v>46</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1603,10 +1603,10 @@
         <v>54</v>
       </c>
       <c r="E6">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="F6">
-        <v>11</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1623,10 +1623,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="F7">
-        <v>111</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1634,7 +1634,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1643,10 +1643,10 @@
         <v>54</v>
       </c>
       <c r="E8">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="F8">
-        <v>166</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1654,19 +1654,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E9">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>228</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1674,7 +1674,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>51</v>
@@ -1694,7 +1694,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
         <v>51</v>
@@ -1714,7 +1714,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1734,7 +1734,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1754,7 +1754,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1774,7 +1774,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1794,7 +1794,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1814,7 +1814,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1834,7 +1834,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
@@ -1854,7 +1854,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -2155,7 +2155,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
@@ -2172,7 +2172,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>39</v>
@@ -2189,7 +2189,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
         <v>39</v>
@@ -2206,7 +2206,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
@@ -2223,7 +2223,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -2257,7 +2257,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
         <v>40</v>
@@ -2291,7 +2291,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
@@ -2308,7 +2308,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
@@ -2342,7 +2342,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
@@ -2359,7 +2359,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
         <v>40</v>
@@ -2376,7 +2376,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
         <v>38</v>
@@ -2393,7 +2393,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
         <v>39</v>
@@ -2410,7 +2410,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
         <v>39</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
@@ -2444,7 +2444,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
         <v>38</v>
@@ -2461,7 +2461,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
         <v>39</v>
@@ -2478,7 +2478,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
         <v>39</v>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
         <v>38</v>
@@ -2512,7 +2512,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
         <v>39</v>
@@ -2529,7 +2529,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>40</v>
@@ -2546,7 +2546,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
         <v>38</v>
@@ -2563,7 +2563,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
@@ -2580,7 +2580,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
@@ -2597,7 +2597,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>38</v>
@@ -2614,7 +2614,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B30" t="s">
         <v>38</v>
@@ -2631,7 +2631,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B31" t="s">
         <v>38</v>
@@ -2648,7 +2648,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B32" t="s">
         <v>38</v>
@@ -2665,7 +2665,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B33" t="s">
         <v>38</v>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
         <v>39</v>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
@@ -2733,7 +2733,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
         <v>40</v>
@@ -2750,7 +2750,7 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
         <v>38</v>
@@ -2767,7 +2767,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
         <v>39</v>
@@ -2784,7 +2784,7 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
         <v>40</v>
@@ -2801,7 +2801,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B41" t="s">
         <v>38</v>
@@ -2818,7 +2818,7 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s">
         <v>39</v>
@@ -2835,7 +2835,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B43" t="s">
         <v>40</v>
@@ -2852,7 +2852,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
         <v>38</v>
@@ -2869,7 +2869,7 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
         <v>40</v>
@@ -2886,7 +2886,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
         <v>38</v>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
         <v>38</v>
@@ -2920,7 +2920,7 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
         <v>38</v>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
         <v>38</v>
@@ -2954,7 +2954,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
         <v>38</v>
@@ -2971,7 +2971,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B51" t="s">
         <v>38</v>
@@ -2988,7 +2988,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
         <v>38</v>
@@ -3005,7 +3005,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
@@ -3022,7 +3022,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
         <v>40</v>
@@ -3039,7 +3039,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B55" t="s">
         <v>38</v>
@@ -3056,7 +3056,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B56" t="s">
         <v>38</v>
@@ -3073,7 +3073,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B57" t="s">
         <v>39</v>
@@ -3090,7 +3090,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B58" t="s">
         <v>39</v>
@@ -3107,7 +3107,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
@@ -3124,7 +3124,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B60" t="s">
         <v>39</v>
@@ -3141,7 +3141,7 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B61" t="s">
         <v>39</v>
@@ -3158,7 +3158,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
         <v>39</v>
@@ -3175,7 +3175,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B63" t="s">
         <v>39</v>
@@ -3192,7 +3192,7 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B65" t="s">
         <v>39</v>
@@ -3226,7 +3226,7 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
         <v>39</v>
@@ -3243,7 +3243,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B67" t="s">
         <v>39</v>
@@ -3260,7 +3260,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
@@ -3277,7 +3277,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>39</v>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B70" t="s">
         <v>39</v>
@@ -3311,7 +3311,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B71" t="s">
         <v>39</v>
@@ -3328,7 +3328,7 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
         <v>39</v>
@@ -3345,7 +3345,7 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
         <v>40</v>
@@ -3362,7 +3362,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B74" t="s">
         <v>39</v>
@@ -3379,7 +3379,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
         <v>39</v>
@@ -3396,7 +3396,7 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
         <v>40</v>
@@ -3413,7 +3413,7 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B77" t="s">
         <v>39</v>
@@ -3430,7 +3430,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
@@ -3447,7 +3447,7 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>40</v>
@@ -3464,7 +3464,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
         <v>39</v>
@@ -3481,7 +3481,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
         <v>39</v>
@@ -3498,7 +3498,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
@@ -3515,7 +3515,7 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
@@ -3532,7 +3532,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
@@ -3549,7 +3549,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
@@ -3566,7 +3566,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
@@ -3617,7 +3617,7 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
@@ -3634,7 +3634,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
@@ -3651,7 +3651,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
@@ -3668,7 +3668,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
@@ -3685,7 +3685,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
         <v>40</v>
@@ -3702,7 +3702,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
@@ -3719,7 +3719,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
         <v>40</v>
@@ -3736,7 +3736,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
@@ -3753,7 +3753,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
         <v>40</v>
@@ -3770,7 +3770,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B98" t="s">
         <v>39</v>
@@ -3787,7 +3787,7 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B99" t="s">
         <v>39</v>
@@ -3804,7 +3804,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B100" t="s">
         <v>39</v>
@@ -3821,7 +3821,7 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B101" t="s">
         <v>39</v>
@@ -3838,7 +3838,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B102" t="s">
         <v>39</v>
@@ -3855,7 +3855,7 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B103" t="s">
         <v>39</v>
@@ -3872,7 +3872,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
@@ -3889,7 +3889,7 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B105" t="s">
         <v>39</v>
@@ -3906,7 +3906,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
@@ -3923,7 +3923,7 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
@@ -3940,7 +3940,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
@@ -3957,7 +3957,7 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
         <v>40</v>
@@ -3974,7 +3974,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
@@ -3991,7 +3991,7 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
         <v>40</v>
@@ -4025,7 +4025,7 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
@@ -4042,7 +4042,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
@@ -4059,7 +4059,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B115" t="s">
         <v>39</v>
@@ -4076,7 +4076,7 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
@@ -4093,7 +4093,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4110,7 +4110,7 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
@@ -4127,7 +4127,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
@@ -4144,7 +4144,7 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B120" t="s">
         <v>39</v>
@@ -4161,7 +4161,7 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B121" t="s">
         <v>39</v>
@@ -4178,7 +4178,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
@@ -4195,7 +4195,7 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
@@ -4212,7 +4212,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
@@ -4229,7 +4229,7 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B126" t="s">
         <v>39</v>
@@ -4263,7 +4263,7 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
@@ -4280,7 +4280,7 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B128" t="s">
         <v>39</v>
@@ -4297,7 +4297,7 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B129" t="s">
         <v>40</v>
@@ -4314,7 +4314,7 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B130" t="s">
         <v>39</v>
@@ -4331,7 +4331,7 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
@@ -4348,7 +4348,7 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B132" t="s">
         <v>39</v>
@@ -4365,7 +4365,7 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B133" t="s">
         <v>39</v>
@@ -4382,7 +4382,7 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B134" t="s">
         <v>39</v>
@@ -4399,7 +4399,7 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B135" t="s">
         <v>39</v>
@@ -4416,7 +4416,7 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B136" t="s">
         <v>39</v>
@@ -4433,7 +4433,7 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B137" t="s">
         <v>39</v>
@@ -4450,7 +4450,7 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B138" t="s">
         <v>39</v>
@@ -4467,7 +4467,7 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B139" t="s">
         <v>39</v>
@@ -4484,7 +4484,7 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B140" t="s">
         <v>39</v>
@@ -4501,7 +4501,7 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B141" t="s">
         <v>39</v>
@@ -4518,7 +4518,7 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B142" t="s">
         <v>39</v>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B143" t="s">
         <v>39</v>
@@ -4552,7 +4552,7 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B144" t="s">
         <v>39</v>
@@ -4569,7 +4569,7 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B145" t="s">
         <v>39</v>
@@ -4586,7 +4586,7 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B146" t="s">
         <v>39</v>
@@ -4603,7 +4603,7 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B147" t="s">
         <v>39</v>
@@ -4620,7 +4620,7 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B148" t="s">
         <v>39</v>
@@ -4637,7 +4637,7 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B149" t="s">
         <v>39</v>
@@ -4654,7 +4654,7 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B150" t="s">
         <v>39</v>
@@ -4671,7 +4671,7 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B151" t="s">
         <v>39</v>
@@ -4688,7 +4688,7 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B152" t="s">
         <v>39</v>
@@ -4705,7 +4705,7 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B153" t="s">
         <v>39</v>
@@ -4722,7 +4722,7 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B154" t="s">
         <v>39</v>
@@ -4739,7 +4739,7 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B155" t="s">
         <v>39</v>
@@ -4756,7 +4756,7 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B156" t="s">
         <v>39</v>
@@ -4773,7 +4773,7 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B157" t="s">
         <v>39</v>
@@ -4790,7 +4790,7 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B158" t="s">
         <v>39</v>
@@ -4807,7 +4807,7 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B159" t="s">
         <v>39</v>
@@ -4824,7 +4824,7 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B160" t="s">
         <v>39</v>
@@ -4841,7 +4841,7 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B161" t="s">
         <v>39</v>
@@ -4858,7 +4858,7 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B162" t="s">
         <v>39</v>
@@ -4875,7 +4875,7 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B163" t="s">
         <v>39</v>
@@ -4892,7 +4892,7 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B164" t="s">
         <v>39</v>
@@ -4909,7 +4909,7 @@
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B165" t="s">
         <v>39</v>
@@ -4926,7 +4926,7 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B166" t="s">
         <v>39</v>
@@ -4943,7 +4943,7 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B167" t="s">
         <v>39</v>
@@ -4960,7 +4960,7 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B168" t="s">
         <v>39</v>
@@ -4977,7 +4977,7 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B169" t="s">
         <v>39</v>
@@ -4994,7 +4994,7 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B170" t="s">
         <v>40</v>
@@ -5011,7 +5011,7 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B171" t="s">
         <v>40</v>
@@ -5028,7 +5028,7 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B172" t="s">
         <v>40</v>
@@ -5045,7 +5045,7 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B173" t="s">
         <v>40</v>
@@ -5062,7 +5062,7 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B174" t="s">
         <v>40</v>
@@ -5079,7 +5079,7 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B175" t="s">
         <v>40</v>
@@ -5096,7 +5096,7 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B176" t="s">
         <v>40</v>
@@ -5113,7 +5113,7 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B177" t="s">
         <v>40</v>
@@ -5130,7 +5130,7 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B178" t="s">
         <v>40</v>
@@ -5147,7 +5147,7 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B179" t="s">
         <v>40</v>
@@ -5164,7 +5164,7 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B180" t="s">
         <v>40</v>
@@ -5181,7 +5181,7 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B181" t="s">
         <v>40</v>
@@ -5198,7 +5198,7 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B182" t="s">
         <v>40</v>
@@ -5215,7 +5215,7 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B183" t="s">
         <v>40</v>
@@ -5232,7 +5232,7 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B184" t="s">
         <v>40</v>
@@ -5249,7 +5249,7 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B185" t="s">
         <v>40</v>
@@ -5266,7 +5266,7 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B186" t="s">
         <v>40</v>
@@ -5283,7 +5283,7 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B187" t="s">
         <v>40</v>
@@ -5300,7 +5300,7 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B188" t="s">
         <v>40</v>
@@ -5317,7 +5317,7 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B189" t="s">
         <v>40</v>
@@ -5334,7 +5334,7 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B190" t="s">
         <v>40</v>
@@ -5351,7 +5351,7 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B191" t="s">
         <v>40</v>
@@ -5368,7 +5368,7 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B192" t="s">
         <v>40</v>
@@ -5385,7 +5385,7 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B193" t="s">
         <v>40</v>
@@ -5402,7 +5402,7 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B194" t="s">
         <v>40</v>
@@ -5419,7 +5419,7 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B195" t="s">
         <v>40</v>
@@ -5436,7 +5436,7 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B196" t="s">
         <v>40</v>
@@ -5453,7 +5453,7 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B197" t="s">
         <v>40</v>
@@ -5470,7 +5470,7 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B198" t="s">
         <v>40</v>
@@ -5487,7 +5487,7 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B199" t="s">
         <v>40</v>
@@ -5504,7 +5504,7 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B200" t="s">
         <v>40</v>
@@ -5521,7 +5521,7 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B201" t="s">
         <v>40</v>
@@ -5538,7 +5538,7 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B202" t="s">
         <v>40</v>
@@ -5555,7 +5555,7 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B203" t="s">
         <v>40</v>
@@ -5572,7 +5572,7 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B204" t="s">
         <v>40</v>
@@ -5589,7 +5589,7 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B205" t="s">
         <v>40</v>
@@ -5606,7 +5606,7 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B206" t="s">
         <v>40</v>
@@ -5623,7 +5623,7 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B207" t="s">
         <v>40</v>
@@ -5640,7 +5640,7 @@
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B208" t="s">
         <v>40</v>
@@ -5657,7 +5657,7 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B209" t="s">
         <v>40</v>
@@ -5674,7 +5674,7 @@
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B210" t="s">
         <v>40</v>
@@ -5691,7 +5691,7 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B211" t="s">
         <v>40</v>
@@ -5708,7 +5708,7 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B212" t="s">
         <v>40</v>
@@ -5725,7 +5725,7 @@
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B213" t="s">
         <v>40</v>
@@ -5742,7 +5742,7 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B214" t="s">
         <v>40</v>
@@ -5759,7 +5759,7 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B215" t="s">
         <v>40</v>
@@ -5776,7 +5776,7 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B216" t="s">
         <v>40</v>
@@ -5793,7 +5793,7 @@
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B217" t="s">
         <v>40</v>
@@ -5810,7 +5810,7 @@
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B218" t="s">
         <v>40</v>
@@ -5827,7 +5827,7 @@
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B219" t="s">
         <v>40</v>
@@ -5844,7 +5844,7 @@
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B220" t="s">
         <v>40</v>
@@ -5861,7 +5861,7 @@
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B221" t="s">
         <v>40</v>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B222" t="s">
         <v>40</v>
@@ -5895,7 +5895,7 @@
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B223" t="s">
         <v>40</v>
@@ -5912,7 +5912,7 @@
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B224" t="s">
         <v>40</v>
@@ -5929,7 +5929,7 @@
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B225" t="s">
         <v>40</v>
@@ -5946,7 +5946,7 @@
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B226" t="s">
         <v>40</v>
@@ -5963,7 +5963,7 @@
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B227" t="s">
         <v>40</v>
@@ -5980,7 +5980,7 @@
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B228" t="s">
         <v>40</v>
@@ -5997,7 +5997,7 @@
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B229" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Atualização automática: rac (13/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="385">
   <si>
     <t>matricula</t>
   </si>
@@ -383,9 +383,6 @@
     <t>040-0043</t>
   </si>
   <si>
-    <t>1214134-1</t>
-  </si>
-  <si>
     <t>MICROB MONITOR 2</t>
   </si>
   <si>
@@ -882,9 +879,6 @@
   </si>
   <si>
     <t>STROB TUB</t>
-  </si>
-  <si>
-    <t>BELLCRANK ASSY</t>
   </si>
   <si>
     <t>TEST KIT, FUEL, WORK</t>
@@ -1684,10 +1678,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2137,7 +2131,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E235"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2168,7 +2162,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2185,7 +2179,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2202,7 +2196,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2219,7 +2213,7 @@
         <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2236,7 +2230,7 @@
         <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2253,7 +2247,7 @@
         <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2270,7 +2264,7 @@
         <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2287,7 +2281,7 @@
         <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2304,7 +2298,7 @@
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2321,7 +2315,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2338,7 +2332,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2355,7 +2349,7 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2372,7 +2366,7 @@
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2389,7 +2383,7 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2406,7 +2400,7 @@
         <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2423,7 +2417,7 @@
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2440,7 +2434,7 @@
         <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2457,7 +2451,7 @@
         <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -2474,7 +2468,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -2491,7 +2485,7 @@
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2508,7 +2502,7 @@
         <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2525,7 +2519,7 @@
         <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2542,7 +2536,7 @@
         <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2559,7 +2553,7 @@
         <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2576,7 +2570,7 @@
         <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2593,7 +2587,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2610,7 +2604,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2627,7 +2621,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2644,7 +2638,7 @@
         <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2661,7 +2655,7 @@
         <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2678,7 +2672,7 @@
         <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2695,7 +2689,7 @@
         <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2712,7 +2706,7 @@
         <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2729,7 +2723,7 @@
         <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2746,7 +2740,7 @@
         <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2763,7 +2757,7 @@
         <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2780,7 +2774,7 @@
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2797,7 +2791,7 @@
         <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2814,7 +2808,7 @@
         <v>74</v>
       </c>
       <c r="D40" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2831,7 +2825,7 @@
         <v>75</v>
       </c>
       <c r="D41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2848,7 +2842,7 @@
         <v>76</v>
       </c>
       <c r="D42" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2865,7 +2859,7 @@
         <v>77</v>
       </c>
       <c r="D43" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E43">
         <v>2</v>
@@ -2882,7 +2876,7 @@
         <v>77</v>
       </c>
       <c r="D44" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E44">
         <v>3</v>
@@ -2899,7 +2893,7 @@
         <v>77</v>
       </c>
       <c r="D45" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2916,7 +2910,7 @@
         <v>77</v>
       </c>
       <c r="D46" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2933,7 +2927,7 @@
         <v>78</v>
       </c>
       <c r="D47" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2950,7 +2944,7 @@
         <v>78</v>
       </c>
       <c r="D48" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2967,7 +2961,7 @@
         <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -2984,7 +2978,7 @@
         <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -3001,7 +2995,7 @@
         <v>79</v>
       </c>
       <c r="D51" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E51">
         <v>4</v>
@@ -3018,7 +3012,7 @@
         <v>79</v>
       </c>
       <c r="D52" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3035,7 +3029,7 @@
         <v>80</v>
       </c>
       <c r="D53" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -3052,7 +3046,7 @@
         <v>80</v>
       </c>
       <c r="D54" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3069,7 +3063,7 @@
         <v>81</v>
       </c>
       <c r="D55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3086,7 +3080,7 @@
         <v>82</v>
       </c>
       <c r="D56" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3103,7 +3097,7 @@
         <v>83</v>
       </c>
       <c r="D57" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E57">
         <v>2</v>
@@ -3120,7 +3114,7 @@
         <v>84</v>
       </c>
       <c r="D58" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3137,7 +3131,7 @@
         <v>85</v>
       </c>
       <c r="D59" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3154,7 +3148,7 @@
         <v>86</v>
       </c>
       <c r="D60" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3171,7 +3165,7 @@
         <v>87</v>
       </c>
       <c r="D61" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3188,7 +3182,7 @@
         <v>88</v>
       </c>
       <c r="D62" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E62">
         <v>4</v>
@@ -3205,7 +3199,7 @@
         <v>88</v>
       </c>
       <c r="D63" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E63">
         <v>4</v>
@@ -3222,7 +3216,7 @@
         <v>89</v>
       </c>
       <c r="D64" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E64">
         <v>4</v>
@@ -3239,7 +3233,7 @@
         <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E65">
         <v>4</v>
@@ -3256,7 +3250,7 @@
         <v>91</v>
       </c>
       <c r="D66" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3273,7 +3267,7 @@
         <v>91</v>
       </c>
       <c r="D67" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3290,7 +3284,7 @@
         <v>91</v>
       </c>
       <c r="D68" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E68">
         <v>1</v>
@@ -3307,7 +3301,7 @@
         <v>92</v>
       </c>
       <c r="D69" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -3324,7 +3318,7 @@
         <v>92</v>
       </c>
       <c r="D70" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -3341,7 +3335,7 @@
         <v>92</v>
       </c>
       <c r="D71" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3358,7 +3352,7 @@
         <v>93</v>
       </c>
       <c r="D72" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3375,7 +3369,7 @@
         <v>93</v>
       </c>
       <c r="D73" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3392,7 +3386,7 @@
         <v>94</v>
       </c>
       <c r="D74" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3409,7 +3403,7 @@
         <v>94</v>
       </c>
       <c r="D75" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3426,7 +3420,7 @@
         <v>95</v>
       </c>
       <c r="D76" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3443,7 +3437,7 @@
         <v>95</v>
       </c>
       <c r="D77" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3460,7 +3454,7 @@
         <v>95</v>
       </c>
       <c r="D78" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3477,7 +3471,7 @@
         <v>96</v>
       </c>
       <c r="D79" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E79">
         <v>2</v>
@@ -3494,7 +3488,7 @@
         <v>96</v>
       </c>
       <c r="D80" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3511,7 +3505,7 @@
         <v>96</v>
       </c>
       <c r="D81" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E81">
         <v>4</v>
@@ -3528,7 +3522,7 @@
         <v>96</v>
       </c>
       <c r="D82" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -3545,7 +3539,7 @@
         <v>97</v>
       </c>
       <c r="D83" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3562,7 +3556,7 @@
         <v>97</v>
       </c>
       <c r="D84" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3579,7 +3573,7 @@
         <v>97</v>
       </c>
       <c r="D85" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3596,7 +3590,7 @@
         <v>98</v>
       </c>
       <c r="D86" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3613,7 +3607,7 @@
         <v>98</v>
       </c>
       <c r="D87" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3630,7 +3624,7 @@
         <v>98</v>
       </c>
       <c r="D88" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E88">
         <v>2</v>
@@ -3647,7 +3641,7 @@
         <v>99</v>
       </c>
       <c r="D89" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3664,7 +3658,7 @@
         <v>99</v>
       </c>
       <c r="D90" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3681,7 +3675,7 @@
         <v>100</v>
       </c>
       <c r="D91" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3698,7 +3692,7 @@
         <v>100</v>
       </c>
       <c r="D92" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3715,7 +3709,7 @@
         <v>101</v>
       </c>
       <c r="D93" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3732,7 +3726,7 @@
         <v>101</v>
       </c>
       <c r="D94" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3749,7 +3743,7 @@
         <v>102</v>
       </c>
       <c r="D95" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3766,7 +3760,7 @@
         <v>102</v>
       </c>
       <c r="D96" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3783,7 +3777,7 @@
         <v>103</v>
       </c>
       <c r="D97" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3800,7 +3794,7 @@
         <v>103</v>
       </c>
       <c r="D98" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3817,7 +3811,7 @@
         <v>104</v>
       </c>
       <c r="D99" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3834,7 +3828,7 @@
         <v>104</v>
       </c>
       <c r="D100" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3851,7 +3845,7 @@
         <v>105</v>
       </c>
       <c r="D101" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3868,7 +3862,7 @@
         <v>105</v>
       </c>
       <c r="D102" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3885,7 +3879,7 @@
         <v>106</v>
       </c>
       <c r="D103" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3902,7 +3896,7 @@
         <v>106</v>
       </c>
       <c r="D104" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3919,7 +3913,7 @@
         <v>107</v>
       </c>
       <c r="D105" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3936,7 +3930,7 @@
         <v>107</v>
       </c>
       <c r="D106" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3953,7 +3947,7 @@
         <v>108</v>
       </c>
       <c r="D107" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3970,7 +3964,7 @@
         <v>109</v>
       </c>
       <c r="D108" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3987,7 +3981,7 @@
         <v>110</v>
       </c>
       <c r="D109" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -4004,7 +3998,7 @@
         <v>111</v>
       </c>
       <c r="D110" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -4021,7 +4015,7 @@
         <v>112</v>
       </c>
       <c r="D111" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4038,7 +4032,7 @@
         <v>113</v>
       </c>
       <c r="D112" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4055,7 +4049,7 @@
         <v>114</v>
       </c>
       <c r="D113" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4072,7 +4066,7 @@
         <v>114</v>
       </c>
       <c r="D114" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E114">
         <v>1</v>
@@ -4089,7 +4083,7 @@
         <v>115</v>
       </c>
       <c r="D115" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4106,7 +4100,7 @@
         <v>115</v>
       </c>
       <c r="D116" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4123,7 +4117,7 @@
         <v>115</v>
       </c>
       <c r="D117" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4140,7 +4134,7 @@
         <v>116</v>
       </c>
       <c r="D118" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4157,7 +4151,7 @@
         <v>116</v>
       </c>
       <c r="D119" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4174,7 +4168,7 @@
         <v>116</v>
       </c>
       <c r="D120" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4191,7 +4185,7 @@
         <v>117</v>
       </c>
       <c r="D121" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4208,7 +4202,7 @@
         <v>117</v>
       </c>
       <c r="D122" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4225,7 +4219,7 @@
         <v>118</v>
       </c>
       <c r="D123" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4242,7 +4236,7 @@
         <v>118</v>
       </c>
       <c r="D124" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E124">
         <v>4</v>
@@ -4259,7 +4253,7 @@
         <v>119</v>
       </c>
       <c r="D125" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E125">
         <v>2</v>
@@ -4276,7 +4270,7 @@
         <v>120</v>
       </c>
       <c r="D126" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E126">
         <v>2</v>
@@ -4293,7 +4287,7 @@
         <v>121</v>
       </c>
       <c r="D127" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E127">
         <v>2</v>
@@ -4310,24 +4304,24 @@
         <v>122</v>
       </c>
       <c r="D128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E128">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B129" t="s">
         <v>41</v>
       </c>
       <c r="C129" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D129" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="E129">
         <v>5</v>
@@ -4335,7 +4329,7 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
         <v>41</v>
@@ -4344,10 +4338,10 @@
         <v>123</v>
       </c>
       <c r="D130" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E130">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -4361,10 +4355,10 @@
         <v>124</v>
       </c>
       <c r="D131" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E131">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -4378,10 +4372,10 @@
         <v>125</v>
       </c>
       <c r="D132" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E132">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -4395,24 +4389,24 @@
         <v>126</v>
       </c>
       <c r="D133" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E133">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B134" t="s">
         <v>41</v>
       </c>
       <c r="C134" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D134" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E134">
         <v>30</v>
@@ -4429,24 +4423,24 @@
         <v>127</v>
       </c>
       <c r="D135" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E135">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B136" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C136" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D136" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4454,16 +4448,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B137" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C137" t="s">
         <v>128</v>
       </c>
       <c r="D137" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4480,7 +4474,7 @@
         <v>129</v>
       </c>
       <c r="D138" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4497,7 +4491,7 @@
         <v>130</v>
       </c>
       <c r="D139" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4514,7 +4508,7 @@
         <v>131</v>
       </c>
       <c r="D140" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4531,7 +4525,7 @@
         <v>132</v>
       </c>
       <c r="D141" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4548,7 +4542,7 @@
         <v>133</v>
       </c>
       <c r="D142" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4565,7 +4559,7 @@
         <v>134</v>
       </c>
       <c r="D143" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4582,7 +4576,7 @@
         <v>135</v>
       </c>
       <c r="D144" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4599,7 +4593,7 @@
         <v>136</v>
       </c>
       <c r="D145" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4616,7 +4610,7 @@
         <v>137</v>
       </c>
       <c r="D146" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4633,7 +4627,7 @@
         <v>138</v>
       </c>
       <c r="D147" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4650,7 +4644,7 @@
         <v>139</v>
       </c>
       <c r="D148" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4667,7 +4661,7 @@
         <v>140</v>
       </c>
       <c r="D149" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4684,7 +4678,7 @@
         <v>141</v>
       </c>
       <c r="D150" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4701,7 +4695,7 @@
         <v>142</v>
       </c>
       <c r="D151" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4718,7 +4712,7 @@
         <v>143</v>
       </c>
       <c r="D152" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4735,7 +4729,7 @@
         <v>144</v>
       </c>
       <c r="D153" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4752,7 +4746,7 @@
         <v>145</v>
       </c>
       <c r="D154" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4769,7 +4763,7 @@
         <v>146</v>
       </c>
       <c r="D155" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4786,7 +4780,7 @@
         <v>147</v>
       </c>
       <c r="D156" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4803,7 +4797,7 @@
         <v>148</v>
       </c>
       <c r="D157" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4820,7 +4814,7 @@
         <v>149</v>
       </c>
       <c r="D158" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4837,7 +4831,7 @@
         <v>150</v>
       </c>
       <c r="D159" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4854,7 +4848,7 @@
         <v>151</v>
       </c>
       <c r="D160" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4871,7 +4865,7 @@
         <v>152</v>
       </c>
       <c r="D161" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4888,7 +4882,7 @@
         <v>153</v>
       </c>
       <c r="D162" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4905,7 +4899,7 @@
         <v>154</v>
       </c>
       <c r="D163" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4922,7 +4916,7 @@
         <v>155</v>
       </c>
       <c r="D164" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4939,10 +4933,10 @@
         <v>156</v>
       </c>
       <c r="D165" t="s">
-        <v>323</v>
+        <v>306</v>
       </c>
       <c r="E165">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4956,7 +4950,7 @@
         <v>157</v>
       </c>
       <c r="D166" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -4973,7 +4967,7 @@
         <v>158</v>
       </c>
       <c r="D167" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -4990,7 +4984,7 @@
         <v>159</v>
       </c>
       <c r="D168" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -5007,7 +5001,7 @@
         <v>160</v>
       </c>
       <c r="D169" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E169">
         <v>2</v>
@@ -5024,10 +5018,10 @@
         <v>161</v>
       </c>
       <c r="D170" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E170">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5041,10 +5035,10 @@
         <v>162</v>
       </c>
       <c r="D171" t="s">
-        <v>328</v>
+        <v>292</v>
       </c>
       <c r="E171">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5058,10 +5052,10 @@
         <v>163</v>
       </c>
       <c r="D172" t="s">
-        <v>294</v>
+        <v>327</v>
       </c>
       <c r="E172">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5075,7 +5069,7 @@
         <v>164</v>
       </c>
       <c r="D173" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E173">
         <v>8</v>
@@ -5092,10 +5086,10 @@
         <v>165</v>
       </c>
       <c r="D174" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E174">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -5109,27 +5103,27 @@
         <v>166</v>
       </c>
       <c r="D175" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E175">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B176" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C176" t="s">
         <v>167</v>
       </c>
       <c r="D176" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E176">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -5143,7 +5137,7 @@
         <v>168</v>
       </c>
       <c r="D177" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5160,7 +5154,7 @@
         <v>169</v>
       </c>
       <c r="D178" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5177,7 +5171,7 @@
         <v>170</v>
       </c>
       <c r="D179" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5194,7 +5188,7 @@
         <v>171</v>
       </c>
       <c r="D180" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5211,7 +5205,7 @@
         <v>172</v>
       </c>
       <c r="D181" t="s">
-        <v>337</v>
+        <v>250</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5228,7 +5222,7 @@
         <v>173</v>
       </c>
       <c r="D182" t="s">
-        <v>251</v>
+        <v>336</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5245,7 +5239,7 @@
         <v>174</v>
       </c>
       <c r="D183" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5262,7 +5256,7 @@
         <v>175</v>
       </c>
       <c r="D184" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5279,7 +5273,7 @@
         <v>176</v>
       </c>
       <c r="D185" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5296,7 +5290,7 @@
         <v>177</v>
       </c>
       <c r="D186" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5313,7 +5307,7 @@
         <v>178</v>
       </c>
       <c r="D187" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5330,7 +5324,7 @@
         <v>179</v>
       </c>
       <c r="D188" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5347,7 +5341,7 @@
         <v>180</v>
       </c>
       <c r="D189" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5364,7 +5358,7 @@
         <v>181</v>
       </c>
       <c r="D190" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5381,7 +5375,7 @@
         <v>182</v>
       </c>
       <c r="D191" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5398,7 +5392,7 @@
         <v>183</v>
       </c>
       <c r="D192" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5415,7 +5409,7 @@
         <v>184</v>
       </c>
       <c r="D193" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5432,7 +5426,7 @@
         <v>185</v>
       </c>
       <c r="D194" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5449,7 +5443,7 @@
         <v>186</v>
       </c>
       <c r="D195" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5466,7 +5460,7 @@
         <v>187</v>
       </c>
       <c r="D196" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5483,7 +5477,7 @@
         <v>188</v>
       </c>
       <c r="D197" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5500,7 +5494,7 @@
         <v>189</v>
       </c>
       <c r="D198" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5517,7 +5511,7 @@
         <v>190</v>
       </c>
       <c r="D199" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5534,7 +5528,7 @@
         <v>191</v>
       </c>
       <c r="D200" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5551,7 +5545,7 @@
         <v>192</v>
       </c>
       <c r="D201" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5568,7 +5562,7 @@
         <v>193</v>
       </c>
       <c r="D202" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5585,7 +5579,7 @@
         <v>194</v>
       </c>
       <c r="D203" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5602,7 +5596,7 @@
         <v>195</v>
       </c>
       <c r="D204" t="s">
-        <v>359</v>
+        <v>316</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5619,7 +5613,7 @@
         <v>196</v>
       </c>
       <c r="D205" t="s">
-        <v>318</v>
+        <v>358</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5636,7 +5630,7 @@
         <v>197</v>
       </c>
       <c r="D206" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5653,10 +5647,10 @@
         <v>198</v>
       </c>
       <c r="D207" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E207">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5670,7 +5664,7 @@
         <v>199</v>
       </c>
       <c r="D208" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5687,7 +5681,7 @@
         <v>200</v>
       </c>
       <c r="D209" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5704,7 +5698,7 @@
         <v>201</v>
       </c>
       <c r="D210" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5721,7 +5715,7 @@
         <v>202</v>
       </c>
       <c r="D211" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5738,7 +5732,7 @@
         <v>203</v>
       </c>
       <c r="D212" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5755,7 +5749,7 @@
         <v>204</v>
       </c>
       <c r="D213" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5772,7 +5766,7 @@
         <v>205</v>
       </c>
       <c r="D214" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5789,7 +5783,7 @@
         <v>206</v>
       </c>
       <c r="D215" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5806,7 +5800,7 @@
         <v>207</v>
       </c>
       <c r="D216" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5823,7 +5817,7 @@
         <v>208</v>
       </c>
       <c r="D217" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5840,10 +5834,10 @@
         <v>209</v>
       </c>
       <c r="D218" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E218">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5857,7 +5851,7 @@
         <v>210</v>
       </c>
       <c r="D219" t="s">
-        <v>372</v>
+        <v>250</v>
       </c>
       <c r="E219">
         <v>3</v>
@@ -5874,10 +5868,10 @@
         <v>211</v>
       </c>
       <c r="D220" t="s">
-        <v>251</v>
+        <v>371</v>
       </c>
       <c r="E220">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5891,7 +5885,7 @@
         <v>212</v>
       </c>
       <c r="D221" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5908,7 +5902,7 @@
         <v>213</v>
       </c>
       <c r="D222" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5925,7 +5919,7 @@
         <v>214</v>
       </c>
       <c r="D223" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5942,7 +5936,7 @@
         <v>215</v>
       </c>
       <c r="D224" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -5959,10 +5953,10 @@
         <v>216</v>
       </c>
       <c r="D225" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E225">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5976,7 +5970,7 @@
         <v>217</v>
       </c>
       <c r="D226" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E226">
         <v>5</v>
@@ -5993,10 +5987,10 @@
         <v>218</v>
       </c>
       <c r="D227" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6010,10 +6004,10 @@
         <v>219</v>
       </c>
       <c r="D228" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E228">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6027,10 +6021,10 @@
         <v>220</v>
       </c>
       <c r="D229" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E229">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6044,7 +6038,7 @@
         <v>221</v>
       </c>
       <c r="D230" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E230">
         <v>10</v>
@@ -6061,10 +6055,10 @@
         <v>222</v>
       </c>
       <c r="D231" t="s">
-        <v>382</v>
+        <v>252</v>
       </c>
       <c r="E231">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6078,7 +6072,7 @@
         <v>223</v>
       </c>
       <c r="D232" t="s">
-        <v>253</v>
+        <v>381</v>
       </c>
       <c r="E232">
         <v>12</v>
@@ -6095,10 +6089,10 @@
         <v>224</v>
       </c>
       <c r="D233" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E233">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -6112,10 +6106,10 @@
         <v>225</v>
       </c>
       <c r="D234" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E234">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6129,26 +6123,9 @@
         <v>226</v>
       </c>
       <c r="D235" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E235">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="236" spans="1:5">
-      <c r="A236" t="s">
-        <v>15</v>
-      </c>
-      <c r="B236" t="s">
-        <v>42</v>
-      </c>
-      <c r="C236" t="s">
-        <v>227</v>
-      </c>
-      <c r="D236" t="s">
-        <v>386</v>
-      </c>
-      <c r="E236">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (13/08/2026 11:25)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="384">
   <si>
     <t>matricula</t>
   </si>
@@ -243,9 +243,6 @@
   </si>
   <si>
     <t>2641030-1</t>
-  </si>
-  <si>
-    <t>2641032-201</t>
   </si>
   <si>
     <t>AE3663163K0600</t>
@@ -2162,7 +2159,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2179,7 +2176,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2196,7 +2193,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2213,7 +2210,7 @@
         <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2230,7 +2227,7 @@
         <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2247,7 +2244,7 @@
         <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2264,7 +2261,7 @@
         <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2281,7 +2278,7 @@
         <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2298,7 +2295,7 @@
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2315,7 +2312,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2332,7 +2329,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2349,7 +2346,7 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2366,7 +2363,7 @@
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2383,7 +2380,7 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2400,7 +2397,7 @@
         <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2417,7 +2414,7 @@
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2434,7 +2431,7 @@
         <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2451,7 +2448,7 @@
         <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -2468,7 +2465,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -2485,7 +2482,7 @@
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2502,7 +2499,7 @@
         <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2519,7 +2516,7 @@
         <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2536,7 +2533,7 @@
         <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2553,7 +2550,7 @@
         <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2570,7 +2567,7 @@
         <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2587,7 +2584,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2604,7 +2601,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2621,7 +2618,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2638,7 +2635,7 @@
         <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2655,7 +2652,7 @@
         <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2672,7 +2669,7 @@
         <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2689,7 +2686,7 @@
         <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2706,7 +2703,7 @@
         <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2723,7 +2720,7 @@
         <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2740,7 +2737,7 @@
         <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2757,7 +2754,7 @@
         <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2774,7 +2771,7 @@
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2791,7 +2788,7 @@
         <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2808,7 +2805,7 @@
         <v>74</v>
       </c>
       <c r="D40" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2825,7 +2822,7 @@
         <v>75</v>
       </c>
       <c r="D41" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2845,55 +2842,55 @@
         <v>244</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D43" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
         <v>41</v>
       </c>
       <c r="C44" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D44" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -2901,10 +2898,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C46" t="s">
         <v>77</v>
@@ -2918,16 +2915,16 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C47" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2935,27 +2932,27 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C49" t="s">
         <v>78</v>
@@ -2964,49 +2961,49 @@
         <v>246</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C52" t="s">
         <v>79</v>
@@ -3020,27 +3017,27 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C53" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D53" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C54" t="s">
         <v>80</v>
@@ -3049,7 +3046,7 @@
         <v>248</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3168,21 +3165,21 @@
         <v>255</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B62" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C62" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D62" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E62">
         <v>4</v>
@@ -3190,10 +3187,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C63" t="s">
         <v>88</v>
@@ -3224,10 +3221,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C65" t="s">
         <v>90</v>
@@ -3236,21 +3233,21 @@
         <v>258</v>
       </c>
       <c r="E65">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
         <v>41</v>
       </c>
       <c r="C66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -3258,16 +3255,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
         <v>41</v>
       </c>
       <c r="C67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3275,10 +3272,10 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C68" t="s">
         <v>91</v>
@@ -3298,10 +3295,10 @@
         <v>41</v>
       </c>
       <c r="C69" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D69" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -3315,10 +3312,10 @@
         <v>41</v>
       </c>
       <c r="C70" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D70" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -3332,10 +3329,10 @@
         <v>41</v>
       </c>
       <c r="C71" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D71" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3349,10 +3346,10 @@
         <v>41</v>
       </c>
       <c r="C72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D72" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3366,10 +3363,10 @@
         <v>41</v>
       </c>
       <c r="C73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D73" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3383,10 +3380,10 @@
         <v>41</v>
       </c>
       <c r="C74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D74" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3400,10 +3397,10 @@
         <v>41</v>
       </c>
       <c r="C75" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D75" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3417,10 +3414,10 @@
         <v>41</v>
       </c>
       <c r="C76" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D76" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3434,10 +3431,10 @@
         <v>41</v>
       </c>
       <c r="C77" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D77" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3451,10 +3448,10 @@
         <v>41</v>
       </c>
       <c r="C78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D78" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3468,10 +3465,10 @@
         <v>41</v>
       </c>
       <c r="C79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D79" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E79">
         <v>2</v>
@@ -3485,10 +3482,10 @@
         <v>41</v>
       </c>
       <c r="C80" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D80" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3502,10 +3499,10 @@
         <v>41</v>
       </c>
       <c r="C81" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D81" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E81">
         <v>4</v>
@@ -3519,10 +3516,10 @@
         <v>42</v>
       </c>
       <c r="C82" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D82" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -3536,10 +3533,10 @@
         <v>41</v>
       </c>
       <c r="C83" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D83" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3553,10 +3550,10 @@
         <v>41</v>
       </c>
       <c r="C84" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D84" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3570,10 +3567,10 @@
         <v>42</v>
       </c>
       <c r="C85" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D85" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3587,10 +3584,10 @@
         <v>41</v>
       </c>
       <c r="C86" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D86" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3604,10 +3601,10 @@
         <v>41</v>
       </c>
       <c r="C87" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D87" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3621,10 +3618,10 @@
         <v>42</v>
       </c>
       <c r="C88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D88" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E88">
         <v>2</v>
@@ -3638,10 +3635,10 @@
         <v>41</v>
       </c>
       <c r="C89" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D89" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3655,10 +3652,10 @@
         <v>41</v>
       </c>
       <c r="C90" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D90" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3672,10 +3669,10 @@
         <v>41</v>
       </c>
       <c r="C91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D91" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3689,10 +3686,10 @@
         <v>41</v>
       </c>
       <c r="C92" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D92" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3706,10 +3703,10 @@
         <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D93" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3723,10 +3720,10 @@
         <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D94" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3740,10 +3737,10 @@
         <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D95" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3757,10 +3754,10 @@
         <v>41</v>
       </c>
       <c r="C96" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D96" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3774,10 +3771,10 @@
         <v>41</v>
       </c>
       <c r="C97" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D97" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3791,10 +3788,10 @@
         <v>41</v>
       </c>
       <c r="C98" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D98" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3808,10 +3805,10 @@
         <v>41</v>
       </c>
       <c r="C99" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D99" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3825,10 +3822,10 @@
         <v>41</v>
       </c>
       <c r="C100" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D100" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3842,10 +3839,10 @@
         <v>41</v>
       </c>
       <c r="C101" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D101" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3859,10 +3856,10 @@
         <v>42</v>
       </c>
       <c r="C102" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D102" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3876,10 +3873,10 @@
         <v>41</v>
       </c>
       <c r="C103" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D103" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3893,10 +3890,10 @@
         <v>42</v>
       </c>
       <c r="C104" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D104" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3910,10 +3907,10 @@
         <v>41</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D105" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3927,10 +3924,10 @@
         <v>42</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D106" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3944,10 +3941,10 @@
         <v>41</v>
       </c>
       <c r="C107" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D107" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3961,10 +3958,10 @@
         <v>41</v>
       </c>
       <c r="C108" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D108" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3978,10 +3975,10 @@
         <v>41</v>
       </c>
       <c r="C109" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D109" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3995,10 +3992,10 @@
         <v>41</v>
       </c>
       <c r="C110" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D110" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -4012,10 +4009,10 @@
         <v>41</v>
       </c>
       <c r="C111" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D111" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4029,10 +4026,10 @@
         <v>41</v>
       </c>
       <c r="C112" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D112" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4046,10 +4043,10 @@
         <v>41</v>
       </c>
       <c r="C113" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D113" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4063,10 +4060,10 @@
         <v>41</v>
       </c>
       <c r="C114" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D114" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E114">
         <v>1</v>
@@ -4080,10 +4077,10 @@
         <v>41</v>
       </c>
       <c r="C115" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D115" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4097,10 +4094,10 @@
         <v>41</v>
       </c>
       <c r="C116" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D116" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4114,10 +4111,10 @@
         <v>42</v>
       </c>
       <c r="C117" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4131,10 +4128,10 @@
         <v>41</v>
       </c>
       <c r="C118" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D118" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4148,10 +4145,10 @@
         <v>41</v>
       </c>
       <c r="C119" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D119" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4165,10 +4162,10 @@
         <v>42</v>
       </c>
       <c r="C120" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D120" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4182,10 +4179,10 @@
         <v>41</v>
       </c>
       <c r="C121" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D121" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4199,10 +4196,10 @@
         <v>41</v>
       </c>
       <c r="C122" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D122" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4216,10 +4213,10 @@
         <v>41</v>
       </c>
       <c r="C123" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D123" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4233,10 +4230,10 @@
         <v>41</v>
       </c>
       <c r="C124" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E124">
         <v>4</v>
@@ -4250,10 +4247,10 @@
         <v>41</v>
       </c>
       <c r="C125" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D125" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E125">
         <v>2</v>
@@ -4267,10 +4264,10 @@
         <v>41</v>
       </c>
       <c r="C126" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D126" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E126">
         <v>2</v>
@@ -4284,10 +4281,10 @@
         <v>41</v>
       </c>
       <c r="C127" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D127" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E127">
         <v>2</v>
@@ -4301,10 +4298,10 @@
         <v>41</v>
       </c>
       <c r="C128" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D128" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E128">
         <v>5</v>
@@ -4318,10 +4315,10 @@
         <v>41</v>
       </c>
       <c r="C129" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D129" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E129">
         <v>5</v>
@@ -4335,10 +4332,10 @@
         <v>41</v>
       </c>
       <c r="C130" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D130" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E130">
         <v>7</v>
@@ -4352,10 +4349,10 @@
         <v>41</v>
       </c>
       <c r="C131" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D131" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E131">
         <v>8</v>
@@ -4369,10 +4366,10 @@
         <v>41</v>
       </c>
       <c r="C132" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D132" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E132">
         <v>10</v>
@@ -4386,10 +4383,10 @@
         <v>41</v>
       </c>
       <c r="C133" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D133" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E133">
         <v>30</v>
@@ -4403,10 +4400,10 @@
         <v>41</v>
       </c>
       <c r="C134" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D134" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E134">
         <v>30</v>
@@ -4420,10 +4417,10 @@
         <v>41</v>
       </c>
       <c r="C135" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D135" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4437,10 +4434,10 @@
         <v>42</v>
       </c>
       <c r="C136" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D136" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4454,10 +4451,10 @@
         <v>41</v>
       </c>
       <c r="C137" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D137" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4471,10 +4468,10 @@
         <v>41</v>
       </c>
       <c r="C138" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4488,10 +4485,10 @@
         <v>41</v>
       </c>
       <c r="C139" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D139" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4505,10 +4502,10 @@
         <v>41</v>
       </c>
       <c r="C140" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D140" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4522,10 +4519,10 @@
         <v>41</v>
       </c>
       <c r="C141" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D141" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4539,10 +4536,10 @@
         <v>41</v>
       </c>
       <c r="C142" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D142" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4556,10 +4553,10 @@
         <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D143" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4573,10 +4570,10 @@
         <v>41</v>
       </c>
       <c r="C144" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D144" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4590,10 +4587,10 @@
         <v>41</v>
       </c>
       <c r="C145" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D145" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4607,10 +4604,10 @@
         <v>41</v>
       </c>
       <c r="C146" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D146" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4624,10 +4621,10 @@
         <v>41</v>
       </c>
       <c r="C147" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D147" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4641,10 +4638,10 @@
         <v>41</v>
       </c>
       <c r="C148" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D148" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4658,10 +4655,10 @@
         <v>41</v>
       </c>
       <c r="C149" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D149" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4675,10 +4672,10 @@
         <v>41</v>
       </c>
       <c r="C150" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D150" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4692,10 +4689,10 @@
         <v>41</v>
       </c>
       <c r="C151" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D151" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4709,10 +4706,10 @@
         <v>41</v>
       </c>
       <c r="C152" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D152" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4726,10 +4723,10 @@
         <v>41</v>
       </c>
       <c r="C153" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D153" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4743,10 +4740,10 @@
         <v>41</v>
       </c>
       <c r="C154" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D154" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4760,10 +4757,10 @@
         <v>41</v>
       </c>
       <c r="C155" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D155" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4777,10 +4774,10 @@
         <v>41</v>
       </c>
       <c r="C156" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D156" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4794,10 +4791,10 @@
         <v>41</v>
       </c>
       <c r="C157" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D157" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4811,10 +4808,10 @@
         <v>41</v>
       </c>
       <c r="C158" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D158" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4828,10 +4825,10 @@
         <v>41</v>
       </c>
       <c r="C159" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4845,10 +4842,10 @@
         <v>41</v>
       </c>
       <c r="C160" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4862,10 +4859,10 @@
         <v>41</v>
       </c>
       <c r="C161" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D161" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4879,10 +4876,10 @@
         <v>41</v>
       </c>
       <c r="C162" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D162" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4896,10 +4893,10 @@
         <v>41</v>
       </c>
       <c r="C163" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D163" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4913,10 +4910,10 @@
         <v>41</v>
       </c>
       <c r="C164" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D164" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4930,10 +4927,10 @@
         <v>41</v>
       </c>
       <c r="C165" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D165" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -4947,10 +4944,10 @@
         <v>41</v>
       </c>
       <c r="C166" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D166" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -4964,10 +4961,10 @@
         <v>41</v>
       </c>
       <c r="C167" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D167" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -4981,10 +4978,10 @@
         <v>41</v>
       </c>
       <c r="C168" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D168" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -4998,10 +4995,10 @@
         <v>41</v>
       </c>
       <c r="C169" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D169" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E169">
         <v>2</v>
@@ -5015,10 +5012,10 @@
         <v>41</v>
       </c>
       <c r="C170" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D170" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E170">
         <v>3</v>
@@ -5032,10 +5029,10 @@
         <v>41</v>
       </c>
       <c r="C171" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D171" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E171">
         <v>5</v>
@@ -5049,10 +5046,10 @@
         <v>41</v>
       </c>
       <c r="C172" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D172" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E172">
         <v>8</v>
@@ -5066,10 +5063,10 @@
         <v>41</v>
       </c>
       <c r="C173" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D173" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E173">
         <v>8</v>
@@ -5083,10 +5080,10 @@
         <v>41</v>
       </c>
       <c r="C174" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D174" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E174">
         <v>10</v>
@@ -5100,10 +5097,10 @@
         <v>41</v>
       </c>
       <c r="C175" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D175" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E175">
         <v>15</v>
@@ -5117,10 +5114,10 @@
         <v>42</v>
       </c>
       <c r="C176" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D176" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5134,10 +5131,10 @@
         <v>42</v>
       </c>
       <c r="C177" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D177" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5151,10 +5148,10 @@
         <v>42</v>
       </c>
       <c r="C178" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D178" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5168,10 +5165,10 @@
         <v>42</v>
       </c>
       <c r="C179" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D179" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5185,10 +5182,10 @@
         <v>42</v>
       </c>
       <c r="C180" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D180" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5202,10 +5199,10 @@
         <v>42</v>
       </c>
       <c r="C181" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D181" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5219,10 +5216,10 @@
         <v>42</v>
       </c>
       <c r="C182" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D182" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5236,10 +5233,10 @@
         <v>42</v>
       </c>
       <c r="C183" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D183" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5253,10 +5250,10 @@
         <v>42</v>
       </c>
       <c r="C184" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D184" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5270,10 +5267,10 @@
         <v>42</v>
       </c>
       <c r="C185" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D185" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5287,10 +5284,10 @@
         <v>42</v>
       </c>
       <c r="C186" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D186" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5304,10 +5301,10 @@
         <v>42</v>
       </c>
       <c r="C187" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D187" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5321,10 +5318,10 @@
         <v>42</v>
       </c>
       <c r="C188" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D188" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5338,10 +5335,10 @@
         <v>42</v>
       </c>
       <c r="C189" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D189" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5355,10 +5352,10 @@
         <v>42</v>
       </c>
       <c r="C190" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D190" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5372,10 +5369,10 @@
         <v>42</v>
       </c>
       <c r="C191" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D191" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5389,10 +5386,10 @@
         <v>42</v>
       </c>
       <c r="C192" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D192" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5406,10 +5403,10 @@
         <v>42</v>
       </c>
       <c r="C193" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D193" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5423,10 +5420,10 @@
         <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D194" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5440,10 +5437,10 @@
         <v>42</v>
       </c>
       <c r="C195" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D195" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5457,10 +5454,10 @@
         <v>42</v>
       </c>
       <c r="C196" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D196" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5474,10 +5471,10 @@
         <v>42</v>
       </c>
       <c r="C197" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D197" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5491,10 +5488,10 @@
         <v>42</v>
       </c>
       <c r="C198" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D198" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5508,10 +5505,10 @@
         <v>42</v>
       </c>
       <c r="C199" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D199" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5525,10 +5522,10 @@
         <v>42</v>
       </c>
       <c r="C200" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D200" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5542,10 +5539,10 @@
         <v>42</v>
       </c>
       <c r="C201" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D201" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5559,10 +5556,10 @@
         <v>42</v>
       </c>
       <c r="C202" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D202" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5576,10 +5573,10 @@
         <v>42</v>
       </c>
       <c r="C203" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D203" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5593,10 +5590,10 @@
         <v>42</v>
       </c>
       <c r="C204" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D204" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5610,10 +5607,10 @@
         <v>42</v>
       </c>
       <c r="C205" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D205" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5627,10 +5624,10 @@
         <v>42</v>
       </c>
       <c r="C206" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D206" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5644,10 +5641,10 @@
         <v>42</v>
       </c>
       <c r="C207" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D207" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5661,10 +5658,10 @@
         <v>42</v>
       </c>
       <c r="C208" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D208" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5678,10 +5675,10 @@
         <v>42</v>
       </c>
       <c r="C209" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D209" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5695,10 +5692,10 @@
         <v>42</v>
       </c>
       <c r="C210" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D210" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5712,10 +5709,10 @@
         <v>42</v>
       </c>
       <c r="C211" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D211" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5729,10 +5726,10 @@
         <v>42</v>
       </c>
       <c r="C212" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D212" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5746,10 +5743,10 @@
         <v>42</v>
       </c>
       <c r="C213" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D213" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5763,10 +5760,10 @@
         <v>42</v>
       </c>
       <c r="C214" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D214" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5780,10 +5777,10 @@
         <v>42</v>
       </c>
       <c r="C215" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D215" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5797,10 +5794,10 @@
         <v>42</v>
       </c>
       <c r="C216" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D216" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5814,10 +5811,10 @@
         <v>42</v>
       </c>
       <c r="C217" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D217" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5831,10 +5828,10 @@
         <v>42</v>
       </c>
       <c r="C218" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D218" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E218">
         <v>3</v>
@@ -5848,10 +5845,10 @@
         <v>42</v>
       </c>
       <c r="C219" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D219" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E219">
         <v>3</v>
@@ -5865,10 +5862,10 @@
         <v>42</v>
       </c>
       <c r="C220" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D220" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E220">
         <v>4</v>
@@ -5882,10 +5879,10 @@
         <v>42</v>
       </c>
       <c r="C221" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D221" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5899,10 +5896,10 @@
         <v>42</v>
       </c>
       <c r="C222" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D222" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5916,10 +5913,10 @@
         <v>42</v>
       </c>
       <c r="C223" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D223" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5933,10 +5930,10 @@
         <v>42</v>
       </c>
       <c r="C224" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D224" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -5950,10 +5947,10 @@
         <v>42</v>
       </c>
       <c r="C225" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D225" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E225">
         <v>5</v>
@@ -5967,10 +5964,10 @@
         <v>42</v>
       </c>
       <c r="C226" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D226" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E226">
         <v>5</v>
@@ -5984,10 +5981,10 @@
         <v>42</v>
       </c>
       <c r="C227" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D227" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E227">
         <v>6</v>
@@ -6001,10 +5998,10 @@
         <v>42</v>
       </c>
       <c r="C228" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D228" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E228">
         <v>8</v>
@@ -6018,10 +6015,10 @@
         <v>42</v>
       </c>
       <c r="C229" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D229" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E229">
         <v>10</v>
@@ -6035,10 +6032,10 @@
         <v>42</v>
       </c>
       <c r="C230" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D230" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E230">
         <v>10</v>
@@ -6052,10 +6049,10 @@
         <v>42</v>
       </c>
       <c r="C231" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D231" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E231">
         <v>12</v>
@@ -6069,10 +6066,10 @@
         <v>42</v>
       </c>
       <c r="C232" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D232" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E232">
         <v>12</v>
@@ -6086,10 +6083,10 @@
         <v>42</v>
       </c>
       <c r="C233" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D233" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E233">
         <v>14</v>
@@ -6103,10 +6100,10 @@
         <v>42</v>
       </c>
       <c r="C234" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D234" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E234">
         <v>15</v>
@@ -6120,10 +6117,10 @@
         <v>42</v>
       </c>
       <c r="C235" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D235" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E235">
         <v>20</v>

</xml_diff>

<commit_message>
Atualização automática: rac (13/08/2026 16:58)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -212,6 +212,9 @@
     <t>C611505-0201</t>
   </si>
   <si>
+    <t>2600100-7</t>
+  </si>
+  <si>
     <t>2643007-1</t>
   </si>
   <si>
@@ -290,9 +293,6 @@
     <t>1H75-21</t>
   </si>
   <si>
-    <t>2600100-7</t>
-  </si>
-  <si>
     <t>2698010-7</t>
   </si>
   <si>
@@ -716,6 +716,9 @@
     <t>ALTERNATOR</t>
   </si>
   <si>
+    <t>LINE ASSY-PROP</t>
+  </si>
+  <si>
     <t>SHIMMY DAMP AS</t>
   </si>
   <si>
@@ -792,9 +795,6 @@
   </si>
   <si>
     <t>PRESSURE REGULATOR</t>
-  </si>
-  <si>
-    <t>LINE ASSY-PROP</t>
   </si>
   <si>
     <t>PASSENGER DOOR - LOW</t>
@@ -2558,7 +2558,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
         <v>41</v>
@@ -2575,7 +2575,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
         <v>41</v>
@@ -2592,16 +2592,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2609,10 +2609,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C29" t="s">
         <v>66</v>
@@ -2626,16 +2626,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2649,10 +2649,10 @@
         <v>41</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2660,10 +2660,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
         <v>67</v>
@@ -2677,16 +2677,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2694,10 +2694,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C34" t="s">
         <v>68</v>
@@ -2706,21 +2706,21 @@
         <v>236</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2728,16 +2728,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2751,10 +2751,10 @@
         <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D37" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2762,19 +2762,19 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D38" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2785,10 +2785,10 @@
         <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2802,10 +2802,10 @@
         <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2819,10 +2819,10 @@
         <v>37</v>
       </c>
       <c r="C41" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2836,55 +2836,55 @@
         <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C45" t="s">
         <v>76</v>
@@ -2893,7 +2893,7 @@
         <v>244</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2915,7 +2915,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" t="s">
         <v>41</v>
@@ -2927,15 +2927,15 @@
         <v>245</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C48" t="s">
         <v>77</v>
@@ -2944,21 +2944,21 @@
         <v>245</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2966,10 +2966,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C50" t="s">
         <v>78</v>
@@ -2978,15 +2978,15 @@
         <v>246</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
         <v>78</v>
@@ -3000,27 +3000,27 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D52" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C53" t="s">
         <v>79</v>
@@ -3029,38 +3029,38 @@
         <v>247</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D54" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B55" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C55" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3074,10 +3074,10 @@
         <v>37</v>
       </c>
       <c r="C56" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D56" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3085,19 +3085,19 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B57" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C57" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D57" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3108,10 +3108,10 @@
         <v>37</v>
       </c>
       <c r="C58" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3125,10 +3125,10 @@
         <v>37</v>
       </c>
       <c r="C59" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3142,10 +3142,10 @@
         <v>37</v>
       </c>
       <c r="C60" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3159,30 +3159,30 @@
         <v>37</v>
       </c>
       <c r="C61" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E61">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C62" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E62">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3193,13 +3193,13 @@
         <v>37</v>
       </c>
       <c r="C63" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3210,64 +3210,64 @@
         <v>37</v>
       </c>
       <c r="C64" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D64" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E64">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C65" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B66" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3278,13 +3278,13 @@
         <v>37</v>
       </c>
       <c r="C68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E68">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -5202,7 +5202,7 @@
         <v>171</v>
       </c>
       <c r="D181" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5848,7 +5848,7 @@
         <v>209</v>
       </c>
       <c r="D219" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E219">
         <v>3</v>
@@ -6052,7 +6052,7 @@
         <v>221</v>
       </c>
       <c r="D231" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E231">
         <v>12</v>

</xml_diff>

<commit_message>
Atualização automática: rac (14/08/2026 12:58)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="392">
   <si>
     <t>matricula</t>
   </si>
@@ -695,6 +695,18 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>3107453-01</t>
+  </si>
+  <si>
+    <t>3026812</t>
+  </si>
+  <si>
+    <t>3013411</t>
+  </si>
+  <si>
+    <t>C662504-0101</t>
+  </si>
+  <si>
     <t>FUEL CONTROL UNIT</t>
   </si>
   <si>
@@ -1167,6 +1179,18 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>HOUSING</t>
+  </si>
+  <si>
+    <t>DISK AND HUB,TURBIN</t>
+  </si>
+  <si>
+    <t>DISK AND HUB,COMPRE</t>
+  </si>
+  <si>
+    <t>GAGE VOLT AMME</t>
   </si>
 </sst>
 </file>
@@ -1555,10 +1579,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1615,10 +1639,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1849,16 +1873,16 @@
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
         <v>53</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2128,7 +2152,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E235"/>
+  <dimension ref="A1:E241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2159,7 +2183,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2167,16 +2191,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2184,16 +2208,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2201,16 +2225,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2218,16 +2242,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2235,16 +2259,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2261,7 +2285,7 @@
         <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2278,7 +2302,7 @@
         <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2295,7 +2319,7 @@
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2312,7 +2336,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2329,7 +2353,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2346,7 +2370,7 @@
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2363,7 +2387,7 @@
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2380,7 +2404,7 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2397,7 +2421,7 @@
         <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2414,7 +2438,7 @@
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2431,7 +2455,7 @@
         <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2448,7 +2472,7 @@
         <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -2465,7 +2489,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -2482,7 +2506,7 @@
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2499,7 +2523,7 @@
         <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2516,7 +2540,7 @@
         <v>64</v>
       </c>
       <c r="D23" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2533,7 +2557,7 @@
         <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2550,7 +2574,7 @@
         <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2567,7 +2591,7 @@
         <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2584,7 +2608,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2601,7 +2625,7 @@
         <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2618,7 +2642,7 @@
         <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2635,7 +2659,7 @@
         <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2652,7 +2676,7 @@
         <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2669,7 +2693,7 @@
         <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2686,7 +2710,7 @@
         <v>67</v>
       </c>
       <c r="D33" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2703,7 +2727,7 @@
         <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2720,7 +2744,7 @@
         <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2737,7 +2761,7 @@
         <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2754,7 +2778,7 @@
         <v>69</v>
       </c>
       <c r="D37" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2771,7 +2795,7 @@
         <v>69</v>
       </c>
       <c r="D38" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -2788,7 +2812,7 @@
         <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2796,7 +2820,7 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B40" t="s">
         <v>37</v>
@@ -2805,7 +2829,7 @@
         <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2819,10 +2843,10 @@
         <v>37</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D41" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2836,10 +2860,10 @@
         <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2853,10 +2877,10 @@
         <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2870,10 +2894,10 @@
         <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2887,10 +2911,10 @@
         <v>37</v>
       </c>
       <c r="C45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2904,35 +2928,35 @@
         <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C47" t="s">
         <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B48" t="s">
         <v>41</v>
@@ -2941,24 +2965,24 @@
         <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C49" t="s">
         <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -2966,16 +2990,16 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D50" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -2983,16 +3007,16 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C51" t="s">
         <v>78</v>
       </c>
       <c r="D51" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -3000,84 +3024,84 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B52" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C52" t="s">
         <v>78</v>
       </c>
       <c r="D52" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C53" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D53" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C54" t="s">
         <v>79</v>
       </c>
       <c r="D54" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C55" t="s">
         <v>79</v>
       </c>
       <c r="D55" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E55">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3085,36 +3109,36 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C57" t="s">
         <v>80</v>
       </c>
       <c r="D57" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B58" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D58" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3125,10 +3149,10 @@
         <v>37</v>
       </c>
       <c r="C59" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D59" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3142,10 +3166,10 @@
         <v>37</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D60" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3159,10 +3183,10 @@
         <v>37</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D61" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3176,10 +3200,10 @@
         <v>37</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D62" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3193,10 +3217,10 @@
         <v>37</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3210,10 +3234,10 @@
         <v>37</v>
       </c>
       <c r="C64" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D64" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3227,27 +3251,27 @@
         <v>37</v>
       </c>
       <c r="C65" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D65" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E65">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C66" t="s">
         <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E66">
         <v>4</v>
@@ -3255,16 +3279,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B67" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C67" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D67" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E67">
         <v>4</v>
@@ -3278,10 +3302,10 @@
         <v>37</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D68" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E68">
         <v>4</v>
@@ -3289,24 +3313,24 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C69" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E69">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
         <v>41</v>
@@ -3315,7 +3339,7 @@
         <v>91</v>
       </c>
       <c r="D70" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -3323,7 +3347,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B71" t="s">
         <v>41</v>
@@ -3332,7 +3356,7 @@
         <v>91</v>
       </c>
       <c r="D71" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3340,16 +3364,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
         <v>41</v>
       </c>
       <c r="C72" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D72" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3357,7 +3381,7 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B73" t="s">
         <v>41</v>
@@ -3366,7 +3390,7 @@
         <v>92</v>
       </c>
       <c r="D73" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3374,16 +3398,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
         <v>41</v>
       </c>
       <c r="C74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D74" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3391,7 +3415,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
         <v>41</v>
@@ -3400,7 +3424,7 @@
         <v>93</v>
       </c>
       <c r="D75" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3408,24 +3432,24 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
         <v>41</v>
       </c>
       <c r="C76" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D76" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
         <v>41</v>
@@ -3434,7 +3458,7 @@
         <v>94</v>
       </c>
       <c r="D77" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -3442,7 +3466,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
         <v>41</v>
@@ -3451,7 +3475,7 @@
         <v>94</v>
       </c>
       <c r="D78" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -3459,16 +3483,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
         <v>41</v>
       </c>
       <c r="C79" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D79" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E79">
         <v>2</v>
@@ -3476,7 +3500,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
         <v>41</v>
@@ -3485,7 +3509,7 @@
         <v>95</v>
       </c>
       <c r="D80" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E80">
         <v>2</v>
@@ -3493,7 +3517,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
         <v>41</v>
@@ -3502,24 +3526,24 @@
         <v>95</v>
       </c>
       <c r="D81" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E81">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
         <v>95</v>
       </c>
       <c r="D82" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -3527,24 +3551,24 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B83" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C83" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D83" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
         <v>41</v>
@@ -3553,7 +3577,7 @@
         <v>96</v>
       </c>
       <c r="D84" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3561,16 +3585,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
         <v>96</v>
       </c>
       <c r="D85" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3578,16 +3602,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C86" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D86" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3595,7 +3619,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
         <v>41</v>
@@ -3604,7 +3628,7 @@
         <v>97</v>
       </c>
       <c r="D87" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3612,41 +3636,41 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C88" t="s">
         <v>97</v>
       </c>
       <c r="D88" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B89" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D89" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
         <v>41</v>
@@ -3655,7 +3679,7 @@
         <v>98</v>
       </c>
       <c r="D90" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3663,16 +3687,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B91" t="s">
         <v>41</v>
       </c>
       <c r="C91" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D91" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3680,7 +3704,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
         <v>41</v>
@@ -3689,7 +3713,7 @@
         <v>99</v>
       </c>
       <c r="D92" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3697,16 +3721,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B93" t="s">
         <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D93" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3714,7 +3738,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
         <v>41</v>
@@ -3723,7 +3747,7 @@
         <v>100</v>
       </c>
       <c r="D94" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3731,16 +3755,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B95" t="s">
         <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D95" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3748,7 +3772,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
         <v>41</v>
@@ -3757,7 +3781,7 @@
         <v>101</v>
       </c>
       <c r="D96" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3765,16 +3789,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B97" t="s">
         <v>41</v>
       </c>
       <c r="C97" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D97" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3782,7 +3806,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
         <v>41</v>
@@ -3791,7 +3815,7 @@
         <v>102</v>
       </c>
       <c r="D98" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3799,16 +3823,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B99" t="s">
         <v>41</v>
       </c>
       <c r="C99" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D99" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3816,7 +3840,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B100" t="s">
         <v>41</v>
@@ -3825,7 +3849,7 @@
         <v>103</v>
       </c>
       <c r="D100" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3833,16 +3857,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B101" t="s">
         <v>41</v>
       </c>
       <c r="C101" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D101" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3850,16 +3874,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C102" t="s">
         <v>104</v>
       </c>
       <c r="D102" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3867,16 +3891,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C103" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3884,16 +3908,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B104" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C104" t="s">
         <v>105</v>
       </c>
       <c r="D104" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3901,16 +3925,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B105" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C105" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D105" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3918,16 +3942,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B106" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C106" t="s">
         <v>106</v>
       </c>
       <c r="D106" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3935,16 +3959,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B107" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C107" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D107" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3958,10 +3982,10 @@
         <v>41</v>
       </c>
       <c r="C108" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D108" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -3975,10 +3999,10 @@
         <v>41</v>
       </c>
       <c r="C109" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D109" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3992,10 +4016,10 @@
         <v>41</v>
       </c>
       <c r="C110" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D110" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -4009,10 +4033,10 @@
         <v>41</v>
       </c>
       <c r="C111" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4026,10 +4050,10 @@
         <v>41</v>
       </c>
       <c r="C112" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4043,18 +4067,18 @@
         <v>41</v>
       </c>
       <c r="C113" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D113" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E113">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
         <v>41</v>
@@ -4063,32 +4087,32 @@
         <v>113</v>
       </c>
       <c r="D114" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
         <v>41</v>
       </c>
       <c r="C115" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D115" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B116" t="s">
         <v>41</v>
@@ -4097,7 +4121,7 @@
         <v>114</v>
       </c>
       <c r="D116" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4105,16 +4129,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C117" t="s">
         <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4122,16 +4146,16 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B118" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C118" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4139,7 +4163,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B119" t="s">
         <v>41</v>
@@ -4148,7 +4172,7 @@
         <v>115</v>
       </c>
       <c r="D119" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4156,16 +4180,16 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C120" t="s">
         <v>115</v>
       </c>
       <c r="D120" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4173,16 +4197,16 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B121" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C121" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D121" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4190,7 +4214,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
         <v>41</v>
@@ -4199,7 +4223,7 @@
         <v>116</v>
       </c>
       <c r="D122" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4207,16 +4231,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B123" t="s">
         <v>41</v>
       </c>
       <c r="C123" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D123" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4224,7 +4248,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
         <v>41</v>
@@ -4233,27 +4257,27 @@
         <v>117</v>
       </c>
       <c r="D124" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E124">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B125" t="s">
         <v>41</v>
       </c>
       <c r="C125" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D125" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4264,10 +4288,10 @@
         <v>41</v>
       </c>
       <c r="C126" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D126" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="E126">
         <v>2</v>
@@ -4281,10 +4305,10 @@
         <v>41</v>
       </c>
       <c r="C127" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D127" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E127">
         <v>2</v>
@@ -4298,18 +4322,18 @@
         <v>41</v>
       </c>
       <c r="C128" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D128" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E128">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
         <v>41</v>
@@ -4318,7 +4342,7 @@
         <v>121</v>
       </c>
       <c r="D129" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E129">
         <v>5</v>
@@ -4326,19 +4350,19 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
         <v>41</v>
       </c>
       <c r="C130" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D130" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E130">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -4349,13 +4373,13 @@
         <v>41</v>
       </c>
       <c r="C131" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D131" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E131">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -4366,13 +4390,13 @@
         <v>41</v>
       </c>
       <c r="C132" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D132" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E132">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -4383,18 +4407,18 @@
         <v>41</v>
       </c>
       <c r="C133" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D133" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E133">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
         <v>41</v>
@@ -4403,7 +4427,7 @@
         <v>125</v>
       </c>
       <c r="D134" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E134">
         <v>30</v>
@@ -4417,27 +4441,27 @@
         <v>41</v>
       </c>
       <c r="C135" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D135" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E135">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B136" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C136" t="s">
         <v>126</v>
       </c>
       <c r="D136" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4445,16 +4469,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B137" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C137" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D137" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4468,10 +4492,10 @@
         <v>41</v>
       </c>
       <c r="C138" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D138" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4485,10 +4509,10 @@
         <v>41</v>
       </c>
       <c r="C139" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D139" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4502,10 +4526,10 @@
         <v>41</v>
       </c>
       <c r="C140" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D140" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4519,10 +4543,10 @@
         <v>41</v>
       </c>
       <c r="C141" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D141" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4536,10 +4560,10 @@
         <v>41</v>
       </c>
       <c r="C142" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D142" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c 